<commit_message>
[Update] Key layout is changed.
</commit_message>
<xml_diff>
--- a/img/keymap.xlsx
+++ b/img/keymap.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1685" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1684" uniqueCount="210">
   <si>
     <t xml:space="preserve">標準</t>
   </si>
@@ -429,78 +429,132 @@
     <t xml:space="preserve">Del</t>
   </si>
   <si>
+    <t xml:space="preserve">C+→</t>
+  </si>
+  <si>
     <t xml:space="preserve">PgUp</t>
   </si>
   <si>
+    <t xml:space="preserve">S+F1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S+F2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S+F4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S+F5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S+F6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S+F7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S+F8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S+F9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S+F10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S+F11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S+F12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PgDn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">””←</t>
+  </si>
+  <si>
+    <t xml:space="preserve">()←</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[]←</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{}←</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+v</t>
+  </si>
+  <si>
+    <t xml:space="preserve">End</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+←</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Num</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mouse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;&gt;←</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Space修飾</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(Space or F13) &amp; 無変換 修飾</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S+↑</t>
+  </si>
+  <si>
     <t xml:space="preserve">S+→</t>
   </si>
   <si>
-    <t xml:space="preserve">C+a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C+s</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C+d</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C+f</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C+y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Home</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C+g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PgDn</t>
-  </si>
-  <si>
     <t xml:space="preserve">S+Home</t>
   </si>
   <si>
     <t xml:space="preserve">S+←</t>
   </si>
   <si>
-    <t xml:space="preserve">C+z</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C+x</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C+c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C+v</t>
-  </si>
-  <si>
-    <t xml:space="preserve">End</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Num</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mouse</t>
+    <t xml:space="preserve">S+↓</t>
   </si>
   <si>
     <t xml:space="preserve">S+End</t>
   </si>
   <si>
-    <t xml:space="preserve">Space修飾</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(Space or F13) &amp; 無変換 修飾</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S+↑</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S+↓</t>
-  </si>
-  <si>
     <t xml:space="preserve">頻度マップ</t>
   </si>
   <si>
@@ -546,12 +600,39 @@
     <t xml:space="preserve">Space &amp; F13 修飾</t>
   </si>
   <si>
+    <t xml:space="preserve">SC+→</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+Home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+End</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SC+←</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> (F14 or 変換 or 無変換) 修飾</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Layer1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">＼</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shiftt</t>
+  </si>
+  <si>
     <t xml:space="preserve">/ 修飾   C+k,C+{}</t>
   </si>
   <si>
-    <t xml:space="preserve">C+→</t>
-  </si>
-  <si>
     <t xml:space="preserve">C+q</t>
   </si>
   <si>
@@ -564,73 +645,13 @@
     <t xml:space="preserve">C+p</t>
   </si>
   <si>
-    <t xml:space="preserve">C+Home</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C+←</t>
-  </si>
-  <si>
     <t xml:space="preserve">C+k</t>
   </si>
   <si>
-    <t xml:space="preserve">C+End</t>
-  </si>
-  <si>
     <t xml:space="preserve">C+b</t>
   </si>
   <si>
     <t xml:space="preserve">C+n</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> (F14 or 変換 or 無変換) 修飾</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Layer1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S+F1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S+F2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S+F4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S+F5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S+F6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S+F7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S+F8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S+F9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S+F10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S+F11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S+F12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">＼</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shiftt</t>
   </si>
 </sst>
 </file>
@@ -729,6 +750,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFB2B2B2"/>
+        <bgColor rgb="FFCCCCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFBBE33D"/>
         <bgColor rgb="FF81D41A"/>
       </patternFill>
@@ -737,12 +764,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF729FCF"/>
         <bgColor rgb="FF808080"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFB2B2B2"/>
-        <bgColor rgb="FFCCCCCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -864,7 +885,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -941,7 +962,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -949,19 +978,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2128,18 +2153,42 @@
       <c r="N18" s="6"/>
       <c r="O18" s="6"/>
       <c r="Q18" s="7"/>
-      <c r="R18" s="7"/>
-      <c r="S18" s="7"/>
-      <c r="T18" s="7"/>
-      <c r="U18" s="7"/>
-      <c r="V18" s="6"/>
-      <c r="W18" s="6"/>
-      <c r="X18" s="6"/>
-      <c r="Y18" s="7"/>
-      <c r="Z18" s="6"/>
-      <c r="AA18" s="6"/>
-      <c r="AB18" s="6"/>
-      <c r="AC18" s="6"/>
+      <c r="R18" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="S18" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="T18" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="U18" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="V18" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="W18" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="X18" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="Y18" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="Z18" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="AA18" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="AB18" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="AC18" s="6" t="s">
+        <v>128</v>
+      </c>
       <c r="AD18" s="6"/>
       <c r="AE18" s="6"/>
     </row>
@@ -2174,56 +2223,78 @@
       <c r="J19" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="K19" s="7" t="s">
-        <v>41</v>
+      <c r="K19" s="6" t="s">
+        <v>135</v>
       </c>
       <c r="L19" s="14" t="s">
         <v>21</v>
       </c>
       <c r="M19" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N19" s="6"/>
       <c r="O19" s="6"/>
       <c r="Q19" s="7"/>
-      <c r="R19" s="7"/>
-      <c r="S19" s="7"/>
-      <c r="T19" s="7"/>
-      <c r="U19" s="7"/>
-      <c r="V19" s="6"/>
-      <c r="W19" s="6"/>
-      <c r="X19" s="6"/>
-      <c r="Y19" s="7"/>
-      <c r="Z19" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="AA19" s="6"/>
-      <c r="AB19" s="6"/>
-      <c r="AC19" s="6"/>
+      <c r="R19" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="S19" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="T19" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="U19" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="V19" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="W19" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="X19" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="Y19" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="Z19" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="AA19" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="AB19" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="AC19" s="19" t="s">
+        <v>147</v>
+      </c>
       <c r="AD19" s="6"/>
       <c r="AE19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="19" t="s">
+      <c r="A20" s="20" t="s">
         <v>90</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="H20" s="9" t="s">
         <v>40</v>
@@ -2238,32 +2309,50 @@
         <v>21</v>
       </c>
       <c r="L20" s="14" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="M20" s="14" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="N20" s="6"/>
       <c r="O20" s="6"/>
       <c r="Q20" s="7"/>
-      <c r="R20" s="7"/>
-      <c r="S20" s="7"/>
-      <c r="T20" s="7"/>
-      <c r="U20" s="9"/>
-      <c r="V20" s="6"/>
+      <c r="R20" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="S20" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="T20" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="U20" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="V20" s="14" t="s">
+        <v>71</v>
+      </c>
       <c r="W20" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="X20" s="9" t="s">
-        <v>146</v>
-      </c>
-      <c r="Y20" s="7"/>
+        <v>72</v>
+      </c>
+      <c r="X20" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="Y20" s="14" t="s">
+        <v>157</v>
+      </c>
       <c r="Z20" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="AA20" s="6"/>
-      <c r="AB20" s="6"/>
-      <c r="AC20" s="6"/>
+        <v>158</v>
+      </c>
+      <c r="AA20" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="AB20" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="AC20" s="16" t="s">
+        <v>159</v>
+      </c>
       <c r="AD20" s="6"/>
       <c r="AE20" s="6"/>
     </row>
@@ -2272,31 +2361,31 @@
         <v>43</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>8</v>
+        <v>165</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="J21" s="14" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="K21" s="6"/>
       <c r="L21" s="6"/>
@@ -2305,21 +2394,37 @@
       </c>
       <c r="N21" s="6"/>
       <c r="O21" s="6"/>
-      <c r="Q21" s="7"/>
-      <c r="R21" s="7"/>
-      <c r="S21" s="7"/>
-      <c r="T21" s="7"/>
-      <c r="U21" s="6"/>
-      <c r="V21" s="7"/>
+      <c r="Q21" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="R21" s="14"/>
+      <c r="S21" s="14"/>
+      <c r="T21" s="14"/>
+      <c r="U21" s="14"/>
+      <c r="V21" s="14" t="s">
+        <v>76</v>
+      </c>
       <c r="W21" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="X21" s="6"/>
-      <c r="Y21" s="7"/>
-      <c r="Z21" s="6"/>
-      <c r="AA21" s="6"/>
-      <c r="AB21" s="6"/>
-      <c r="AC21" s="6"/>
+        <v>113</v>
+      </c>
+      <c r="X21" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y21" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="Z21" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="AA21" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB21" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="AC21" s="6" t="s">
+        <v>43</v>
+      </c>
       <c r="AD21" s="6"/>
       <c r="AE21" s="6"/>
     </row>
@@ -2327,9 +2432,7 @@
       <c r="A22" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B22" s="7" t="s">
-        <v>56</v>
-      </c>
+      <c r="B22" s="7"/>
       <c r="C22" s="7" t="s">
         <v>57</v>
       </c>
@@ -2337,37 +2440,41 @@
         <v>58</v>
       </c>
       <c r="E22" s="7"/>
-      <c r="F22" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="F22" s="7"/>
       <c r="G22" s="7"/>
-      <c r="H22" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="I22" s="7" t="s">
-        <v>2</v>
-      </c>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
       <c r="J22" s="11"/>
-      <c r="K22" s="6" t="s">
-        <v>55</v>
-      </c>
+      <c r="K22" s="6"/>
       <c r="L22" s="11"/>
       <c r="M22" s="6"/>
       <c r="N22" s="11"/>
       <c r="O22" s="11"/>
-      <c r="Q22" s="7"/>
+      <c r="Q22" s="7" t="s">
+        <v>55</v>
+      </c>
       <c r="R22" s="7"/>
-      <c r="S22" s="7"/>
-      <c r="T22" s="7"/>
-      <c r="U22" s="19" t="s">
+      <c r="S22" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="T22" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="U22" s="20" t="s">
         <v>59</v>
       </c>
       <c r="V22" s="7"/>
       <c r="W22" s="7"/>
-      <c r="X22" s="6"/>
-      <c r="Y22" s="7"/>
+      <c r="X22" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="Y22" s="21" t="s">
+        <v>114</v>
+      </c>
       <c r="Z22" s="11"/>
-      <c r="AA22" s="6"/>
+      <c r="AA22" s="6" t="s">
+        <v>55</v>
+      </c>
       <c r="AB22" s="11"/>
       <c r="AC22" s="6"/>
       <c r="AD22" s="11"/>
@@ -2393,11 +2500,11 @@
       <c r="R23" s="7"/>
       <c r="S23" s="7"/>
       <c r="T23" s="7"/>
-      <c r="U23" s="7"/>
-      <c r="V23" s="7"/>
+      <c r="U23" s="20"/>
+      <c r="V23" s="20"/>
       <c r="W23" s="7"/>
-      <c r="X23" s="6"/>
-      <c r="Y23" s="7"/>
+      <c r="X23" s="21"/>
+      <c r="Y23" s="21"/>
       <c r="Z23" s="11"/>
       <c r="AA23" s="6"/>
       <c r="AB23" s="6"/>
@@ -2407,7 +2514,7 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3"/>
-      <c r="B24" s="20"/>
+      <c r="B24" s="22"/>
       <c r="C24" s="12"/>
       <c r="D24" s="12"/>
       <c r="E24" s="12"/>
@@ -2424,7 +2531,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="4"/>
@@ -2444,7 +2551,7 @@
         <v>7</v>
       </c>
       <c r="Q25" s="18" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="R25" s="18"/>
       <c r="S25" s="4"/>
@@ -2546,14 +2653,14 @@
       <c r="J27" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="K27" s="7" t="s">
-        <v>41</v>
+      <c r="K27" s="6" t="s">
+        <v>135</v>
       </c>
       <c r="L27" s="14" t="s">
         <v>21</v>
       </c>
       <c r="M27" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="N27" s="6"/>
       <c r="O27" s="6"/>
@@ -2566,10 +2673,10 @@
       <c r="W27" s="6"/>
       <c r="X27" s="6"/>
       <c r="Y27" s="14" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="Z27" s="14" t="s">
-        <v>136</v>
+        <v>172</v>
       </c>
       <c r="AA27" s="6"/>
       <c r="AB27" s="6"/>
@@ -2580,22 +2687,22 @@
     <row r="28" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7"/>
       <c r="B28" s="14" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="E28" s="17" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="H28" s="9" t="s">
         <v>40</v>
@@ -2610,14 +2717,14 @@
         <v>21</v>
       </c>
       <c r="L28" s="14" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="M28" s="14" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="N28" s="6"/>
       <c r="O28" s="6"/>
-      <c r="Q28" s="19" t="s">
+      <c r="Q28" s="20" t="s">
         <v>90</v>
       </c>
       <c r="R28" s="7"/>
@@ -2626,16 +2733,16 @@
       <c r="U28" s="9"/>
       <c r="V28" s="6"/>
       <c r="W28" s="14" t="s">
-        <v>145</v>
+        <v>173</v>
       </c>
       <c r="X28" s="17" t="s">
-        <v>146</v>
+        <v>174</v>
       </c>
       <c r="Y28" s="14" t="s">
-        <v>158</v>
+        <v>175</v>
       </c>
       <c r="Z28" s="14" t="s">
-        <v>136</v>
+        <v>172</v>
       </c>
       <c r="AA28" s="6"/>
       <c r="AB28" s="6"/>
@@ -2648,31 +2755,31 @@
         <v>43</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>8</v>
+        <v>165</v>
       </c>
       <c r="I29" s="14" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="J29" s="14" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="K29" s="6"/>
       <c r="L29" s="6"/>
@@ -2688,7 +2795,7 @@
       <c r="U29" s="6"/>
       <c r="V29" s="7"/>
       <c r="W29" s="14" t="s">
-        <v>154</v>
+        <v>176</v>
       </c>
       <c r="X29" s="6"/>
       <c r="Y29" s="7"/>
@@ -2703,9 +2810,7 @@
       <c r="A30" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B30" s="7" t="s">
-        <v>56</v>
-      </c>
+      <c r="B30" s="7"/>
       <c r="C30" s="7" t="s">
         <v>57</v>
       </c>
@@ -2713,20 +2818,14 @@
         <v>58</v>
       </c>
       <c r="E30" s="7"/>
-      <c r="F30" s="19" t="s">
+      <c r="F30" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="G30" s="19"/>
-      <c r="H30" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="I30" s="7" t="s">
-        <v>2</v>
-      </c>
+      <c r="G30" s="20"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="7"/>
       <c r="J30" s="11"/>
-      <c r="K30" s="6" t="s">
-        <v>4</v>
-      </c>
+      <c r="K30" s="6"/>
       <c r="L30" s="11"/>
       <c r="M30" s="6"/>
       <c r="N30" s="11"/>
@@ -2735,13 +2834,13 @@
       <c r="R30" s="7"/>
       <c r="S30" s="7"/>
       <c r="T30" s="7"/>
-      <c r="U30" s="19" t="s">
+      <c r="U30" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="V30" s="19" t="s">
+      <c r="V30" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="W30" s="19"/>
+      <c r="W30" s="20"/>
       <c r="X30" s="6"/>
       <c r="Y30" s="7"/>
       <c r="Z30" s="11"/>
@@ -2758,8 +2857,8 @@
       <c r="D31" s="7"/>
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
-      <c r="G31" s="19"/>
-      <c r="H31" s="6"/>
+      <c r="G31" s="20"/>
+      <c r="H31" s="7"/>
       <c r="I31" s="7"/>
       <c r="J31" s="11"/>
       <c r="K31" s="6"/>
@@ -2773,7 +2872,7 @@
       <c r="T31" s="7"/>
       <c r="U31" s="7"/>
       <c r="V31" s="7"/>
-      <c r="W31" s="19"/>
+      <c r="W31" s="20"/>
       <c r="X31" s="6"/>
       <c r="Y31" s="7"/>
       <c r="Z31" s="11"/>
@@ -2785,7 +2884,7 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3"/>
-      <c r="B32" s="20"/>
+      <c r="B32" s="22"/>
       <c r="C32" s="12"/>
       <c r="D32" s="12"/>
       <c r="E32" s="12"/>
@@ -2817,7 +2916,7 @@
       <c r="N33" s="4"/>
       <c r="O33" s="5"/>
       <c r="Q33" s="3" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
       <c r="R33" s="18"/>
       <c r="S33" s="4"/>
@@ -2836,137 +2935,89 @@
     </row>
     <row r="34" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7"/>
-      <c r="B34" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="D34" s="7" t="s">
-        <v>162</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="F34" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="G34" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="I34" s="7" t="s">
-        <v>167</v>
-      </c>
-      <c r="J34" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="K34" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="L34" s="21" t="s">
-        <v>170</v>
-      </c>
-      <c r="M34" s="21" t="s">
-        <v>171</v>
-      </c>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="6"/>
+      <c r="I34" s="7"/>
+      <c r="J34" s="6"/>
+      <c r="K34" s="6"/>
+      <c r="L34" s="19"/>
+      <c r="M34" s="19"/>
       <c r="N34" s="6"/>
       <c r="O34" s="6"/>
       <c r="Q34" s="6" t="s">
         <v>2</v>
       </c>
       <c r="R34" s="7" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="S34" s="7" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="T34" s="7" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
       <c r="U34" s="6" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="V34" s="6" t="s">
-        <v>164</v>
+        <v>182</v>
       </c>
       <c r="W34" s="6" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
       <c r="X34" s="6" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="Y34" s="7" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="Z34" s="6" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="AA34" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="AB34" s="21" t="s">
-        <v>170</v>
-      </c>
-      <c r="AC34" s="21" t="s">
-        <v>171</v>
+        <v>187</v>
+      </c>
+      <c r="AB34" s="19" t="s">
+        <v>188</v>
+      </c>
+      <c r="AC34" s="19" t="s">
+        <v>189</v>
       </c>
       <c r="AD34" s="6"/>
       <c r="AE34" s="6"/>
     </row>
     <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="7"/>
-      <c r="B35" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="D35" s="7" t="s">
-        <v>172</v>
-      </c>
-      <c r="E35" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="G35" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="H35" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I35" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="J35" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="K35" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="L35" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="M35" s="6" t="s">
-        <v>135</v>
-      </c>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="6"/>
+      <c r="H35" s="6"/>
+      <c r="I35" s="7"/>
+      <c r="J35" s="6"/>
+      <c r="K35" s="7"/>
+      <c r="L35" s="6"/>
+      <c r="M35" s="6"/>
       <c r="N35" s="6"/>
       <c r="O35" s="6"/>
       <c r="Q35" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="R35" s="22" t="s">
+      <c r="R35" s="23" t="s">
         <v>130</v>
       </c>
       <c r="S35" s="7" t="s">
         <v>131</v>
       </c>
       <c r="T35" s="7" t="s">
-        <v>172</v>
+        <v>190</v>
       </c>
       <c r="U35" s="7" t="s">
         <v>133</v>
@@ -2974,166 +3025,126 @@
       <c r="V35" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="W35" s="22" t="s">
+      <c r="W35" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="X35" s="22" t="s">
+      <c r="X35" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="Y35" s="22" t="s">
+      <c r="Y35" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="Z35" s="22" t="s">
+      <c r="Z35" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="AA35" s="22" t="s">
+      <c r="AA35" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="AB35" s="22" t="s">
+      <c r="AB35" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="AC35" s="22" t="s">
-        <v>135</v>
+      <c r="AC35" s="23" t="s">
+        <v>136</v>
       </c>
       <c r="AD35" s="6"/>
       <c r="AE35" s="6"/>
     </row>
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7"/>
-      <c r="B36" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="D36" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="E36" s="23" t="s">
-        <v>140</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="G36" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="H36" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="I36" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="J36" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="K36" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="L36" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="M36" s="6" t="s">
-        <v>144</v>
-      </c>
+      <c r="B36" s="7"/>
+      <c r="C36" s="7"/>
+      <c r="D36" s="7"/>
+      <c r="E36" s="24"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="24"/>
+      <c r="I36" s="7"/>
+      <c r="J36" s="6"/>
+      <c r="K36" s="6"/>
+      <c r="L36" s="6"/>
+      <c r="M36" s="6"/>
       <c r="N36" s="6"/>
       <c r="O36" s="6"/>
       <c r="Q36" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="R36" s="22" t="s">
-        <v>173</v>
-      </c>
-      <c r="S36" s="22" t="s">
-        <v>138</v>
+      <c r="R36" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="S36" s="23" t="s">
+        <v>149</v>
       </c>
       <c r="T36" s="7" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="U36" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="V36" s="22" t="s">
-        <v>141</v>
-      </c>
-      <c r="W36" s="22" t="s">
-        <v>142</v>
-      </c>
-      <c r="X36" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="V36" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="W36" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="X36" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="Y36" s="22" t="s">
+      <c r="Y36" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="Z36" s="22" t="s">
+      <c r="Z36" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="AA36" s="22" t="s">
+      <c r="AA36" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="AB36" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="AC36" s="22" t="s">
-        <v>144</v>
+      <c r="AB36" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="AC36" s="23" t="s">
+        <v>155</v>
       </c>
       <c r="AD36" s="6"/>
       <c r="AE36" s="6"/>
     </row>
     <row r="37" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="B37" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="D37" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="F37" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="G37" s="6" t="s">
-        <v>151</v>
-      </c>
+      <c r="A37" s="7"/>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="6"/>
       <c r="H37" s="7"/>
       <c r="I37" s="7"/>
       <c r="J37" s="7"/>
       <c r="K37" s="6"/>
       <c r="L37" s="6"/>
-      <c r="M37" s="6" t="s">
-        <v>43</v>
-      </c>
+      <c r="M37" s="6"/>
       <c r="N37" s="6"/>
       <c r="O37" s="6"/>
       <c r="Q37" s="7" t="s">
         <v>43</v>
       </c>
       <c r="R37" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="S37" s="22" t="s">
-        <v>148</v>
-      </c>
-      <c r="T37" s="22" t="s">
-        <v>149</v>
-      </c>
-      <c r="U37" s="22" t="s">
-        <v>150</v>
-      </c>
-      <c r="V37" s="22" t="s">
-        <v>147</v>
-      </c>
-      <c r="W37" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="X37" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="S37" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="T37" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="U37" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="V37" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="W37" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="X37" s="23" t="s">
         <v>41</v>
       </c>
       <c r="Y37" s="7"/>
@@ -3147,31 +3158,17 @@
       <c r="AE37" s="6"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="B38" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="C38" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="D38" s="7" t="s">
-        <v>58</v>
-      </c>
+      <c r="A38" s="7"/>
+      <c r="B38" s="7"/>
+      <c r="C38" s="7"/>
+      <c r="D38" s="7"/>
       <c r="E38" s="7"/>
       <c r="F38" s="7"/>
       <c r="G38" s="7"/>
-      <c r="H38" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="I38" s="7" t="s">
-        <v>2</v>
-      </c>
+      <c r="H38" s="7"/>
+      <c r="I38" s="7"/>
       <c r="J38" s="11"/>
-      <c r="K38" s="6" t="s">
-        <v>55</v>
-      </c>
+      <c r="K38" s="6"/>
       <c r="L38" s="11"/>
       <c r="M38" s="6"/>
       <c r="N38" s="11"/>
@@ -3220,7 +3217,7 @@
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
       <c r="G39" s="7"/>
-      <c r="H39" s="6"/>
+      <c r="H39" s="7"/>
       <c r="I39" s="7"/>
       <c r="J39" s="11"/>
       <c r="K39" s="6"/>
@@ -3251,7 +3248,7 @@
       <c r="AE39" s="6"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="20"/>
+      <c r="B40" s="22"/>
       <c r="C40" s="12"/>
       <c r="D40" s="12"/>
       <c r="E40" s="12"/>
@@ -3268,7 +3265,7 @@
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="18" t="s">
-        <v>173</v>
+        <v>191</v>
       </c>
       <c r="B41" s="18"/>
       <c r="C41" s="4"/>
@@ -3285,7 +3282,7 @@
       <c r="N41" s="4"/>
       <c r="O41" s="5"/>
       <c r="Q41" s="18" t="s">
-        <v>174</v>
+        <v>59</v>
       </c>
       <c r="R41" s="18"/>
       <c r="S41" s="4"/>
@@ -3319,14 +3316,14 @@
       <c r="N42" s="6"/>
       <c r="O42" s="6"/>
       <c r="Q42" s="7"/>
-      <c r="R42" s="6"/>
-      <c r="S42" s="6"/>
-      <c r="T42" s="6"/>
+      <c r="R42" s="7"/>
+      <c r="S42" s="7"/>
+      <c r="T42" s="7"/>
       <c r="U42" s="6"/>
       <c r="V42" s="6"/>
       <c r="W42" s="6"/>
       <c r="X42" s="6"/>
-      <c r="Y42" s="6"/>
+      <c r="Y42" s="7"/>
       <c r="Z42" s="6"/>
       <c r="AA42" s="6"/>
       <c r="AB42" s="6"/>
@@ -3341,11 +3338,11 @@
       <c r="D43" s="7"/>
       <c r="E43" s="7"/>
       <c r="F43" s="6"/>
-      <c r="G43" s="6"/>
-      <c r="H43" s="6"/>
+      <c r="G43" s="7"/>
+      <c r="H43" s="7"/>
       <c r="I43" s="7"/>
-      <c r="J43" s="14" t="s">
-        <v>175</v>
+      <c r="J43" s="7" t="s">
+        <v>135</v>
       </c>
       <c r="K43" s="6"/>
       <c r="L43" s="6"/>
@@ -3353,31 +3350,35 @@
       <c r="N43" s="6"/>
       <c r="O43" s="6"/>
       <c r="Q43" s="7"/>
-      <c r="R43" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="S43" s="6"/>
-      <c r="T43" s="6"/>
-      <c r="U43" s="6"/>
-      <c r="V43" s="6"/>
-      <c r="W43" s="6"/>
-      <c r="X43" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="Y43" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z43" s="6"/>
-      <c r="AA43" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="AB43" s="6"/>
+      <c r="R43" s="7"/>
+      <c r="S43" s="7"/>
+      <c r="T43" s="7"/>
+      <c r="U43" s="7"/>
+      <c r="V43" s="7"/>
+      <c r="W43" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="X43" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="Y43" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="Z43" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="AA43" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="AB43" s="14" t="s">
+        <v>21</v>
+      </c>
       <c r="AC43" s="6"/>
       <c r="AD43" s="6"/>
       <c r="AE43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="19" t="s">
+      <c r="A44" s="20" t="s">
         <v>90</v>
       </c>
       <c r="B44" s="7"/>
@@ -3385,15 +3386,15 @@
       <c r="D44" s="7"/>
       <c r="E44" s="9"/>
       <c r="F44" s="6"/>
-      <c r="G44" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="H44" s="17" t="s">
-        <v>181</v>
+      <c r="G44" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="H44" s="9" t="s">
+        <v>165</v>
       </c>
       <c r="I44" s="7"/>
-      <c r="J44" s="14" t="s">
-        <v>175</v>
+      <c r="J44" s="7" t="s">
+        <v>135</v>
       </c>
       <c r="K44" s="6"/>
       <c r="L44" s="6"/>
@@ -3401,22 +3402,30 @@
       <c r="N44" s="6"/>
       <c r="O44" s="6"/>
       <c r="Q44" s="7"/>
-      <c r="R44" s="6"/>
-      <c r="S44" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="T44" s="6"/>
-      <c r="U44" s="23" t="s">
-        <v>140</v>
-      </c>
-      <c r="V44" s="6"/>
-      <c r="W44" s="6"/>
-      <c r="X44" s="23"/>
-      <c r="Y44" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="Z44" s="6"/>
-      <c r="AA44" s="6"/>
+      <c r="R44" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="S44" s="7"/>
+      <c r="T44" s="7"/>
+      <c r="U44" s="9"/>
+      <c r="V44" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="W44" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="X44" s="17" t="s">
+        <v>174</v>
+      </c>
+      <c r="Y44" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="Z44" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="AA44" s="14" t="s">
+        <v>21</v>
+      </c>
       <c r="AB44" s="6"/>
       <c r="AC44" s="6"/>
       <c r="AD44" s="6"/>
@@ -3429,38 +3438,42 @@
       <c r="D45" s="7"/>
       <c r="E45" s="6"/>
       <c r="F45" s="7"/>
-      <c r="G45" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="H45" s="6"/>
+      <c r="G45" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H45" s="7"/>
       <c r="I45" s="7"/>
-      <c r="J45" s="6"/>
+      <c r="J45" s="7"/>
       <c r="K45" s="6"/>
       <c r="L45" s="6"/>
       <c r="M45" s="6"/>
       <c r="N45" s="6"/>
       <c r="O45" s="6"/>
       <c r="Q45" s="7"/>
-      <c r="R45" s="7"/>
-      <c r="S45" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="T45" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="U45" s="7"/>
-      <c r="V45" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="W45" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="X45" s="7"/>
-      <c r="Y45" s="7"/>
+      <c r="R45" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="S45" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="T45" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="U45" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="V45" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="W45" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="X45" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="Y45" s="6"/>
       <c r="Z45" s="6"/>
-      <c r="AA45" s="24" t="s">
-        <v>52</v>
-      </c>
+      <c r="AA45" s="6"/>
       <c r="AB45" s="6"/>
       <c r="AC45" s="6"/>
       <c r="AD45" s="6"/>
@@ -3472,10 +3485,10 @@
       <c r="C46" s="7"/>
       <c r="D46" s="7"/>
       <c r="E46" s="7"/>
-      <c r="F46" s="19" t="s">
+      <c r="F46" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="G46" s="19"/>
+      <c r="G46" s="20"/>
       <c r="H46" s="6"/>
       <c r="I46" s="7"/>
       <c r="J46" s="11"/>
@@ -3488,13 +3501,21 @@
       <c r="R46" s="7"/>
       <c r="S46" s="7"/>
       <c r="T46" s="7"/>
-      <c r="U46" s="7"/>
+      <c r="U46" s="20" t="s">
+        <v>59</v>
+      </c>
       <c r="V46" s="7"/>
       <c r="W46" s="7"/>
-      <c r="X46" s="6"/>
-      <c r="Y46" s="7"/>
+      <c r="X46" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="Y46" s="20" t="s">
+        <v>114</v>
+      </c>
       <c r="Z46" s="11"/>
-      <c r="AA46" s="6"/>
+      <c r="AA46" s="6" t="s">
+        <v>4</v>
+      </c>
       <c r="AB46" s="11"/>
       <c r="AC46" s="6"/>
       <c r="AD46" s="11"/>
@@ -3507,7 +3528,7 @@
       <c r="D47" s="7"/>
       <c r="E47" s="7"/>
       <c r="F47" s="7"/>
-      <c r="G47" s="19"/>
+      <c r="G47" s="20"/>
       <c r="H47" s="6"/>
       <c r="I47" s="7"/>
       <c r="J47" s="11"/>
@@ -3523,8 +3544,8 @@
       <c r="U47" s="7"/>
       <c r="V47" s="7"/>
       <c r="W47" s="7"/>
-      <c r="X47" s="6"/>
-      <c r="Y47" s="7"/>
+      <c r="X47" s="20"/>
+      <c r="Y47" s="20"/>
       <c r="Z47" s="11"/>
       <c r="AA47" s="6"/>
       <c r="AB47" s="6"/>
@@ -3533,8 +3554,8 @@
       <c r="AE47" s="6"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="20"/>
-      <c r="B48" s="20"/>
+      <c r="A48" s="22"/>
+      <c r="B48" s="22"/>
       <c r="C48" s="12"/>
       <c r="D48" s="12"/>
       <c r="E48" s="12"/>
@@ -3551,7 +3572,7 @@
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="B49" s="18"/>
       <c r="C49" s="4"/>
@@ -3568,7 +3589,7 @@
       <c r="N49" s="4"/>
       <c r="O49" s="5"/>
       <c r="Q49" s="3" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3617,7 +3638,9 @@
       <c r="T50" s="7"/>
       <c r="U50" s="6"/>
       <c r="V50" s="6"/>
-      <c r="W50" s="6"/>
+      <c r="W50" s="14" t="s">
+        <v>130</v>
+      </c>
       <c r="X50" s="14" t="n">
         <v>7</v>
       </c>
@@ -3633,47 +3656,47 @@
       <c r="AB50" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="AC50" s="6"/>
-      <c r="AD50" s="6"/>
-      <c r="AE50" s="6"/>
+      <c r="AC50" s="7"/>
+      <c r="AD50" s="7"/>
+      <c r="AE50" s="7"/>
     </row>
     <row r="51" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="7"/>
       <c r="B51" s="7" t="s">
-        <v>188</v>
+        <v>137</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>189</v>
+        <v>138</v>
       </c>
       <c r="D51" s="7" t="s">
         <v>132</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>190</v>
+        <v>139</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>191</v>
+        <v>140</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>192</v>
+        <v>141</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>193</v>
+        <v>142</v>
       </c>
       <c r="I51" s="7" t="s">
-        <v>194</v>
+        <v>143</v>
       </c>
       <c r="J51" s="6" t="s">
-        <v>195</v>
+        <v>144</v>
       </c>
       <c r="K51" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="L51" s="21" t="s">
-        <v>197</v>
-      </c>
-      <c r="M51" s="21" t="s">
-        <v>198</v>
+        <v>145</v>
+      </c>
+      <c r="L51" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="M51" s="19" t="s">
+        <v>147</v>
       </c>
       <c r="N51" s="6"/>
       <c r="O51" s="6"/>
@@ -3704,8 +3727,8 @@
       <c r="AC51" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="AD51" s="6"/>
-      <c r="AE51" s="6"/>
+      <c r="AD51" s="7"/>
+      <c r="AE51" s="7"/>
     </row>
     <row r="52" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="7"/>
@@ -3753,12 +3776,12 @@
       <c r="R52" s="7"/>
       <c r="S52" s="7"/>
       <c r="T52" s="7"/>
-      <c r="U52" s="6"/>
+      <c r="U52" s="25"/>
       <c r="V52" s="6"/>
       <c r="W52" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="X52" s="14" t="n">
+      <c r="X52" s="17" t="n">
         <v>1</v>
       </c>
       <c r="Y52" s="14" t="n">
@@ -3776,8 +3799,8 @@
       <c r="AC52" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="AD52" s="6"/>
-      <c r="AE52" s="6"/>
+      <c r="AD52" s="7"/>
+      <c r="AE52" s="7"/>
     </row>
     <row r="53" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
@@ -3841,9 +3864,9 @@
         <v>52</v>
       </c>
       <c r="AB53" s="7"/>
-      <c r="AC53" s="6"/>
-      <c r="AD53" s="6"/>
-      <c r="AE53" s="6"/>
+      <c r="AC53" s="7"/>
+      <c r="AD53" s="7"/>
+      <c r="AE53" s="7"/>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
@@ -3856,15 +3879,15 @@
       <c r="D54" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="E54" s="19" t="s">
+      <c r="E54" s="20" t="s">
         <v>59</v>
       </c>
       <c r="F54" s="7"/>
       <c r="G54" s="7"/>
-      <c r="H54" s="24" t="s">
+      <c r="H54" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="I54" s="24" t="s">
+      <c r="I54" s="21" t="s">
         <v>114</v>
       </c>
       <c r="J54" s="11"/>
@@ -3898,11 +3921,11 @@
       <c r="B55" s="7"/>
       <c r="C55" s="7"/>
       <c r="D55" s="7"/>
-      <c r="E55" s="19"/>
-      <c r="F55" s="19"/>
+      <c r="E55" s="20"/>
+      <c r="F55" s="20"/>
       <c r="G55" s="7"/>
-      <c r="H55" s="24"/>
-      <c r="I55" s="24"/>
+      <c r="H55" s="21"/>
+      <c r="I55" s="21"/>
       <c r="J55" s="11"/>
       <c r="K55" s="6"/>
       <c r="L55" s="6"/>
@@ -4264,7 +4287,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -4281,7 +4304,7 @@
       <c r="N1" s="4"/>
       <c r="O1" s="5"/>
       <c r="Q1" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="R1" s="4"/>
       <c r="S1" s="4"/>
@@ -4431,7 +4454,7 @@
         <v>37</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="O3" s="6"/>
       <c r="Q3" s="6" t="s">
@@ -4491,7 +4514,7 @@
       <c r="D4" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="E4" s="24" t="s">
         <v>29</v>
       </c>
       <c r="F4" s="6" t="s">
@@ -4500,7 +4523,7 @@
       <c r="G4" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="H4" s="23" t="s">
+      <c r="H4" s="24" t="s">
         <v>32</v>
       </c>
       <c r="I4" s="6" t="s">
@@ -4534,7 +4557,7 @@
       <c r="T4" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="U4" s="23" t="s">
+      <c r="U4" s="24" t="s">
         <v>29</v>
       </c>
       <c r="V4" s="6" t="s">
@@ -4543,7 +4566,7 @@
       <c r="W4" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="X4" s="23" t="s">
+      <c r="X4" s="24" t="s">
         <v>32</v>
       </c>
       <c r="Y4" s="6" t="s">
@@ -4599,7 +4622,7 @@
         <v>52</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="M5" s="6" t="s">
         <v>43</v>
@@ -4948,7 +4971,7 @@
         <v>37</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="O11" s="6"/>
       <c r="Q11" s="7"/>
@@ -5006,7 +5029,7 @@
       <c r="D12" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="23" t="s">
+      <c r="E12" s="24" t="s">
         <v>29</v>
       </c>
       <c r="F12" s="6" t="s">
@@ -5015,7 +5038,7 @@
       <c r="G12" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="H12" s="23" t="s">
+      <c r="H12" s="24" t="s">
         <v>32</v>
       </c>
       <c r="I12" s="6" t="s">
@@ -5047,7 +5070,7 @@
       <c r="T12" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="U12" s="23" t="s">
+      <c r="U12" s="24" t="s">
         <v>94</v>
       </c>
       <c r="V12" s="6" t="s">
@@ -5056,7 +5079,7 @@
       <c r="W12" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="X12" s="23" t="s">
+      <c r="X12" s="24" t="s">
         <v>97</v>
       </c>
       <c r="Y12" s="7" t="s">
@@ -5112,7 +5135,7 @@
         <v>52</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="M13" s="6" t="s">
         <v>43</v>
@@ -5305,40 +5328,40 @@
         <v>116</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>164</v>
+        <v>182</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="L18" s="21" t="s">
-        <v>170</v>
-      </c>
-      <c r="M18" s="21" t="s">
-        <v>171</v>
+        <v>187</v>
+      </c>
+      <c r="L18" s="19" t="s">
+        <v>188</v>
+      </c>
+      <c r="M18" s="19" t="s">
+        <v>189</v>
       </c>
       <c r="N18" s="6" t="s">
         <v>6</v>
@@ -5373,7 +5396,7 @@
         <v>131</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>172</v>
+        <v>190</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>133</v>
@@ -5397,7 +5420,7 @@
         <v>41</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="M19" s="6"/>
       <c r="N19" s="6"/>
@@ -5413,7 +5436,7 @@
       <c r="X19" s="6"/>
       <c r="Y19" s="7"/>
       <c r="Z19" s="6" t="s">
-        <v>136</v>
+        <v>172</v>
       </c>
       <c r="AA19" s="6"/>
       <c r="AB19" s="6"/>
@@ -5422,28 +5445,28 @@
       <c r="AE19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="19" t="s">
+      <c r="A20" s="20" t="s">
         <v>90</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="E20" s="23" t="s">
-        <v>140</v>
+        <v>150</v>
+      </c>
+      <c r="E20" s="24" t="s">
+        <v>151</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="H20" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="H20" s="24" t="s">
         <v>40</v>
       </c>
       <c r="I20" s="7" t="s">
@@ -5456,7 +5479,7 @@
         <v>21</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="M20" s="6" t="s">
         <v>21</v>
@@ -5470,17 +5493,17 @@
       <c r="R20" s="7"/>
       <c r="S20" s="7"/>
       <c r="T20" s="7"/>
-      <c r="U20" s="23"/>
+      <c r="U20" s="24"/>
       <c r="V20" s="6"/>
       <c r="W20" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="X20" s="23" t="s">
-        <v>146</v>
+        <v>173</v>
+      </c>
+      <c r="X20" s="24" t="s">
+        <v>174</v>
       </c>
       <c r="Y20" s="7"/>
       <c r="Z20" s="6" t="s">
-        <v>136</v>
+        <v>172</v>
       </c>
       <c r="AA20" s="6"/>
       <c r="AB20" s="6"/>
@@ -5493,35 +5516,35 @@
         <v>43</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="H21" s="7" t="s">
         <v>41</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="J21" s="7" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="K21" s="6"/>
       <c r="L21" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="M21" s="6" t="s">
         <v>43</v>
@@ -5535,7 +5558,7 @@
       <c r="U21" s="6"/>
       <c r="V21" s="7"/>
       <c r="W21" s="6" t="s">
-        <v>154</v>
+        <v>176</v>
       </c>
       <c r="X21" s="6"/>
       <c r="Y21" s="7"/>
@@ -5640,7 +5663,7 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3"/>
-      <c r="B24" s="20"/>
+      <c r="B24" s="22"/>
       <c r="C24" s="12"/>
       <c r="D24" s="12"/>
       <c r="E24" s="12"/>
@@ -5657,7 +5680,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="4"/>
@@ -5695,40 +5718,40 @@
     <row r="26" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7"/>
       <c r="B26" s="7" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>164</v>
+        <v>182</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="K26" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="L26" s="21" t="s">
-        <v>170</v>
-      </c>
-      <c r="M26" s="21" t="s">
-        <v>171</v>
+        <v>187</v>
+      </c>
+      <c r="L26" s="19" t="s">
+        <v>188</v>
+      </c>
+      <c r="M26" s="19" t="s">
+        <v>189</v>
       </c>
       <c r="N26" s="6" t="s">
         <v>6</v>
@@ -5761,7 +5784,7 @@
         <v>131</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>172</v>
+        <v>190</v>
       </c>
       <c r="E27" s="7" t="s">
         <v>133</v>
@@ -5785,11 +5808,11 @@
         <v>41</v>
       </c>
       <c r="L27" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="M27" s="6"/>
       <c r="N27" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="O27" s="6"/>
       <c r="Q27" s="7"/>
@@ -5811,24 +5834,24 @@
     <row r="28" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7"/>
       <c r="B28" s="7" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="E28" s="23" t="s">
-        <v>140</v>
+        <v>150</v>
+      </c>
+      <c r="E28" s="24" t="s">
+        <v>151</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="H28" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="H28" s="24" t="s">
         <v>40</v>
       </c>
       <c r="I28" s="7" t="s">
@@ -5841,7 +5864,7 @@
         <v>21</v>
       </c>
       <c r="L28" s="6" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="M28" s="6" t="s">
         <v>21</v>
@@ -5850,14 +5873,14 @@
         <v>37</v>
       </c>
       <c r="O28" s="6"/>
-      <c r="Q28" s="19"/>
+      <c r="Q28" s="20"/>
       <c r="R28" s="7"/>
       <c r="S28" s="7"/>
       <c r="T28" s="7"/>
-      <c r="U28" s="23"/>
+      <c r="U28" s="24"/>
       <c r="V28" s="6"/>
       <c r="W28" s="6"/>
-      <c r="X28" s="23"/>
+      <c r="X28" s="24"/>
       <c r="Y28" s="7"/>
       <c r="Z28" s="6"/>
       <c r="AA28" s="6"/>
@@ -5871,35 +5894,35 @@
         <v>43</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="H29" s="7" t="s">
         <v>41</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="K29" s="6"/>
       <c r="L29" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="M29" s="6" t="s">
         <v>43</v>
@@ -6016,7 +6039,7 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3"/>
-      <c r="B32" s="20"/>
+      <c r="B32" s="22"/>
       <c r="C32" s="12"/>
       <c r="D32" s="12"/>
       <c r="E32" s="12"/>
@@ -6048,7 +6071,7 @@
       <c r="N33" s="4"/>
       <c r="O33" s="5"/>
       <c r="Q33" s="3" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
       <c r="R33" s="18"/>
       <c r="S33" s="4"/>
@@ -6068,40 +6091,40 @@
     <row r="34" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7"/>
       <c r="B34" s="7" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>164</v>
+        <v>182</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="I34" s="7" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="K34" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="L34" s="21" t="s">
-        <v>170</v>
-      </c>
-      <c r="M34" s="21" t="s">
-        <v>171</v>
+        <v>187</v>
+      </c>
+      <c r="L34" s="19" t="s">
+        <v>188</v>
+      </c>
+      <c r="M34" s="19" t="s">
+        <v>189</v>
       </c>
       <c r="N34" s="6" t="s">
         <v>6</v>
@@ -6113,40 +6136,40 @@
         <v>2</v>
       </c>
       <c r="R34" s="7" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="S34" s="7" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="T34" s="7" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
       <c r="U34" s="6" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="V34" s="6" t="s">
-        <v>164</v>
+        <v>182</v>
       </c>
       <c r="W34" s="6" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
       <c r="X34" s="6" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="Y34" s="7" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="Z34" s="6" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="AA34" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="AB34" s="21" t="s">
-        <v>170</v>
-      </c>
-      <c r="AC34" s="21" t="s">
-        <v>171</v>
+        <v>187</v>
+      </c>
+      <c r="AB34" s="19" t="s">
+        <v>188</v>
+      </c>
+      <c r="AC34" s="19" t="s">
+        <v>189</v>
       </c>
       <c r="AD34" s="6"/>
       <c r="AE34" s="6"/>
@@ -6160,7 +6183,7 @@
         <v>131</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>172</v>
+        <v>190</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>133</v>
@@ -6184,24 +6207,24 @@
         <v>41</v>
       </c>
       <c r="L35" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="M35" s="6"/>
       <c r="N35" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="O35" s="6"/>
       <c r="Q35" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="R35" s="22" t="s">
+      <c r="R35" s="23" t="s">
         <v>130</v>
       </c>
       <c r="S35" s="7" t="s">
         <v>131</v>
       </c>
       <c r="T35" s="7" t="s">
-        <v>172</v>
+        <v>190</v>
       </c>
       <c r="U35" s="7" t="s">
         <v>133</v>
@@ -6209,26 +6232,26 @@
       <c r="V35" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="W35" s="22" t="s">
+      <c r="W35" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="X35" s="22" t="s">
+      <c r="X35" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="Y35" s="22" t="s">
+      <c r="Y35" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="Z35" s="22" t="s">
+      <c r="Z35" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="AA35" s="22" t="s">
+      <c r="AA35" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="AB35" s="22" t="s">
+      <c r="AB35" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="AC35" s="22" t="s">
-        <v>135</v>
+      <c r="AC35" s="23" t="s">
+        <v>136</v>
       </c>
       <c r="AD35" s="6"/>
       <c r="AE35" s="6"/>
@@ -6236,24 +6259,24 @@
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7"/>
       <c r="B36" s="7" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="E36" s="23" t="s">
-        <v>140</v>
+        <v>150</v>
+      </c>
+      <c r="E36" s="24" t="s">
+        <v>151</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="H36" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="H36" s="24" t="s">
         <v>40</v>
       </c>
       <c r="I36" s="7" t="s">
@@ -6266,7 +6289,7 @@
         <v>21</v>
       </c>
       <c r="L36" s="6" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="M36" s="6" t="s">
         <v>21</v>
@@ -6278,41 +6301,41 @@
       <c r="Q36" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="R36" s="22" t="s">
-        <v>173</v>
-      </c>
-      <c r="S36" s="22" t="s">
-        <v>138</v>
+      <c r="R36" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="S36" s="23" t="s">
+        <v>149</v>
       </c>
       <c r="T36" s="7" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="U36" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="V36" s="22" t="s">
-        <v>141</v>
-      </c>
-      <c r="W36" s="22" t="s">
-        <v>142</v>
-      </c>
-      <c r="X36" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="V36" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="W36" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="X36" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="Y36" s="22" t="s">
+      <c r="Y36" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="Z36" s="22" t="s">
+      <c r="Z36" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="AA36" s="22" t="s">
+      <c r="AA36" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="AB36" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="AC36" s="22" t="s">
-        <v>144</v>
+      <c r="AB36" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="AC36" s="23" t="s">
+        <v>155</v>
       </c>
       <c r="AD36" s="6"/>
       <c r="AE36" s="6"/>
@@ -6322,22 +6345,22 @@
         <v>43</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="H37" s="7" t="s">
         <v>41</v>
@@ -6346,7 +6369,7 @@
       <c r="J37" s="7"/>
       <c r="K37" s="6"/>
       <c r="L37" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="M37" s="6" t="s">
         <v>43</v>
@@ -6357,24 +6380,24 @@
         <v>43</v>
       </c>
       <c r="R37" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="S37" s="22" t="s">
-        <v>148</v>
-      </c>
-      <c r="T37" s="22" t="s">
-        <v>149</v>
-      </c>
-      <c r="U37" s="22" t="s">
-        <v>150</v>
-      </c>
-      <c r="V37" s="22" t="s">
-        <v>147</v>
-      </c>
-      <c r="W37" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="X37" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="S37" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="T37" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="U37" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="V37" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="W37" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="X37" s="23" t="s">
         <v>41</v>
       </c>
       <c r="Y37" s="7"/>
@@ -6508,7 +6531,7 @@
       <c r="AE39" s="6"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="20"/>
+      <c r="B40" s="22"/>
       <c r="C40" s="12"/>
       <c r="D40" s="12"/>
       <c r="E40" s="12"/>
@@ -6525,7 +6548,7 @@
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="18" t="s">
-        <v>173</v>
+        <v>191</v>
       </c>
       <c r="B41" s="18"/>
       <c r="C41" s="4"/>
@@ -6542,7 +6565,7 @@
       <c r="N41" s="4"/>
       <c r="O41" s="5"/>
       <c r="Q41" s="18" t="s">
-        <v>174</v>
+        <v>202</v>
       </c>
       <c r="R41" s="18"/>
       <c r="S41" s="4"/>
@@ -6606,22 +6629,22 @@
       <c r="H43" s="6"/>
       <c r="I43" s="7"/>
       <c r="J43" s="6" t="s">
-        <v>175</v>
+        <v>135</v>
       </c>
       <c r="K43" s="6"/>
       <c r="L43" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="M43" s="6" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="N43" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="O43" s="6"/>
       <c r="Q43" s="7"/>
       <c r="R43" s="6" t="s">
-        <v>176</v>
+        <v>203</v>
       </c>
       <c r="S43" s="6"/>
       <c r="T43" s="6"/>
@@ -6629,14 +6652,14 @@
       <c r="V43" s="6"/>
       <c r="W43" s="6"/>
       <c r="X43" s="6" t="s">
-        <v>177</v>
+        <v>204</v>
       </c>
       <c r="Y43" s="6" t="s">
-        <v>178</v>
+        <v>205</v>
       </c>
       <c r="Z43" s="6"/>
       <c r="AA43" s="6" t="s">
-        <v>179</v>
+        <v>206</v>
       </c>
       <c r="AB43" s="6"/>
       <c r="AC43" s="6"/>
@@ -6644,27 +6667,27 @@
       <c r="AE43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="19" t="s">
+      <c r="A44" s="20" t="s">
         <v>90</v>
       </c>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
-      <c r="E44" s="23"/>
+      <c r="E44" s="24"/>
       <c r="F44" s="6"/>
       <c r="G44" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="H44" s="23" t="s">
-        <v>181</v>
+        <v>193</v>
+      </c>
+      <c r="H44" s="24" t="s">
+        <v>165</v>
       </c>
       <c r="I44" s="7"/>
       <c r="J44" s="6" t="s">
-        <v>175</v>
+        <v>135</v>
       </c>
       <c r="K44" s="6"/>
       <c r="L44" s="6" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="M44" s="6" t="s">
         <v>21</v>
@@ -6676,17 +6699,17 @@
       <c r="Q44" s="7"/>
       <c r="R44" s="6"/>
       <c r="S44" s="6" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="T44" s="6"/>
-      <c r="U44" s="23" t="s">
-        <v>140</v>
+      <c r="U44" s="24" t="s">
+        <v>151</v>
       </c>
       <c r="V44" s="6"/>
       <c r="W44" s="6"/>
-      <c r="X44" s="23"/>
+      <c r="X44" s="24"/>
       <c r="Y44" s="6" t="s">
-        <v>182</v>
+        <v>207</v>
       </c>
       <c r="Z44" s="6"/>
       <c r="AA44" s="6"/>
@@ -6703,14 +6726,14 @@
       <c r="E45" s="6"/>
       <c r="F45" s="7"/>
       <c r="G45" s="6" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="H45" s="6"/>
       <c r="I45" s="7"/>
       <c r="J45" s="6"/>
       <c r="K45" s="6"/>
       <c r="L45" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="M45" s="6" t="s">
         <v>43</v>
@@ -6720,22 +6743,22 @@
       <c r="Q45" s="7"/>
       <c r="R45" s="7"/>
       <c r="S45" s="7" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="T45" s="7" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="U45" s="7"/>
       <c r="V45" s="7" t="s">
-        <v>184</v>
+        <v>208</v>
       </c>
       <c r="W45" s="7" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="X45" s="7"/>
       <c r="Y45" s="7"/>
       <c r="Z45" s="6"/>
-      <c r="AA45" s="24" t="s">
+      <c r="AA45" s="21" t="s">
         <v>52</v>
       </c>
       <c r="AB45" s="6"/>
@@ -6836,8 +6859,8 @@
       <c r="AE47" s="6"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="20"/>
-      <c r="B48" s="20"/>
+      <c r="A48" s="22"/>
+      <c r="B48" s="22"/>
       <c r="C48" s="12"/>
       <c r="D48" s="12"/>
       <c r="E48" s="12"/>
@@ -6869,7 +6892,7 @@
       <c r="N49" s="4"/>
       <c r="O49" s="5"/>
       <c r="Q49" s="3" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6924,8 +6947,8 @@
       <c r="I51" s="7"/>
       <c r="J51" s="6"/>
       <c r="K51" s="6"/>
-      <c r="L51" s="21"/>
-      <c r="M51" s="21"/>
+      <c r="L51" s="19"/>
+      <c r="M51" s="19"/>
       <c r="N51" s="6"/>
       <c r="O51" s="6"/>
       <c r="Q51" s="7"/>
@@ -6959,27 +6982,27 @@
       <c r="B52" s="7"/>
       <c r="C52" s="7"/>
       <c r="D52" s="7"/>
-      <c r="E52" s="23"/>
+      <c r="E52" s="24"/>
       <c r="F52" s="6"/>
       <c r="G52" s="6"/>
-      <c r="H52" s="23"/>
+      <c r="H52" s="24"/>
       <c r="I52" s="7"/>
       <c r="J52" s="6"/>
       <c r="K52" s="6"/>
-      <c r="L52" s="21"/>
-      <c r="M52" s="21"/>
+      <c r="L52" s="19"/>
+      <c r="M52" s="19"/>
       <c r="N52" s="6"/>
       <c r="O52" s="6"/>
       <c r="Q52" s="7"/>
       <c r="R52" s="7"/>
       <c r="S52" s="7"/>
       <c r="T52" s="7"/>
-      <c r="U52" s="23"/>
+      <c r="U52" s="24"/>
       <c r="V52" s="6"/>
       <c r="W52" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="X52" s="23" t="n">
+      <c r="X52" s="24" t="n">
         <v>1</v>
       </c>
       <c r="Y52" s="7" t="n">
@@ -7437,7 +7460,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -7600,7 +7623,7 @@
         <v>37</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="O3" s="6"/>
       <c r="Q3" s="7"/>
@@ -7658,7 +7681,7 @@
       <c r="D4" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="E4" s="24" t="s">
         <v>29</v>
       </c>
       <c r="F4" s="6" t="s">
@@ -7667,7 +7690,7 @@
       <c r="G4" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="H4" s="23" t="s">
+      <c r="H4" s="24" t="s">
         <v>32</v>
       </c>
       <c r="I4" s="6" t="s">
@@ -7699,7 +7722,7 @@
       <c r="T4" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="U4" s="23" t="s">
+      <c r="U4" s="24" t="s">
         <v>94</v>
       </c>
       <c r="V4" s="6" t="s">
@@ -7708,7 +7731,7 @@
       <c r="W4" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="X4" s="23" t="s">
+      <c r="X4" s="24" t="s">
         <v>97</v>
       </c>
       <c r="Y4" s="7" t="s">
@@ -7764,7 +7787,7 @@
         <v>52</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="M5" s="6" t="s">
         <v>43</v>
@@ -7920,7 +7943,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -8141,7 +8164,7 @@
       <c r="D12" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="23" t="s">
+      <c r="E12" s="24" t="s">
         <v>29</v>
       </c>
       <c r="F12" s="6" t="s">
@@ -8150,7 +8173,7 @@
       <c r="G12" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="H12" s="23" t="s">
+      <c r="H12" s="24" t="s">
         <v>32</v>
       </c>
       <c r="I12" s="6" t="s">
@@ -8180,7 +8203,7 @@
       <c r="T12" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="U12" s="23" t="s">
+      <c r="U12" s="24" t="s">
         <v>94</v>
       </c>
       <c r="V12" s="6" t="s">
@@ -8189,7 +8212,7 @@
       <c r="W12" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="X12" s="23" t="s">
+      <c r="X12" s="24" t="s">
         <v>97</v>
       </c>
       <c r="Y12" s="7" t="s">
@@ -8469,7 +8492,7 @@
         <v>4</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="O18" s="6" t="s">
         <v>6</v>
@@ -8514,7 +8537,7 @@
         <v>4</v>
       </c>
       <c r="AD18" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AE18" s="6" t="s">
         <v>6</v>
@@ -8620,7 +8643,7 @@
       <c r="D20" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E20" s="23" t="s">
+      <c r="E20" s="24" t="s">
         <v>29</v>
       </c>
       <c r="F20" s="6" t="s">
@@ -8629,7 +8652,7 @@
       <c r="G20" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="H20" s="23" t="s">
+      <c r="H20" s="24" t="s">
         <v>32</v>
       </c>
       <c r="I20" s="6" t="s">
@@ -8660,7 +8683,7 @@
       <c r="T20" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="U20" s="23" t="s">
+      <c r="U20" s="24" t="s">
         <v>94</v>
       </c>
       <c r="V20" s="6" t="s">
@@ -8669,7 +8692,7 @@
       <c r="W20" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="X20" s="23" t="s">
+      <c r="X20" s="24" t="s">
         <v>97</v>
       </c>
       <c r="Y20" s="7" t="s">
@@ -8860,7 +8883,7 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3"/>
-      <c r="B24" s="20"/>
+      <c r="B24" s="22"/>
       <c r="C24" s="12"/>
       <c r="D24" s="12"/>
       <c r="E24" s="12"/>
@@ -9067,10 +9090,10 @@
       <c r="AA27" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="AB27" s="25" t="s">
+      <c r="AB27" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="AC27" s="21" t="s">
+      <c r="AC27" s="19" t="s">
         <v>89</v>
       </c>
       <c r="AD27" s="6"/>
@@ -9089,7 +9112,7 @@
       <c r="D28" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E28" s="23" t="s">
+      <c r="E28" s="24" t="s">
         <v>29</v>
       </c>
       <c r="F28" s="6" t="s">
@@ -9098,7 +9121,7 @@
       <c r="G28" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="H28" s="23" t="s">
+      <c r="H28" s="24" t="s">
         <v>32</v>
       </c>
       <c r="I28" s="6" t="s">
@@ -9128,7 +9151,7 @@
       <c r="T28" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="U28" s="23" t="s">
+      <c r="U28" s="24" t="s">
         <v>94</v>
       </c>
       <c r="V28" s="6" t="s">
@@ -9137,7 +9160,7 @@
       <c r="W28" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="X28" s="23" t="s">
+      <c r="X28" s="24" t="s">
         <v>97</v>
       </c>
       <c r="Y28" s="7" t="s">
@@ -9149,10 +9172,10 @@
       <c r="AA28" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="AB28" s="21" t="s">
+      <c r="AB28" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="AC28" s="21" t="s">
+      <c r="AC28" s="19" t="s">
         <v>102</v>
       </c>
       <c r="AD28" s="6"/>
@@ -9330,7 +9353,7 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3"/>
-      <c r="B32" s="20"/>
+      <c r="B32" s="22"/>
       <c r="C32" s="12"/>
       <c r="D32" s="12"/>
       <c r="E32" s="12"/>
@@ -9362,7 +9385,7 @@
       <c r="N33" s="4"/>
       <c r="O33" s="5"/>
       <c r="Q33" s="3" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
       <c r="R33" s="18"/>
       <c r="S33" s="4"/>
@@ -9382,40 +9405,40 @@
     <row r="34" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7"/>
       <c r="B34" s="7" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>164</v>
+        <v>182</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="I34" s="7" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="K34" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="L34" s="21" t="s">
-        <v>170</v>
-      </c>
-      <c r="M34" s="21" t="s">
-        <v>171</v>
+        <v>187</v>
+      </c>
+      <c r="L34" s="19" t="s">
+        <v>188</v>
+      </c>
+      <c r="M34" s="19" t="s">
+        <v>189</v>
       </c>
       <c r="N34" s="6" t="s">
         <v>6</v>
@@ -9427,40 +9450,40 @@
         <v>2</v>
       </c>
       <c r="R34" s="7" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="S34" s="7" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="T34" s="7" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
       <c r="U34" s="6" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="V34" s="6" t="s">
-        <v>164</v>
+        <v>182</v>
       </c>
       <c r="W34" s="6" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
       <c r="X34" s="6" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="Y34" s="7" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="Z34" s="6" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="AA34" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="AB34" s="21" t="s">
-        <v>170</v>
-      </c>
-      <c r="AC34" s="21" t="s">
-        <v>171</v>
+        <v>187</v>
+      </c>
+      <c r="AB34" s="19" t="s">
+        <v>188</v>
+      </c>
+      <c r="AC34" s="19" t="s">
+        <v>189</v>
       </c>
       <c r="AD34" s="6"/>
       <c r="AE34" s="6"/>
@@ -9474,7 +9497,7 @@
         <v>131</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>172</v>
+        <v>190</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>133</v>
@@ -9498,24 +9521,24 @@
         <v>41</v>
       </c>
       <c r="L35" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="M35" s="6"/>
       <c r="N35" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="O35" s="6"/>
       <c r="Q35" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="R35" s="22" t="s">
+      <c r="R35" s="23" t="s">
         <v>130</v>
       </c>
       <c r="S35" s="7" t="s">
         <v>131</v>
       </c>
       <c r="T35" s="7" t="s">
-        <v>172</v>
+        <v>190</v>
       </c>
       <c r="U35" s="7" t="s">
         <v>133</v>
@@ -9523,26 +9546,26 @@
       <c r="V35" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="W35" s="22" t="s">
+      <c r="W35" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="X35" s="22" t="s">
+      <c r="X35" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="Y35" s="22" t="s">
+      <c r="Y35" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="Z35" s="22" t="s">
+      <c r="Z35" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="AA35" s="22" t="s">
+      <c r="AA35" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="AB35" s="22" t="s">
+      <c r="AB35" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="AC35" s="22" t="s">
-        <v>135</v>
+      <c r="AC35" s="23" t="s">
+        <v>136</v>
       </c>
       <c r="AD35" s="6"/>
       <c r="AE35" s="6"/>
@@ -9550,24 +9573,24 @@
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7"/>
       <c r="B36" s="7" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="E36" s="23" t="s">
-        <v>140</v>
+        <v>150</v>
+      </c>
+      <c r="E36" s="24" t="s">
+        <v>151</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="H36" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="H36" s="24" t="s">
         <v>40</v>
       </c>
       <c r="I36" s="7" t="s">
@@ -9580,7 +9603,7 @@
         <v>21</v>
       </c>
       <c r="L36" s="6" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="M36" s="6" t="s">
         <v>21</v>
@@ -9592,41 +9615,41 @@
       <c r="Q36" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="R36" s="22" t="s">
-        <v>173</v>
-      </c>
-      <c r="S36" s="22" t="s">
-        <v>138</v>
+      <c r="R36" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="S36" s="23" t="s">
+        <v>149</v>
       </c>
       <c r="T36" s="7" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="U36" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="V36" s="22" t="s">
-        <v>141</v>
-      </c>
-      <c r="W36" s="22" t="s">
-        <v>142</v>
-      </c>
-      <c r="X36" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="V36" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="W36" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="X36" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="Y36" s="22" t="s">
+      <c r="Y36" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="Z36" s="22" t="s">
+      <c r="Z36" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="AA36" s="22" t="s">
+      <c r="AA36" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="AB36" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="AC36" s="22" t="s">
-        <v>144</v>
+      <c r="AB36" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="AC36" s="23" t="s">
+        <v>155</v>
       </c>
       <c r="AD36" s="6"/>
       <c r="AE36" s="6"/>
@@ -9636,22 +9659,22 @@
         <v>43</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="H37" s="7" t="s">
         <v>41</v>
@@ -9660,7 +9683,7 @@
       <c r="J37" s="7"/>
       <c r="K37" s="6"/>
       <c r="L37" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="M37" s="6" t="s">
         <v>43</v>
@@ -9671,24 +9694,24 @@
         <v>43</v>
       </c>
       <c r="R37" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="S37" s="22" t="s">
-        <v>148</v>
-      </c>
-      <c r="T37" s="22" t="s">
-        <v>149</v>
-      </c>
-      <c r="U37" s="22" t="s">
-        <v>150</v>
-      </c>
-      <c r="V37" s="22" t="s">
-        <v>147</v>
-      </c>
-      <c r="W37" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="X37" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="S37" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="T37" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="U37" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="V37" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="W37" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="X37" s="23" t="s">
         <v>41</v>
       </c>
       <c r="Y37" s="7"/>
@@ -9822,7 +9845,7 @@
       <c r="AE39" s="6"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="20"/>
+      <c r="B40" s="22"/>
       <c r="C40" s="12"/>
       <c r="D40" s="12"/>
       <c r="E40" s="12"/>
@@ -9839,7 +9862,7 @@
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="18" t="s">
-        <v>173</v>
+        <v>191</v>
       </c>
       <c r="B41" s="18"/>
       <c r="C41" s="4"/>
@@ -9856,7 +9879,7 @@
       <c r="N41" s="4"/>
       <c r="O41" s="5"/>
       <c r="Q41" s="18" t="s">
-        <v>174</v>
+        <v>202</v>
       </c>
       <c r="R41" s="18"/>
       <c r="S41" s="4"/>
@@ -9920,22 +9943,22 @@
       <c r="H43" s="6"/>
       <c r="I43" s="7"/>
       <c r="J43" s="6" t="s">
-        <v>175</v>
+        <v>135</v>
       </c>
       <c r="K43" s="6"/>
       <c r="L43" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="M43" s="6" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="N43" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="O43" s="6"/>
       <c r="Q43" s="7"/>
       <c r="R43" s="6" t="s">
-        <v>176</v>
+        <v>203</v>
       </c>
       <c r="S43" s="6"/>
       <c r="T43" s="6"/>
@@ -9943,14 +9966,14 @@
       <c r="V43" s="6"/>
       <c r="W43" s="6"/>
       <c r="X43" s="6" t="s">
-        <v>177</v>
+        <v>204</v>
       </c>
       <c r="Y43" s="6" t="s">
-        <v>178</v>
+        <v>205</v>
       </c>
       <c r="Z43" s="6"/>
       <c r="AA43" s="6" t="s">
-        <v>179</v>
+        <v>206</v>
       </c>
       <c r="AB43" s="6"/>
       <c r="AC43" s="6"/>
@@ -9958,27 +9981,27 @@
       <c r="AE43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="19" t="s">
+      <c r="A44" s="20" t="s">
         <v>90</v>
       </c>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
-      <c r="E44" s="23"/>
+      <c r="E44" s="24"/>
       <c r="F44" s="6"/>
       <c r="G44" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="H44" s="23" t="s">
-        <v>181</v>
+        <v>193</v>
+      </c>
+      <c r="H44" s="24" t="s">
+        <v>165</v>
       </c>
       <c r="I44" s="7"/>
       <c r="J44" s="6" t="s">
-        <v>175</v>
+        <v>135</v>
       </c>
       <c r="K44" s="6"/>
       <c r="L44" s="6" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="M44" s="6" t="s">
         <v>21</v>
@@ -9990,17 +10013,17 @@
       <c r="Q44" s="7"/>
       <c r="R44" s="6"/>
       <c r="S44" s="6" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="T44" s="6"/>
-      <c r="U44" s="23" t="s">
-        <v>140</v>
+      <c r="U44" s="24" t="s">
+        <v>151</v>
       </c>
       <c r="V44" s="6"/>
       <c r="W44" s="6"/>
-      <c r="X44" s="23"/>
+      <c r="X44" s="24"/>
       <c r="Y44" s="6" t="s">
-        <v>182</v>
+        <v>207</v>
       </c>
       <c r="Z44" s="6"/>
       <c r="AA44" s="6"/>
@@ -10017,14 +10040,14 @@
       <c r="E45" s="6"/>
       <c r="F45" s="7"/>
       <c r="G45" s="6" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="H45" s="6"/>
       <c r="I45" s="7"/>
       <c r="J45" s="6"/>
       <c r="K45" s="6"/>
       <c r="L45" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="M45" s="6" t="s">
         <v>43</v>
@@ -10034,22 +10057,22 @@
       <c r="Q45" s="7"/>
       <c r="R45" s="7"/>
       <c r="S45" s="7" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="T45" s="7" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="U45" s="7"/>
       <c r="V45" s="7" t="s">
-        <v>184</v>
+        <v>208</v>
       </c>
       <c r="W45" s="7" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="X45" s="7"/>
       <c r="Y45" s="7"/>
       <c r="Z45" s="6"/>
-      <c r="AA45" s="24" t="s">
+      <c r="AA45" s="21" t="s">
         <v>52</v>
       </c>
       <c r="AB45" s="6"/>
@@ -10150,8 +10173,8 @@
       <c r="AE47" s="6"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="20"/>
-      <c r="B48" s="20"/>
+      <c r="A48" s="22"/>
+      <c r="B48" s="22"/>
       <c r="C48" s="12"/>
       <c r="D48" s="12"/>
       <c r="E48" s="12"/>
@@ -10183,7 +10206,7 @@
       <c r="N49" s="4"/>
       <c r="O49" s="5"/>
       <c r="Q49" s="3" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10238,8 +10261,8 @@
       <c r="I51" s="7"/>
       <c r="J51" s="6"/>
       <c r="K51" s="6"/>
-      <c r="L51" s="21"/>
-      <c r="M51" s="21"/>
+      <c r="L51" s="19"/>
+      <c r="M51" s="19"/>
       <c r="N51" s="6"/>
       <c r="O51" s="6"/>
       <c r="Q51" s="7"/>
@@ -10273,27 +10296,27 @@
       <c r="B52" s="7"/>
       <c r="C52" s="7"/>
       <c r="D52" s="7"/>
-      <c r="E52" s="23"/>
+      <c r="E52" s="24"/>
       <c r="F52" s="6"/>
       <c r="G52" s="6"/>
-      <c r="H52" s="23"/>
+      <c r="H52" s="24"/>
       <c r="I52" s="7"/>
       <c r="J52" s="6"/>
       <c r="K52" s="6"/>
-      <c r="L52" s="21"/>
-      <c r="M52" s="21"/>
+      <c r="L52" s="19"/>
+      <c r="M52" s="19"/>
       <c r="N52" s="6"/>
       <c r="O52" s="6"/>
       <c r="Q52" s="7"/>
       <c r="R52" s="7"/>
       <c r="S52" s="7"/>
       <c r="T52" s="7"/>
-      <c r="U52" s="23"/>
+      <c r="U52" s="24"/>
       <c r="V52" s="6"/>
       <c r="W52" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="X52" s="23" t="n">
+      <c r="X52" s="24" t="n">
         <v>1</v>
       </c>
       <c r="Y52" s="7" t="n">

</xml_diff>

<commit_message>
[Fix] Incorrect layout images are fixed.
</commit_message>
<xml_diff>
--- a/img/keymap.xlsx
+++ b/img/keymap.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2340" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2405" uniqueCount="230">
   <si>
     <t xml:space="preserve">標準</t>
   </si>
@@ -611,16 +611,19 @@
     <t xml:space="preserve">C+End</t>
   </si>
   <si>
+    <t xml:space="preserve">Layer1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">標準(改変なし)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">標準（ahk）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">　</t>
+  </si>
+  <si>
     <t xml:space="preserve"> (F14 or 変換 or 無変換) 修飾</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Layer1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">標準(改変なし)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">標準（ahk）</t>
   </si>
   <si>
     <t xml:space="preserve">US</t>
@@ -2531,8 +2534,12 @@
       <c r="E22" s="7"/>
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
-      <c r="I22" s="7"/>
+      <c r="H22" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="I22" s="14" t="s">
+        <v>2</v>
+      </c>
       <c r="J22" s="11"/>
       <c r="K22" s="7" t="s">
         <v>55</v>
@@ -2579,8 +2586,8 @@
       <c r="E23" s="7"/>
       <c r="F23" s="7"/>
       <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="7"/>
+      <c r="H23" s="14"/>
+      <c r="I23" s="14"/>
       <c r="J23" s="11"/>
       <c r="K23" s="7"/>
       <c r="L23" s="6"/>
@@ -2614,7 +2621,7 @@
       <c r="H24" s="12"/>
       <c r="I24" s="12"/>
       <c r="J24" s="12"/>
-      <c r="K24" s="12"/>
+      <c r="K24" s="0"/>
       <c r="L24" s="12"/>
       <c r="M24" s="12"/>
       <c r="N24" s="12"/>
@@ -2991,8 +2998,12 @@
         <v>60</v>
       </c>
       <c r="G30" s="20"/>
-      <c r="H30" s="7"/>
-      <c r="I30" s="7"/>
+      <c r="H30" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="I30" s="14" t="s">
+        <v>2</v>
+      </c>
       <c r="J30" s="11"/>
       <c r="K30" s="7" t="s">
         <v>55</v>
@@ -3035,8 +3046,8 @@
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
       <c r="G31" s="20"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="7"/>
+      <c r="H31" s="14"/>
+      <c r="I31" s="14"/>
       <c r="J31" s="11"/>
       <c r="K31" s="7"/>
       <c r="L31" s="6"/>
@@ -3820,9 +3831,7 @@
       <c r="O48" s="13"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3" t="s">
-        <v>195</v>
-      </c>
+      <c r="A49" s="3"/>
       <c r="B49" s="18"/>
       <c r="C49" s="4"/>
       <c r="D49" s="4"/>
@@ -3838,26 +3847,56 @@
       <c r="N49" s="4"/>
       <c r="O49" s="5"/>
       <c r="Q49" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="W49" s="1"/>
     </row>
     <row r="50" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="7"/>
-      <c r="B50" s="7"/>
-      <c r="C50" s="7"/>
-      <c r="D50" s="7"/>
-      <c r="E50" s="6"/>
-      <c r="F50" s="6"/>
-      <c r="G50" s="6"/>
-      <c r="H50" s="6"/>
-      <c r="I50" s="7"/>
-      <c r="J50" s="6"/>
-      <c r="K50" s="6"/>
-      <c r="L50" s="6"/>
-      <c r="M50" s="6"/>
-      <c r="N50" s="6"/>
-      <c r="O50" s="6"/>
+      <c r="A50" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B50" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D50" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F50" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G50" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="H50" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="I50" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="J50" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="K50" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="M50" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="N50" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="O50" s="6" t="s">
+        <v>6</v>
+      </c>
       <c r="Q50" s="7"/>
       <c r="R50" s="7"/>
       <c r="S50" s="7"/>
@@ -3889,20 +3928,48 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="7"/>
-      <c r="B51" s="7"/>
-      <c r="C51" s="7"/>
-      <c r="D51" s="7"/>
-      <c r="E51" s="6"/>
-      <c r="F51" s="6"/>
-      <c r="G51" s="6"/>
-      <c r="H51" s="6"/>
-      <c r="I51" s="7"/>
-      <c r="J51" s="6"/>
-      <c r="K51" s="6"/>
-      <c r="L51" s="19"/>
-      <c r="M51" s="19"/>
-      <c r="N51" s="6"/>
+      <c r="A51" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F51" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G51" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H51" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="I51" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J51" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="K51" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L51" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="M51" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="N51" s="6" t="s">
+        <v>21</v>
+      </c>
       <c r="O51" s="6"/>
       <c r="Q51" s="7"/>
       <c r="R51" s="7"/>
@@ -3937,19 +4004,45 @@
       <c r="AE51" s="7"/>
     </row>
     <row r="52" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="7"/>
-      <c r="B52" s="14"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="17"/>
-      <c r="F52" s="14"/>
-      <c r="G52" s="14"/>
-      <c r="H52" s="17"/>
-      <c r="I52" s="14"/>
-      <c r="J52" s="14"/>
-      <c r="K52" s="14"/>
-      <c r="L52" s="16"/>
-      <c r="M52" s="16"/>
+      <c r="A52" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G52" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="H52" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="I52" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J52" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="K52" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="L52" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="M52" s="6" t="s">
+        <v>37</v>
+      </c>
       <c r="N52" s="6"/>
       <c r="O52" s="6"/>
       <c r="Q52" s="7" t="s">
@@ -3985,19 +4078,45 @@
       <c r="AE52" s="7"/>
     </row>
     <row r="53" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="7"/>
-      <c r="B53" s="14"/>
-      <c r="C53" s="14"/>
-      <c r="D53" s="14"/>
-      <c r="E53" s="14"/>
-      <c r="F53" s="14"/>
-      <c r="G53" s="14"/>
-      <c r="H53" s="14"/>
-      <c r="I53" s="14"/>
-      <c r="J53" s="14"/>
-      <c r="K53" s="14"/>
-      <c r="L53" s="14"/>
-      <c r="M53" s="6"/>
+      <c r="A53" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E53" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F53" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G53" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="H53" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="I53" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="J53" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="K53" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="L53" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="M53" s="6" t="s">
+        <v>43</v>
+      </c>
       <c r="N53" s="6"/>
       <c r="O53" s="6"/>
       <c r="Q53" s="7"/>
@@ -4025,19 +4144,39 @@
       <c r="AE53" s="7"/>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="7"/>
-      <c r="B54" s="7"/>
-      <c r="C54" s="7"/>
-      <c r="D54" s="7"/>
-      <c r="E54" s="20"/>
-      <c r="F54" s="7"/>
+      <c r="A54" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B54" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D54" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E54" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F54" s="7" t="s">
+        <v>60</v>
+      </c>
       <c r="G54" s="7"/>
-      <c r="H54" s="21"/>
-      <c r="I54" s="21"/>
+      <c r="H54" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="I54" s="7" t="s">
+        <v>6</v>
+      </c>
       <c r="J54" s="11"/>
-      <c r="K54" s="6"/>
+      <c r="K54" s="6" t="s">
+        <v>55</v>
+      </c>
       <c r="L54" s="11"/>
-      <c r="M54" s="6"/>
+      <c r="M54" s="6" t="s">
+        <v>23</v>
+      </c>
       <c r="N54" s="11"/>
       <c r="O54" s="11"/>
       <c r="Q54" s="7"/>
@@ -4065,16 +4204,22 @@
       <c r="B55" s="7"/>
       <c r="C55" s="7"/>
       <c r="D55" s="7"/>
-      <c r="E55" s="20"/>
-      <c r="F55" s="20"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="7"/>
       <c r="G55" s="7"/>
-      <c r="H55" s="21"/>
-      <c r="I55" s="21"/>
+      <c r="H55" s="7"/>
+      <c r="I55" s="7"/>
       <c r="J55" s="11"/>
       <c r="K55" s="6"/>
-      <c r="L55" s="6"/>
-      <c r="M55" s="6"/>
-      <c r="N55" s="6"/>
+      <c r="L55" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="M55" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="N55" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="O55" s="6"/>
       <c r="Q55" s="7"/>
       <c r="R55" s="7"/>
@@ -4424,7 +4569,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AE62"/>
+  <dimension ref="A1:AH62"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="1" style="1" width="7.66"/>
@@ -4437,7 +4582,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -4850,7 +4995,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -5031,13 +5176,13 @@
         <v>83</v>
       </c>
       <c r="W11" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="X11" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y11" s="14" t="s">
         <v>84</v>
-      </c>
-      <c r="X11" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="Y11" s="16" t="s">
-        <v>89</v>
       </c>
       <c r="Z11" s="14" t="s">
         <v>85</v>
@@ -5053,6 +5198,9 @@
       </c>
       <c r="AD11" s="6"/>
       <c r="AE11" s="6"/>
+      <c r="AH11" s="16" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
@@ -5113,13 +5261,13 @@
         <v>95</v>
       </c>
       <c r="W12" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="X12" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="Y12" s="14" t="s">
         <v>96</v>
-      </c>
-      <c r="X12" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="Y12" s="16" t="s">
-        <v>102</v>
       </c>
       <c r="Z12" s="17" t="s">
         <v>97</v>
@@ -5135,6 +5283,9 @@
       </c>
       <c r="AD12" s="6"/>
       <c r="AE12" s="6"/>
+      <c r="AH12" s="16" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
@@ -5195,13 +5346,13 @@
         <v>107</v>
       </c>
       <c r="W13" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="X13" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="Y13" s="14" t="s">
         <v>108</v>
-      </c>
-      <c r="X13" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="Y13" s="14" t="s">
-        <v>113</v>
       </c>
       <c r="Z13" s="14" t="s">
         <v>109</v>
@@ -5215,6 +5366,9 @@
       <c r="AC13" s="6"/>
       <c r="AD13" s="6"/>
       <c r="AE13" s="6"/>
+      <c r="AH13" s="14" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
@@ -5924,6 +6078,9 @@
       <c r="AC27" s="6"/>
       <c r="AD27" s="6"/>
       <c r="AE27" s="6"/>
+      <c r="AF27" s="2" t="s">
+        <v>198</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7"/>
@@ -6863,7 +7020,7 @@
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="B49" s="18"/>
       <c r="C49" s="4"/>
@@ -6880,7 +7037,7 @@
       <c r="N49" s="4"/>
       <c r="O49" s="5"/>
       <c r="Q49" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="W49" s="1"/>
     </row>
@@ -7479,7 +7636,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -7496,7 +7653,7 @@
       <c r="N1" s="4"/>
       <c r="O1" s="5"/>
       <c r="Q1" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="R1" s="4"/>
       <c r="S1" s="4"/>
@@ -7646,7 +7803,7 @@
         <v>37</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="O3" s="6"/>
       <c r="Q3" s="6" t="s">
@@ -7814,7 +7971,7 @@
         <v>52</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="M5" s="6" t="s">
         <v>43</v>
@@ -8163,7 +8320,7 @@
         <v>37</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="O11" s="6"/>
       <c r="Q11" s="7"/>
@@ -8327,7 +8484,7 @@
         <v>52</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="M13" s="6" t="s">
         <v>43</v>
@@ -8520,40 +8677,40 @@
         <v>116</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="L18" s="19" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="M18" s="19" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="N18" s="6" t="s">
         <v>6</v>
@@ -8588,10 +8745,10 @@
         <v>131</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>8</v>
@@ -8736,7 +8893,7 @@
       </c>
       <c r="K21" s="6"/>
       <c r="L21" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="M21" s="6" t="s">
         <v>43</v>
@@ -8910,40 +9067,40 @@
     <row r="26" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7"/>
       <c r="B26" s="7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K26" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="L26" s="19" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="M26" s="19" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="N26" s="6" t="s">
         <v>6</v>
@@ -8976,10 +9133,10 @@
         <v>131</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>8</v>
@@ -9004,7 +9161,7 @@
       </c>
       <c r="M27" s="6"/>
       <c r="N27" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="O27" s="6"/>
       <c r="Q27" s="7"/>
@@ -9114,7 +9271,7 @@
       </c>
       <c r="K29" s="6"/>
       <c r="L29" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="M29" s="6" t="s">
         <v>43</v>
@@ -9263,7 +9420,7 @@
       <c r="N33" s="4"/>
       <c r="O33" s="5"/>
       <c r="Q33" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="R33" s="18"/>
       <c r="S33" s="4"/>
@@ -9283,40 +9440,40 @@
     <row r="34" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7"/>
       <c r="B34" s="7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I34" s="7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K34" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="L34" s="19" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="M34" s="19" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="N34" s="6" t="s">
         <v>6</v>
@@ -9328,40 +9485,40 @@
         <v>2</v>
       </c>
       <c r="R34" s="7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="S34" s="7" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="T34" s="7" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="U34" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="V34" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="W34" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="X34" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="Y34" s="7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="Z34" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="AA34" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AB34" s="19" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AC34" s="19" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AD34" s="6"/>
       <c r="AE34" s="6"/>
@@ -9375,10 +9532,10 @@
         <v>131</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F35" s="6" t="s">
         <v>8</v>
@@ -9403,7 +9560,7 @@
       </c>
       <c r="M35" s="6"/>
       <c r="N35" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="O35" s="6"/>
       <c r="Q35" s="7" t="s">
@@ -9416,10 +9573,10 @@
         <v>131</v>
       </c>
       <c r="T35" s="7" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="U35" s="7" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="V35" s="6" t="s">
         <v>8</v>
@@ -9561,7 +9718,7 @@
       <c r="J37" s="7"/>
       <c r="K37" s="6"/>
       <c r="L37" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="M37" s="6" t="s">
         <v>43</v>
@@ -9757,7 +9914,7 @@
       <c r="N41" s="4"/>
       <c r="O41" s="5"/>
       <c r="Q41" s="18" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R41" s="18"/>
       <c r="S41" s="4"/>
@@ -9831,12 +9988,12 @@
         <v>138</v>
       </c>
       <c r="N43" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="O43" s="6"/>
       <c r="Q43" s="7"/>
       <c r="R43" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="S43" s="6"/>
       <c r="T43" s="6"/>
@@ -9844,14 +10001,14 @@
       <c r="V43" s="6"/>
       <c r="W43" s="6"/>
       <c r="X43" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="Y43" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="Z43" s="6"/>
       <c r="AA43" s="6" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AB43" s="6"/>
       <c r="AC43" s="6"/>
@@ -9901,7 +10058,7 @@
       <c r="W44" s="6"/>
       <c r="X44" s="27"/>
       <c r="Y44" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="Z44" s="6"/>
       <c r="AA44" s="6"/>
@@ -9925,7 +10082,7 @@
       <c r="J45" s="6"/>
       <c r="K45" s="6"/>
       <c r="L45" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="M45" s="6" t="s">
         <v>43</v>
@@ -9942,10 +10099,10 @@
       </c>
       <c r="U45" s="7"/>
       <c r="V45" s="7" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="W45" s="7" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="X45" s="7"/>
       <c r="Y45" s="7"/>
@@ -10084,7 +10241,7 @@
       <c r="N49" s="4"/>
       <c r="O49" s="5"/>
       <c r="Q49" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10652,7 +10809,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -10815,7 +10972,7 @@
         <v>37</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="O3" s="6"/>
       <c r="Q3" s="7"/>
@@ -10979,7 +11136,7 @@
         <v>52</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="M5" s="6" t="s">
         <v>43</v>
@@ -11135,7 +11292,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -11277,7 +11434,7 @@
         <v>13</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>14</v>
@@ -11462,7 +11619,7 @@
         <v>7</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="M13" s="6" t="s">
         <v>43</v>
@@ -11733,7 +11890,7 @@
         <v>4</v>
       </c>
       <c r="AD18" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="AE18" s="6" t="s">
         <v>6</v>
@@ -12583,7 +12740,7 @@
       <c r="N33" s="4"/>
       <c r="O33" s="5"/>
       <c r="Q33" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="R33" s="18"/>
       <c r="S33" s="4"/>
@@ -12603,40 +12760,40 @@
     <row r="34" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7"/>
       <c r="B34" s="7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I34" s="7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K34" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="L34" s="19" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="M34" s="19" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="N34" s="6" t="s">
         <v>6</v>
@@ -12648,40 +12805,40 @@
         <v>2</v>
       </c>
       <c r="R34" s="7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="S34" s="7" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="T34" s="7" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="U34" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="V34" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="W34" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="X34" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="Y34" s="7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="Z34" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="AA34" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AB34" s="19" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AC34" s="19" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AD34" s="6"/>
       <c r="AE34" s="6"/>
@@ -12695,10 +12852,10 @@
         <v>131</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F35" s="6" t="s">
         <v>8</v>
@@ -12723,7 +12880,7 @@
       </c>
       <c r="M35" s="6"/>
       <c r="N35" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="O35" s="6"/>
       <c r="Q35" s="7" t="s">
@@ -12736,10 +12893,10 @@
         <v>131</v>
       </c>
       <c r="T35" s="7" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="U35" s="7" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="V35" s="6" t="s">
         <v>8</v>
@@ -12881,7 +13038,7 @@
       <c r="J37" s="7"/>
       <c r="K37" s="6"/>
       <c r="L37" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="M37" s="6" t="s">
         <v>43</v>
@@ -13077,7 +13234,7 @@
       <c r="N41" s="4"/>
       <c r="O41" s="5"/>
       <c r="Q41" s="18" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R41" s="18"/>
       <c r="S41" s="4"/>
@@ -13151,12 +13308,12 @@
         <v>138</v>
       </c>
       <c r="N43" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="O43" s="6"/>
       <c r="Q43" s="7"/>
       <c r="R43" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="S43" s="6"/>
       <c r="T43" s="6"/>
@@ -13164,14 +13321,14 @@
       <c r="V43" s="6"/>
       <c r="W43" s="6"/>
       <c r="X43" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="Y43" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="Z43" s="6"/>
       <c r="AA43" s="6" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AB43" s="6"/>
       <c r="AC43" s="6"/>
@@ -13221,7 +13378,7 @@
       <c r="W44" s="6"/>
       <c r="X44" s="27"/>
       <c r="Y44" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="Z44" s="6"/>
       <c r="AA44" s="6"/>
@@ -13245,7 +13402,7 @@
       <c r="J45" s="6"/>
       <c r="K45" s="6"/>
       <c r="L45" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="M45" s="6" t="s">
         <v>43</v>
@@ -13262,10 +13419,10 @@
       </c>
       <c r="U45" s="7"/>
       <c r="V45" s="7" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="W45" s="7" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="X45" s="7"/>
       <c r="Y45" s="7"/>
@@ -13404,7 +13561,7 @@
       <c r="N49" s="4"/>
       <c r="O49" s="5"/>
       <c r="Q49" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14234,7 +14391,7 @@
       <c r="N5" s="6"/>
       <c r="O5" s="6"/>
       <c r="P5" s="30" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="R5" s="7"/>
       <c r="S5" s="7"/>
@@ -14365,7 +14522,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -14629,7 +14786,7 @@
       <c r="N13" s="6"/>
       <c r="O13" s="6"/>
       <c r="P13" s="30" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="R13" s="7"/>
       <c r="S13" s="14"/>
@@ -14838,7 +14995,7 @@
       <c r="N19" s="6"/>
       <c r="O19" s="6"/>
       <c r="P19" s="31" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="R19" s="7"/>
       <c r="S19" s="7"/>

</xml_diff>

<commit_message>
[Update] F13 + space is assigned as backspace.
</commit_message>
<xml_diff>
--- a/img/keymap.xlsx
+++ b/img/keymap.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2405" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2406" uniqueCount="230">
   <si>
     <t xml:space="preserve">標準</t>
   </si>
@@ -2532,7 +2532,9 @@
         <v>58</v>
       </c>
       <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
+      <c r="F22" s="7" t="s">
+        <v>6</v>
+      </c>
       <c r="G22" s="7"/>
       <c r="H22" s="14" t="s">
         <v>2</v>
@@ -2621,7 +2623,7 @@
       <c r="H24" s="12"/>
       <c r="I24" s="12"/>
       <c r="J24" s="12"/>
-      <c r="K24" s="0"/>
+      <c r="K24" s="2"/>
       <c r="L24" s="12"/>
       <c r="M24" s="12"/>
       <c r="N24" s="12"/>

</xml_diff>

<commit_message>
[Update] Stability is much improved. [Update] F14 and Conv assignment is changed.
</commit_message>
<xml_diff>
--- a/img/keymap.xlsx
+++ b/img/keymap.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1943" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1972" uniqueCount="214">
   <si>
     <t xml:space="preserve">標準</t>
   </si>
@@ -556,10 +556,7 @@
     <t xml:space="preserve">WhDn</t>
   </si>
   <si>
-    <t xml:space="preserve">Find-Next</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Find-Prev</t>
+    <t xml:space="preserve">Prev</t>
   </si>
   <si>
     <t xml:space="preserve">Replace</t>
@@ -590,12 +587,6 @@
   </si>
   <si>
     <t xml:space="preserve">Paste</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Num</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C+”-”</t>
   </si>
   <si>
     <t xml:space="preserve">Space &amp; F13 修飾</t>
@@ -649,10 +640,25 @@
     <t xml:space="preserve">＼</t>
   </si>
   <si>
+    <t xml:space="preserve">Find-Next</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Find-Prev</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Num</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+”-”</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pn</t>
   </si>
   <si>
     <t xml:space="preserve">Kana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">カスタマイズ後</t>
   </si>
   <si>
     <t xml:space="preserve">設定変更</t>
@@ -1017,15 +1023,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1041,7 +1039,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4469,67 +4475,67 @@
       <c r="BG33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7"/>
-      <c r="B34" s="7"/>
-      <c r="C34" s="7"/>
-      <c r="D34" s="7" t="s">
+      <c r="A34" s="6"/>
+      <c r="B34" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="7" t="s">
+      <c r="C34" s="6"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="H34" s="7"/>
-      <c r="I34" s="7"/>
-      <c r="J34" s="25" t="s">
-        <v>177</v>
-      </c>
-      <c r="K34" s="25"/>
-      <c r="L34" s="25"/>
-      <c r="M34" s="6" t="s">
+      <c r="F34" s="6"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="I34" s="6"/>
+      <c r="J34" s="6"/>
+      <c r="K34" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="N34" s="6"/>
+      <c r="L34" s="6"/>
+      <c r="M34" s="6"/>
+      <c r="N34" s="6" t="s">
+        <v>122</v>
+      </c>
       <c r="O34" s="6"/>
-      <c r="P34" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q34" s="6"/>
+      <c r="P34" s="6"/>
+      <c r="Q34" s="6" t="s">
+        <v>123</v>
+      </c>
       <c r="R34" s="6"/>
-      <c r="S34" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="T34" s="6"/>
+      <c r="S34" s="6"/>
+      <c r="T34" s="6" t="s">
+        <v>124</v>
+      </c>
       <c r="U34" s="6"/>
-      <c r="V34" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="W34" s="6"/>
+      <c r="V34" s="6"/>
+      <c r="W34" s="6" t="s">
+        <v>125</v>
+      </c>
       <c r="X34" s="6"/>
-      <c r="Y34" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="Z34" s="7"/>
-      <c r="AA34" s="7"/>
-      <c r="AB34" s="6" t="s">
+      <c r="Y34" s="6"/>
+      <c r="Z34" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="AC34" s="6"/>
+      <c r="AA34" s="6"/>
+      <c r="AB34" s="6"/>
+      <c r="AC34" s="6" t="s">
+        <v>127</v>
+      </c>
       <c r="AD34" s="6"/>
-      <c r="AE34" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="AF34" s="6"/>
+      <c r="AE34" s="6"/>
+      <c r="AF34" s="6" t="s">
+        <v>128</v>
+      </c>
       <c r="AG34" s="6"/>
-      <c r="AH34" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="AI34" s="6"/>
+      <c r="AH34" s="6"/>
+      <c r="AI34" s="6" t="s">
+        <v>129</v>
+      </c>
       <c r="AJ34" s="6"/>
-      <c r="AK34" s="6" t="s">
-        <v>129</v>
-      </c>
+      <c r="AK34" s="6"/>
       <c r="AL34" s="6"/>
       <c r="AM34" s="6"/>
       <c r="AN34" s="6"/>
@@ -4593,67 +4599,67 @@
       <c r="CI34" s="7"/>
     </row>
     <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7"/>
-      <c r="B35" s="7"/>
-      <c r="C35" s="7"/>
-      <c r="D35" s="14" t="s">
+      <c r="A35" s="6"/>
+      <c r="B35" s="6"/>
+      <c r="C35" s="14" t="s">
         <v>143</v>
       </c>
+      <c r="D35" s="14"/>
       <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14" t="s">
+      <c r="F35" s="14" t="s">
         <v>144</v>
       </c>
+      <c r="G35" s="14"/>
       <c r="H35" s="14"/>
-      <c r="I35" s="14"/>
-      <c r="J35" s="26" t="s">
+      <c r="I35" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="J35" s="14"/>
+      <c r="K35" s="14"/>
+      <c r="L35" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="K35" s="26"/>
-      <c r="L35" s="26"/>
-      <c r="M35" s="14" t="s">
+      <c r="M35" s="25"/>
+      <c r="N35" s="25"/>
+      <c r="O35" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="N35" s="14"/>
-      <c r="O35" s="14"/>
-      <c r="P35" s="14" t="s">
-        <v>180</v>
-      </c>
+      <c r="P35" s="14"/>
       <c r="Q35" s="14"/>
-      <c r="R35" s="14"/>
-      <c r="S35" s="14" t="s">
+      <c r="R35" s="14" t="s">
         <v>147</v>
       </c>
+      <c r="S35" s="14"/>
       <c r="T35" s="14"/>
-      <c r="U35" s="14"/>
-      <c r="V35" s="14" t="s">
+      <c r="U35" s="14" t="s">
         <v>6</v>
       </c>
+      <c r="V35" s="14"/>
       <c r="W35" s="14"/>
-      <c r="X35" s="14"/>
-      <c r="Y35" s="7" t="s">
+      <c r="X35" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="Z35" s="7"/>
-      <c r="AA35" s="7"/>
-      <c r="AB35" s="6" t="s">
+      <c r="Y35" s="6"/>
+      <c r="Z35" s="6"/>
+      <c r="AA35" s="6" t="s">
         <v>42</v>
       </c>
+      <c r="AB35" s="6"/>
       <c r="AC35" s="6"/>
-      <c r="AD35" s="6"/>
-      <c r="AE35" s="7" t="s">
+      <c r="AD35" s="7" t="s">
         <v>148</v>
       </c>
+      <c r="AE35" s="7"/>
       <c r="AF35" s="7"/>
-      <c r="AG35" s="7"/>
-      <c r="AH35" s="14" t="s">
+      <c r="AG35" s="14" t="s">
         <v>149</v>
       </c>
+      <c r="AH35" s="14"/>
       <c r="AI35" s="14"/>
-      <c r="AJ35" s="14"/>
-      <c r="AK35" s="14" t="s">
+      <c r="AJ35" s="14" t="s">
         <v>150</v>
       </c>
+      <c r="AK35" s="14"/>
       <c r="AL35" s="14"/>
       <c r="AM35" s="6"/>
       <c r="AN35" s="6"/>
@@ -4717,31 +4723,31 @@
       <c r="CI35" s="7"/>
     </row>
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7"/>
+      <c r="A36" s="7" t="s">
+        <v>91</v>
+      </c>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E36" s="14"/>
       <c r="F36" s="14"/>
       <c r="G36" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H36" s="14"/>
       <c r="I36" s="14"/>
-      <c r="J36" s="14" t="s">
-        <v>156</v>
-      </c>
+      <c r="J36" s="14"/>
       <c r="K36" s="14"/>
       <c r="L36" s="14"/>
-      <c r="M36" s="9" t="s">
+      <c r="M36" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="N36" s="9"/>
-      <c r="O36" s="9"/>
+      <c r="N36" s="20"/>
+      <c r="O36" s="20"/>
       <c r="P36" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Q36" s="14"/>
       <c r="R36" s="14"/>
@@ -4755,11 +4761,11 @@
       </c>
       <c r="W36" s="9"/>
       <c r="X36" s="9"/>
-      <c r="Y36" s="7" t="s">
+      <c r="Y36" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="Z36" s="7"/>
-      <c r="AA36" s="7"/>
+      <c r="Z36" s="6"/>
+      <c r="AA36" s="6"/>
       <c r="AB36" s="6" t="s">
         <v>42</v>
       </c>
@@ -4771,7 +4777,7 @@
       <c r="AF36" s="14"/>
       <c r="AG36" s="14"/>
       <c r="AH36" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AI36" s="14"/>
       <c r="AJ36" s="14"/>
@@ -4779,11 +4785,11 @@
         <v>160</v>
       </c>
       <c r="AL36" s="14"/>
-      <c r="AM36" s="6"/>
-      <c r="AN36" s="6"/>
-      <c r="AO36" s="6"/>
-      <c r="AP36" s="6"/>
-      <c r="AQ36" s="6"/>
+      <c r="AM36" s="14"/>
+      <c r="AN36" s="10"/>
+      <c r="AO36" s="10"/>
+      <c r="AP36" s="10"/>
+      <c r="AQ36" s="10"/>
       <c r="AS36" s="7"/>
       <c r="AT36" s="7"/>
       <c r="AU36" s="7"/>
@@ -4846,63 +4852,63 @@
       </c>
       <c r="B37" s="7"/>
       <c r="C37" s="7"/>
-      <c r="D37" s="14" t="s">
+      <c r="D37" s="7"/>
+      <c r="E37" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="F37" s="14"/>
+      <c r="G37" s="14"/>
+      <c r="H37" s="14" t="s">
         <v>185</v>
       </c>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14" t="s">
+      <c r="I37" s="14"/>
+      <c r="J37" s="14"/>
+      <c r="K37" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="H37" s="14"/>
-      <c r="I37" s="14"/>
-      <c r="J37" s="14" t="s">
+      <c r="L37" s="14"/>
+      <c r="M37" s="14"/>
+      <c r="N37" s="14" t="s">
         <v>187</v>
       </c>
-      <c r="K37" s="14"/>
-      <c r="L37" s="14"/>
-      <c r="M37" s="14" t="s">
-        <v>188</v>
-      </c>
-      <c r="N37" s="14"/>
       <c r="O37" s="14"/>
-      <c r="P37" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="Q37" s="14"/>
+      <c r="P37" s="14"/>
+      <c r="Q37" s="14" t="s">
+        <v>184</v>
+      </c>
       <c r="R37" s="14"/>
-      <c r="S37" s="6" t="s">
+      <c r="S37" s="14"/>
+      <c r="T37" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="T37" s="6"/>
-      <c r="U37" s="6"/>
-      <c r="V37" s="7" t="s">
+      <c r="U37" s="7"/>
+      <c r="V37" s="7"/>
+      <c r="W37" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="W37" s="7"/>
       <c r="X37" s="7"/>
-      <c r="Y37" s="14" t="s">
-        <v>189</v>
-      </c>
-      <c r="Z37" s="14"/>
+      <c r="Y37" s="7"/>
+      <c r="Z37" s="14" t="s">
+        <v>170</v>
+      </c>
       <c r="AA37" s="14"/>
-      <c r="AB37" s="14" t="s">
+      <c r="AB37" s="14"/>
+      <c r="AC37" s="21" t="s">
         <v>171</v>
       </c>
-      <c r="AC37" s="14"/>
-      <c r="AD37" s="14"/>
-      <c r="AE37" s="6"/>
+      <c r="AD37" s="21"/>
+      <c r="AE37" s="21"/>
       <c r="AF37" s="6"/>
       <c r="AG37" s="6"/>
-      <c r="AH37" s="14" t="s">
-        <v>190</v>
-      </c>
-      <c r="AI37" s="14"/>
-      <c r="AJ37" s="14"/>
+      <c r="AH37" s="6"/>
+      <c r="AI37" s="6"/>
+      <c r="AJ37" s="6"/>
       <c r="AK37" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="AL37" s="6"/>
+      <c r="AL37" s="6" t="s">
+        <v>43</v>
+      </c>
       <c r="AM37" s="6"/>
       <c r="AN37" s="6"/>
       <c r="AO37" s="6"/>
@@ -4967,50 +4973,60 @@
       <c r="B38" s="7"/>
       <c r="C38" s="7"/>
       <c r="D38" s="7"/>
-      <c r="E38" s="7"/>
+      <c r="E38" s="7" t="s">
+        <v>57</v>
+      </c>
       <c r="F38" s="7"/>
-      <c r="G38" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="H38" s="7"/>
+      <c r="G38" s="7"/>
+      <c r="H38" s="7" t="s">
+        <v>58</v>
+      </c>
       <c r="I38" s="7"/>
-      <c r="J38" s="7" t="s">
-        <v>58</v>
-      </c>
+      <c r="J38" s="7"/>
       <c r="K38" s="7"/>
       <c r="L38" s="7"/>
       <c r="M38" s="7"/>
-      <c r="N38" s="7"/>
+      <c r="N38" s="7" t="s">
+        <v>60</v>
+      </c>
       <c r="O38" s="7"/>
-      <c r="P38" s="27" t="s">
+      <c r="P38" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="Q38" s="27"/>
-      <c r="R38" s="27"/>
-      <c r="S38" s="27"/>
-      <c r="T38" s="27"/>
-      <c r="U38" s="27"/>
-      <c r="V38" s="7"/>
-      <c r="W38" s="7"/>
+      <c r="Q38" s="7"/>
+      <c r="R38" s="7"/>
+      <c r="S38" s="7"/>
+      <c r="T38" s="7"/>
+      <c r="U38" s="7"/>
+      <c r="V38" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="W38" s="7" t="s">
+        <v>2</v>
+      </c>
       <c r="X38" s="7"/>
       <c r="Y38" s="7"/>
-      <c r="Z38" s="7"/>
+      <c r="Z38" s="7" t="s">
+        <v>2</v>
+      </c>
       <c r="AA38" s="7"/>
-      <c r="AB38" s="12"/>
-      <c r="AC38" s="12"/>
-      <c r="AD38" s="12"/>
-      <c r="AE38" s="7" t="s">
+      <c r="AB38" s="7"/>
+      <c r="AC38" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD38" s="7"/>
+      <c r="AE38" s="7"/>
+      <c r="AF38" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="AF38" s="7"/>
       <c r="AG38" s="7"/>
-      <c r="AH38" s="12"/>
+      <c r="AH38" s="7"/>
       <c r="AI38" s="12"/>
       <c r="AJ38" s="12"/>
-      <c r="AK38" s="6"/>
+      <c r="AK38" s="12"/>
       <c r="AL38" s="6"/>
-      <c r="AM38" s="12"/>
-      <c r="AN38" s="12"/>
+      <c r="AM38" s="6"/>
+      <c r="AN38" s="6"/>
       <c r="AO38" s="12"/>
       <c r="AP38" s="12"/>
       <c r="AQ38" s="12"/>
@@ -5076,25 +5092,25 @@
       <c r="M39" s="7"/>
       <c r="N39" s="7"/>
       <c r="O39" s="7"/>
-      <c r="P39" s="27"/>
-      <c r="Q39" s="27"/>
-      <c r="R39" s="27"/>
-      <c r="S39" s="27"/>
-      <c r="T39" s="27"/>
-      <c r="U39" s="27"/>
+      <c r="P39" s="7"/>
+      <c r="Q39" s="7"/>
+      <c r="R39" s="7"/>
+      <c r="S39" s="7"/>
+      <c r="T39" s="7"/>
+      <c r="U39" s="7"/>
       <c r="V39" s="7"/>
       <c r="W39" s="7"/>
       <c r="X39" s="7"/>
       <c r="Y39" s="7"/>
       <c r="Z39" s="7"/>
       <c r="AA39" s="7"/>
-      <c r="AB39" s="12"/>
-      <c r="AC39" s="12"/>
-      <c r="AD39" s="12"/>
+      <c r="AB39" s="7"/>
+      <c r="AC39" s="7"/>
+      <c r="AD39" s="7"/>
       <c r="AE39" s="7"/>
       <c r="AF39" s="7"/>
       <c r="AG39" s="7"/>
-      <c r="AH39" s="6"/>
+      <c r="AH39" s="7"/>
       <c r="AI39" s="6"/>
       <c r="AJ39" s="6"/>
       <c r="AK39" s="6"/>
@@ -5155,50 +5171,50 @@
       <c r="CI39" s="24"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D40" s="28"/>
-      <c r="E40" s="28"/>
-      <c r="F40" s="28"/>
-      <c r="G40" s="29"/>
-      <c r="H40" s="29"/>
-      <c r="I40" s="29"/>
-      <c r="J40" s="29"/>
-      <c r="K40" s="29"/>
-      <c r="L40" s="29"/>
-      <c r="M40" s="29"/>
-      <c r="N40" s="29"/>
-      <c r="O40" s="29"/>
-      <c r="P40" s="29"/>
-      <c r="Q40" s="29"/>
-      <c r="R40" s="29"/>
-      <c r="S40" s="29"/>
-      <c r="T40" s="29"/>
-      <c r="U40" s="29"/>
-      <c r="V40" s="29"/>
-      <c r="W40" s="29"/>
-      <c r="X40" s="29"/>
-      <c r="Y40" s="29"/>
-      <c r="Z40" s="29"/>
-      <c r="AA40" s="29"/>
-      <c r="AB40" s="29"/>
-      <c r="AC40" s="29"/>
-      <c r="AD40" s="29"/>
-      <c r="AE40" s="29"/>
-      <c r="AF40" s="29"/>
-      <c r="AG40" s="29"/>
-      <c r="AH40" s="29"/>
-      <c r="AI40" s="29"/>
-      <c r="AJ40" s="29"/>
-      <c r="AK40" s="29"/>
-      <c r="AL40" s="29"/>
-      <c r="AM40" s="29"/>
-      <c r="AN40" s="29"/>
-      <c r="AO40" s="29"/>
-      <c r="AP40" s="29"/>
-      <c r="AQ40" s="30"/>
+      <c r="D40" s="26"/>
+      <c r="E40" s="26"/>
+      <c r="F40" s="26"/>
+      <c r="G40" s="27"/>
+      <c r="H40" s="27"/>
+      <c r="I40" s="27"/>
+      <c r="J40" s="27"/>
+      <c r="K40" s="27"/>
+      <c r="L40" s="27"/>
+      <c r="M40" s="27"/>
+      <c r="N40" s="27"/>
+      <c r="O40" s="27"/>
+      <c r="P40" s="27"/>
+      <c r="Q40" s="27"/>
+      <c r="R40" s="27"/>
+      <c r="S40" s="27"/>
+      <c r="T40" s="27"/>
+      <c r="U40" s="27"/>
+      <c r="V40" s="27"/>
+      <c r="W40" s="27"/>
+      <c r="X40" s="27"/>
+      <c r="Y40" s="27"/>
+      <c r="Z40" s="27"/>
+      <c r="AA40" s="27"/>
+      <c r="AB40" s="27"/>
+      <c r="AC40" s="27"/>
+      <c r="AD40" s="27"/>
+      <c r="AE40" s="27"/>
+      <c r="AF40" s="27"/>
+      <c r="AG40" s="27"/>
+      <c r="AH40" s="27"/>
+      <c r="AI40" s="27"/>
+      <c r="AJ40" s="27"/>
+      <c r="AK40" s="27"/>
+      <c r="AL40" s="27"/>
+      <c r="AM40" s="27"/>
+      <c r="AN40" s="27"/>
+      <c r="AO40" s="27"/>
+      <c r="AP40" s="27"/>
+      <c r="AQ40" s="28"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="16" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="16"/>
@@ -5392,50 +5408,50 @@
       <c r="AQ43" s="6"/>
       <c r="AS43" s="7"/>
       <c r="AT43" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="AU43" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="AV43" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="AW43" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="AU43" s="7" t="s">
+      <c r="AX43" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="AV43" s="7" t="s">
+      <c r="AY43" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="AW43" s="6" t="s">
+      <c r="AZ43" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="AX43" s="6" t="s">
+      <c r="BA43" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="AY43" s="6" t="s">
+      <c r="BB43" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="AZ43" s="6" t="s">
+      <c r="BC43" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="BA43" s="7" t="s">
+      <c r="BD43" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="BB43" s="6" t="s">
+      <c r="BE43" s="6" t="s">
         <v>200</v>
-      </c>
-      <c r="BC43" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="BD43" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="BE43" s="6" t="s">
-        <v>203</v>
       </c>
       <c r="BF43" s="6"/>
       <c r="BG43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="27" t="s">
+      <c r="A44" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="B44" s="27"/>
-      <c r="C44" s="27"/>
+      <c r="B44" s="29"/>
+      <c r="C44" s="29"/>
       <c r="D44" s="7"/>
       <c r="E44" s="7"/>
       <c r="F44" s="7"/>
@@ -5452,7 +5468,7 @@
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
       <c r="S44" s="19" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="T44" s="19"/>
       <c r="U44" s="19"/>
@@ -5482,7 +5498,7 @@
       <c r="AO44" s="6"/>
       <c r="AP44" s="6"/>
       <c r="AQ44" s="6"/>
-      <c r="AS44" s="27" t="s">
+      <c r="AS44" s="29" t="s">
         <v>91</v>
       </c>
       <c r="AT44" s="14" t="s">
@@ -5542,7 +5558,7 @@
       <c r="Q45" s="7"/>
       <c r="R45" s="7"/>
       <c r="S45" s="19" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="T45" s="19"/>
       <c r="U45" s="19"/>
@@ -5622,14 +5638,14 @@
       <c r="M46" s="7"/>
       <c r="N46" s="7"/>
       <c r="O46" s="7"/>
-      <c r="P46" s="27" t="s">
+      <c r="P46" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="Q46" s="27"/>
-      <c r="R46" s="27"/>
-      <c r="S46" s="27"/>
-      <c r="T46" s="27"/>
-      <c r="U46" s="27"/>
+      <c r="Q46" s="29"/>
+      <c r="R46" s="29"/>
+      <c r="S46" s="29"/>
+      <c r="T46" s="29"/>
+      <c r="U46" s="29"/>
       <c r="V46" s="6"/>
       <c r="W46" s="6"/>
       <c r="X46" s="6"/>
@@ -5664,17 +5680,17 @@
       <c r="AV46" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AW46" s="27" t="s">
+      <c r="AW46" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="AX46" s="27" t="s">
+      <c r="AX46" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="AY46" s="27"/>
-      <c r="AZ46" s="27" t="s">
+      <c r="AY46" s="29"/>
+      <c r="AZ46" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="BA46" s="27" t="s">
+      <c r="BA46" s="29" t="s">
         <v>115</v>
       </c>
       <c r="BB46" s="12"/>
@@ -5702,12 +5718,12 @@
       <c r="M47" s="7"/>
       <c r="N47" s="7"/>
       <c r="O47" s="7"/>
-      <c r="P47" s="27"/>
-      <c r="Q47" s="27"/>
-      <c r="R47" s="27"/>
-      <c r="S47" s="27"/>
-      <c r="T47" s="27"/>
-      <c r="U47" s="27"/>
+      <c r="P47" s="29"/>
+      <c r="Q47" s="29"/>
+      <c r="R47" s="29"/>
+      <c r="S47" s="29"/>
+      <c r="T47" s="29"/>
+      <c r="U47" s="29"/>
       <c r="V47" s="6"/>
       <c r="W47" s="6"/>
       <c r="X47" s="6"/>
@@ -5736,9 +5752,9 @@
       <c r="AV47" s="7"/>
       <c r="AW47" s="7"/>
       <c r="AX47" s="7"/>
-      <c r="AY47" s="27"/>
-      <c r="AZ47" s="27"/>
-      <c r="BA47" s="27"/>
+      <c r="AY47" s="29"/>
+      <c r="AZ47" s="29"/>
+      <c r="BA47" s="29"/>
       <c r="BB47" s="12"/>
       <c r="BC47" s="6"/>
       <c r="BD47" s="6"/>
@@ -5747,49 +5763,49 @@
       <c r="BG47" s="6"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="28"/>
-      <c r="B48" s="28"/>
-      <c r="C48" s="28"/>
-      <c r="D48" s="28"/>
-      <c r="E48" s="28"/>
-      <c r="F48" s="28"/>
-      <c r="G48" s="29"/>
-      <c r="H48" s="29"/>
-      <c r="I48" s="29"/>
-      <c r="J48" s="29"/>
-      <c r="K48" s="29"/>
-      <c r="L48" s="29"/>
-      <c r="M48" s="29"/>
-      <c r="N48" s="29"/>
-      <c r="O48" s="29"/>
-      <c r="P48" s="29"/>
-      <c r="Q48" s="29"/>
-      <c r="R48" s="29"/>
-      <c r="S48" s="29"/>
-      <c r="T48" s="29"/>
-      <c r="U48" s="29"/>
-      <c r="V48" s="29"/>
-      <c r="W48" s="29"/>
-      <c r="X48" s="29"/>
-      <c r="Y48" s="29"/>
-      <c r="Z48" s="29"/>
-      <c r="AA48" s="29"/>
-      <c r="AB48" s="29"/>
-      <c r="AC48" s="29"/>
-      <c r="AD48" s="29"/>
-      <c r="AE48" s="29"/>
-      <c r="AF48" s="29"/>
-      <c r="AG48" s="29"/>
-      <c r="AH48" s="29"/>
-      <c r="AI48" s="29"/>
-      <c r="AJ48" s="29"/>
-      <c r="AK48" s="29"/>
-      <c r="AL48" s="29"/>
-      <c r="AM48" s="29"/>
-      <c r="AN48" s="29"/>
-      <c r="AO48" s="29"/>
-      <c r="AP48" s="29"/>
-      <c r="AQ48" s="30"/>
+      <c r="A48" s="26"/>
+      <c r="B48" s="26"/>
+      <c r="C48" s="26"/>
+      <c r="D48" s="26"/>
+      <c r="E48" s="26"/>
+      <c r="F48" s="26"/>
+      <c r="G48" s="27"/>
+      <c r="H48" s="27"/>
+      <c r="I48" s="27"/>
+      <c r="J48" s="27"/>
+      <c r="K48" s="27"/>
+      <c r="L48" s="27"/>
+      <c r="M48" s="27"/>
+      <c r="N48" s="27"/>
+      <c r="O48" s="27"/>
+      <c r="P48" s="27"/>
+      <c r="Q48" s="27"/>
+      <c r="R48" s="27"/>
+      <c r="S48" s="27"/>
+      <c r="T48" s="27"/>
+      <c r="U48" s="27"/>
+      <c r="V48" s="27"/>
+      <c r="W48" s="27"/>
+      <c r="X48" s="27"/>
+      <c r="Y48" s="27"/>
+      <c r="Z48" s="27"/>
+      <c r="AA48" s="27"/>
+      <c r="AB48" s="27"/>
+      <c r="AC48" s="27"/>
+      <c r="AD48" s="27"/>
+      <c r="AE48" s="27"/>
+      <c r="AF48" s="27"/>
+      <c r="AG48" s="27"/>
+      <c r="AH48" s="27"/>
+      <c r="AI48" s="27"/>
+      <c r="AJ48" s="27"/>
+      <c r="AK48" s="27"/>
+      <c r="AL48" s="27"/>
+      <c r="AM48" s="27"/>
+      <c r="AN48" s="27"/>
+      <c r="AO48" s="27"/>
+      <c r="AP48" s="27"/>
+      <c r="AQ48" s="28"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3"/>
@@ -5836,7 +5852,7 @@
       <c r="AP49" s="4"/>
       <c r="AQ49" s="5"/>
       <c r="AS49" s="3" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="AY49" s="1"/>
     </row>
@@ -6124,7 +6140,7 @@
       <c r="AT52" s="7"/>
       <c r="AU52" s="7"/>
       <c r="AV52" s="7"/>
-      <c r="AW52" s="31"/>
+      <c r="AW52" s="30"/>
       <c r="AX52" s="6"/>
       <c r="AY52" s="14" t="s">
         <v>6</v>
@@ -6723,7 +6739,7 @@
       <c r="AR62" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="638">
+  <mergeCells count="695">
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
@@ -7227,6 +7243,20 @@
     <mergeCell ref="CA31:CC31"/>
     <mergeCell ref="CD31:CF31"/>
     <mergeCell ref="CG31:CI31"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="E34:G34"/>
+    <mergeCell ref="H34:J34"/>
+    <mergeCell ref="K34:M34"/>
+    <mergeCell ref="N34:P34"/>
+    <mergeCell ref="Q34:S34"/>
+    <mergeCell ref="T34:V34"/>
+    <mergeCell ref="W34:Y34"/>
+    <mergeCell ref="Z34:AB34"/>
+    <mergeCell ref="AC34:AE34"/>
+    <mergeCell ref="AF34:AH34"/>
+    <mergeCell ref="AI34:AK34"/>
+    <mergeCell ref="AL34:AN34"/>
+    <mergeCell ref="AO34:AQ34"/>
     <mergeCell ref="AT34:AV34"/>
     <mergeCell ref="AW34:AY34"/>
     <mergeCell ref="AZ34:BB34"/>
@@ -7241,7 +7271,20 @@
     <mergeCell ref="CA34:CC34"/>
     <mergeCell ref="CD34:CF34"/>
     <mergeCell ref="CG34:CI34"/>
-    <mergeCell ref="AM35:AQ36"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="I35:K35"/>
+    <mergeCell ref="L35:N35"/>
+    <mergeCell ref="O35:Q35"/>
+    <mergeCell ref="R35:T35"/>
+    <mergeCell ref="U35:W35"/>
+    <mergeCell ref="X35:Z35"/>
+    <mergeCell ref="AA35:AC35"/>
+    <mergeCell ref="AD35:AF35"/>
+    <mergeCell ref="AG35:AI35"/>
+    <mergeCell ref="AJ35:AL35"/>
+    <mergeCell ref="AM35:AQ35"/>
     <mergeCell ref="AS35:AT35"/>
     <mergeCell ref="AU35:AW35"/>
     <mergeCell ref="AX35:AZ35"/>
@@ -7256,6 +7299,20 @@
     <mergeCell ref="BY35:CA35"/>
     <mergeCell ref="CB35:CD35"/>
     <mergeCell ref="CE35:CI35"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="D36:F36"/>
+    <mergeCell ref="G36:I36"/>
+    <mergeCell ref="J36:L36"/>
+    <mergeCell ref="M36:O36"/>
+    <mergeCell ref="P36:R36"/>
+    <mergeCell ref="S36:U36"/>
+    <mergeCell ref="V36:X36"/>
+    <mergeCell ref="Y36:AA36"/>
+    <mergeCell ref="AB36:AD36"/>
+    <mergeCell ref="AE36:AG36"/>
+    <mergeCell ref="AH36:AJ36"/>
+    <mergeCell ref="AK36:AM36"/>
+    <mergeCell ref="AN36:AQ36"/>
     <mergeCell ref="AS36:AU36"/>
     <mergeCell ref="AV36:AX36"/>
     <mergeCell ref="AY36:BA36"/>
@@ -7270,7 +7327,19 @@
     <mergeCell ref="BZ36:CB36"/>
     <mergeCell ref="CC36:CE36"/>
     <mergeCell ref="CF36:CI36"/>
-    <mergeCell ref="AK37:AQ37"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="E37:G37"/>
+    <mergeCell ref="H37:J37"/>
+    <mergeCell ref="K37:M37"/>
+    <mergeCell ref="N37:P37"/>
+    <mergeCell ref="Q37:S37"/>
+    <mergeCell ref="T37:V37"/>
+    <mergeCell ref="W37:Y37"/>
+    <mergeCell ref="Z37:AB37"/>
+    <mergeCell ref="AC37:AE37"/>
+    <mergeCell ref="AF37:AH37"/>
+    <mergeCell ref="AI37:AK37"/>
+    <mergeCell ref="AL37:AQ37"/>
     <mergeCell ref="AS37:AV37"/>
     <mergeCell ref="AW37:AY37"/>
     <mergeCell ref="AZ37:BB37"/>
@@ -7285,15 +7354,17 @@
     <mergeCell ref="CA37:CC37"/>
     <mergeCell ref="CD37:CI37"/>
     <mergeCell ref="A38:A39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="G38:G39"/>
-    <mergeCell ref="J38:J39"/>
-    <mergeCell ref="M38:M39"/>
-    <mergeCell ref="P38:S39"/>
-    <mergeCell ref="V38:V39"/>
-    <mergeCell ref="Y38:Y39"/>
-    <mergeCell ref="AE38:AE39"/>
-    <mergeCell ref="AM38:AQ38"/>
+    <mergeCell ref="B38:D39"/>
+    <mergeCell ref="E38:G39"/>
+    <mergeCell ref="H38:J39"/>
+    <mergeCell ref="K38:M39"/>
+    <mergeCell ref="N38:V39"/>
+    <mergeCell ref="W38:Y39"/>
+    <mergeCell ref="Z38:AB39"/>
+    <mergeCell ref="AC38:AE39"/>
+    <mergeCell ref="AF38:AH39"/>
+    <mergeCell ref="AI38:AK38"/>
+    <mergeCell ref="AL38:AN38"/>
     <mergeCell ref="AS38:AS39"/>
     <mergeCell ref="AT38:AV39"/>
     <mergeCell ref="AW38:AY39"/>
@@ -7306,7 +7377,9 @@
     <mergeCell ref="BX38:BZ39"/>
     <mergeCell ref="CA38:CC38"/>
     <mergeCell ref="CD38:CF38"/>
-    <mergeCell ref="AM39:AQ39"/>
+    <mergeCell ref="AI39:AK39"/>
+    <mergeCell ref="AL39:AN39"/>
+    <mergeCell ref="AO39:AQ39"/>
     <mergeCell ref="CA39:CC39"/>
     <mergeCell ref="CD39:CF39"/>
     <mergeCell ref="CG39:CI39"/>
@@ -8306,7 +8379,7 @@
       <c r="AK11" s="6"/>
       <c r="AL11" s="6"/>
       <c r="AM11" s="6" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="AN11" s="6"/>
       <c r="AO11" s="6"/>
@@ -10608,11 +10681,11 @@
       </c>
       <c r="H34" s="7"/>
       <c r="I34" s="7"/>
-      <c r="J34" s="25" t="s">
-        <v>177</v>
-      </c>
-      <c r="K34" s="25"/>
-      <c r="L34" s="25"/>
+      <c r="J34" s="31" t="s">
+        <v>205</v>
+      </c>
+      <c r="K34" s="31"/>
+      <c r="L34" s="31"/>
       <c r="M34" s="6" t="s">
         <v>121</v>
       </c>
@@ -10732,18 +10805,18 @@
       </c>
       <c r="H35" s="14"/>
       <c r="I35" s="14"/>
-      <c r="J35" s="26" t="s">
+      <c r="J35" s="25" t="s">
+        <v>206</v>
+      </c>
+      <c r="K35" s="25"/>
+      <c r="L35" s="25"/>
+      <c r="M35" s="14" t="s">
         <v>178</v>
-      </c>
-      <c r="K35" s="26"/>
-      <c r="L35" s="26"/>
-      <c r="M35" s="14" t="s">
-        <v>179</v>
       </c>
       <c r="N35" s="14"/>
       <c r="O35" s="14"/>
       <c r="P35" s="14" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="Q35" s="14"/>
       <c r="R35" s="14"/>
@@ -10847,12 +10920,12 @@
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E36" s="14"/>
       <c r="F36" s="14"/>
       <c r="G36" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H36" s="14"/>
       <c r="I36" s="14"/>
@@ -10867,7 +10940,7 @@
       <c r="N36" s="9"/>
       <c r="O36" s="9"/>
       <c r="P36" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Q36" s="14"/>
       <c r="R36" s="14"/>
@@ -10897,7 +10970,7 @@
       <c r="AF36" s="14"/>
       <c r="AG36" s="14"/>
       <c r="AH36" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AI36" s="14"/>
       <c r="AJ36" s="14"/>
@@ -10973,27 +11046,27 @@
       <c r="B37" s="7"/>
       <c r="C37" s="7"/>
       <c r="D37" s="14" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E37" s="14"/>
       <c r="F37" s="14"/>
       <c r="G37" s="14" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H37" s="14"/>
       <c r="I37" s="14"/>
       <c r="J37" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="K37" s="14"/>
       <c r="L37" s="14"/>
       <c r="M37" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="N37" s="14"/>
       <c r="O37" s="14"/>
       <c r="P37" s="14" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="Q37" s="14"/>
       <c r="R37" s="14"/>
@@ -11008,7 +11081,7 @@
       <c r="W37" s="7"/>
       <c r="X37" s="7"/>
       <c r="Y37" s="14" t="s">
-        <v>189</v>
+        <v>207</v>
       </c>
       <c r="Z37" s="14"/>
       <c r="AA37" s="14"/>
@@ -11021,7 +11094,7 @@
       <c r="AF37" s="6"/>
       <c r="AG37" s="6"/>
       <c r="AH37" s="14" t="s">
-        <v>190</v>
+        <v>208</v>
       </c>
       <c r="AI37" s="14"/>
       <c r="AJ37" s="14"/>
@@ -11108,14 +11181,14 @@
       <c r="M38" s="7"/>
       <c r="N38" s="7"/>
       <c r="O38" s="7"/>
-      <c r="P38" s="27" t="s">
+      <c r="P38" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="Q38" s="27"/>
-      <c r="R38" s="27"/>
-      <c r="S38" s="27"/>
-      <c r="T38" s="27"/>
-      <c r="U38" s="27"/>
+      <c r="Q38" s="29"/>
+      <c r="R38" s="29"/>
+      <c r="S38" s="29"/>
+      <c r="T38" s="29"/>
+      <c r="U38" s="29"/>
       <c r="V38" s="7"/>
       <c r="W38" s="7"/>
       <c r="X38" s="7"/>
@@ -11202,12 +11275,12 @@
       <c r="M39" s="7"/>
       <c r="N39" s="7"/>
       <c r="O39" s="7"/>
-      <c r="P39" s="27"/>
-      <c r="Q39" s="27"/>
-      <c r="R39" s="27"/>
-      <c r="S39" s="27"/>
-      <c r="T39" s="27"/>
-      <c r="U39" s="27"/>
+      <c r="P39" s="29"/>
+      <c r="Q39" s="29"/>
+      <c r="R39" s="29"/>
+      <c r="S39" s="29"/>
+      <c r="T39" s="29"/>
+      <c r="U39" s="29"/>
       <c r="V39" s="7"/>
       <c r="W39" s="7"/>
       <c r="X39" s="7"/>
@@ -11281,50 +11354,50 @@
       <c r="CI39" s="24"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D40" s="28"/>
-      <c r="E40" s="28"/>
-      <c r="F40" s="28"/>
-      <c r="G40" s="29"/>
-      <c r="H40" s="29"/>
-      <c r="I40" s="29"/>
-      <c r="J40" s="29"/>
-      <c r="K40" s="29"/>
-      <c r="L40" s="29"/>
-      <c r="M40" s="29"/>
-      <c r="N40" s="29"/>
-      <c r="O40" s="29"/>
-      <c r="P40" s="29"/>
-      <c r="Q40" s="29"/>
-      <c r="R40" s="29"/>
-      <c r="S40" s="29"/>
-      <c r="T40" s="29"/>
-      <c r="U40" s="29"/>
-      <c r="V40" s="29"/>
-      <c r="W40" s="29"/>
-      <c r="X40" s="29"/>
-      <c r="Y40" s="29"/>
-      <c r="Z40" s="29"/>
-      <c r="AA40" s="29"/>
-      <c r="AB40" s="29"/>
-      <c r="AC40" s="29"/>
-      <c r="AD40" s="29"/>
-      <c r="AE40" s="29"/>
-      <c r="AF40" s="29"/>
-      <c r="AG40" s="29"/>
-      <c r="AH40" s="29"/>
-      <c r="AI40" s="29"/>
-      <c r="AJ40" s="29"/>
-      <c r="AK40" s="29"/>
-      <c r="AL40" s="29"/>
-      <c r="AM40" s="29"/>
-      <c r="AN40" s="29"/>
-      <c r="AO40" s="29"/>
-      <c r="AP40" s="29"/>
-      <c r="AQ40" s="30"/>
+      <c r="D40" s="26"/>
+      <c r="E40" s="26"/>
+      <c r="F40" s="26"/>
+      <c r="G40" s="27"/>
+      <c r="H40" s="27"/>
+      <c r="I40" s="27"/>
+      <c r="J40" s="27"/>
+      <c r="K40" s="27"/>
+      <c r="L40" s="27"/>
+      <c r="M40" s="27"/>
+      <c r="N40" s="27"/>
+      <c r="O40" s="27"/>
+      <c r="P40" s="27"/>
+      <c r="Q40" s="27"/>
+      <c r="R40" s="27"/>
+      <c r="S40" s="27"/>
+      <c r="T40" s="27"/>
+      <c r="U40" s="27"/>
+      <c r="V40" s="27"/>
+      <c r="W40" s="27"/>
+      <c r="X40" s="27"/>
+      <c r="Y40" s="27"/>
+      <c r="Z40" s="27"/>
+      <c r="AA40" s="27"/>
+      <c r="AB40" s="27"/>
+      <c r="AC40" s="27"/>
+      <c r="AD40" s="27"/>
+      <c r="AE40" s="27"/>
+      <c r="AF40" s="27"/>
+      <c r="AG40" s="27"/>
+      <c r="AH40" s="27"/>
+      <c r="AI40" s="27"/>
+      <c r="AJ40" s="27"/>
+      <c r="AK40" s="27"/>
+      <c r="AL40" s="27"/>
+      <c r="AM40" s="27"/>
+      <c r="AN40" s="27"/>
+      <c r="AO40" s="27"/>
+      <c r="AP40" s="27"/>
+      <c r="AQ40" s="28"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="16" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="16"/>
@@ -11518,50 +11591,50 @@
       <c r="AQ43" s="6"/>
       <c r="AS43" s="7"/>
       <c r="AT43" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="AU43" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="AV43" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="AW43" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="AU43" s="7" t="s">
+      <c r="AX43" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="AV43" s="7" t="s">
+      <c r="AY43" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="AW43" s="6" t="s">
+      <c r="AZ43" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="AX43" s="6" t="s">
+      <c r="BA43" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="AY43" s="6" t="s">
+      <c r="BB43" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="AZ43" s="6" t="s">
+      <c r="BC43" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="BA43" s="7" t="s">
+      <c r="BD43" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="BB43" s="6" t="s">
+      <c r="BE43" s="6" t="s">
         <v>200</v>
-      </c>
-      <c r="BC43" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="BD43" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="BE43" s="6" t="s">
-        <v>203</v>
       </c>
       <c r="BF43" s="6"/>
       <c r="BG43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="27" t="s">
+      <c r="A44" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="B44" s="27"/>
-      <c r="C44" s="27"/>
+      <c r="B44" s="29"/>
+      <c r="C44" s="29"/>
       <c r="D44" s="7"/>
       <c r="E44" s="7"/>
       <c r="F44" s="7"/>
@@ -11578,7 +11651,7 @@
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
       <c r="S44" s="19" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="T44" s="19"/>
       <c r="U44" s="19"/>
@@ -11608,7 +11681,7 @@
       <c r="AO44" s="6"/>
       <c r="AP44" s="6"/>
       <c r="AQ44" s="6"/>
-      <c r="AS44" s="27" t="s">
+      <c r="AS44" s="29" t="s">
         <v>91</v>
       </c>
       <c r="AT44" s="14" t="s">
@@ -11668,7 +11741,7 @@
       <c r="Q45" s="7"/>
       <c r="R45" s="7"/>
       <c r="S45" s="19" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="T45" s="19"/>
       <c r="U45" s="19"/>
@@ -11748,14 +11821,14 @@
       <c r="M46" s="7"/>
       <c r="N46" s="7"/>
       <c r="O46" s="7"/>
-      <c r="P46" s="27" t="s">
+      <c r="P46" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="Q46" s="27"/>
-      <c r="R46" s="27"/>
-      <c r="S46" s="27"/>
-      <c r="T46" s="27"/>
-      <c r="U46" s="27"/>
+      <c r="Q46" s="29"/>
+      <c r="R46" s="29"/>
+      <c r="S46" s="29"/>
+      <c r="T46" s="29"/>
+      <c r="U46" s="29"/>
       <c r="V46" s="6"/>
       <c r="W46" s="6"/>
       <c r="X46" s="6"/>
@@ -11790,17 +11863,17 @@
       <c r="AV46" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AW46" s="27" t="s">
+      <c r="AW46" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="AX46" s="27" t="s">
+      <c r="AX46" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="AY46" s="27"/>
-      <c r="AZ46" s="27" t="s">
+      <c r="AY46" s="29"/>
+      <c r="AZ46" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="BA46" s="27" t="s">
+      <c r="BA46" s="29" t="s">
         <v>115</v>
       </c>
       <c r="BB46" s="12"/>
@@ -11828,12 +11901,12 @@
       <c r="M47" s="7"/>
       <c r="N47" s="7"/>
       <c r="O47" s="7"/>
-      <c r="P47" s="27"/>
-      <c r="Q47" s="27"/>
-      <c r="R47" s="27"/>
-      <c r="S47" s="27"/>
-      <c r="T47" s="27"/>
-      <c r="U47" s="27"/>
+      <c r="P47" s="29"/>
+      <c r="Q47" s="29"/>
+      <c r="R47" s="29"/>
+      <c r="S47" s="29"/>
+      <c r="T47" s="29"/>
+      <c r="U47" s="29"/>
       <c r="V47" s="6"/>
       <c r="W47" s="6"/>
       <c r="X47" s="6"/>
@@ -11862,9 +11935,9 @@
       <c r="AV47" s="7"/>
       <c r="AW47" s="7"/>
       <c r="AX47" s="7"/>
-      <c r="AY47" s="27"/>
-      <c r="AZ47" s="27"/>
-      <c r="BA47" s="27"/>
+      <c r="AY47" s="29"/>
+      <c r="AZ47" s="29"/>
+      <c r="BA47" s="29"/>
       <c r="BB47" s="12"/>
       <c r="BC47" s="6"/>
       <c r="BD47" s="6"/>
@@ -11873,49 +11946,49 @@
       <c r="BG47" s="6"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="28"/>
-      <c r="B48" s="28"/>
-      <c r="C48" s="28"/>
-      <c r="D48" s="28"/>
-      <c r="E48" s="28"/>
-      <c r="F48" s="28"/>
-      <c r="G48" s="29"/>
-      <c r="H48" s="29"/>
-      <c r="I48" s="29"/>
-      <c r="J48" s="29"/>
-      <c r="K48" s="29"/>
-      <c r="L48" s="29"/>
-      <c r="M48" s="29"/>
-      <c r="N48" s="29"/>
-      <c r="O48" s="29"/>
-      <c r="P48" s="29"/>
-      <c r="Q48" s="29"/>
-      <c r="R48" s="29"/>
-      <c r="S48" s="29"/>
-      <c r="T48" s="29"/>
-      <c r="U48" s="29"/>
-      <c r="V48" s="29"/>
-      <c r="W48" s="29"/>
-      <c r="X48" s="29"/>
-      <c r="Y48" s="29"/>
-      <c r="Z48" s="29"/>
-      <c r="AA48" s="29"/>
-      <c r="AB48" s="29"/>
-      <c r="AC48" s="29"/>
-      <c r="AD48" s="29"/>
-      <c r="AE48" s="29"/>
-      <c r="AF48" s="29"/>
-      <c r="AG48" s="29"/>
-      <c r="AH48" s="29"/>
-      <c r="AI48" s="29"/>
-      <c r="AJ48" s="29"/>
-      <c r="AK48" s="29"/>
-      <c r="AL48" s="29"/>
-      <c r="AM48" s="29"/>
-      <c r="AN48" s="29"/>
-      <c r="AO48" s="29"/>
-      <c r="AP48" s="29"/>
-      <c r="AQ48" s="30"/>
+      <c r="A48" s="26"/>
+      <c r="B48" s="26"/>
+      <c r="C48" s="26"/>
+      <c r="D48" s="26"/>
+      <c r="E48" s="26"/>
+      <c r="F48" s="26"/>
+      <c r="G48" s="27"/>
+      <c r="H48" s="27"/>
+      <c r="I48" s="27"/>
+      <c r="J48" s="27"/>
+      <c r="K48" s="27"/>
+      <c r="L48" s="27"/>
+      <c r="M48" s="27"/>
+      <c r="N48" s="27"/>
+      <c r="O48" s="27"/>
+      <c r="P48" s="27"/>
+      <c r="Q48" s="27"/>
+      <c r="R48" s="27"/>
+      <c r="S48" s="27"/>
+      <c r="T48" s="27"/>
+      <c r="U48" s="27"/>
+      <c r="V48" s="27"/>
+      <c r="W48" s="27"/>
+      <c r="X48" s="27"/>
+      <c r="Y48" s="27"/>
+      <c r="Z48" s="27"/>
+      <c r="AA48" s="27"/>
+      <c r="AB48" s="27"/>
+      <c r="AC48" s="27"/>
+      <c r="AD48" s="27"/>
+      <c r="AE48" s="27"/>
+      <c r="AF48" s="27"/>
+      <c r="AG48" s="27"/>
+      <c r="AH48" s="27"/>
+      <c r="AI48" s="27"/>
+      <c r="AJ48" s="27"/>
+      <c r="AK48" s="27"/>
+      <c r="AL48" s="27"/>
+      <c r="AM48" s="27"/>
+      <c r="AN48" s="27"/>
+      <c r="AO48" s="27"/>
+      <c r="AP48" s="27"/>
+      <c r="AQ48" s="28"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3"/>
@@ -11962,7 +12035,7 @@
       <c r="AP49" s="4"/>
       <c r="AQ49" s="5"/>
       <c r="AS49" s="3" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="AY49" s="1"/>
     </row>
@@ -12250,7 +12323,7 @@
       <c r="AT52" s="7"/>
       <c r="AU52" s="7"/>
       <c r="AV52" s="7"/>
-      <c r="AW52" s="31"/>
+      <c r="AW52" s="30"/>
       <c r="AX52" s="6"/>
       <c r="AY52" s="14" t="s">
         <v>6</v>
@@ -13931,7 +14004,7 @@
       <c r="AP5" s="6"/>
       <c r="AQ5" s="6"/>
       <c r="AR5" s="32" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AT5" s="7"/>
       <c r="AU5" s="7"/>
@@ -13975,7 +14048,9 @@
       </c>
       <c r="J6" s="7"/>
       <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
+      <c r="L6" s="7" t="s">
+        <v>61</v>
+      </c>
       <c r="M6" s="7" t="s">
         <v>60</v>
       </c>
@@ -13985,21 +14060,23 @@
       </c>
       <c r="P6" s="7"/>
       <c r="Q6" s="7"/>
-      <c r="R6" s="7"/>
-      <c r="S6" s="7"/>
-      <c r="T6" s="7" t="s">
+      <c r="R6" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="S6" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="U6" s="7"/>
-      <c r="V6" s="7" t="s">
+      <c r="T6" s="7"/>
+      <c r="U6" s="7" t="s">
         <v>61</v>
       </c>
+      <c r="V6" s="7"/>
       <c r="W6" s="7"/>
       <c r="X6" s="7" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="Y6" s="7" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="Z6" s="7"/>
       <c r="AA6" s="7"/>
@@ -14170,7 +14247,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>66</v>
+        <v>211</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -14734,7 +14811,7 @@
       <c r="AP13" s="6"/>
       <c r="AQ13" s="6"/>
       <c r="AR13" s="32" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AT13" s="7"/>
       <c r="AU13" s="7"/>
@@ -14822,7 +14899,9 @@
       </c>
       <c r="J14" s="7"/>
       <c r="K14" s="7"/>
-      <c r="L14" s="7"/>
+      <c r="L14" s="7" t="s">
+        <v>61</v>
+      </c>
       <c r="M14" s="7" t="s">
         <v>60</v>
       </c>
@@ -14832,7 +14911,9 @@
       </c>
       <c r="P14" s="7"/>
       <c r="Q14" s="7"/>
-      <c r="R14" s="7"/>
+      <c r="R14" s="7" t="s">
+        <v>61</v>
+      </c>
       <c r="S14" s="7"/>
       <c r="T14" s="7" t="s">
         <v>60</v>
@@ -14843,10 +14924,10 @@
       </c>
       <c r="W14" s="7"/>
       <c r="X14" s="7" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="Y14" s="7" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="Z14" s="7"/>
       <c r="AA14" s="7"/>
@@ -15193,6 +15274,9 @@
       <c r="AO18" s="6"/>
       <c r="AP18" s="6"/>
       <c r="AQ18" s="6"/>
+      <c r="AR18" s="6" t="s">
+        <v>149</v>
+      </c>
       <c r="AT18" s="6"/>
       <c r="AU18" s="6" t="s">
         <v>130</v>
@@ -15331,6 +15415,9 @@
       <c r="AO19" s="6"/>
       <c r="AP19" s="6"/>
       <c r="AQ19" s="6"/>
+      <c r="AR19" s="6" t="s">
+        <v>150</v>
+      </c>
       <c r="AT19" s="6"/>
       <c r="AU19" s="6"/>
       <c r="AV19" s="7"/>
@@ -15455,6 +15542,9 @@
       <c r="AO20" s="10"/>
       <c r="AP20" s="10"/>
       <c r="AQ20" s="10"/>
+      <c r="AR20" s="6" t="s">
+        <v>168</v>
+      </c>
       <c r="AT20" s="7"/>
       <c r="AU20" s="7"/>
       <c r="AV20" s="7"/>
@@ -15587,6 +15677,9 @@
       <c r="AO21" s="6"/>
       <c r="AP21" s="6"/>
       <c r="AQ21" s="6"/>
+      <c r="AR21" s="32" t="s">
+        <v>209</v>
+      </c>
       <c r="AT21" s="7"/>
       <c r="AU21" s="7"/>
       <c r="AV21" s="7"/>
@@ -15669,7 +15762,9 @@
       </c>
       <c r="J22" s="7"/>
       <c r="K22" s="7"/>
-      <c r="L22" s="7"/>
+      <c r="L22" s="7" t="s">
+        <v>61</v>
+      </c>
       <c r="M22" s="7" t="s">
         <v>60</v>
       </c>
@@ -15679,7 +15774,9 @@
       </c>
       <c r="P22" s="7"/>
       <c r="Q22" s="7"/>
-      <c r="R22" s="7"/>
+      <c r="R22" s="7" t="s">
+        <v>61</v>
+      </c>
       <c r="S22" s="7"/>
       <c r="T22" s="7" t="s">
         <v>60</v>
@@ -15690,39 +15787,34 @@
       </c>
       <c r="W22" s="7"/>
       <c r="X22" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="Y22" s="7"/>
+        <v>210</v>
+      </c>
+      <c r="Y22" s="7" t="s">
+        <v>210</v>
+      </c>
       <c r="Z22" s="7"/>
-      <c r="AA22" s="7" t="s">
+      <c r="AA22" s="7"/>
+      <c r="AB22" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="AB22" s="7"/>
       <c r="AC22" s="7"/>
-      <c r="AD22" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="AD22" s="7"/>
       <c r="AE22" s="7"/>
       <c r="AF22" s="7"/>
-      <c r="AG22" s="7" t="s">
-        <v>42</v>
-      </c>
+      <c r="AG22" s="7"/>
       <c r="AH22" s="7"/>
       <c r="AI22" s="7"/>
-      <c r="AJ22" s="7" t="s">
-        <v>42</v>
-      </c>
+      <c r="AJ22" s="7"/>
       <c r="AK22" s="7"/>
       <c r="AL22" s="7"/>
-      <c r="AM22" s="7" t="s">
-        <v>114</v>
-      </c>
+      <c r="AM22" s="7"/>
       <c r="AN22" s="7"/>
       <c r="AO22" s="7"/>
-      <c r="AP22" s="7" t="s">
+      <c r="AP22" s="7"/>
+      <c r="AQ22" s="7"/>
+      <c r="AR22" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="AQ22" s="7"/>
       <c r="AT22" s="7" t="s">
         <v>55</v>
       </c>
@@ -15825,6 +15917,7 @@
       <c r="AO23" s="7"/>
       <c r="AP23" s="7"/>
       <c r="AQ23" s="7"/>
+      <c r="AR23" s="6"/>
       <c r="AT23" s="7"/>
       <c r="AU23" s="7"/>
       <c r="AV23" s="7"/>
@@ -16047,6 +16140,9 @@
       <c r="AO26" s="6"/>
       <c r="AP26" s="6"/>
       <c r="AQ26" s="6"/>
+      <c r="AR26" s="6" t="s">
+        <v>149</v>
+      </c>
       <c r="AT26" s="7"/>
       <c r="AU26" s="7"/>
       <c r="AV26" s="7"/>
@@ -16159,6 +16255,9 @@
       <c r="AO27" s="6"/>
       <c r="AP27" s="6"/>
       <c r="AQ27" s="6"/>
+      <c r="AR27" s="6" t="s">
+        <v>150</v>
+      </c>
       <c r="AT27" s="7"/>
       <c r="AU27" s="7"/>
       <c r="AV27" s="7"/>
@@ -16281,6 +16380,9 @@
       <c r="AO28" s="10"/>
       <c r="AP28" s="10"/>
       <c r="AQ28" s="10"/>
+      <c r="AR28" s="6" t="s">
+        <v>168</v>
+      </c>
       <c r="AT28" s="7"/>
       <c r="AU28" s="7"/>
       <c r="AV28" s="7"/>
@@ -16401,6 +16503,9 @@
       <c r="AO29" s="6"/>
       <c r="AP29" s="6"/>
       <c r="AQ29" s="6"/>
+      <c r="AR29" s="32" t="s">
+        <v>209</v>
+      </c>
       <c r="AT29" s="7"/>
       <c r="AU29" s="7"/>
       <c r="AV29" s="7"/>
@@ -16471,7 +16576,9 @@
       </c>
       <c r="J30" s="7"/>
       <c r="K30" s="7"/>
-      <c r="L30" s="7"/>
+      <c r="L30" s="7" t="s">
+        <v>61</v>
+      </c>
       <c r="M30" s="7" t="s">
         <v>60</v>
       </c>
@@ -16481,7 +16588,9 @@
       </c>
       <c r="P30" s="7"/>
       <c r="Q30" s="7"/>
-      <c r="R30" s="7"/>
+      <c r="R30" s="7" t="s">
+        <v>61</v>
+      </c>
       <c r="S30" s="7"/>
       <c r="T30" s="7" t="s">
         <v>60</v>
@@ -16492,39 +16601,34 @@
       </c>
       <c r="W30" s="7"/>
       <c r="X30" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="Y30" s="7"/>
+        <v>210</v>
+      </c>
+      <c r="Y30" s="7" t="s">
+        <v>210</v>
+      </c>
       <c r="Z30" s="7"/>
-      <c r="AA30" s="7" t="s">
+      <c r="AA30" s="7"/>
+      <c r="AB30" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="AB30" s="7"/>
       <c r="AC30" s="7"/>
-      <c r="AD30" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="AD30" s="7"/>
       <c r="AE30" s="7"/>
       <c r="AF30" s="7"/>
-      <c r="AG30" s="7" t="s">
-        <v>41</v>
-      </c>
+      <c r="AG30" s="7"/>
       <c r="AH30" s="7"/>
       <c r="AI30" s="7"/>
-      <c r="AJ30" s="7" t="s">
-        <v>42</v>
-      </c>
+      <c r="AJ30" s="7"/>
       <c r="AK30" s="7"/>
       <c r="AL30" s="7"/>
-      <c r="AM30" s="7" t="s">
-        <v>114</v>
-      </c>
+      <c r="AM30" s="7"/>
       <c r="AN30" s="7"/>
       <c r="AO30" s="7"/>
-      <c r="AP30" s="7" t="s">
+      <c r="AP30" s="7"/>
+      <c r="AQ30" s="7"/>
+      <c r="AR30" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="AQ30" s="7"/>
       <c r="AT30" s="7" t="s">
         <v>55</v>
       </c>
@@ -16567,7 +16671,7 @@
       </c>
       <c r="BP30" s="7"/>
       <c r="BQ30" s="7" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="BR30" s="7"/>
       <c r="BS30" s="7"/>
@@ -16645,6 +16749,7 @@
       <c r="AO31" s="7"/>
       <c r="AP31" s="7"/>
       <c r="AQ31" s="7"/>
+      <c r="AR31" s="6"/>
       <c r="AT31" s="7"/>
       <c r="AU31" s="7"/>
       <c r="AV31" s="7"/>
@@ -16795,73 +16900,76 @@
       <c r="BH33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7"/>
-      <c r="B34" s="7"/>
-      <c r="C34" s="7"/>
-      <c r="D34" s="7" t="s">
+      <c r="A34" s="6"/>
+      <c r="B34" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="7" t="s">
+      <c r="C34" s="6"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="H34" s="7"/>
-      <c r="I34" s="7"/>
-      <c r="J34" s="25" t="s">
-        <v>177</v>
-      </c>
-      <c r="K34" s="25"/>
-      <c r="L34" s="25"/>
-      <c r="M34" s="6" t="s">
+      <c r="F34" s="6"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="I34" s="6"/>
+      <c r="J34" s="6"/>
+      <c r="K34" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="N34" s="6"/>
+      <c r="L34" s="6"/>
+      <c r="M34" s="6"/>
+      <c r="N34" s="6" t="s">
+        <v>122</v>
+      </c>
       <c r="O34" s="6"/>
-      <c r="P34" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q34" s="6"/>
+      <c r="P34" s="6"/>
+      <c r="Q34" s="6" t="s">
+        <v>123</v>
+      </c>
       <c r="R34" s="6"/>
-      <c r="S34" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="T34" s="6"/>
+      <c r="S34" s="6"/>
+      <c r="T34" s="6" t="s">
+        <v>124</v>
+      </c>
       <c r="U34" s="6"/>
-      <c r="V34" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="W34" s="6"/>
+      <c r="V34" s="6"/>
+      <c r="W34" s="6" t="s">
+        <v>125</v>
+      </c>
       <c r="X34" s="6"/>
-      <c r="Y34" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="Z34" s="7"/>
-      <c r="AA34" s="7"/>
-      <c r="AB34" s="6" t="s">
+      <c r="Y34" s="6"/>
+      <c r="Z34" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="AC34" s="6"/>
+      <c r="AA34" s="6"/>
+      <c r="AB34" s="6"/>
+      <c r="AC34" s="6" t="s">
+        <v>127</v>
+      </c>
       <c r="AD34" s="6"/>
-      <c r="AE34" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="AF34" s="6"/>
+      <c r="AE34" s="6"/>
+      <c r="AF34" s="6" t="s">
+        <v>128</v>
+      </c>
       <c r="AG34" s="6"/>
-      <c r="AH34" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="AI34" s="6"/>
+      <c r="AH34" s="6"/>
+      <c r="AI34" s="6" t="s">
+        <v>129</v>
+      </c>
       <c r="AJ34" s="6"/>
-      <c r="AK34" s="6" t="s">
-        <v>129</v>
-      </c>
+      <c r="AK34" s="6"/>
       <c r="AL34" s="6"/>
       <c r="AM34" s="6"/>
       <c r="AN34" s="6"/>
       <c r="AO34" s="6"/>
       <c r="AP34" s="6"/>
       <c r="AQ34" s="6"/>
+      <c r="AR34" s="6" t="s">
+        <v>149</v>
+      </c>
       <c r="AT34" s="7"/>
       <c r="AU34" s="7" t="s">
         <v>130</v>
@@ -16903,73 +17011,76 @@
       <c r="BH34" s="6"/>
     </row>
     <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7"/>
-      <c r="B35" s="7"/>
-      <c r="C35" s="7"/>
-      <c r="D35" s="14" t="s">
+      <c r="A35" s="6"/>
+      <c r="B35" s="6"/>
+      <c r="C35" s="14" t="s">
         <v>143</v>
       </c>
+      <c r="D35" s="14"/>
       <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14" t="s">
+      <c r="F35" s="14" t="s">
         <v>144</v>
       </c>
+      <c r="G35" s="14"/>
       <c r="H35" s="14"/>
-      <c r="I35" s="14"/>
-      <c r="J35" s="26" t="s">
+      <c r="I35" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="J35" s="14"/>
+      <c r="K35" s="14"/>
+      <c r="L35" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="K35" s="26"/>
-      <c r="L35" s="26"/>
-      <c r="M35" s="14" t="s">
+      <c r="M35" s="25"/>
+      <c r="N35" s="25"/>
+      <c r="O35" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="N35" s="14"/>
-      <c r="O35" s="14"/>
-      <c r="P35" s="14" t="s">
-        <v>180</v>
-      </c>
+      <c r="P35" s="14"/>
       <c r="Q35" s="14"/>
-      <c r="R35" s="14"/>
-      <c r="S35" s="14" t="s">
+      <c r="R35" s="14" t="s">
         <v>147</v>
       </c>
+      <c r="S35" s="14"/>
       <c r="T35" s="14"/>
-      <c r="U35" s="14"/>
-      <c r="V35" s="14" t="s">
+      <c r="U35" s="14" t="s">
         <v>6</v>
       </c>
+      <c r="V35" s="14"/>
       <c r="W35" s="14"/>
-      <c r="X35" s="14"/>
-      <c r="Y35" s="7" t="s">
+      <c r="X35" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="Z35" s="7"/>
-      <c r="AA35" s="7"/>
-      <c r="AB35" s="6" t="s">
+      <c r="Y35" s="6"/>
+      <c r="Z35" s="6"/>
+      <c r="AA35" s="6" t="s">
         <v>42</v>
       </c>
+      <c r="AB35" s="6"/>
       <c r="AC35" s="6"/>
-      <c r="AD35" s="6"/>
-      <c r="AE35" s="7" t="s">
+      <c r="AD35" s="7" t="s">
         <v>148</v>
       </c>
+      <c r="AE35" s="7"/>
       <c r="AF35" s="7"/>
-      <c r="AG35" s="7"/>
-      <c r="AH35" s="14" t="s">
+      <c r="AG35" s="14" t="s">
         <v>149</v>
       </c>
+      <c r="AH35" s="14"/>
       <c r="AI35" s="14"/>
-      <c r="AJ35" s="14"/>
-      <c r="AK35" s="14" t="s">
+      <c r="AJ35" s="14" t="s">
         <v>150</v>
       </c>
+      <c r="AK35" s="14"/>
       <c r="AL35" s="14"/>
       <c r="AM35" s="6"/>
       <c r="AN35" s="6"/>
       <c r="AO35" s="6"/>
       <c r="AP35" s="6"/>
       <c r="AQ35" s="6"/>
+      <c r="AR35" s="6" t="s">
+        <v>150</v>
+      </c>
       <c r="AT35" s="7"/>
       <c r="AU35" s="7"/>
       <c r="AV35" s="7"/>
@@ -16995,31 +17106,31 @@
       <c r="BH35" s="6"/>
     </row>
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7"/>
+      <c r="A36" s="7" t="s">
+        <v>91</v>
+      </c>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E36" s="14"/>
       <c r="F36" s="14"/>
       <c r="G36" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H36" s="14"/>
       <c r="I36" s="14"/>
-      <c r="J36" s="14" t="s">
-        <v>156</v>
-      </c>
+      <c r="J36" s="14"/>
       <c r="K36" s="14"/>
       <c r="L36" s="14"/>
-      <c r="M36" s="9" t="s">
+      <c r="M36" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="N36" s="9"/>
-      <c r="O36" s="9"/>
+      <c r="N36" s="20"/>
+      <c r="O36" s="20"/>
       <c r="P36" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Q36" s="14"/>
       <c r="R36" s="14"/>
@@ -17033,11 +17144,11 @@
       </c>
       <c r="W36" s="9"/>
       <c r="X36" s="9"/>
-      <c r="Y36" s="7" t="s">
+      <c r="Y36" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="Z36" s="7"/>
-      <c r="AA36" s="7"/>
+      <c r="Z36" s="6"/>
+      <c r="AA36" s="6"/>
       <c r="AB36" s="6" t="s">
         <v>42</v>
       </c>
@@ -17049,7 +17160,7 @@
       <c r="AF36" s="14"/>
       <c r="AG36" s="14"/>
       <c r="AH36" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AI36" s="14"/>
       <c r="AJ36" s="14"/>
@@ -17057,12 +17168,15 @@
         <v>160</v>
       </c>
       <c r="AL36" s="14"/>
-      <c r="AM36" s="6"/>
-      <c r="AN36" s="6"/>
-      <c r="AO36" s="6"/>
-      <c r="AP36" s="6"/>
-      <c r="AQ36" s="6"/>
-      <c r="AT36" s="27" t="s">
+      <c r="AM36" s="14"/>
+      <c r="AN36" s="10"/>
+      <c r="AO36" s="10"/>
+      <c r="AP36" s="10"/>
+      <c r="AQ36" s="10"/>
+      <c r="AR36" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="AT36" s="29" t="s">
         <v>91</v>
       </c>
       <c r="AU36" s="14" t="s">
@@ -17106,68 +17220,71 @@
       </c>
       <c r="B37" s="7"/>
       <c r="C37" s="7"/>
-      <c r="D37" s="14" t="s">
+      <c r="D37" s="7"/>
+      <c r="E37" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="F37" s="14"/>
+      <c r="G37" s="14"/>
+      <c r="H37" s="14" t="s">
         <v>185</v>
       </c>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14" t="s">
+      <c r="I37" s="14"/>
+      <c r="J37" s="14"/>
+      <c r="K37" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="H37" s="14"/>
-      <c r="I37" s="14"/>
-      <c r="J37" s="14" t="s">
+      <c r="L37" s="14"/>
+      <c r="M37" s="14"/>
+      <c r="N37" s="14" t="s">
         <v>187</v>
       </c>
-      <c r="K37" s="14"/>
-      <c r="L37" s="14"/>
-      <c r="M37" s="14" t="s">
-        <v>188</v>
-      </c>
-      <c r="N37" s="14"/>
       <c r="O37" s="14"/>
-      <c r="P37" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="Q37" s="14"/>
+      <c r="P37" s="14"/>
+      <c r="Q37" s="14" t="s">
+        <v>184</v>
+      </c>
       <c r="R37" s="14"/>
-      <c r="S37" s="6" t="s">
+      <c r="S37" s="14"/>
+      <c r="T37" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="T37" s="6"/>
-      <c r="U37" s="6"/>
-      <c r="V37" s="7" t="s">
+      <c r="U37" s="7"/>
+      <c r="V37" s="7"/>
+      <c r="W37" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="W37" s="7"/>
       <c r="X37" s="7"/>
-      <c r="Y37" s="14" t="s">
-        <v>189</v>
-      </c>
-      <c r="Z37" s="14"/>
+      <c r="Y37" s="7"/>
+      <c r="Z37" s="14" t="s">
+        <v>170</v>
+      </c>
       <c r="AA37" s="14"/>
-      <c r="AB37" s="14" t="s">
+      <c r="AB37" s="14"/>
+      <c r="AC37" s="21" t="s">
         <v>171</v>
       </c>
-      <c r="AC37" s="14"/>
-      <c r="AD37" s="14"/>
-      <c r="AE37" s="6"/>
+      <c r="AD37" s="21"/>
+      <c r="AE37" s="21"/>
       <c r="AF37" s="6"/>
       <c r="AG37" s="6"/>
-      <c r="AH37" s="14" t="s">
-        <v>190</v>
-      </c>
-      <c r="AI37" s="14"/>
-      <c r="AJ37" s="14"/>
+      <c r="AH37" s="6"/>
+      <c r="AI37" s="6"/>
+      <c r="AJ37" s="6"/>
       <c r="AK37" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="AL37" s="6"/>
+      <c r="AL37" s="6" t="s">
+        <v>43</v>
+      </c>
       <c r="AM37" s="6"/>
       <c r="AN37" s="6"/>
       <c r="AO37" s="6"/>
       <c r="AP37" s="6"/>
       <c r="AQ37" s="6"/>
+      <c r="AR37" s="32" t="s">
+        <v>209</v>
+      </c>
       <c r="AT37" s="7" t="s">
         <v>43</v>
       </c>
@@ -17206,56 +17323,77 @@
       <c r="A38" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B38" s="7"/>
-      <c r="C38" s="7"/>
+      <c r="B38" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>57</v>
+      </c>
       <c r="D38" s="7"/>
       <c r="E38" s="7"/>
-      <c r="F38" s="7"/>
-      <c r="G38" s="7" t="s">
-        <v>57</v>
-      </c>
+      <c r="F38" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="G38" s="7"/>
       <c r="H38" s="7"/>
-      <c r="I38" s="7"/>
-      <c r="J38" s="7" t="s">
-        <v>58</v>
-      </c>
+      <c r="I38" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="J38" s="7"/>
       <c r="K38" s="7"/>
-      <c r="L38" s="7"/>
-      <c r="M38" s="7"/>
+      <c r="L38" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="M38" s="7" t="s">
+        <v>60</v>
+      </c>
       <c r="N38" s="7"/>
-      <c r="O38" s="7"/>
-      <c r="P38" s="27" t="s">
+      <c r="O38" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="Q38" s="27"/>
-      <c r="R38" s="27"/>
-      <c r="S38" s="27"/>
-      <c r="T38" s="27"/>
-      <c r="U38" s="27"/>
-      <c r="V38" s="7"/>
+      <c r="P38" s="7"/>
+      <c r="Q38" s="7"/>
+      <c r="R38" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="S38" s="7"/>
+      <c r="T38" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="U38" s="7"/>
+      <c r="V38" s="7" t="s">
+        <v>61</v>
+      </c>
       <c r="W38" s="7"/>
-      <c r="X38" s="7"/>
-      <c r="Y38" s="7"/>
+      <c r="X38" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="Y38" s="7" t="s">
+        <v>210</v>
+      </c>
       <c r="Z38" s="7"/>
       <c r="AA38" s="7"/>
-      <c r="AB38" s="12"/>
-      <c r="AC38" s="12"/>
-      <c r="AD38" s="12"/>
-      <c r="AE38" s="7" t="s">
+      <c r="AB38" s="7" t="s">
         <v>55</v>
       </c>
+      <c r="AC38" s="7"/>
+      <c r="AD38" s="7"/>
+      <c r="AE38" s="7"/>
       <c r="AF38" s="7"/>
       <c r="AG38" s="7"/>
-      <c r="AH38" s="12"/>
-      <c r="AI38" s="12"/>
-      <c r="AJ38" s="12"/>
-      <c r="AK38" s="6"/>
-      <c r="AL38" s="6"/>
-      <c r="AM38" s="12"/>
-      <c r="AN38" s="12"/>
-      <c r="AO38" s="12"/>
-      <c r="AP38" s="12"/>
-      <c r="AQ38" s="12"/>
+      <c r="AH38" s="7"/>
+      <c r="AI38" s="7"/>
+      <c r="AJ38" s="7"/>
+      <c r="AK38" s="7"/>
+      <c r="AL38" s="7"/>
+      <c r="AM38" s="7"/>
+      <c r="AN38" s="7"/>
+      <c r="AO38" s="7"/>
+      <c r="AP38" s="7"/>
+      <c r="AQ38" s="7"/>
+      <c r="AR38" s="6" t="s">
+        <v>56</v>
+      </c>
       <c r="AT38" s="7" t="s">
         <v>55</v>
       </c>
@@ -17266,17 +17404,17 @@
       <c r="AW38" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AX38" s="27" t="s">
+      <c r="AX38" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="AY38" s="27" t="s">
+      <c r="AY38" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="AZ38" s="27"/>
-      <c r="BA38" s="27" t="s">
+      <c r="AZ38" s="29"/>
+      <c r="BA38" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="BB38" s="27" t="s">
+      <c r="BB38" s="29" t="s">
         <v>115</v>
       </c>
       <c r="BC38" s="12"/>
@@ -17304,43 +17442,44 @@
       <c r="M39" s="7"/>
       <c r="N39" s="7"/>
       <c r="O39" s="7"/>
-      <c r="P39" s="27"/>
-      <c r="Q39" s="27"/>
-      <c r="R39" s="27"/>
-      <c r="S39" s="27"/>
-      <c r="T39" s="27"/>
-      <c r="U39" s="27"/>
+      <c r="P39" s="7"/>
+      <c r="Q39" s="7"/>
+      <c r="R39" s="7"/>
+      <c r="S39" s="7"/>
+      <c r="T39" s="7"/>
+      <c r="U39" s="7"/>
       <c r="V39" s="7"/>
       <c r="W39" s="7"/>
       <c r="X39" s="7"/>
       <c r="Y39" s="7"/>
       <c r="Z39" s="7"/>
       <c r="AA39" s="7"/>
-      <c r="AB39" s="12"/>
-      <c r="AC39" s="12"/>
-      <c r="AD39" s="12"/>
+      <c r="AB39" s="7"/>
+      <c r="AC39" s="7"/>
+      <c r="AD39" s="7"/>
       <c r="AE39" s="7"/>
       <c r="AF39" s="7"/>
       <c r="AG39" s="7"/>
-      <c r="AH39" s="6"/>
-      <c r="AI39" s="6"/>
-      <c r="AJ39" s="6"/>
-      <c r="AK39" s="6"/>
-      <c r="AL39" s="6"/>
-      <c r="AM39" s="6"/>
-      <c r="AN39" s="6"/>
-      <c r="AO39" s="6"/>
-      <c r="AP39" s="6"/>
-      <c r="AQ39" s="6"/>
+      <c r="AH39" s="7"/>
+      <c r="AI39" s="7"/>
+      <c r="AJ39" s="7"/>
+      <c r="AK39" s="7"/>
+      <c r="AL39" s="7"/>
+      <c r="AM39" s="7"/>
+      <c r="AN39" s="7"/>
+      <c r="AO39" s="7"/>
+      <c r="AP39" s="7"/>
+      <c r="AQ39" s="7"/>
+      <c r="AR39" s="6"/>
       <c r="AT39" s="7"/>
       <c r="AU39" s="7"/>
       <c r="AV39" s="7"/>
       <c r="AW39" s="7"/>
       <c r="AX39" s="7"/>
       <c r="AY39" s="7"/>
-      <c r="AZ39" s="27"/>
-      <c r="BA39" s="27"/>
-      <c r="BB39" s="27"/>
+      <c r="AZ39" s="29"/>
+      <c r="BA39" s="29"/>
+      <c r="BB39" s="29"/>
       <c r="BC39" s="12"/>
       <c r="BD39" s="6"/>
       <c r="BE39" s="6"/>
@@ -17349,50 +17488,50 @@
       <c r="BH39" s="6"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D40" s="28"/>
-      <c r="E40" s="28"/>
-      <c r="F40" s="28"/>
-      <c r="G40" s="29"/>
-      <c r="H40" s="29"/>
-      <c r="I40" s="29"/>
-      <c r="J40" s="29"/>
-      <c r="K40" s="29"/>
-      <c r="L40" s="29"/>
-      <c r="M40" s="29"/>
-      <c r="N40" s="29"/>
-      <c r="O40" s="29"/>
-      <c r="P40" s="29"/>
-      <c r="Q40" s="29"/>
-      <c r="R40" s="29"/>
-      <c r="S40" s="29"/>
-      <c r="T40" s="29"/>
-      <c r="U40" s="29"/>
-      <c r="V40" s="29"/>
-      <c r="W40" s="29"/>
-      <c r="X40" s="29"/>
-      <c r="Y40" s="29"/>
-      <c r="Z40" s="29"/>
-      <c r="AA40" s="29"/>
-      <c r="AB40" s="29"/>
-      <c r="AC40" s="29"/>
-      <c r="AD40" s="29"/>
-      <c r="AE40" s="29"/>
-      <c r="AF40" s="29"/>
-      <c r="AG40" s="29"/>
-      <c r="AH40" s="29"/>
-      <c r="AI40" s="29"/>
-      <c r="AJ40" s="29"/>
-      <c r="AK40" s="29"/>
-      <c r="AL40" s="29"/>
-      <c r="AM40" s="29"/>
-      <c r="AN40" s="29"/>
-      <c r="AO40" s="29"/>
-      <c r="AP40" s="29"/>
-      <c r="AQ40" s="30"/>
+      <c r="D40" s="26"/>
+      <c r="E40" s="26"/>
+      <c r="F40" s="26"/>
+      <c r="G40" s="27"/>
+      <c r="H40" s="27"/>
+      <c r="I40" s="27"/>
+      <c r="J40" s="27"/>
+      <c r="K40" s="27"/>
+      <c r="L40" s="27"/>
+      <c r="M40" s="27"/>
+      <c r="N40" s="27"/>
+      <c r="O40" s="27"/>
+      <c r="P40" s="27"/>
+      <c r="Q40" s="27"/>
+      <c r="R40" s="27"/>
+      <c r="S40" s="27"/>
+      <c r="T40" s="27"/>
+      <c r="U40" s="27"/>
+      <c r="V40" s="27"/>
+      <c r="W40" s="27"/>
+      <c r="X40" s="27"/>
+      <c r="Y40" s="27"/>
+      <c r="Z40" s="27"/>
+      <c r="AA40" s="27"/>
+      <c r="AB40" s="27"/>
+      <c r="AC40" s="27"/>
+      <c r="AD40" s="27"/>
+      <c r="AE40" s="27"/>
+      <c r="AF40" s="27"/>
+      <c r="AG40" s="27"/>
+      <c r="AH40" s="27"/>
+      <c r="AI40" s="27"/>
+      <c r="AJ40" s="27"/>
+      <c r="AK40" s="27"/>
+      <c r="AL40" s="27"/>
+      <c r="AM40" s="27"/>
+      <c r="AN40" s="27"/>
+      <c r="AO40" s="27"/>
+      <c r="AP40" s="27"/>
+      <c r="AQ40" s="28"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="16" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="16"/>
@@ -17586,50 +17725,50 @@
       <c r="AQ43" s="6"/>
       <c r="AT43" s="7"/>
       <c r="AU43" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="AV43" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="AW43" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="AX43" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="AV43" s="7" t="s">
+      <c r="AY43" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="AW43" s="7" t="s">
+      <c r="AZ43" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="AX43" s="6" t="s">
+      <c r="BA43" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="AY43" s="6" t="s">
+      <c r="BB43" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="AZ43" s="6" t="s">
+      <c r="BC43" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="BA43" s="6" t="s">
+      <c r="BD43" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="BB43" s="7" t="s">
+      <c r="BE43" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="BC43" s="6" t="s">
+      <c r="BF43" s="6" t="s">
         <v>200</v>
-      </c>
-      <c r="BD43" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="BE43" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="BF43" s="6" t="s">
-        <v>203</v>
       </c>
       <c r="BG43" s="6"/>
       <c r="BH43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="27" t="s">
+      <c r="A44" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="B44" s="27"/>
-      <c r="C44" s="27"/>
+      <c r="B44" s="29"/>
+      <c r="C44" s="29"/>
       <c r="D44" s="7"/>
       <c r="E44" s="7"/>
       <c r="F44" s="7"/>
@@ -17646,7 +17785,7 @@
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
       <c r="S44" s="19" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="T44" s="19"/>
       <c r="U44" s="19"/>
@@ -17676,7 +17815,7 @@
       <c r="AO44" s="6"/>
       <c r="AP44" s="6"/>
       <c r="AQ44" s="6"/>
-      <c r="AT44" s="27" t="s">
+      <c r="AT44" s="29" t="s">
         <v>91</v>
       </c>
       <c r="AU44" s="14" t="s">
@@ -17736,7 +17875,7 @@
       <c r="Q45" s="7"/>
       <c r="R45" s="7"/>
       <c r="S45" s="19" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="T45" s="19"/>
       <c r="U45" s="19"/>
@@ -17816,14 +17955,14 @@
       <c r="M46" s="7"/>
       <c r="N46" s="7"/>
       <c r="O46" s="7"/>
-      <c r="P46" s="27" t="s">
+      <c r="P46" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="Q46" s="27"/>
-      <c r="R46" s="27"/>
-      <c r="S46" s="27"/>
-      <c r="T46" s="27"/>
-      <c r="U46" s="27"/>
+      <c r="Q46" s="29"/>
+      <c r="R46" s="29"/>
+      <c r="S46" s="29"/>
+      <c r="T46" s="29"/>
+      <c r="U46" s="29"/>
       <c r="V46" s="6"/>
       <c r="W46" s="6"/>
       <c r="X46" s="6"/>
@@ -17858,17 +17997,17 @@
       <c r="AW46" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AX46" s="27" t="s">
+      <c r="AX46" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="AY46" s="27" t="s">
+      <c r="AY46" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="AZ46" s="27"/>
-      <c r="BA46" s="27" t="s">
+      <c r="AZ46" s="29"/>
+      <c r="BA46" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="BB46" s="27" t="s">
+      <c r="BB46" s="29" t="s">
         <v>115</v>
       </c>
       <c r="BC46" s="12"/>
@@ -17896,12 +18035,12 @@
       <c r="M47" s="7"/>
       <c r="N47" s="7"/>
       <c r="O47" s="7"/>
-      <c r="P47" s="27"/>
-      <c r="Q47" s="27"/>
-      <c r="R47" s="27"/>
-      <c r="S47" s="27"/>
-      <c r="T47" s="27"/>
-      <c r="U47" s="27"/>
+      <c r="P47" s="29"/>
+      <c r="Q47" s="29"/>
+      <c r="R47" s="29"/>
+      <c r="S47" s="29"/>
+      <c r="T47" s="29"/>
+      <c r="U47" s="29"/>
       <c r="V47" s="6"/>
       <c r="W47" s="6"/>
       <c r="X47" s="6"/>
@@ -17930,9 +18069,9 @@
       <c r="AW47" s="7"/>
       <c r="AX47" s="7"/>
       <c r="AY47" s="7"/>
-      <c r="AZ47" s="27"/>
-      <c r="BA47" s="27"/>
-      <c r="BB47" s="27"/>
+      <c r="AZ47" s="29"/>
+      <c r="BA47" s="29"/>
+      <c r="BB47" s="29"/>
       <c r="BC47" s="12"/>
       <c r="BD47" s="6"/>
       <c r="BE47" s="6"/>
@@ -17941,49 +18080,49 @@
       <c r="BH47" s="6"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="28"/>
-      <c r="B48" s="28"/>
-      <c r="C48" s="28"/>
-      <c r="D48" s="28"/>
-      <c r="E48" s="28"/>
-      <c r="F48" s="28"/>
-      <c r="G48" s="29"/>
-      <c r="H48" s="29"/>
-      <c r="I48" s="29"/>
-      <c r="J48" s="29"/>
-      <c r="K48" s="29"/>
-      <c r="L48" s="29"/>
-      <c r="M48" s="29"/>
-      <c r="N48" s="29"/>
-      <c r="O48" s="29"/>
-      <c r="P48" s="29"/>
-      <c r="Q48" s="29"/>
-      <c r="R48" s="29"/>
-      <c r="S48" s="29"/>
-      <c r="T48" s="29"/>
-      <c r="U48" s="29"/>
-      <c r="V48" s="29"/>
-      <c r="W48" s="29"/>
-      <c r="X48" s="29"/>
-      <c r="Y48" s="29"/>
-      <c r="Z48" s="29"/>
-      <c r="AA48" s="29"/>
-      <c r="AB48" s="29"/>
-      <c r="AC48" s="29"/>
-      <c r="AD48" s="29"/>
-      <c r="AE48" s="29"/>
-      <c r="AF48" s="29"/>
-      <c r="AG48" s="29"/>
-      <c r="AH48" s="29"/>
-      <c r="AI48" s="29"/>
-      <c r="AJ48" s="29"/>
-      <c r="AK48" s="29"/>
-      <c r="AL48" s="29"/>
-      <c r="AM48" s="29"/>
-      <c r="AN48" s="29"/>
-      <c r="AO48" s="29"/>
-      <c r="AP48" s="29"/>
-      <c r="AQ48" s="30"/>
+      <c r="A48" s="26"/>
+      <c r="B48" s="26"/>
+      <c r="C48" s="26"/>
+      <c r="D48" s="26"/>
+      <c r="E48" s="26"/>
+      <c r="F48" s="26"/>
+      <c r="G48" s="27"/>
+      <c r="H48" s="27"/>
+      <c r="I48" s="27"/>
+      <c r="J48" s="27"/>
+      <c r="K48" s="27"/>
+      <c r="L48" s="27"/>
+      <c r="M48" s="27"/>
+      <c r="N48" s="27"/>
+      <c r="O48" s="27"/>
+      <c r="P48" s="27"/>
+      <c r="Q48" s="27"/>
+      <c r="R48" s="27"/>
+      <c r="S48" s="27"/>
+      <c r="T48" s="27"/>
+      <c r="U48" s="27"/>
+      <c r="V48" s="27"/>
+      <c r="W48" s="27"/>
+      <c r="X48" s="27"/>
+      <c r="Y48" s="27"/>
+      <c r="Z48" s="27"/>
+      <c r="AA48" s="27"/>
+      <c r="AB48" s="27"/>
+      <c r="AC48" s="27"/>
+      <c r="AD48" s="27"/>
+      <c r="AE48" s="27"/>
+      <c r="AF48" s="27"/>
+      <c r="AG48" s="27"/>
+      <c r="AH48" s="27"/>
+      <c r="AI48" s="27"/>
+      <c r="AJ48" s="27"/>
+      <c r="AK48" s="27"/>
+      <c r="AL48" s="27"/>
+      <c r="AM48" s="27"/>
+      <c r="AN48" s="27"/>
+      <c r="AO48" s="27"/>
+      <c r="AP48" s="27"/>
+      <c r="AQ48" s="28"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3"/>
@@ -18030,7 +18169,7 @@
       <c r="AP49" s="4"/>
       <c r="AQ49" s="5"/>
       <c r="AT49" s="3" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="AZ49" s="1"/>
     </row>
@@ -18318,7 +18457,7 @@
       <c r="AU52" s="7"/>
       <c r="AV52" s="7"/>
       <c r="AW52" s="7"/>
-      <c r="AX52" s="31"/>
+      <c r="AX52" s="30"/>
       <c r="AY52" s="6"/>
       <c r="AZ52" s="14" t="s">
         <v>6</v>
@@ -18924,7 +19063,7 @@
       <c r="AS62" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="569">
+  <mergeCells count="624">
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
@@ -18987,7 +19126,7 @@
     <mergeCell ref="F6:H7"/>
     <mergeCell ref="I6:K7"/>
     <mergeCell ref="L6:Q7"/>
-    <mergeCell ref="R6:X7"/>
+    <mergeCell ref="R6:W7"/>
     <mergeCell ref="Y6:AA7"/>
     <mergeCell ref="AB6:AD7"/>
     <mergeCell ref="AE6:AG7"/>
@@ -19257,14 +19396,14 @@
     <mergeCell ref="F22:H23"/>
     <mergeCell ref="I22:K23"/>
     <mergeCell ref="L22:Q23"/>
-    <mergeCell ref="R22:W23"/>
-    <mergeCell ref="X22:Z23"/>
-    <mergeCell ref="AA22:AC23"/>
-    <mergeCell ref="AD22:AF23"/>
-    <mergeCell ref="AG22:AI23"/>
-    <mergeCell ref="AJ22:AL23"/>
-    <mergeCell ref="AM22:AO23"/>
-    <mergeCell ref="AP22:AQ23"/>
+    <mergeCell ref="R22:X23"/>
+    <mergeCell ref="Y22:AA23"/>
+    <mergeCell ref="AB22:AD23"/>
+    <mergeCell ref="AE22:AG23"/>
+    <mergeCell ref="AH22:AJ23"/>
+    <mergeCell ref="AK22:AM23"/>
+    <mergeCell ref="AN22:AQ23"/>
+    <mergeCell ref="AR22:AR23"/>
     <mergeCell ref="AT22:AT23"/>
     <mergeCell ref="AU22:AW23"/>
     <mergeCell ref="AX22:AZ23"/>
@@ -19395,14 +19534,14 @@
     <mergeCell ref="F30:H31"/>
     <mergeCell ref="I30:K31"/>
     <mergeCell ref="L30:Q31"/>
-    <mergeCell ref="R30:W31"/>
-    <mergeCell ref="X30:Z31"/>
-    <mergeCell ref="AA30:AC31"/>
-    <mergeCell ref="AD30:AF31"/>
-    <mergeCell ref="AG30:AI31"/>
-    <mergeCell ref="AJ30:AL31"/>
-    <mergeCell ref="AM30:AO31"/>
-    <mergeCell ref="AP30:AQ31"/>
+    <mergeCell ref="R30:X31"/>
+    <mergeCell ref="Y30:AA31"/>
+    <mergeCell ref="AB30:AD31"/>
+    <mergeCell ref="AE30:AG31"/>
+    <mergeCell ref="AH30:AJ31"/>
+    <mergeCell ref="AK30:AM31"/>
+    <mergeCell ref="AN30:AQ31"/>
+    <mergeCell ref="AR30:AR31"/>
     <mergeCell ref="AT30:AU31"/>
     <mergeCell ref="AV30:AX31"/>
     <mergeCell ref="AY30:BA31"/>
@@ -19416,20 +19555,76 @@
     <mergeCell ref="CC30:CE31"/>
     <mergeCell ref="CF30:CH31"/>
     <mergeCell ref="CI30:CJ31"/>
-    <mergeCell ref="AM35:AQ36"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="E34:G34"/>
+    <mergeCell ref="H34:J34"/>
+    <mergeCell ref="K34:M34"/>
+    <mergeCell ref="N34:P34"/>
+    <mergeCell ref="Q34:S34"/>
+    <mergeCell ref="T34:V34"/>
+    <mergeCell ref="W34:Y34"/>
+    <mergeCell ref="Z34:AB34"/>
+    <mergeCell ref="AC34:AE34"/>
+    <mergeCell ref="AF34:AH34"/>
+    <mergeCell ref="AI34:AK34"/>
+    <mergeCell ref="AL34:AN34"/>
+    <mergeCell ref="AO34:AQ34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="I35:K35"/>
+    <mergeCell ref="L35:N35"/>
+    <mergeCell ref="O35:Q35"/>
+    <mergeCell ref="R35:T35"/>
+    <mergeCell ref="U35:W35"/>
+    <mergeCell ref="X35:Z35"/>
+    <mergeCell ref="AA35:AC35"/>
+    <mergeCell ref="AD35:AF35"/>
+    <mergeCell ref="AG35:AI35"/>
+    <mergeCell ref="AJ35:AL35"/>
+    <mergeCell ref="AM35:AQ35"/>
     <mergeCell ref="BG35:BH36"/>
-    <mergeCell ref="AK37:AQ37"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="D36:F36"/>
+    <mergeCell ref="G36:I36"/>
+    <mergeCell ref="J36:L36"/>
+    <mergeCell ref="M36:O36"/>
+    <mergeCell ref="P36:R36"/>
+    <mergeCell ref="S36:U36"/>
+    <mergeCell ref="V36:X36"/>
+    <mergeCell ref="Y36:AA36"/>
+    <mergeCell ref="AB36:AD36"/>
+    <mergeCell ref="AE36:AG36"/>
+    <mergeCell ref="AH36:AJ36"/>
+    <mergeCell ref="AK36:AM36"/>
+    <mergeCell ref="AN36:AQ36"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="E37:G37"/>
+    <mergeCell ref="H37:J37"/>
+    <mergeCell ref="K37:M37"/>
+    <mergeCell ref="N37:P37"/>
+    <mergeCell ref="Q37:S37"/>
+    <mergeCell ref="T37:V37"/>
+    <mergeCell ref="W37:Y37"/>
+    <mergeCell ref="Z37:AB37"/>
+    <mergeCell ref="AC37:AE37"/>
+    <mergeCell ref="AF37:AH37"/>
+    <mergeCell ref="AI37:AK37"/>
+    <mergeCell ref="AL37:AQ37"/>
     <mergeCell ref="BF37:BH37"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="G38:G39"/>
-    <mergeCell ref="J38:J39"/>
-    <mergeCell ref="M38:M39"/>
-    <mergeCell ref="P38:S39"/>
-    <mergeCell ref="V38:V39"/>
-    <mergeCell ref="Y38:Y39"/>
-    <mergeCell ref="AE38:AE39"/>
-    <mergeCell ref="AM38:AQ38"/>
+    <mergeCell ref="A38:B39"/>
+    <mergeCell ref="C38:E39"/>
+    <mergeCell ref="F38:H39"/>
+    <mergeCell ref="I38:K39"/>
+    <mergeCell ref="L38:Q39"/>
+    <mergeCell ref="R38:X39"/>
+    <mergeCell ref="Y38:AA39"/>
+    <mergeCell ref="AB38:AD39"/>
+    <mergeCell ref="AE38:AG39"/>
+    <mergeCell ref="AH38:AJ39"/>
+    <mergeCell ref="AK38:AM39"/>
+    <mergeCell ref="AN38:AQ39"/>
+    <mergeCell ref="AR38:AR39"/>
     <mergeCell ref="AT38:AT39"/>
     <mergeCell ref="AU38:AU39"/>
     <mergeCell ref="AV38:AV39"/>
@@ -19440,7 +19635,6 @@
     <mergeCell ref="BB38:BB39"/>
     <mergeCell ref="BD38:BD39"/>
     <mergeCell ref="BG38:BH38"/>
-    <mergeCell ref="AM39:AQ39"/>
     <mergeCell ref="BG39:BH39"/>
     <mergeCell ref="AM43:AQ44"/>
     <mergeCell ref="BG43:BH44"/>
@@ -19787,7 +19981,7 @@
       <c r="N5" s="6"/>
       <c r="O5" s="6"/>
       <c r="P5" s="32" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="R5" s="7"/>
       <c r="S5" s="7"/>
@@ -19901,24 +20095,24 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3"/>
-      <c r="B8" s="29"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="29"/>
-      <c r="I8" s="29"/>
-      <c r="J8" s="29"/>
-      <c r="K8" s="29"/>
-      <c r="L8" s="29"/>
-      <c r="M8" s="29"/>
-      <c r="N8" s="29"/>
-      <c r="O8" s="30"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="27"/>
+      <c r="K8" s="27"/>
+      <c r="L8" s="27"/>
+      <c r="M8" s="27"/>
+      <c r="N8" s="27"/>
+      <c r="O8" s="28"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -20182,7 +20376,7 @@
       <c r="N13" s="6"/>
       <c r="O13" s="6"/>
       <c r="P13" s="32" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="R13" s="7"/>
       <c r="S13" s="14"/>
@@ -20296,20 +20490,20 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3"/>
-      <c r="B16" s="29"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29"/>
-      <c r="E16" s="29"/>
-      <c r="F16" s="29"/>
-      <c r="G16" s="29"/>
-      <c r="H16" s="29"/>
-      <c r="I16" s="29"/>
-      <c r="J16" s="29"/>
-      <c r="K16" s="29"/>
-      <c r="L16" s="29"/>
-      <c r="M16" s="29"/>
-      <c r="N16" s="29"/>
-      <c r="O16" s="30"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="27"/>
+      <c r="J16" s="27"/>
+      <c r="K16" s="27"/>
+      <c r="L16" s="27"/>
+      <c r="M16" s="27"/>
+      <c r="N16" s="27"/>
+      <c r="O16" s="28"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="4"/>
@@ -20391,7 +20585,7 @@
       <c r="N19" s="6"/>
       <c r="O19" s="6"/>
       <c r="P19" s="34" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="R19" s="7"/>
       <c r="S19" s="7"/>
@@ -20410,7 +20604,7 @@
       <c r="AF19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="27"/>
+      <c r="A20" s="29"/>
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
       <c r="D20" s="14"/>
@@ -20493,7 +20687,7 @@
       <c r="S22" s="7"/>
       <c r="T22" s="7"/>
       <c r="U22" s="7"/>
-      <c r="V22" s="27"/>
+      <c r="V22" s="29"/>
       <c r="W22" s="7"/>
       <c r="X22" s="7"/>
       <c r="Y22" s="35"/>
@@ -20525,8 +20719,8 @@
       <c r="S23" s="7"/>
       <c r="T23" s="7"/>
       <c r="U23" s="7"/>
-      <c r="V23" s="27"/>
-      <c r="W23" s="27"/>
+      <c r="V23" s="29"/>
+      <c r="W23" s="29"/>
       <c r="X23" s="7"/>
       <c r="Y23" s="35"/>
       <c r="Z23" s="35"/>
@@ -20539,20 +20733,20 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3"/>
-      <c r="B24" s="28"/>
-      <c r="C24" s="29"/>
-      <c r="D24" s="29"/>
-      <c r="E24" s="29"/>
-      <c r="F24" s="29"/>
-      <c r="G24" s="29"/>
-      <c r="H24" s="29"/>
-      <c r="I24" s="29"/>
-      <c r="J24" s="29"/>
-      <c r="K24" s="29"/>
-      <c r="L24" s="29"/>
-      <c r="M24" s="29"/>
-      <c r="N24" s="29"/>
-      <c r="O24" s="30"/>
+      <c r="B24" s="26"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
+      <c r="I24" s="27"/>
+      <c r="J24" s="27"/>
+      <c r="K24" s="27"/>
+      <c r="L24" s="27"/>
+      <c r="M24" s="27"/>
+      <c r="N24" s="27"/>
+      <c r="O24" s="28"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3"/>
@@ -20666,7 +20860,7 @@
       <c r="M28" s="14"/>
       <c r="N28" s="6"/>
       <c r="O28" s="6"/>
-      <c r="R28" s="27"/>
+      <c r="R28" s="29"/>
       <c r="S28" s="7"/>
       <c r="T28" s="7"/>
       <c r="U28" s="7"/>
@@ -20720,8 +20914,8 @@
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
       <c r="E30" s="7"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="27"/>
+      <c r="F30" s="29"/>
+      <c r="G30" s="29"/>
       <c r="H30" s="7"/>
       <c r="I30" s="7"/>
       <c r="J30" s="12"/>
@@ -20734,9 +20928,9 @@
       <c r="S30" s="7"/>
       <c r="T30" s="7"/>
       <c r="U30" s="7"/>
-      <c r="V30" s="27"/>
-      <c r="W30" s="27"/>
-      <c r="X30" s="27"/>
+      <c r="V30" s="29"/>
+      <c r="W30" s="29"/>
+      <c r="X30" s="29"/>
       <c r="Y30" s="6"/>
       <c r="Z30" s="7"/>
       <c r="AA30" s="12"/>
@@ -20753,7 +20947,7 @@
       <c r="D31" s="7"/>
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
-      <c r="G31" s="27"/>
+      <c r="G31" s="29"/>
       <c r="H31" s="7"/>
       <c r="I31" s="7"/>
       <c r="J31" s="12"/>
@@ -20768,7 +20962,7 @@
       <c r="U31" s="7"/>
       <c r="V31" s="7"/>
       <c r="W31" s="7"/>
-      <c r="X31" s="27"/>
+      <c r="X31" s="29"/>
       <c r="Y31" s="6"/>
       <c r="Z31" s="7"/>
       <c r="AA31" s="12"/>
@@ -20780,20 +20974,20 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3"/>
-      <c r="B32" s="28"/>
-      <c r="C32" s="29"/>
-      <c r="D32" s="29"/>
-      <c r="E32" s="29"/>
-      <c r="F32" s="29"/>
-      <c r="G32" s="29"/>
-      <c r="H32" s="29"/>
-      <c r="I32" s="29"/>
-      <c r="J32" s="29"/>
-      <c r="K32" s="29"/>
-      <c r="L32" s="29"/>
-      <c r="M32" s="29"/>
-      <c r="N32" s="29"/>
-      <c r="O32" s="30"/>
+      <c r="B32" s="26"/>
+      <c r="C32" s="27"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="27"/>
+      <c r="F32" s="27"/>
+      <c r="G32" s="27"/>
+      <c r="H32" s="27"/>
+      <c r="I32" s="27"/>
+      <c r="J32" s="27"/>
+      <c r="K32" s="27"/>
+      <c r="L32" s="27"/>
+      <c r="M32" s="27"/>
+      <c r="N32" s="27"/>
+      <c r="O32" s="28"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3"/>
@@ -20831,7 +21025,7 @@
       <c r="A34" s="7"/>
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
-      <c r="D34" s="25"/>
+      <c r="D34" s="31"/>
       <c r="E34" s="6"/>
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
@@ -20863,7 +21057,7 @@
       <c r="A35" s="7"/>
       <c r="B35" s="14"/>
       <c r="C35" s="14"/>
-      <c r="D35" s="26"/>
+      <c r="D35" s="25"/>
       <c r="E35" s="14"/>
       <c r="F35" s="14"/>
       <c r="G35" s="14"/>
@@ -20907,7 +21101,7 @@
       <c r="M36" s="14"/>
       <c r="N36" s="6"/>
       <c r="O36" s="6"/>
-      <c r="R36" s="27"/>
+      <c r="R36" s="29"/>
       <c r="S36" s="14"/>
       <c r="T36" s="14"/>
       <c r="U36" s="14"/>
@@ -20961,8 +21155,8 @@
       <c r="C38" s="7"/>
       <c r="D38" s="7"/>
       <c r="E38" s="7"/>
-      <c r="F38" s="27"/>
-      <c r="G38" s="27"/>
+      <c r="F38" s="29"/>
+      <c r="G38" s="29"/>
       <c r="H38" s="7"/>
       <c r="I38" s="7"/>
       <c r="J38" s="12"/>
@@ -20975,11 +21169,11 @@
       <c r="S38" s="7"/>
       <c r="T38" s="7"/>
       <c r="U38" s="7"/>
-      <c r="V38" s="27"/>
-      <c r="W38" s="27"/>
-      <c r="X38" s="27"/>
-      <c r="Y38" s="27"/>
-      <c r="Z38" s="27"/>
+      <c r="V38" s="29"/>
+      <c r="W38" s="29"/>
+      <c r="X38" s="29"/>
+      <c r="Y38" s="29"/>
+      <c r="Z38" s="29"/>
       <c r="AA38" s="12"/>
       <c r="AB38" s="6"/>
       <c r="AC38" s="12"/>
@@ -20994,7 +21188,7 @@
       <c r="D39" s="7"/>
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
-      <c r="G39" s="27"/>
+      <c r="G39" s="29"/>
       <c r="H39" s="7"/>
       <c r="I39" s="7"/>
       <c r="J39" s="12"/>
@@ -21009,9 +21203,9 @@
       <c r="U39" s="7"/>
       <c r="V39" s="7"/>
       <c r="W39" s="7"/>
-      <c r="X39" s="27"/>
-      <c r="Y39" s="27"/>
-      <c r="Z39" s="27"/>
+      <c r="X39" s="29"/>
+      <c r="Y39" s="29"/>
+      <c r="Z39" s="29"/>
       <c r="AA39" s="12"/>
       <c r="AB39" s="6"/>
       <c r="AC39" s="6"/>
@@ -21020,20 +21214,20 @@
       <c r="AF39" s="6"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="28"/>
-      <c r="C40" s="29"/>
-      <c r="D40" s="29"/>
-      <c r="E40" s="29"/>
-      <c r="F40" s="29"/>
-      <c r="G40" s="29"/>
-      <c r="H40" s="29"/>
-      <c r="I40" s="29"/>
-      <c r="J40" s="29"/>
-      <c r="K40" s="29"/>
-      <c r="L40" s="29"/>
-      <c r="M40" s="29"/>
-      <c r="N40" s="29"/>
-      <c r="O40" s="30"/>
+      <c r="B40" s="26"/>
+      <c r="C40" s="27"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="27"/>
+      <c r="F40" s="27"/>
+      <c r="G40" s="27"/>
+      <c r="H40" s="27"/>
+      <c r="I40" s="27"/>
+      <c r="J40" s="27"/>
+      <c r="K40" s="27"/>
+      <c r="L40" s="27"/>
+      <c r="M40" s="27"/>
+      <c r="N40" s="27"/>
+      <c r="O40" s="28"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="16"/>
@@ -21132,7 +21326,7 @@
       <c r="AF43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="27"/>
+      <c r="A44" s="29"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
@@ -21147,7 +21341,7 @@
       <c r="M44" s="6"/>
       <c r="N44" s="6"/>
       <c r="O44" s="6"/>
-      <c r="R44" s="27"/>
+      <c r="R44" s="29"/>
       <c r="S44" s="14"/>
       <c r="T44" s="14"/>
       <c r="U44" s="14"/>
@@ -21201,8 +21395,8 @@
       <c r="C46" s="7"/>
       <c r="D46" s="7"/>
       <c r="E46" s="7"/>
-      <c r="F46" s="27"/>
-      <c r="G46" s="27"/>
+      <c r="F46" s="29"/>
+      <c r="G46" s="29"/>
       <c r="H46" s="6"/>
       <c r="I46" s="7"/>
       <c r="J46" s="12"/>
@@ -21215,11 +21409,11 @@
       <c r="S46" s="7"/>
       <c r="T46" s="7"/>
       <c r="U46" s="7"/>
-      <c r="V46" s="27"/>
-      <c r="W46" s="27"/>
-      <c r="X46" s="27"/>
-      <c r="Y46" s="27"/>
-      <c r="Z46" s="27"/>
+      <c r="V46" s="29"/>
+      <c r="W46" s="29"/>
+      <c r="X46" s="29"/>
+      <c r="Y46" s="29"/>
+      <c r="Z46" s="29"/>
       <c r="AA46" s="12"/>
       <c r="AB46" s="6"/>
       <c r="AC46" s="12"/>
@@ -21234,7 +21428,7 @@
       <c r="D47" s="7"/>
       <c r="E47" s="7"/>
       <c r="F47" s="7"/>
-      <c r="G47" s="27"/>
+      <c r="G47" s="29"/>
       <c r="H47" s="6"/>
       <c r="I47" s="7"/>
       <c r="J47" s="12"/>
@@ -21249,9 +21443,9 @@
       <c r="U47" s="7"/>
       <c r="V47" s="7"/>
       <c r="W47" s="7"/>
-      <c r="X47" s="27"/>
-      <c r="Y47" s="27"/>
-      <c r="Z47" s="27"/>
+      <c r="X47" s="29"/>
+      <c r="Y47" s="29"/>
+      <c r="Z47" s="29"/>
       <c r="AA47" s="12"/>
       <c r="AB47" s="6"/>
       <c r="AC47" s="6"/>
@@ -21260,21 +21454,21 @@
       <c r="AF47" s="6"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="28"/>
-      <c r="B48" s="28"/>
-      <c r="C48" s="29"/>
-      <c r="D48" s="29"/>
-      <c r="E48" s="29"/>
-      <c r="F48" s="29"/>
-      <c r="G48" s="29"/>
-      <c r="H48" s="29"/>
-      <c r="I48" s="29"/>
-      <c r="J48" s="29"/>
-      <c r="K48" s="29"/>
-      <c r="L48" s="29"/>
-      <c r="M48" s="29"/>
-      <c r="N48" s="29"/>
-      <c r="O48" s="30"/>
+      <c r="A48" s="26"/>
+      <c r="B48" s="26"/>
+      <c r="C48" s="27"/>
+      <c r="D48" s="27"/>
+      <c r="E48" s="27"/>
+      <c r="F48" s="27"/>
+      <c r="G48" s="27"/>
+      <c r="H48" s="27"/>
+      <c r="I48" s="27"/>
+      <c r="J48" s="27"/>
+      <c r="K48" s="27"/>
+      <c r="L48" s="27"/>
+      <c r="M48" s="27"/>
+      <c r="N48" s="27"/>
+      <c r="O48" s="28"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3"/>
@@ -21379,7 +21573,7 @@
       <c r="S52" s="7"/>
       <c r="T52" s="7"/>
       <c r="U52" s="7"/>
-      <c r="V52" s="31"/>
+      <c r="V52" s="30"/>
       <c r="W52" s="6"/>
       <c r="X52" s="14"/>
       <c r="Y52" s="15"/>
@@ -21428,7 +21622,7 @@
       <c r="B54" s="7"/>
       <c r="C54" s="7"/>
       <c r="D54" s="7"/>
-      <c r="E54" s="27"/>
+      <c r="E54" s="29"/>
       <c r="F54" s="7"/>
       <c r="G54" s="7"/>
       <c r="H54" s="35"/>
@@ -21460,8 +21654,8 @@
       <c r="B55" s="7"/>
       <c r="C55" s="7"/>
       <c r="D55" s="7"/>
-      <c r="E55" s="27"/>
-      <c r="F55" s="27"/>
+      <c r="E55" s="29"/>
+      <c r="F55" s="29"/>
       <c r="G55" s="7"/>
       <c r="H55" s="35"/>
       <c r="I55" s="35"/>

</xml_diff>

<commit_message>
[Fixed] The issue script does not work is fixed. [Change] Layout is changed.
</commit_message>
<xml_diff>
--- a/img/keymap.xlsx
+++ b/img/keymap.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1797" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1804" uniqueCount="198">
   <si>
     <t xml:space="preserve">標準</t>
   </si>
@@ -457,6 +457,12 @@
     <t xml:space="preserve">SC+→</t>
   </si>
   <si>
+    <t xml:space="preserve">C+Home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+End</t>
+  </si>
+  <si>
     <t xml:space="preserve">C+a</t>
   </si>
   <si>
@@ -505,10 +511,10 @@
     <t xml:space="preserve">C+←</t>
   </si>
   <si>
-    <t xml:space="preserve">10Key</t>
+    <t xml:space="preserve">Mouse</t>
   </si>
   <si>
-    <t xml:space="preserve">Mouse</t>
+    <t xml:space="preserve">10Key</t>
   </si>
   <si>
     <t xml:space="preserve">S+End</t>
@@ -945,12 +951,12 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -3325,12 +3331,16 @@
       </c>
       <c r="BW19" s="18"/>
       <c r="BX19" s="18"/>
-      <c r="BY19" s="7"/>
-      <c r="BZ19" s="7"/>
-      <c r="CA19" s="7"/>
-      <c r="CB19" s="7"/>
-      <c r="CC19" s="7"/>
-      <c r="CD19" s="7"/>
+      <c r="BY19" s="19" t="s">
+        <v>144</v>
+      </c>
+      <c r="BZ19" s="19"/>
+      <c r="CA19" s="19"/>
+      <c r="CB19" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="CC19" s="10"/>
+      <c r="CD19" s="10"/>
       <c r="CE19" s="6"/>
       <c r="CF19" s="6"/>
       <c r="CG19" s="6"/>
@@ -3344,32 +3354,32 @@
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
       <c r="D20" s="13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E20" s="13"/>
       <c r="F20" s="13"/>
       <c r="G20" s="13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H20" s="13"/>
       <c r="I20" s="13"/>
       <c r="J20" s="13" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="K20" s="13"/>
       <c r="L20" s="13"/>
-      <c r="M20" s="19" t="s">
+      <c r="M20" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="N20" s="19"/>
-      <c r="O20" s="19"/>
+      <c r="N20" s="20"/>
+      <c r="O20" s="20"/>
       <c r="P20" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Q20" s="13"/>
       <c r="R20" s="13"/>
       <c r="S20" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="T20" s="6"/>
       <c r="U20" s="6"/>
@@ -3394,12 +3404,12 @@
       <c r="AF20" s="13"/>
       <c r="AG20" s="13"/>
       <c r="AH20" s="13" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="AI20" s="13"/>
       <c r="AJ20" s="13"/>
       <c r="AK20" s="13" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="AL20" s="13"/>
       <c r="AM20" s="13"/>
@@ -3411,42 +3421,42 @@
       <c r="AT20" s="7"/>
       <c r="AU20" s="7"/>
       <c r="AV20" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="AW20" s="13"/>
       <c r="AX20" s="13"/>
       <c r="AY20" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="AZ20" s="13"/>
       <c r="BA20" s="13"/>
       <c r="BB20" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="BC20" s="13"/>
       <c r="BD20" s="13"/>
       <c r="BE20" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BF20" s="13"/>
       <c r="BG20" s="13"/>
       <c r="BH20" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="BI20" s="13"/>
       <c r="BJ20" s="13"/>
-      <c r="BK20" s="20" t="s">
-        <v>155</v>
-      </c>
-      <c r="BL20" s="20"/>
-      <c r="BM20" s="20"/>
+      <c r="BK20" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="BL20" s="19"/>
+      <c r="BM20" s="19"/>
       <c r="BN20" s="8" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="BO20" s="8"/>
       <c r="BP20" s="8"/>
       <c r="BQ20" s="6" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="BR20" s="6"/>
       <c r="BS20" s="6"/>
@@ -3479,53 +3489,55 @@
       <c r="C21" s="7"/>
       <c r="D21" s="7"/>
       <c r="E21" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F21" s="13"/>
       <c r="G21" s="13"/>
       <c r="H21" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I21" s="13"/>
       <c r="J21" s="13"/>
       <c r="K21" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="L21" s="13"/>
       <c r="M21" s="13"/>
       <c r="N21" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="O21" s="13"/>
       <c r="P21" s="13"/>
       <c r="Q21" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="R21" s="13"/>
       <c r="S21" s="13"/>
       <c r="T21" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="U21" s="7"/>
       <c r="V21" s="7"/>
       <c r="W21" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="X21" s="7"/>
       <c r="Y21" s="7"/>
-      <c r="Z21" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="AA21" s="13"/>
-      <c r="AB21" s="13"/>
+      <c r="Z21" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="AA21" s="7"/>
+      <c r="AB21" s="7"/>
       <c r="AC21" s="21" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AD21" s="21"/>
       <c r="AE21" s="21"/>
-      <c r="AF21" s="6"/>
-      <c r="AG21" s="6"/>
-      <c r="AH21" s="6"/>
+      <c r="AF21" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="AG21" s="13"/>
+      <c r="AH21" s="13"/>
       <c r="AI21" s="6"/>
       <c r="AJ21" s="6"/>
       <c r="AK21" s="6" t="s">
@@ -3544,43 +3556,45 @@
       <c r="AU21" s="7"/>
       <c r="AV21" s="7"/>
       <c r="AW21" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="AX21" s="13"/>
       <c r="AY21" s="13"/>
       <c r="AZ21" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="BA21" s="13"/>
       <c r="BB21" s="13"/>
       <c r="BC21" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="BD21" s="13"/>
       <c r="BE21" s="13"/>
       <c r="BF21" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BG21" s="13"/>
       <c r="BH21" s="13"/>
       <c r="BI21" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="BJ21" s="13"/>
       <c r="BK21" s="13"/>
       <c r="BL21" s="10" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="BM21" s="10"/>
       <c r="BN21" s="10"/>
       <c r="BO21" s="18" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="BP21" s="18"/>
       <c r="BQ21" s="18"/>
-      <c r="BR21" s="7"/>
-      <c r="BS21" s="7"/>
-      <c r="BT21" s="7"/>
+      <c r="BR21" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="BS21" s="18"/>
+      <c r="BT21" s="18"/>
       <c r="BU21" s="7"/>
       <c r="BV21" s="7"/>
       <c r="BW21" s="7"/>
@@ -3856,7 +3870,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -3900,9 +3914,6 @@
       <c r="AO25" s="4"/>
       <c r="AP25" s="4"/>
       <c r="AQ25" s="5"/>
-      <c r="AR25" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="AS25" s="15"/>
       <c r="AT25" s="15"/>
       <c r="AU25" s="4"/>
@@ -4117,12 +4128,12 @@
       <c r="BH27" s="7"/>
       <c r="BI27" s="7"/>
       <c r="BJ27" s="7" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="BK27" s="7"/>
       <c r="BL27" s="7"/>
       <c r="BM27" s="22" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="BN27" s="22"/>
       <c r="BO27" s="22"/>
@@ -4132,7 +4143,7 @@
       <c r="BQ27" s="7"/>
       <c r="BR27" s="7"/>
       <c r="BS27" s="22" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="BT27" s="22"/>
       <c r="BU27" s="22"/>
@@ -4158,32 +4169,32 @@
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
       <c r="D28" s="13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E28" s="13"/>
       <c r="F28" s="13"/>
       <c r="G28" s="13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H28" s="13"/>
       <c r="I28" s="13"/>
       <c r="J28" s="13" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="K28" s="13"/>
       <c r="L28" s="13"/>
-      <c r="M28" s="19" t="s">
+      <c r="M28" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="N28" s="19"/>
-      <c r="O28" s="19"/>
+      <c r="N28" s="20"/>
+      <c r="O28" s="20"/>
       <c r="P28" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Q28" s="13"/>
       <c r="R28" s="13"/>
       <c r="S28" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="T28" s="6"/>
       <c r="U28" s="6"/>
@@ -4208,12 +4219,12 @@
       <c r="AF28" s="13"/>
       <c r="AG28" s="13"/>
       <c r="AH28" s="13" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="AI28" s="13"/>
       <c r="AJ28" s="13"/>
       <c r="AK28" s="13" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="AL28" s="13"/>
       <c r="AM28" s="13"/>
@@ -4240,7 +4251,7 @@
       <c r="BI28" s="7"/>
       <c r="BJ28" s="7"/>
       <c r="BK28" s="7" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="BL28" s="7"/>
       <c r="BM28" s="7"/>
@@ -4281,53 +4292,55 @@
       <c r="C29" s="7"/>
       <c r="D29" s="7"/>
       <c r="E29" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F29" s="13"/>
       <c r="G29" s="13"/>
       <c r="H29" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I29" s="13"/>
       <c r="J29" s="13"/>
       <c r="K29" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="L29" s="13"/>
       <c r="M29" s="13"/>
       <c r="N29" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="O29" s="13"/>
       <c r="P29" s="13"/>
       <c r="Q29" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="R29" s="13"/>
       <c r="S29" s="13"/>
       <c r="T29" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="U29" s="7"/>
       <c r="V29" s="7"/>
       <c r="W29" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="X29" s="7"/>
       <c r="Y29" s="7"/>
-      <c r="Z29" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="AA29" s="13"/>
-      <c r="AB29" s="13"/>
+      <c r="Z29" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="AA29" s="7"/>
+      <c r="AB29" s="7"/>
       <c r="AC29" s="21" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AD29" s="21"/>
       <c r="AE29" s="21"/>
-      <c r="AF29" s="6"/>
-      <c r="AG29" s="6"/>
-      <c r="AH29" s="6"/>
+      <c r="AF29" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="AG29" s="13"/>
+      <c r="AH29" s="13"/>
       <c r="AI29" s="6"/>
       <c r="AJ29" s="6"/>
       <c r="AK29" s="6" t="s">
@@ -4361,7 +4374,7 @@
       <c r="BJ29" s="7"/>
       <c r="BK29" s="7"/>
       <c r="BL29" s="7" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="BM29" s="7"/>
       <c r="BN29" s="7"/>
@@ -4489,7 +4502,7 @@
       <c r="CB30" s="11"/>
       <c r="CC30" s="11"/>
       <c r="CD30" s="6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="CE30" s="6"/>
       <c r="CF30" s="6"/>
@@ -4576,17 +4589,17 @@
       <c r="BY31" s="7"/>
       <c r="BZ31" s="7"/>
       <c r="CA31" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="CB31" s="6"/>
       <c r="CC31" s="6"/>
       <c r="CD31" s="6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="CE31" s="6"/>
       <c r="CF31" s="6"/>
       <c r="CG31" s="24" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="CH31" s="24"/>
       <c r="CI31" s="24"/>
@@ -4635,6 +4648,8 @@
       <c r="AO32" s="12"/>
       <c r="AP32" s="12"/>
       <c r="AQ32" s="12"/>
+      <c r="AS32" s="12"/>
+      <c r="AT32" s="12"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3"/>
@@ -4680,8 +4695,8 @@
       <c r="AO33" s="4"/>
       <c r="AP33" s="4"/>
       <c r="AQ33" s="5"/>
-      <c r="AS33" s="3"/>
-      <c r="AT33" s="15"/>
+      <c r="AS33" s="4"/>
+      <c r="AT33" s="5"/>
       <c r="AU33" s="4"/>
       <c r="AV33" s="4"/>
       <c r="AW33" s="4"/>
@@ -4709,7 +4724,7 @@
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
       <c r="H34" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I34" s="6"/>
       <c r="J34" s="6"/>
@@ -4834,17 +4849,17 @@
       <c r="G35" s="13"/>
       <c r="H35" s="13"/>
       <c r="I35" s="13" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="J35" s="13"/>
       <c r="K35" s="13"/>
       <c r="L35" s="25" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="M35" s="25"/>
       <c r="N35" s="25"/>
       <c r="O35" s="13" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="P35" s="13"/>
       <c r="Q35" s="13"/>
@@ -4951,30 +4966,30 @@
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="13" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E36" s="13"/>
       <c r="F36" s="13"/>
       <c r="G36" s="13" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H36" s="13"/>
       <c r="I36" s="13"/>
       <c r="J36" s="13"/>
       <c r="K36" s="13"/>
       <c r="L36" s="13"/>
-      <c r="M36" s="19" t="s">
+      <c r="M36" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="N36" s="19"/>
-      <c r="O36" s="19"/>
+      <c r="N36" s="20"/>
+      <c r="O36" s="20"/>
       <c r="P36" s="13" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="Q36" s="13"/>
       <c r="R36" s="13"/>
       <c r="S36" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="T36" s="6"/>
       <c r="U36" s="6"/>
@@ -4999,12 +5014,12 @@
       <c r="AF36" s="13"/>
       <c r="AG36" s="13"/>
       <c r="AH36" s="13" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AI36" s="13"/>
       <c r="AJ36" s="13"/>
       <c r="AK36" s="13" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="AL36" s="13"/>
       <c r="AM36" s="13"/>
@@ -5076,53 +5091,55 @@
       <c r="C37" s="7"/>
       <c r="D37" s="7"/>
       <c r="E37" s="13" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="F37" s="13"/>
       <c r="G37" s="13"/>
       <c r="H37" s="13" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="I37" s="13"/>
       <c r="J37" s="13"/>
       <c r="K37" s="13" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="L37" s="13"/>
       <c r="M37" s="13"/>
       <c r="N37" s="13" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="O37" s="13"/>
       <c r="P37" s="13"/>
       <c r="Q37" s="13" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="R37" s="13"/>
       <c r="S37" s="13"/>
       <c r="T37" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="U37" s="7"/>
       <c r="V37" s="7"/>
       <c r="W37" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="X37" s="7"/>
       <c r="Y37" s="7"/>
-      <c r="Z37" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="AA37" s="13"/>
-      <c r="AB37" s="13"/>
+      <c r="Z37" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="AA37" s="7"/>
+      <c r="AB37" s="7"/>
       <c r="AC37" s="21" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AD37" s="21"/>
       <c r="AE37" s="21"/>
-      <c r="AF37" s="6"/>
-      <c r="AG37" s="6"/>
-      <c r="AH37" s="6"/>
+      <c r="AF37" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="AG37" s="13"/>
+      <c r="AH37" s="13"/>
       <c r="AI37" s="6"/>
       <c r="AJ37" s="6"/>
       <c r="AK37" s="6" t="s">
@@ -5428,7 +5445,7 @@
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B41" s="15"/>
       <c r="C41" s="15"/>
@@ -5773,32 +5790,32 @@
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E44" s="13"/>
       <c r="F44" s="13"/>
       <c r="G44" s="13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H44" s="13"/>
       <c r="I44" s="13"/>
       <c r="J44" s="13" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="K44" s="13"/>
       <c r="L44" s="13"/>
-      <c r="M44" s="19" t="s">
+      <c r="M44" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="N44" s="19"/>
-      <c r="O44" s="19"/>
+      <c r="N44" s="20"/>
+      <c r="O44" s="20"/>
       <c r="P44" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Q44" s="13"/>
       <c r="R44" s="13"/>
       <c r="S44" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="T44" s="6"/>
       <c r="U44" s="6"/>
@@ -5823,12 +5840,12 @@
       <c r="AF44" s="13"/>
       <c r="AG44" s="13"/>
       <c r="AH44" s="13" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="AI44" s="13"/>
       <c r="AJ44" s="13"/>
       <c r="AK44" s="13" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="AL44" s="13"/>
       <c r="AM44" s="13"/>
@@ -5842,32 +5859,32 @@
       <c r="AT44" s="7"/>
       <c r="AU44" s="7"/>
       <c r="AV44" s="13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="AW44" s="13"/>
       <c r="AX44" s="13"/>
       <c r="AY44" s="13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="AZ44" s="13"/>
       <c r="BA44" s="13"/>
       <c r="BB44" s="13" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="BC44" s="13"/>
       <c r="BD44" s="13"/>
-      <c r="BE44" s="19" t="s">
+      <c r="BE44" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="BF44" s="19"/>
-      <c r="BG44" s="19"/>
+      <c r="BF44" s="20"/>
+      <c r="BG44" s="20"/>
       <c r="BH44" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="BI44" s="13"/>
       <c r="BJ44" s="13"/>
       <c r="BK44" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="BL44" s="6"/>
       <c r="BM44" s="6"/>
@@ -5892,12 +5909,12 @@
       <c r="BX44" s="13"/>
       <c r="BY44" s="13"/>
       <c r="BZ44" s="13" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="CA44" s="13"/>
       <c r="CB44" s="13"/>
       <c r="CC44" s="13" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="CD44" s="13"/>
       <c r="CE44" s="13"/>
@@ -5914,53 +5931,55 @@
       <c r="C45" s="7"/>
       <c r="D45" s="7"/>
       <c r="E45" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F45" s="13"/>
       <c r="G45" s="13"/>
       <c r="H45" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I45" s="13"/>
       <c r="J45" s="13"/>
       <c r="K45" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="L45" s="13"/>
       <c r="M45" s="13"/>
       <c r="N45" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="O45" s="13"/>
       <c r="P45" s="13"/>
       <c r="Q45" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="R45" s="13"/>
       <c r="S45" s="13"/>
       <c r="T45" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="U45" s="7"/>
       <c r="V45" s="7"/>
       <c r="W45" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="X45" s="7"/>
       <c r="Y45" s="7"/>
-      <c r="Z45" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="AA45" s="13"/>
-      <c r="AB45" s="13"/>
+      <c r="Z45" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="AA45" s="7"/>
+      <c r="AB45" s="7"/>
       <c r="AC45" s="21" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AD45" s="21"/>
       <c r="AE45" s="21"/>
-      <c r="AF45" s="6"/>
-      <c r="AG45" s="6"/>
-      <c r="AH45" s="6"/>
+      <c r="AF45" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="AG45" s="13"/>
+      <c r="AH45" s="13"/>
       <c r="AI45" s="6"/>
       <c r="AJ45" s="6"/>
       <c r="AK45" s="6" t="s">
@@ -5981,53 +6000,55 @@
       <c r="AU45" s="7"/>
       <c r="AV45" s="7"/>
       <c r="AW45" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="AX45" s="13"/>
       <c r="AY45" s="13"/>
       <c r="AZ45" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="BA45" s="13"/>
       <c r="BB45" s="13"/>
       <c r="BC45" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="BD45" s="13"/>
       <c r="BE45" s="13"/>
       <c r="BF45" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BG45" s="13"/>
       <c r="BH45" s="13"/>
       <c r="BI45" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="BJ45" s="13"/>
       <c r="BK45" s="13"/>
       <c r="BL45" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="BM45" s="7"/>
       <c r="BN45" s="7"/>
       <c r="BO45" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="BP45" s="7"/>
       <c r="BQ45" s="7"/>
-      <c r="BR45" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="BS45" s="13"/>
-      <c r="BT45" s="13"/>
+      <c r="BR45" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="BS45" s="7"/>
+      <c r="BT45" s="7"/>
       <c r="BU45" s="21" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="BV45" s="21"/>
       <c r="BW45" s="21"/>
-      <c r="BX45" s="6"/>
-      <c r="BY45" s="6"/>
-      <c r="BZ45" s="6"/>
+      <c r="BX45" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="BY45" s="13"/>
+      <c r="BZ45" s="13"/>
       <c r="CA45" s="6"/>
       <c r="CB45" s="6"/>
       <c r="CC45" s="6" t="s">
@@ -8424,8 +8445,8 @@
       <c r="CI7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0"/>
-      <c r="B8" s="0"/>
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
       <c r="C8" s="12"/>
       <c r="D8" s="12"/>
       <c r="E8" s="12"/>
@@ -8469,8 +8490,8 @@
       <c r="AQ8" s="12"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0"/>
-      <c r="B9" s="0"/>
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
       <c r="C9" s="3" t="s">
         <v>57</v>
       </c>
@@ -8650,7 +8671,7 @@
       <c r="BP10" s="13"/>
       <c r="BQ10" s="13"/>
       <c r="BR10" s="13" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="BS10" s="13"/>
       <c r="BT10" s="13"/>
@@ -8744,7 +8765,7 @@
       <c r="AK11" s="6"/>
       <c r="AL11" s="6"/>
       <c r="AM11" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="AN11" s="6"/>
       <c r="AO11" s="6"/>
@@ -9413,7 +9434,7 @@
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>108</v>
@@ -9619,7 +9640,7 @@
       <c r="AK19" s="13"/>
       <c r="AL19" s="13"/>
       <c r="AM19" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="AN19" s="6"/>
       <c r="AO19" s="6"/>
@@ -9674,7 +9695,7 @@
       <c r="CC19" s="7"/>
       <c r="CD19" s="7"/>
       <c r="CE19" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="CF19" s="6"/>
       <c r="CG19" s="6"/>
@@ -9688,32 +9709,32 @@
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
       <c r="D20" s="13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E20" s="13"/>
       <c r="F20" s="13"/>
       <c r="G20" s="13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H20" s="13"/>
       <c r="I20" s="13"/>
       <c r="J20" s="13" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="K20" s="13"/>
       <c r="L20" s="13"/>
-      <c r="M20" s="19" t="s">
+      <c r="M20" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="N20" s="19"/>
-      <c r="O20" s="19"/>
+      <c r="N20" s="20"/>
+      <c r="O20" s="20"/>
       <c r="P20" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Q20" s="13"/>
       <c r="R20" s="13"/>
       <c r="S20" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="T20" s="6"/>
       <c r="U20" s="6"/>
@@ -9738,7 +9759,7 @@
       <c r="AF20" s="13"/>
       <c r="AG20" s="13"/>
       <c r="AH20" s="13" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="AI20" s="13"/>
       <c r="AJ20" s="13"/>
@@ -9755,42 +9776,42 @@
       <c r="AT20" s="7"/>
       <c r="AU20" s="7"/>
       <c r="AV20" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="AW20" s="13"/>
       <c r="AX20" s="13"/>
       <c r="AY20" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="AZ20" s="13"/>
       <c r="BA20" s="13"/>
       <c r="BB20" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="BC20" s="13"/>
       <c r="BD20" s="13"/>
       <c r="BE20" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BF20" s="13"/>
       <c r="BG20" s="13"/>
       <c r="BH20" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="BI20" s="13"/>
       <c r="BJ20" s="13"/>
-      <c r="BK20" s="20" t="s">
-        <v>155</v>
-      </c>
-      <c r="BL20" s="20"/>
-      <c r="BM20" s="20"/>
+      <c r="BK20" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="BL20" s="19"/>
+      <c r="BM20" s="19"/>
       <c r="BN20" s="8" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="BO20" s="8"/>
       <c r="BP20" s="8"/>
       <c r="BQ20" s="6" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="BR20" s="6"/>
       <c r="BS20" s="6"/>
@@ -9825,47 +9846,47 @@
       <c r="C21" s="7"/>
       <c r="D21" s="7"/>
       <c r="E21" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F21" s="13"/>
       <c r="G21" s="13"/>
       <c r="H21" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I21" s="13"/>
       <c r="J21" s="13"/>
       <c r="K21" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="L21" s="13"/>
       <c r="M21" s="13"/>
       <c r="N21" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="O21" s="13"/>
       <c r="P21" s="13"/>
       <c r="Q21" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="R21" s="13"/>
       <c r="S21" s="13"/>
       <c r="T21" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="U21" s="7"/>
       <c r="V21" s="7"/>
       <c r="W21" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="X21" s="7"/>
       <c r="Y21" s="7"/>
       <c r="Z21" s="13" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="AA21" s="13"/>
       <c r="AB21" s="13"/>
       <c r="AC21" s="21" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AD21" s="21"/>
       <c r="AE21" s="21"/>
@@ -9892,37 +9913,37 @@
       <c r="AU21" s="7"/>
       <c r="AV21" s="7"/>
       <c r="AW21" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="AX21" s="13"/>
       <c r="AY21" s="13"/>
       <c r="AZ21" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="BA21" s="13"/>
       <c r="BB21" s="13"/>
       <c r="BC21" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="BD21" s="13"/>
       <c r="BE21" s="13"/>
       <c r="BF21" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BG21" s="13"/>
       <c r="BH21" s="13"/>
       <c r="BI21" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="BJ21" s="13"/>
       <c r="BK21" s="13"/>
       <c r="BL21" s="10" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="BM21" s="10"/>
       <c r="BN21" s="10"/>
       <c r="BO21" s="18" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="BP21" s="18"/>
       <c r="BQ21" s="18"/>
@@ -10208,7 +10229,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -10455,7 +10476,7 @@
       <c r="AK27" s="13"/>
       <c r="AL27" s="13"/>
       <c r="AM27" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="AN27" s="6"/>
       <c r="AO27" s="6"/>
@@ -10479,12 +10500,12 @@
       <c r="BH27" s="7"/>
       <c r="BI27" s="7"/>
       <c r="BJ27" s="7" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="BK27" s="7"/>
       <c r="BL27" s="7"/>
       <c r="BM27" s="22" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="BN27" s="22"/>
       <c r="BO27" s="22"/>
@@ -10494,7 +10515,7 @@
       <c r="BQ27" s="7"/>
       <c r="BR27" s="7"/>
       <c r="BS27" s="22" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="BT27" s="22"/>
       <c r="BU27" s="22"/>
@@ -10508,7 +10529,7 @@
       <c r="CC27" s="7"/>
       <c r="CD27" s="7"/>
       <c r="CE27" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="CF27" s="6"/>
       <c r="CG27" s="6"/>
@@ -10522,32 +10543,32 @@
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
       <c r="D28" s="13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E28" s="13"/>
       <c r="F28" s="13"/>
       <c r="G28" s="13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H28" s="13"/>
       <c r="I28" s="13"/>
       <c r="J28" s="13" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="K28" s="13"/>
       <c r="L28" s="13"/>
-      <c r="M28" s="19" t="s">
+      <c r="M28" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="N28" s="19"/>
-      <c r="O28" s="19"/>
+      <c r="N28" s="20"/>
+      <c r="O28" s="20"/>
       <c r="P28" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Q28" s="13"/>
       <c r="R28" s="13"/>
       <c r="S28" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="T28" s="6"/>
       <c r="U28" s="6"/>
@@ -10572,7 +10593,7 @@
       <c r="AF28" s="13"/>
       <c r="AG28" s="13"/>
       <c r="AH28" s="13" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="AI28" s="13"/>
       <c r="AJ28" s="13"/>
@@ -10604,7 +10625,7 @@
       <c r="BI28" s="7"/>
       <c r="BJ28" s="7"/>
       <c r="BK28" s="7" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="BL28" s="7"/>
       <c r="BM28" s="7"/>
@@ -10647,47 +10668,47 @@
       <c r="C29" s="7"/>
       <c r="D29" s="7"/>
       <c r="E29" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F29" s="13"/>
       <c r="G29" s="13"/>
       <c r="H29" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I29" s="13"/>
       <c r="J29" s="13"/>
       <c r="K29" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="L29" s="13"/>
       <c r="M29" s="13"/>
       <c r="N29" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="O29" s="13"/>
       <c r="P29" s="13"/>
       <c r="Q29" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="R29" s="13"/>
       <c r="S29" s="13"/>
       <c r="T29" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="U29" s="7"/>
       <c r="V29" s="7"/>
       <c r="W29" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="X29" s="7"/>
       <c r="Y29" s="7"/>
       <c r="Z29" s="13" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="AA29" s="13"/>
       <c r="AB29" s="13"/>
       <c r="AC29" s="21" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AD29" s="21"/>
       <c r="AE29" s="21"/>
@@ -10729,7 +10750,7 @@
       <c r="BJ29" s="7"/>
       <c r="BK29" s="7"/>
       <c r="BL29" s="7" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="BM29" s="7"/>
       <c r="BN29" s="7"/>
@@ -10869,7 +10890,7 @@
       <c r="CB30" s="11"/>
       <c r="CC30" s="11"/>
       <c r="CD30" s="6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="CE30" s="6"/>
       <c r="CF30" s="6"/>
@@ -10964,17 +10985,17 @@
       <c r="BY31" s="7"/>
       <c r="BZ31" s="7"/>
       <c r="CA31" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="CB31" s="6"/>
       <c r="CC31" s="6"/>
       <c r="CD31" s="6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="CE31" s="6"/>
       <c r="CF31" s="6"/>
       <c r="CG31" s="24" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="CH31" s="24"/>
       <c r="CI31" s="24"/>
@@ -11280,7 +11301,7 @@
       <c r="AK35" s="13"/>
       <c r="AL35" s="13"/>
       <c r="AM35" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="AN35" s="6"/>
       <c r="AO35" s="6"/>
@@ -11337,7 +11358,7 @@
       <c r="CC35" s="7"/>
       <c r="CD35" s="7"/>
       <c r="CE35" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="CF35" s="6"/>
       <c r="CG35" s="6"/>
@@ -11351,32 +11372,32 @@
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E36" s="13"/>
       <c r="F36" s="13"/>
       <c r="G36" s="13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H36" s="13"/>
       <c r="I36" s="13"/>
       <c r="J36" s="13" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="K36" s="13"/>
       <c r="L36" s="13"/>
-      <c r="M36" s="19" t="s">
+      <c r="M36" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="N36" s="19"/>
-      <c r="O36" s="19"/>
+      <c r="N36" s="20"/>
+      <c r="O36" s="20"/>
       <c r="P36" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Q36" s="13"/>
       <c r="R36" s="13"/>
       <c r="S36" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="T36" s="6"/>
       <c r="U36" s="6"/>
@@ -11401,7 +11422,7 @@
       <c r="AF36" s="13"/>
       <c r="AG36" s="13"/>
       <c r="AH36" s="13" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="AI36" s="13"/>
       <c r="AJ36" s="13"/>
@@ -11480,47 +11501,47 @@
       <c r="C37" s="7"/>
       <c r="D37" s="7"/>
       <c r="E37" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F37" s="13"/>
       <c r="G37" s="13"/>
       <c r="H37" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I37" s="13"/>
       <c r="J37" s="13"/>
       <c r="K37" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="L37" s="13"/>
       <c r="M37" s="13"/>
       <c r="N37" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="O37" s="13"/>
       <c r="P37" s="13"/>
       <c r="Q37" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="R37" s="13"/>
       <c r="S37" s="13"/>
       <c r="T37" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="U37" s="7"/>
       <c r="V37" s="7"/>
       <c r="W37" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="X37" s="7"/>
       <c r="Y37" s="7"/>
       <c r="Z37" s="13" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="AA37" s="13"/>
       <c r="AB37" s="13"/>
       <c r="AC37" s="21" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AD37" s="21"/>
       <c r="AE37" s="21"/>
@@ -12891,7 +12912,7 @@
       <c r="AP1" s="4"/>
       <c r="AQ1" s="5"/>
       <c r="AT1" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="AU1" s="4"/>
       <c r="AV1" s="4"/>
@@ -13085,14 +13106,14 @@
       <c r="AX3" s="6"/>
       <c r="AY3" s="6"/>
       <c r="AZ3" s="6"/>
-      <c r="BA3" s="20" t="s">
-        <v>166</v>
+      <c r="BA3" s="19" t="s">
+        <v>168</v>
       </c>
       <c r="BB3" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="BC3" s="20" t="s">
-        <v>167</v>
+      <c r="BC3" s="19" t="s">
+        <v>169</v>
       </c>
       <c r="BD3" s="6"/>
       <c r="BE3" s="6"/>
@@ -13171,10 +13192,10 @@
       <c r="AP4" s="9"/>
       <c r="AQ4" s="9"/>
       <c r="AR4" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="AT4" s="7" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="AU4" s="7"/>
       <c r="AV4" s="7"/>
@@ -13182,7 +13203,7 @@
       <c r="AX4" s="8"/>
       <c r="AY4" s="6"/>
       <c r="AZ4" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="BA4" s="8" t="s">
         <v>54</v>
@@ -13272,7 +13293,7 @@
       <c r="AP5" s="6"/>
       <c r="AQ5" s="6"/>
       <c r="AR5" s="29" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="AT5" s="7"/>
       <c r="AU5" s="7"/>
@@ -13281,10 +13302,10 @@
       <c r="AX5" s="7"/>
       <c r="AY5" s="7"/>
       <c r="AZ5" s="6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="BA5" s="7" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="BB5" s="7"/>
       <c r="BC5" s="7"/>
@@ -13341,10 +13362,10 @@
       <c r="V6" s="7"/>
       <c r="W6" s="7"/>
       <c r="X6" s="7" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="Y6" s="7" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="Z6" s="7"/>
       <c r="AA6" s="7"/>
@@ -13387,7 +13408,7 @@
       <c r="AW6" s="7"/>
       <c r="AX6" s="7"/>
       <c r="AY6" s="7" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="AZ6" s="7"/>
       <c r="BA6" s="7"/>
@@ -13396,7 +13417,7 @@
       <c r="BD6" s="6"/>
       <c r="BE6" s="11"/>
       <c r="BF6" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="BG6" s="11"/>
       <c r="BH6" s="11"/>
@@ -13458,13 +13479,13 @@
       <c r="BC7" s="11"/>
       <c r="BD7" s="6"/>
       <c r="BE7" s="7" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="BF7" s="6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="BG7" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="BH7" s="6"/>
     </row>
@@ -13515,7 +13536,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -13936,7 +13957,7 @@
       <c r="AP12" s="9"/>
       <c r="AQ12" s="9"/>
       <c r="AR12" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="AT12" s="7"/>
       <c r="AU12" s="7"/>
@@ -14079,7 +14100,7 @@
       <c r="AP13" s="6"/>
       <c r="AQ13" s="6"/>
       <c r="AR13" s="29" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="AT13" s="7"/>
       <c r="AU13" s="7"/>
@@ -14192,10 +14213,10 @@
       </c>
       <c r="W14" s="7"/>
       <c r="X14" s="7" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="Y14" s="7" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="Z14" s="7"/>
       <c r="AA14" s="7"/>
@@ -14474,7 +14495,7 @@
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>108</v>
@@ -14747,32 +14768,32 @@
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
       <c r="D20" s="13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E20" s="13"/>
       <c r="F20" s="13"/>
       <c r="G20" s="13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H20" s="13"/>
       <c r="I20" s="13"/>
       <c r="J20" s="13" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="K20" s="13"/>
       <c r="L20" s="13"/>
-      <c r="M20" s="19" t="s">
+      <c r="M20" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="N20" s="19"/>
-      <c r="O20" s="19"/>
+      <c r="N20" s="20"/>
+      <c r="O20" s="20"/>
       <c r="P20" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Q20" s="13"/>
       <c r="R20" s="13"/>
       <c r="S20" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="T20" s="6"/>
       <c r="U20" s="6"/>
@@ -14797,12 +14818,12 @@
       <c r="AF20" s="13"/>
       <c r="AG20" s="13"/>
       <c r="AH20" s="13" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="AI20" s="13"/>
       <c r="AJ20" s="13"/>
       <c r="AK20" s="13" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="AL20" s="13"/>
       <c r="AM20" s="13"/>
@@ -14811,48 +14832,48 @@
       <c r="AP20" s="9"/>
       <c r="AQ20" s="9"/>
       <c r="AR20" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="AT20" s="7"/>
       <c r="AU20" s="7"/>
       <c r="AV20" s="7"/>
       <c r="AW20" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="AX20" s="13"/>
       <c r="AY20" s="13"/>
       <c r="AZ20" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="BA20" s="13"/>
       <c r="BB20" s="13"/>
       <c r="BC20" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="BD20" s="13"/>
       <c r="BE20" s="13"/>
       <c r="BF20" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BG20" s="13"/>
       <c r="BH20" s="13"/>
       <c r="BI20" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="BJ20" s="13"/>
       <c r="BK20" s="13"/>
-      <c r="BL20" s="20" t="s">
-        <v>155</v>
-      </c>
-      <c r="BM20" s="20"/>
-      <c r="BN20" s="20"/>
+      <c r="BL20" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="BM20" s="19"/>
+      <c r="BN20" s="19"/>
       <c r="BO20" s="8" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="BP20" s="8"/>
       <c r="BQ20" s="8"/>
       <c r="BR20" s="6" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="BS20" s="6"/>
       <c r="BT20" s="6"/>
@@ -14885,47 +14906,47 @@
       <c r="C21" s="7"/>
       <c r="D21" s="7"/>
       <c r="E21" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F21" s="13"/>
       <c r="G21" s="13"/>
       <c r="H21" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I21" s="13"/>
       <c r="J21" s="13"/>
       <c r="K21" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="L21" s="13"/>
       <c r="M21" s="13"/>
       <c r="N21" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="O21" s="13"/>
       <c r="P21" s="13"/>
       <c r="Q21" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="R21" s="13"/>
       <c r="S21" s="13"/>
       <c r="T21" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="U21" s="7"/>
       <c r="V21" s="7"/>
       <c r="W21" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="X21" s="7"/>
       <c r="Y21" s="7"/>
       <c r="Z21" s="13" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="AA21" s="13"/>
       <c r="AB21" s="13"/>
       <c r="AC21" s="21" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AD21" s="21"/>
       <c r="AE21" s="21"/>
@@ -14946,44 +14967,44 @@
       <c r="AP21" s="6"/>
       <c r="AQ21" s="6"/>
       <c r="AR21" s="29" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="AT21" s="7"/>
       <c r="AU21" s="7"/>
       <c r="AV21" s="7"/>
       <c r="AW21" s="7"/>
       <c r="AX21" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="AY21" s="13"/>
       <c r="AZ21" s="13"/>
       <c r="BA21" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="BB21" s="13"/>
       <c r="BC21" s="13"/>
       <c r="BD21" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="BE21" s="13"/>
       <c r="BF21" s="13"/>
       <c r="BG21" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BH21" s="13"/>
       <c r="BI21" s="13"/>
       <c r="BJ21" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="BK21" s="13"/>
       <c r="BL21" s="13"/>
       <c r="BM21" s="10" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="BN21" s="10"/>
       <c r="BO21" s="10"/>
       <c r="BP21" s="18" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="BQ21" s="18"/>
       <c r="BR21" s="18"/>
@@ -15055,10 +15076,10 @@
       </c>
       <c r="W22" s="7"/>
       <c r="X22" s="7" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="Y22" s="7" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="Z22" s="7"/>
       <c r="AA22" s="7"/>
@@ -15277,7 +15298,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -15544,12 +15565,12 @@
       <c r="BI27" s="7"/>
       <c r="BJ27" s="7"/>
       <c r="BK27" s="7" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="BL27" s="7"/>
       <c r="BM27" s="7"/>
       <c r="BN27" s="22" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="BO27" s="22"/>
       <c r="BP27" s="22"/>
@@ -15559,7 +15580,7 @@
       <c r="BR27" s="7"/>
       <c r="BS27" s="7"/>
       <c r="BT27" s="22" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="BU27" s="22"/>
       <c r="BV27" s="22"/>
@@ -15585,32 +15606,32 @@
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
       <c r="D28" s="13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E28" s="13"/>
       <c r="F28" s="13"/>
       <c r="G28" s="13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H28" s="13"/>
       <c r="I28" s="13"/>
       <c r="J28" s="13" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="K28" s="13"/>
       <c r="L28" s="13"/>
-      <c r="M28" s="19" t="s">
+      <c r="M28" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="N28" s="19"/>
-      <c r="O28" s="19"/>
+      <c r="N28" s="20"/>
+      <c r="O28" s="20"/>
       <c r="P28" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Q28" s="13"/>
       <c r="R28" s="13"/>
       <c r="S28" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="T28" s="6"/>
       <c r="U28" s="6"/>
@@ -15635,12 +15656,12 @@
       <c r="AF28" s="13"/>
       <c r="AG28" s="13"/>
       <c r="AH28" s="13" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="AI28" s="13"/>
       <c r="AJ28" s="13"/>
       <c r="AK28" s="13" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="AL28" s="13"/>
       <c r="AM28" s="13"/>
@@ -15649,7 +15670,7 @@
       <c r="AP28" s="9"/>
       <c r="AQ28" s="9"/>
       <c r="AR28" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="AT28" s="7"/>
       <c r="AU28" s="7"/>
@@ -15670,7 +15691,7 @@
       <c r="BJ28" s="7"/>
       <c r="BK28" s="7"/>
       <c r="BL28" s="7" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="BM28" s="7"/>
       <c r="BN28" s="7"/>
@@ -15711,47 +15732,47 @@
       <c r="C29" s="7"/>
       <c r="D29" s="7"/>
       <c r="E29" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F29" s="13"/>
       <c r="G29" s="13"/>
       <c r="H29" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I29" s="13"/>
       <c r="J29" s="13"/>
       <c r="K29" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="L29" s="13"/>
       <c r="M29" s="13"/>
       <c r="N29" s="13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="O29" s="13"/>
       <c r="P29" s="13"/>
       <c r="Q29" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="R29" s="13"/>
       <c r="S29" s="13"/>
       <c r="T29" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="U29" s="7"/>
       <c r="V29" s="7"/>
       <c r="W29" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="X29" s="7"/>
       <c r="Y29" s="7"/>
       <c r="Z29" s="13" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="AA29" s="13"/>
       <c r="AB29" s="13"/>
       <c r="AC29" s="21" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AD29" s="21"/>
       <c r="AE29" s="21"/>
@@ -15772,7 +15793,7 @@
       <c r="AP29" s="6"/>
       <c r="AQ29" s="6"/>
       <c r="AR29" s="29" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="AT29" s="7"/>
       <c r="AU29" s="7"/>
@@ -15794,7 +15815,7 @@
       <c r="BK29" s="7"/>
       <c r="BL29" s="7"/>
       <c r="BM29" s="7" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="BN29" s="7"/>
       <c r="BO29" s="7"/>
@@ -15869,10 +15890,10 @@
       </c>
       <c r="W30" s="7"/>
       <c r="X30" s="7" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="Y30" s="7" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="Z30" s="7"/>
       <c r="AA30" s="7"/>
@@ -15939,7 +15960,7 @@
       </c>
       <c r="BP30" s="7"/>
       <c r="BQ30" s="7" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="BR30" s="7"/>
       <c r="BS30" s="7"/>
@@ -16180,7 +16201,7 @@
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
       <c r="H34" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I34" s="6"/>
       <c r="J34" s="6"/>
@@ -16292,17 +16313,17 @@
       <c r="G35" s="13"/>
       <c r="H35" s="13"/>
       <c r="I35" s="13" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="J35" s="13"/>
       <c r="K35" s="13"/>
       <c r="L35" s="25" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="M35" s="25"/>
       <c r="N35" s="25"/>
       <c r="O35" s="13" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="P35" s="13"/>
       <c r="Q35" s="13"/>
@@ -16380,30 +16401,30 @@
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="13" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E36" s="13"/>
       <c r="F36" s="13"/>
       <c r="G36" s="13" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H36" s="13"/>
       <c r="I36" s="13"/>
       <c r="J36" s="13"/>
       <c r="K36" s="13"/>
       <c r="L36" s="13"/>
-      <c r="M36" s="19" t="s">
+      <c r="M36" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="N36" s="19"/>
-      <c r="O36" s="19"/>
+      <c r="N36" s="20"/>
+      <c r="O36" s="20"/>
       <c r="P36" s="13" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="Q36" s="13"/>
       <c r="R36" s="13"/>
       <c r="S36" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="T36" s="6"/>
       <c r="U36" s="6"/>
@@ -16428,12 +16449,12 @@
       <c r="AF36" s="13"/>
       <c r="AG36" s="13"/>
       <c r="AH36" s="13" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AI36" s="13"/>
       <c r="AJ36" s="13"/>
       <c r="AK36" s="13" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="AL36" s="13"/>
       <c r="AM36" s="13"/>
@@ -16442,34 +16463,34 @@
       <c r="AP36" s="9"/>
       <c r="AQ36" s="9"/>
       <c r="AR36" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="AT36" s="30" t="s">
         <v>82</v>
       </c>
       <c r="AU36" s="13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="AV36" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="AW36" s="13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="AX36" s="14" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="AY36" s="13" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="AZ36" s="17" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BA36" s="8" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="BB36" s="7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="BC36" s="7" t="s">
         <v>142</v>
@@ -16490,47 +16511,47 @@
       <c r="C37" s="7"/>
       <c r="D37" s="7"/>
       <c r="E37" s="13" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="F37" s="13"/>
       <c r="G37" s="13"/>
       <c r="H37" s="13" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="I37" s="13"/>
       <c r="J37" s="13"/>
       <c r="K37" s="13" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="L37" s="13"/>
       <c r="M37" s="13"/>
       <c r="N37" s="13" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="O37" s="13"/>
       <c r="P37" s="13"/>
       <c r="Q37" s="13" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="R37" s="13"/>
       <c r="S37" s="13"/>
       <c r="T37" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="U37" s="7"/>
       <c r="V37" s="7"/>
       <c r="W37" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="X37" s="7"/>
       <c r="Y37" s="7"/>
       <c r="Z37" s="13" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="AA37" s="13"/>
       <c r="AB37" s="13"/>
       <c r="AC37" s="21" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AD37" s="21"/>
       <c r="AE37" s="21"/>
@@ -16551,31 +16572,31 @@
       <c r="AP37" s="6"/>
       <c r="AQ37" s="6"/>
       <c r="AR37" s="29" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="AT37" s="7" t="s">
         <v>33</v>
       </c>
       <c r="AU37" s="13" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="AV37" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="AW37" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="AX37" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="AY37" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="AX37" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="AY37" s="13" t="s">
-        <v>151</v>
-      </c>
       <c r="AZ37" s="18" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="BA37" s="7" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="BB37" s="7" t="s">
         <v>143</v>
@@ -16634,10 +16655,10 @@
       </c>
       <c r="W38" s="7"/>
       <c r="X38" s="7" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="Y38" s="7" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="Z38" s="7"/>
       <c r="AA38" s="7"/>
@@ -17880,9 +17901,9 @@
       <c r="V3" s="6"/>
       <c r="W3" s="6"/>
       <c r="X3" s="6"/>
-      <c r="Y3" s="20"/>
+      <c r="Y3" s="19"/>
       <c r="Z3" s="7"/>
-      <c r="AA3" s="20"/>
+      <c r="AA3" s="19"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
       <c r="AD3" s="6"/>
@@ -17932,7 +17953,7 @@
       <c r="N4" s="6"/>
       <c r="O4" s="6"/>
       <c r="P4" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="R4" s="7"/>
       <c r="S4" s="7"/>
@@ -17993,7 +18014,7 @@
       <c r="N5" s="6"/>
       <c r="O5" s="6"/>
       <c r="P5" s="29" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="R5" s="7"/>
       <c r="S5" s="7"/>
@@ -18124,7 +18145,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -18327,7 +18348,7 @@
       <c r="N12" s="6"/>
       <c r="O12" s="6"/>
       <c r="P12" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="R12" s="7"/>
       <c r="S12" s="13"/>
@@ -18388,7 +18409,7 @@
       <c r="N13" s="6"/>
       <c r="O13" s="6"/>
       <c r="P13" s="29" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="R13" s="7"/>
       <c r="S13" s="13"/>
@@ -18597,7 +18618,7 @@
       <c r="N19" s="6"/>
       <c r="O19" s="6"/>
       <c r="P19" s="32" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="R19" s="7"/>
       <c r="S19" s="7"/>

</xml_diff>

<commit_message>
[Temp] Layout is begin changed.
</commit_message>
<xml_diff>
--- a/img/keymap.xlsx
+++ b/img/keymap.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2347" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2356" uniqueCount="208">
   <si>
     <t xml:space="preserve">標準</t>
   </si>
@@ -584,13 +584,17 @@
     <t xml:space="preserve">Space &amp; F13 修飾</t>
   </si>
   <si>
+    <t xml:space="preserve">SelMode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">StdMode</t>
+  </si>
+  <si>
     <t xml:space="preserve">10Key Mode</t>
   </si>
   <si>
-    <t xml:space="preserve">SelMode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CurMode</t>
+    <t xml:space="preserve">SelCur
+Togle</t>
   </si>
   <si>
     <t xml:space="preserve">Cursor Mode</t>
@@ -599,7 +603,49 @@
     <t xml:space="preserve">Select Mode</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
+    <t xml:space="preserve">CurMode</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve">C+x
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <rFont val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve">CurMode</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve">C+c
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <rFont val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t xml:space="preserve">CurMode</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve"> (</t>
@@ -896,7 +942,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1015,6 +1061,14 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -8353,11 +8407,11 @@
       </c>
       <c r="BV6" s="7"/>
       <c r="BW6" s="7"/>
-      <c r="BX6" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="BY6" s="7"/>
-      <c r="BZ6" s="7"/>
+      <c r="BX6" s="29" t="s">
+        <v>186</v>
+      </c>
+      <c r="BY6" s="29"/>
+      <c r="BZ6" s="29"/>
       <c r="CA6" s="11"/>
       <c r="CB6" s="11"/>
       <c r="CC6" s="11"/>
@@ -8453,9 +8507,9 @@
       <c r="BU7" s="7"/>
       <c r="BV7" s="7"/>
       <c r="BW7" s="7"/>
-      <c r="BX7" s="7"/>
-      <c r="BY7" s="7"/>
-      <c r="BZ7" s="7"/>
+      <c r="BX7" s="29"/>
+      <c r="BY7" s="29"/>
+      <c r="BZ7" s="29"/>
       <c r="CA7" s="6" t="s">
         <v>56</v>
       </c>
@@ -9738,11 +9792,11 @@
       </c>
       <c r="H20" s="13"/>
       <c r="I20" s="13"/>
-      <c r="J20" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="K20" s="13"/>
-      <c r="L20" s="13"/>
+      <c r="J20" s="29" t="s">
+        <v>186</v>
+      </c>
+      <c r="K20" s="29"/>
+      <c r="L20" s="29"/>
       <c r="M20" s="20" t="s">
         <v>7</v>
       </c>
@@ -10553,11 +10607,11 @@
       </c>
       <c r="H28" s="13"/>
       <c r="I28" s="13"/>
-      <c r="J28" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="K28" s="13"/>
-      <c r="L28" s="13"/>
+      <c r="J28" s="29" t="s">
+        <v>186</v>
+      </c>
+      <c r="K28" s="29"/>
+      <c r="L28" s="29"/>
       <c r="M28" s="20" t="s">
         <v>7</v>
       </c>
@@ -10607,7 +10661,9 @@
       <c r="AO28" s="9"/>
       <c r="AP28" s="9"/>
       <c r="AQ28" s="9"/>
-      <c r="AS28" s="7"/>
+      <c r="AS28" s="7" t="s">
+        <v>187</v>
+      </c>
       <c r="AT28" s="7"/>
       <c r="AU28" s="7"/>
       <c r="AV28" s="7"/>
@@ -10852,7 +10908,9 @@
       <c r="BC30" s="7"/>
       <c r="BD30" s="7"/>
       <c r="BE30" s="7"/>
-      <c r="BF30" s="7"/>
+      <c r="BF30" s="7" t="s">
+        <v>187</v>
+      </c>
       <c r="BG30" s="7"/>
       <c r="BH30" s="7"/>
       <c r="BI30" s="7"/>
@@ -10870,9 +10928,11 @@
       <c r="BU30" s="7"/>
       <c r="BV30" s="7"/>
       <c r="BW30" s="7"/>
-      <c r="BX30" s="7"/>
-      <c r="BY30" s="7"/>
-      <c r="BZ30" s="7"/>
+      <c r="BX30" s="29" t="s">
+        <v>186</v>
+      </c>
+      <c r="BY30" s="29"/>
+      <c r="BZ30" s="29"/>
       <c r="CA30" s="11"/>
       <c r="CB30" s="11"/>
       <c r="CC30" s="11"/>
@@ -10960,9 +11020,9 @@
       <c r="BU31" s="7"/>
       <c r="BV31" s="7"/>
       <c r="BW31" s="7"/>
-      <c r="BX31" s="7"/>
-      <c r="BY31" s="7"/>
-      <c r="BZ31" s="7"/>
+      <c r="BX31" s="29"/>
+      <c r="BY31" s="29"/>
+      <c r="BZ31" s="29"/>
       <c r="CA31" s="6" t="s">
         <v>172</v>
       </c>
@@ -11071,7 +11131,7 @@
       <c r="AP33" s="4"/>
       <c r="AQ33" s="5"/>
       <c r="AS33" s="4" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="AT33" s="5"/>
       <c r="AU33" s="4"/>
@@ -11395,7 +11455,7 @@
       <c r="AF36" s="13"/>
       <c r="AG36" s="13"/>
       <c r="AH36" s="29" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AI36" s="29"/>
       <c r="AJ36" s="29"/>
@@ -11408,7 +11468,9 @@
       <c r="AO36" s="9"/>
       <c r="AP36" s="9"/>
       <c r="AQ36" s="9"/>
-      <c r="AS36" s="7"/>
+      <c r="AS36" s="7" t="s">
+        <v>187</v>
+      </c>
       <c r="AT36" s="7"/>
       <c r="AU36" s="7"/>
       <c r="AV36" s="7"/>
@@ -11521,11 +11583,9 @@
       </c>
       <c r="AG37" s="13"/>
       <c r="AH37" s="13"/>
-      <c r="AI37" s="29" t="s">
-        <v>188</v>
-      </c>
-      <c r="AJ37" s="29"/>
-      <c r="AK37" s="29"/>
+      <c r="AI37" s="6"/>
+      <c r="AJ37" s="6"/>
+      <c r="AK37" s="6"/>
       <c r="AL37" s="6" t="s">
         <v>35</v>
       </c>
@@ -11586,7 +11646,7 @@
       <c r="CH37" s="7"/>
       <c r="CI37" s="7"/>
     </row>
-    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
         <v>46</v>
       </c>
@@ -11636,11 +11696,11 @@
       </c>
       <c r="AD38" s="7"/>
       <c r="AE38" s="7"/>
-      <c r="AF38" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="AG38" s="7"/>
-      <c r="AH38" s="7"/>
+      <c r="AF38" s="30" t="s">
+        <v>189</v>
+      </c>
+      <c r="AG38" s="30"/>
+      <c r="AH38" s="30"/>
       <c r="AI38" s="11"/>
       <c r="AJ38" s="11"/>
       <c r="AK38" s="11"/>
@@ -11663,7 +11723,9 @@
       <c r="BC38" s="7"/>
       <c r="BD38" s="7"/>
       <c r="BE38" s="7"/>
-      <c r="BF38" s="7"/>
+      <c r="BF38" s="7" t="s">
+        <v>187</v>
+      </c>
       <c r="BG38" s="7"/>
       <c r="BH38" s="7"/>
       <c r="BI38" s="7"/>
@@ -11681,9 +11743,11 @@
       <c r="BU38" s="7"/>
       <c r="BV38" s="7"/>
       <c r="BW38" s="7"/>
-      <c r="BX38" s="7"/>
-      <c r="BY38" s="7"/>
-      <c r="BZ38" s="7"/>
+      <c r="BX38" s="29" t="s">
+        <v>186</v>
+      </c>
+      <c r="BY38" s="29"/>
+      <c r="BZ38" s="29"/>
       <c r="CA38" s="11"/>
       <c r="CB38" s="11"/>
       <c r="CC38" s="11"/>
@@ -11726,9 +11790,9 @@
       <c r="AC39" s="7"/>
       <c r="AD39" s="7"/>
       <c r="AE39" s="7"/>
-      <c r="AF39" s="7"/>
-      <c r="AG39" s="7"/>
-      <c r="AH39" s="7"/>
+      <c r="AF39" s="30"/>
+      <c r="AG39" s="30"/>
+      <c r="AH39" s="30"/>
       <c r="AI39" s="6"/>
       <c r="AJ39" s="6"/>
       <c r="AK39" s="6"/>
@@ -11769,9 +11833,9 @@
       <c r="BU39" s="7"/>
       <c r="BV39" s="7"/>
       <c r="BW39" s="7"/>
-      <c r="BX39" s="7"/>
-      <c r="BY39" s="7"/>
-      <c r="BZ39" s="7"/>
+      <c r="BX39" s="29"/>
+      <c r="BY39" s="29"/>
+      <c r="BZ39" s="29"/>
       <c r="CA39" s="6"/>
       <c r="CB39" s="6"/>
       <c r="CC39" s="6"/>
@@ -11826,7 +11890,7 @@
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B41" s="15"/>
       <c r="C41" s="15"/>
@@ -11871,7 +11935,7 @@
       <c r="AP41" s="4"/>
       <c r="AQ41" s="5"/>
       <c r="AS41" s="15" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="AT41" s="15"/>
       <c r="AU41" s="4"/>
@@ -11979,21 +12043,23 @@
     <row r="43" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="6"/>
       <c r="B43" s="6"/>
-      <c r="C43" s="13"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13"/>
-      <c r="F43" s="29"/>
-      <c r="G43" s="29"/>
-      <c r="H43" s="29"/>
-      <c r="I43" s="13"/>
-      <c r="J43" s="13"/>
-      <c r="K43" s="13"/>
-      <c r="L43" s="13"/>
-      <c r="M43" s="13"/>
-      <c r="N43" s="13"/>
-      <c r="O43" s="13"/>
-      <c r="P43" s="13"/>
-      <c r="Q43" s="13"/>
+      <c r="C43" s="6"/>
+      <c r="D43" s="6"/>
+      <c r="E43" s="6"/>
+      <c r="F43" s="6"/>
+      <c r="G43" s="6"/>
+      <c r="H43" s="6"/>
+      <c r="I43" s="29" t="s">
+        <v>186</v>
+      </c>
+      <c r="J43" s="29"/>
+      <c r="K43" s="29"/>
+      <c r="L43" s="6"/>
+      <c r="M43" s="6"/>
+      <c r="N43" s="6"/>
+      <c r="O43" s="6"/>
+      <c r="P43" s="6"/>
+      <c r="Q43" s="6"/>
       <c r="R43" s="13" t="s">
         <v>138</v>
       </c>
@@ -12039,12 +12105,14 @@
       <c r="AU43" s="6"/>
       <c r="AV43" s="6"/>
       <c r="AW43" s="6"/>
-      <c r="AX43" s="29"/>
-      <c r="AY43" s="29"/>
-      <c r="AZ43" s="29"/>
-      <c r="BA43" s="6"/>
-      <c r="BB43" s="6"/>
-      <c r="BC43" s="6"/>
+      <c r="AX43" s="6"/>
+      <c r="AY43" s="6"/>
+      <c r="AZ43" s="6"/>
+      <c r="BA43" s="29" t="s">
+        <v>192</v>
+      </c>
+      <c r="BB43" s="29"/>
+      <c r="BC43" s="29"/>
       <c r="BD43" s="6"/>
       <c r="BE43" s="6"/>
       <c r="BF43" s="6"/>
@@ -12069,15 +12137,15 @@
       <c r="BS43" s="6"/>
       <c r="BT43" s="6"/>
       <c r="BU43" s="6"/>
-      <c r="BV43" s="7"/>
-      <c r="BW43" s="7"/>
-      <c r="BX43" s="7"/>
-      <c r="BY43" s="13"/>
-      <c r="BZ43" s="13"/>
-      <c r="CA43" s="13"/>
-      <c r="CB43" s="13"/>
-      <c r="CC43" s="13"/>
-      <c r="CD43" s="13"/>
+      <c r="BV43" s="6"/>
+      <c r="BW43" s="6"/>
+      <c r="BX43" s="6"/>
+      <c r="BY43" s="6"/>
+      <c r="BZ43" s="6"/>
+      <c r="CA43" s="6"/>
+      <c r="CB43" s="6"/>
+      <c r="CC43" s="6"/>
+      <c r="CD43" s="6"/>
       <c r="CE43" s="6"/>
       <c r="CF43" s="6"/>
       <c r="CG43" s="6"/>
@@ -12090,15 +12158,15 @@
       </c>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="13"/>
-      <c r="F44" s="13"/>
-      <c r="G44" s="13"/>
-      <c r="H44" s="13"/>
-      <c r="I44" s="13"/>
-      <c r="J44" s="13"/>
-      <c r="K44" s="13"/>
-      <c r="L44" s="13"/>
+      <c r="D44" s="6"/>
+      <c r="E44" s="6"/>
+      <c r="F44" s="6"/>
+      <c r="G44" s="6"/>
+      <c r="H44" s="6"/>
+      <c r="I44" s="6"/>
+      <c r="J44" s="6"/>
+      <c r="K44" s="6"/>
+      <c r="L44" s="6"/>
       <c r="M44" s="20"/>
       <c r="N44" s="20"/>
       <c r="O44" s="20"/>
@@ -12128,18 +12196,18 @@
       <c r="AC44" s="6"/>
       <c r="AD44" s="6"/>
       <c r="AE44" s="13" t="s">
-        <v>191</v>
+        <v>20</v>
       </c>
       <c r="AF44" s="13"/>
       <c r="AG44" s="13"/>
       <c r="AH44" s="29" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AI44" s="29"/>
       <c r="AJ44" s="29"/>
-      <c r="AK44" s="13"/>
-      <c r="AL44" s="13"/>
-      <c r="AM44" s="13"/>
+      <c r="AK44" s="6"/>
+      <c r="AL44" s="6"/>
+      <c r="AM44" s="6"/>
       <c r="AN44" s="9"/>
       <c r="AO44" s="9"/>
       <c r="AP44" s="9"/>
@@ -12192,13 +12260,13 @@
       <c r="BX44" s="13"/>
       <c r="BY44" s="13"/>
       <c r="BZ44" s="29" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="CA44" s="29"/>
       <c r="CB44" s="29"/>
-      <c r="CC44" s="13"/>
-      <c r="CD44" s="13"/>
-      <c r="CE44" s="13"/>
+      <c r="CC44" s="6"/>
+      <c r="CD44" s="6"/>
+      <c r="CE44" s="6"/>
       <c r="CF44" s="9"/>
       <c r="CG44" s="9"/>
       <c r="CH44" s="9"/>
@@ -12249,12 +12317,12 @@
       </c>
       <c r="AA45" s="7"/>
       <c r="AB45" s="7"/>
-      <c r="AC45" s="21"/>
-      <c r="AD45" s="21"/>
-      <c r="AE45" s="21"/>
-      <c r="AF45" s="13"/>
-      <c r="AG45" s="13"/>
-      <c r="AH45" s="13"/>
+      <c r="AC45" s="6"/>
+      <c r="AD45" s="6"/>
+      <c r="AE45" s="6"/>
+      <c r="AF45" s="6"/>
+      <c r="AG45" s="6"/>
+      <c r="AH45" s="6"/>
       <c r="AI45" s="6"/>
       <c r="AJ45" s="6"/>
       <c r="AK45" s="6"/>
@@ -12273,16 +12341,16 @@
       </c>
       <c r="AX45" s="13"/>
       <c r="AY45" s="13"/>
-      <c r="AZ45" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="BA45" s="13"/>
-      <c r="BB45" s="13"/>
-      <c r="BC45" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="BD45" s="13"/>
-      <c r="BE45" s="13"/>
+      <c r="AZ45" s="31" t="s">
+        <v>193</v>
+      </c>
+      <c r="BA45" s="31"/>
+      <c r="BB45" s="31"/>
+      <c r="BC45" s="31" t="s">
+        <v>194</v>
+      </c>
+      <c r="BD45" s="31"/>
+      <c r="BE45" s="31"/>
       <c r="BF45" s="13" t="s">
         <v>157</v>
       </c>
@@ -12298,22 +12366,22 @@
       </c>
       <c r="BM45" s="10"/>
       <c r="BN45" s="10"/>
-      <c r="BO45" s="30" t="s">
+      <c r="BO45" s="32" t="s">
         <v>166</v>
       </c>
-      <c r="BP45" s="30"/>
-      <c r="BQ45" s="30"/>
-      <c r="BR45" s="30" t="s">
+      <c r="BP45" s="32"/>
+      <c r="BQ45" s="32"/>
+      <c r="BR45" s="32" t="s">
         <v>144</v>
       </c>
-      <c r="BS45" s="30"/>
-      <c r="BT45" s="30"/>
-      <c r="BU45" s="21"/>
-      <c r="BV45" s="21"/>
-      <c r="BW45" s="21"/>
-      <c r="BX45" s="13"/>
-      <c r="BY45" s="13"/>
-      <c r="BZ45" s="13"/>
+      <c r="BS45" s="32"/>
+      <c r="BT45" s="32"/>
+      <c r="BU45" s="6"/>
+      <c r="BV45" s="6"/>
+      <c r="BW45" s="6"/>
+      <c r="BX45" s="6"/>
+      <c r="BY45" s="6"/>
+      <c r="BZ45" s="6"/>
       <c r="CA45" s="6"/>
       <c r="CB45" s="6"/>
       <c r="CC45" s="6"/>
@@ -12356,9 +12424,11 @@
       <c r="AC46" s="7"/>
       <c r="AD46" s="7"/>
       <c r="AE46" s="7"/>
-      <c r="AF46" s="7"/>
-      <c r="AG46" s="7"/>
-      <c r="AH46" s="7"/>
+      <c r="AF46" s="29" t="s">
+        <v>186</v>
+      </c>
+      <c r="AG46" s="29"/>
+      <c r="AH46" s="29"/>
       <c r="AI46" s="11"/>
       <c r="AJ46" s="11"/>
       <c r="AK46" s="11"/>
@@ -12405,9 +12475,11 @@
       <c r="BU46" s="7"/>
       <c r="BV46" s="7"/>
       <c r="BW46" s="7"/>
-      <c r="BX46" s="7"/>
-      <c r="BY46" s="7"/>
-      <c r="BZ46" s="7"/>
+      <c r="BX46" s="29" t="s">
+        <v>192</v>
+      </c>
+      <c r="BY46" s="29"/>
+      <c r="BZ46" s="29"/>
       <c r="CA46" s="11"/>
       <c r="CB46" s="11"/>
       <c r="CC46" s="11"/>
@@ -12450,9 +12522,9 @@
       <c r="AC47" s="7"/>
       <c r="AD47" s="7"/>
       <c r="AE47" s="7"/>
-      <c r="AF47" s="7"/>
-      <c r="AG47" s="7"/>
-      <c r="AH47" s="7"/>
+      <c r="AF47" s="29"/>
+      <c r="AG47" s="29"/>
+      <c r="AH47" s="29"/>
       <c r="AI47" s="6"/>
       <c r="AJ47" s="6"/>
       <c r="AK47" s="6"/>
@@ -12493,9 +12565,9 @@
       <c r="BU47" s="7"/>
       <c r="BV47" s="7"/>
       <c r="BW47" s="7"/>
-      <c r="BX47" s="7"/>
-      <c r="BY47" s="7"/>
-      <c r="BZ47" s="7"/>
+      <c r="BX47" s="29"/>
+      <c r="BY47" s="29"/>
+      <c r="BZ47" s="29"/>
       <c r="CA47" s="6"/>
       <c r="CB47" s="6"/>
       <c r="CC47" s="6"/>
@@ -14898,7 +14970,7 @@
       <c r="BP10" s="13"/>
       <c r="BQ10" s="13"/>
       <c r="BR10" s="13" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="BS10" s="13"/>
       <c r="BT10" s="13"/>
@@ -14992,7 +15064,7 @@
       <c r="AK11" s="6"/>
       <c r="AL11" s="6"/>
       <c r="AM11" s="6" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="AN11" s="6"/>
       <c r="AO11" s="6"/>
@@ -15661,7 +15733,7 @@
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>109</v>
@@ -15867,7 +15939,7 @@
       <c r="AK19" s="13"/>
       <c r="AL19" s="13"/>
       <c r="AM19" s="6" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="AN19" s="6"/>
       <c r="AO19" s="6"/>
@@ -15922,7 +15994,7 @@
       <c r="CC19" s="7"/>
       <c r="CD19" s="7"/>
       <c r="CE19" s="6" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="CF19" s="6"/>
       <c r="CG19" s="6"/>
@@ -16703,7 +16775,7 @@
       <c r="AK27" s="13"/>
       <c r="AL27" s="13"/>
       <c r="AM27" s="6" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="AN27" s="6"/>
       <c r="AO27" s="6"/>
@@ -16756,7 +16828,7 @@
       <c r="CC27" s="7"/>
       <c r="CD27" s="7"/>
       <c r="CE27" s="6" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="CF27" s="6"/>
       <c r="CG27" s="6"/>
@@ -17528,7 +17600,7 @@
       <c r="AK35" s="13"/>
       <c r="AL35" s="13"/>
       <c r="AM35" s="6" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="AN35" s="6"/>
       <c r="AO35" s="6"/>
@@ -17585,7 +17657,7 @@
       <c r="CC35" s="7"/>
       <c r="CD35" s="7"/>
       <c r="CE35" s="6" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="CF35" s="6"/>
       <c r="CG35" s="6"/>
@@ -19139,7 +19211,7 @@
       <c r="AP1" s="4"/>
       <c r="AQ1" s="5"/>
       <c r="AT1" s="3" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="AU1" s="4"/>
       <c r="AV1" s="4"/>
@@ -19422,7 +19494,7 @@
         <v>161</v>
       </c>
       <c r="AT4" s="7" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="AU4" s="7"/>
       <c r="AV4" s="7"/>
@@ -19430,7 +19502,7 @@
       <c r="AX4" s="8"/>
       <c r="AY4" s="6"/>
       <c r="AZ4" s="6" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="BA4" s="8" t="s">
         <v>56</v>
@@ -19519,8 +19591,8 @@
       <c r="AO5" s="6"/>
       <c r="AP5" s="6"/>
       <c r="AQ5" s="6"/>
-      <c r="AR5" s="31" t="s">
-        <v>198</v>
+      <c r="AR5" s="33" t="s">
+        <v>201</v>
       </c>
       <c r="AT5" s="7"/>
       <c r="AU5" s="7"/>
@@ -19529,7 +19601,7 @@
       <c r="AX5" s="7"/>
       <c r="AY5" s="7"/>
       <c r="AZ5" s="6" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="BA5" s="7" t="s">
         <v>172</v>
@@ -19589,10 +19661,10 @@
       <c r="V6" s="7"/>
       <c r="W6" s="7"/>
       <c r="X6" s="7" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="Y6" s="7" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="Z6" s="7"/>
       <c r="AA6" s="7"/>
@@ -19635,7 +19707,7 @@
       <c r="AW6" s="7"/>
       <c r="AX6" s="7"/>
       <c r="AY6" s="7" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="AZ6" s="7"/>
       <c r="BA6" s="7"/>
@@ -19644,7 +19716,7 @@
       <c r="BD6" s="6"/>
       <c r="BE6" s="11"/>
       <c r="BF6" s="6" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="BG6" s="11"/>
       <c r="BH6" s="11"/>
@@ -19709,7 +19781,7 @@
         <v>172</v>
       </c>
       <c r="BF7" s="6" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="BG7" s="6" t="s">
         <v>173</v>
@@ -19763,7 +19835,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -20326,8 +20398,8 @@
       <c r="AO13" s="6"/>
       <c r="AP13" s="6"/>
       <c r="AQ13" s="6"/>
-      <c r="AR13" s="31" t="s">
-        <v>198</v>
+      <c r="AR13" s="33" t="s">
+        <v>201</v>
       </c>
       <c r="AT13" s="7"/>
       <c r="AU13" s="7"/>
@@ -20440,10 +20512,10 @@
       </c>
       <c r="W14" s="7"/>
       <c r="X14" s="7" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="Y14" s="7" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="Z14" s="7"/>
       <c r="AA14" s="7"/>
@@ -20722,7 +20794,7 @@
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>109</v>
@@ -21193,8 +21265,8 @@
       <c r="AO21" s="6"/>
       <c r="AP21" s="6"/>
       <c r="AQ21" s="6"/>
-      <c r="AR21" s="31" t="s">
-        <v>198</v>
+      <c r="AR21" s="33" t="s">
+        <v>201</v>
       </c>
       <c r="AT21" s="7"/>
       <c r="AU21" s="7"/>
@@ -21303,10 +21375,10 @@
       </c>
       <c r="W22" s="7"/>
       <c r="X22" s="7" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="Y22" s="7" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="Z22" s="7"/>
       <c r="AA22" s="7"/>
@@ -22019,8 +22091,8 @@
       <c r="AO29" s="6"/>
       <c r="AP29" s="6"/>
       <c r="AQ29" s="6"/>
-      <c r="AR29" s="31" t="s">
-        <v>198</v>
+      <c r="AR29" s="33" t="s">
+        <v>201</v>
       </c>
       <c r="AT29" s="7"/>
       <c r="AU29" s="7"/>
@@ -22117,10 +22189,10 @@
       </c>
       <c r="W30" s="7"/>
       <c r="X30" s="7" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="Y30" s="7" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="Z30" s="7"/>
       <c r="AA30" s="7"/>
@@ -22187,7 +22259,7 @@
       </c>
       <c r="BP30" s="7"/>
       <c r="BQ30" s="7" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="BR30" s="7"/>
       <c r="BS30" s="7"/>
@@ -22692,7 +22764,7 @@
       <c r="AR36" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="AT36" s="32" t="s">
+      <c r="AT36" s="34" t="s">
         <v>34</v>
       </c>
       <c r="AU36" s="13" t="s">
@@ -22798,8 +22870,8 @@
       <c r="AO37" s="6"/>
       <c r="AP37" s="6"/>
       <c r="AQ37" s="6"/>
-      <c r="AR37" s="31" t="s">
-        <v>198</v>
+      <c r="AR37" s="33" t="s">
+        <v>201</v>
       </c>
       <c r="AT37" s="7" t="s">
         <v>35</v>
@@ -22882,10 +22954,10 @@
       </c>
       <c r="W38" s="7"/>
       <c r="X38" s="7" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="Y38" s="7" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="Z38" s="7"/>
       <c r="AA38" s="7"/>
@@ -22920,17 +22992,17 @@
       <c r="AW38" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="AX38" s="32" t="s">
+      <c r="AX38" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="AY38" s="32" t="s">
+      <c r="AY38" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="AZ38" s="32"/>
-      <c r="BA38" s="32" t="s">
+      <c r="AZ38" s="34"/>
+      <c r="BA38" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="BB38" s="32" t="s">
+      <c r="BB38" s="34" t="s">
         <v>107</v>
       </c>
       <c r="BC38" s="11"/>
@@ -22993,9 +23065,9 @@
       <c r="AW39" s="7"/>
       <c r="AX39" s="7"/>
       <c r="AY39" s="7"/>
-      <c r="AZ39" s="32"/>
-      <c r="BA39" s="32"/>
-      <c r="BB39" s="32"/>
+      <c r="AZ39" s="34"/>
+      <c r="BA39" s="34"/>
+      <c r="BB39" s="34"/>
       <c r="BC39" s="11"/>
       <c r="BD39" s="6"/>
       <c r="BE39" s="6"/>
@@ -24240,8 +24312,8 @@
       </c>
       <c r="N5" s="6"/>
       <c r="O5" s="6"/>
-      <c r="P5" s="31" t="s">
-        <v>198</v>
+      <c r="P5" s="33" t="s">
+        <v>201</v>
       </c>
       <c r="R5" s="7"/>
       <c r="S5" s="7"/>
@@ -24372,7 +24444,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -24527,7 +24599,7 @@
       <c r="Z11" s="13"/>
       <c r="AA11" s="13"/>
       <c r="AB11" s="13"/>
-      <c r="AC11" s="33"/>
+      <c r="AC11" s="35"/>
       <c r="AD11" s="21"/>
       <c r="AE11" s="6"/>
       <c r="AF11" s="6"/>
@@ -24635,8 +24707,8 @@
       </c>
       <c r="N13" s="6"/>
       <c r="O13" s="6"/>
-      <c r="P13" s="31" t="s">
-        <v>198</v>
+      <c r="P13" s="33" t="s">
+        <v>201</v>
       </c>
       <c r="R13" s="7"/>
       <c r="S13" s="13"/>
@@ -24844,8 +24916,8 @@
       <c r="M19" s="13"/>
       <c r="N19" s="6"/>
       <c r="O19" s="6"/>
-      <c r="P19" s="34" t="s">
-        <v>204</v>
+      <c r="P19" s="36" t="s">
+        <v>207</v>
       </c>
       <c r="R19" s="7"/>
       <c r="S19" s="7"/>
@@ -24864,7 +24936,7 @@
       <c r="AF19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="32"/>
+      <c r="A20" s="34"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
@@ -24947,11 +25019,11 @@
       <c r="S22" s="7"/>
       <c r="T22" s="7"/>
       <c r="U22" s="7"/>
-      <c r="V22" s="32"/>
+      <c r="V22" s="34"/>
       <c r="W22" s="7"/>
       <c r="X22" s="7"/>
-      <c r="Y22" s="35"/>
-      <c r="Z22" s="35"/>
+      <c r="Y22" s="37"/>
+      <c r="Z22" s="37"/>
       <c r="AA22" s="11"/>
       <c r="AB22" s="6"/>
       <c r="AC22" s="11"/>
@@ -24979,11 +25051,11 @@
       <c r="S23" s="7"/>
       <c r="T23" s="7"/>
       <c r="U23" s="7"/>
-      <c r="V23" s="32"/>
-      <c r="W23" s="32"/>
+      <c r="V23" s="34"/>
+      <c r="W23" s="34"/>
       <c r="X23" s="7"/>
-      <c r="Y23" s="35"/>
-      <c r="Z23" s="35"/>
+      <c r="Y23" s="37"/>
+      <c r="Z23" s="37"/>
       <c r="AA23" s="11"/>
       <c r="AB23" s="6"/>
       <c r="AC23" s="6"/>
@@ -25120,7 +25192,7 @@
       <c r="M28" s="13"/>
       <c r="N28" s="6"/>
       <c r="O28" s="6"/>
-      <c r="R28" s="32"/>
+      <c r="R28" s="34"/>
       <c r="S28" s="7"/>
       <c r="T28" s="7"/>
       <c r="U28" s="7"/>
@@ -25174,8 +25246,8 @@
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
       <c r="E30" s="7"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32"/>
+      <c r="F30" s="34"/>
+      <c r="G30" s="34"/>
       <c r="H30" s="7"/>
       <c r="I30" s="7"/>
       <c r="J30" s="11"/>
@@ -25188,9 +25260,9 @@
       <c r="S30" s="7"/>
       <c r="T30" s="7"/>
       <c r="U30" s="7"/>
-      <c r="V30" s="32"/>
-      <c r="W30" s="32"/>
-      <c r="X30" s="32"/>
+      <c r="V30" s="34"/>
+      <c r="W30" s="34"/>
+      <c r="X30" s="34"/>
       <c r="Y30" s="6"/>
       <c r="Z30" s="7"/>
       <c r="AA30" s="11"/>
@@ -25207,7 +25279,7 @@
       <c r="D31" s="7"/>
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
-      <c r="G31" s="32"/>
+      <c r="G31" s="34"/>
       <c r="H31" s="7"/>
       <c r="I31" s="7"/>
       <c r="J31" s="11"/>
@@ -25222,7 +25294,7 @@
       <c r="U31" s="7"/>
       <c r="V31" s="7"/>
       <c r="W31" s="7"/>
-      <c r="X31" s="32"/>
+      <c r="X31" s="34"/>
       <c r="Y31" s="6"/>
       <c r="Z31" s="7"/>
       <c r="AA31" s="11"/>
@@ -25285,7 +25357,7 @@
       <c r="A34" s="7"/>
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
-      <c r="D34" s="30"/>
+      <c r="D34" s="32"/>
       <c r="E34" s="6"/>
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
@@ -25361,7 +25433,7 @@
       <c r="M36" s="13"/>
       <c r="N36" s="6"/>
       <c r="O36" s="6"/>
-      <c r="R36" s="32"/>
+      <c r="R36" s="34"/>
       <c r="S36" s="13"/>
       <c r="T36" s="13"/>
       <c r="U36" s="13"/>
@@ -25400,7 +25472,7 @@
       <c r="V37" s="13"/>
       <c r="W37" s="13"/>
       <c r="X37" s="18"/>
-      <c r="Y37" s="36"/>
+      <c r="Y37" s="38"/>
       <c r="Z37" s="6"/>
       <c r="AA37" s="6"/>
       <c r="AB37" s="6"/>
@@ -25415,8 +25487,8 @@
       <c r="C38" s="7"/>
       <c r="D38" s="7"/>
       <c r="E38" s="7"/>
-      <c r="F38" s="32"/>
-      <c r="G38" s="32"/>
+      <c r="F38" s="34"/>
+      <c r="G38" s="34"/>
       <c r="H38" s="7"/>
       <c r="I38" s="7"/>
       <c r="J38" s="11"/>
@@ -25429,11 +25501,11 @@
       <c r="S38" s="7"/>
       <c r="T38" s="7"/>
       <c r="U38" s="7"/>
-      <c r="V38" s="32"/>
-      <c r="W38" s="32"/>
-      <c r="X38" s="32"/>
-      <c r="Y38" s="32"/>
-      <c r="Z38" s="32"/>
+      <c r="V38" s="34"/>
+      <c r="W38" s="34"/>
+      <c r="X38" s="34"/>
+      <c r="Y38" s="34"/>
+      <c r="Z38" s="34"/>
       <c r="AA38" s="11"/>
       <c r="AB38" s="6"/>
       <c r="AC38" s="11"/>
@@ -25448,7 +25520,7 @@
       <c r="D39" s="7"/>
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
-      <c r="G39" s="32"/>
+      <c r="G39" s="34"/>
       <c r="H39" s="7"/>
       <c r="I39" s="7"/>
       <c r="J39" s="11"/>
@@ -25463,9 +25535,9 @@
       <c r="U39" s="7"/>
       <c r="V39" s="7"/>
       <c r="W39" s="7"/>
-      <c r="X39" s="32"/>
-      <c r="Y39" s="32"/>
-      <c r="Z39" s="32"/>
+      <c r="X39" s="34"/>
+      <c r="Y39" s="34"/>
+      <c r="Z39" s="34"/>
       <c r="AA39" s="11"/>
       <c r="AB39" s="6"/>
       <c r="AC39" s="6"/>
@@ -25586,7 +25658,7 @@
       <c r="AF43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="32"/>
+      <c r="A44" s="34"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
@@ -25601,7 +25673,7 @@
       <c r="M44" s="6"/>
       <c r="N44" s="6"/>
       <c r="O44" s="6"/>
-      <c r="R44" s="32"/>
+      <c r="R44" s="34"/>
       <c r="S44" s="13"/>
       <c r="T44" s="13"/>
       <c r="U44" s="13"/>
@@ -25655,8 +25727,8 @@
       <c r="C46" s="7"/>
       <c r="D46" s="7"/>
       <c r="E46" s="7"/>
-      <c r="F46" s="32"/>
-      <c r="G46" s="32"/>
+      <c r="F46" s="34"/>
+      <c r="G46" s="34"/>
       <c r="H46" s="6"/>
       <c r="I46" s="7"/>
       <c r="J46" s="11"/>
@@ -25669,11 +25741,11 @@
       <c r="S46" s="7"/>
       <c r="T46" s="7"/>
       <c r="U46" s="7"/>
-      <c r="V46" s="32"/>
-      <c r="W46" s="32"/>
-      <c r="X46" s="32"/>
-      <c r="Y46" s="32"/>
-      <c r="Z46" s="32"/>
+      <c r="V46" s="34"/>
+      <c r="W46" s="34"/>
+      <c r="X46" s="34"/>
+      <c r="Y46" s="34"/>
+      <c r="Z46" s="34"/>
       <c r="AA46" s="11"/>
       <c r="AB46" s="6"/>
       <c r="AC46" s="11"/>
@@ -25688,7 +25760,7 @@
       <c r="D47" s="7"/>
       <c r="E47" s="7"/>
       <c r="F47" s="7"/>
-      <c r="G47" s="32"/>
+      <c r="G47" s="34"/>
       <c r="H47" s="6"/>
       <c r="I47" s="7"/>
       <c r="J47" s="11"/>
@@ -25703,9 +25775,9 @@
       <c r="U47" s="7"/>
       <c r="V47" s="7"/>
       <c r="W47" s="7"/>
-      <c r="X47" s="32"/>
-      <c r="Y47" s="32"/>
-      <c r="Z47" s="32"/>
+      <c r="X47" s="34"/>
+      <c r="Y47" s="34"/>
+      <c r="Z47" s="34"/>
       <c r="AA47" s="11"/>
       <c r="AB47" s="6"/>
       <c r="AC47" s="6"/>
@@ -25833,7 +25905,7 @@
       <c r="S52" s="7"/>
       <c r="T52" s="7"/>
       <c r="U52" s="7"/>
-      <c r="V52" s="37"/>
+      <c r="V52" s="39"/>
       <c r="W52" s="6"/>
       <c r="X52" s="13"/>
       <c r="Y52" s="14"/>
@@ -25882,11 +25954,11 @@
       <c r="B54" s="7"/>
       <c r="C54" s="7"/>
       <c r="D54" s="7"/>
-      <c r="E54" s="32"/>
+      <c r="E54" s="34"/>
       <c r="F54" s="7"/>
       <c r="G54" s="7"/>
-      <c r="H54" s="35"/>
-      <c r="I54" s="35"/>
+      <c r="H54" s="37"/>
+      <c r="I54" s="37"/>
       <c r="J54" s="11"/>
       <c r="K54" s="6"/>
       <c r="L54" s="11"/>
@@ -25914,11 +25986,11 @@
       <c r="B55" s="7"/>
       <c r="C55" s="7"/>
       <c r="D55" s="7"/>
-      <c r="E55" s="32"/>
-      <c r="F55" s="32"/>
+      <c r="E55" s="34"/>
+      <c r="F55" s="34"/>
       <c r="G55" s="7"/>
-      <c r="H55" s="35"/>
-      <c r="I55" s="35"/>
+      <c r="H55" s="37"/>
+      <c r="I55" s="37"/>
       <c r="J55" s="11"/>
       <c r="K55" s="6"/>
       <c r="L55" s="6"/>

</xml_diff>

<commit_message>
[Update] Layout is changed.
</commit_message>
<xml_diff>
--- a/img/keymap.xlsx
+++ b/img/keymap.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2356" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2358" uniqueCount="211">
   <si>
     <t xml:space="preserve">標準</t>
   </si>
@@ -584,23 +584,36 @@
     <t xml:space="preserve">Space &amp; F13 修飾</t>
   </si>
   <si>
-    <t xml:space="preserve">SelMode</t>
+    <t xml:space="preserve">SelCur
+Togle</t>
   </si>
   <si>
-    <t xml:space="preserve">StdMode</t>
+    <t xml:space="preserve">Select
+Mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stdard
+Mode</t>
   </si>
   <si>
     <t xml:space="preserve">10Key Mode</t>
   </si>
   <si>
-    <t xml:space="preserve">SelCur
-Togle</t>
+    <t xml:space="preserve">SelMode</t>
   </si>
   <si>
     <t xml:space="preserve">Cursor Mode</t>
   </si>
   <si>
     <t xml:space="preserve">Select Mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Normal
+Mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cursor
+Mode</t>
   </si>
   <si>
     <t xml:space="preserve">CurMode</t>
@@ -942,7 +955,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1060,10 +1073,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -8392,26 +8413,26 @@
       <c r="BN6" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="BO6" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="BP6" s="7"/>
-      <c r="BQ6" s="7"/>
-      <c r="BR6" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="BS6" s="7"/>
-      <c r="BT6" s="7"/>
+      <c r="BO6" s="29" t="s">
+        <v>186</v>
+      </c>
+      <c r="BP6" s="29"/>
+      <c r="BQ6" s="29"/>
+      <c r="BR6" s="29" t="s">
+        <v>186</v>
+      </c>
+      <c r="BS6" s="29"/>
+      <c r="BT6" s="29"/>
       <c r="BU6" s="7" t="s">
         <v>49</v>
       </c>
       <c r="BV6" s="7"/>
       <c r="BW6" s="7"/>
-      <c r="BX6" s="29" t="s">
-        <v>186</v>
-      </c>
-      <c r="BY6" s="29"/>
-      <c r="BZ6" s="29"/>
+      <c r="BX6" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="BY6" s="7"/>
+      <c r="BZ6" s="7"/>
       <c r="CA6" s="11"/>
       <c r="CB6" s="11"/>
       <c r="CC6" s="11"/>
@@ -8498,18 +8519,18 @@
       <c r="BL7" s="7"/>
       <c r="BM7" s="7"/>
       <c r="BN7" s="7"/>
-      <c r="BO7" s="7"/>
-      <c r="BP7" s="7"/>
-      <c r="BQ7" s="7"/>
-      <c r="BR7" s="7"/>
-      <c r="BS7" s="7"/>
-      <c r="BT7" s="7"/>
+      <c r="BO7" s="29"/>
+      <c r="BP7" s="29"/>
+      <c r="BQ7" s="29"/>
+      <c r="BR7" s="29"/>
+      <c r="BS7" s="29"/>
+      <c r="BT7" s="29"/>
       <c r="BU7" s="7"/>
       <c r="BV7" s="7"/>
       <c r="BW7" s="7"/>
-      <c r="BX7" s="29"/>
-      <c r="BY7" s="29"/>
-      <c r="BZ7" s="29"/>
+      <c r="BX7" s="7"/>
+      <c r="BY7" s="7"/>
+      <c r="BZ7" s="7"/>
       <c r="CA7" s="6" t="s">
         <v>56</v>
       </c>
@@ -9703,16 +9724,16 @@
       </c>
       <c r="AE19" s="13"/>
       <c r="AF19" s="13"/>
-      <c r="AG19" s="29" t="s">
+      <c r="AG19" s="30" t="s">
         <v>145</v>
       </c>
-      <c r="AH19" s="29"/>
-      <c r="AI19" s="29"/>
-      <c r="AJ19" s="29" t="s">
+      <c r="AH19" s="30"/>
+      <c r="AI19" s="30"/>
+      <c r="AJ19" s="30" t="s">
         <v>146</v>
       </c>
-      <c r="AK19" s="29"/>
-      <c r="AL19" s="29"/>
+      <c r="AK19" s="30"/>
+      <c r="AL19" s="30"/>
       <c r="AM19" s="6"/>
       <c r="AN19" s="6"/>
       <c r="AO19" s="6"/>
@@ -9793,7 +9814,7 @@
       <c r="H20" s="13"/>
       <c r="I20" s="13"/>
       <c r="J20" s="29" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K20" s="29"/>
       <c r="L20" s="29"/>
@@ -10608,7 +10629,7 @@
       <c r="H28" s="13"/>
       <c r="I28" s="13"/>
       <c r="J28" s="29" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K28" s="29"/>
       <c r="L28" s="29"/>
@@ -10661,11 +10682,11 @@
       <c r="AO28" s="9"/>
       <c r="AP28" s="9"/>
       <c r="AQ28" s="9"/>
-      <c r="AS28" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="AT28" s="7"/>
-      <c r="AU28" s="7"/>
+      <c r="AS28" s="31" t="s">
+        <v>188</v>
+      </c>
+      <c r="AT28" s="31"/>
+      <c r="AU28" s="31"/>
       <c r="AV28" s="7"/>
       <c r="AW28" s="7"/>
       <c r="AX28" s="7"/>
@@ -10831,7 +10852,7 @@
       <c r="CH29" s="7"/>
       <c r="CI29" s="7"/>
     </row>
-    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
         <v>46</v>
       </c>
@@ -10908,17 +10929,17 @@
       <c r="BC30" s="7"/>
       <c r="BD30" s="7"/>
       <c r="BE30" s="7"/>
-      <c r="BF30" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="BG30" s="7"/>
-      <c r="BH30" s="7"/>
-      <c r="BI30" s="7"/>
-      <c r="BJ30" s="7"/>
-      <c r="BK30" s="7"/>
-      <c r="BL30" s="7"/>
-      <c r="BM30" s="7"/>
-      <c r="BN30" s="7"/>
+      <c r="BF30" s="31" t="s">
+        <v>188</v>
+      </c>
+      <c r="BG30" s="31"/>
+      <c r="BH30" s="31"/>
+      <c r="BI30" s="31"/>
+      <c r="BJ30" s="31"/>
+      <c r="BK30" s="31"/>
+      <c r="BL30" s="31"/>
+      <c r="BM30" s="31"/>
+      <c r="BN30" s="31"/>
       <c r="BO30" s="7"/>
       <c r="BP30" s="7"/>
       <c r="BQ30" s="7"/>
@@ -10928,11 +10949,11 @@
       <c r="BU30" s="7"/>
       <c r="BV30" s="7"/>
       <c r="BW30" s="7"/>
-      <c r="BX30" s="29" t="s">
-        <v>186</v>
-      </c>
-      <c r="BY30" s="29"/>
-      <c r="BZ30" s="29"/>
+      <c r="BX30" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="BY30" s="32"/>
+      <c r="BZ30" s="32"/>
       <c r="CA30" s="11"/>
       <c r="CB30" s="11"/>
       <c r="CC30" s="11"/>
@@ -11002,15 +11023,15 @@
       <c r="BC31" s="7"/>
       <c r="BD31" s="7"/>
       <c r="BE31" s="7"/>
-      <c r="BF31" s="7"/>
-      <c r="BG31" s="7"/>
-      <c r="BH31" s="7"/>
-      <c r="BI31" s="7"/>
-      <c r="BJ31" s="7"/>
-      <c r="BK31" s="7"/>
-      <c r="BL31" s="7"/>
-      <c r="BM31" s="7"/>
-      <c r="BN31" s="7"/>
+      <c r="BF31" s="31"/>
+      <c r="BG31" s="31"/>
+      <c r="BH31" s="31"/>
+      <c r="BI31" s="31"/>
+      <c r="BJ31" s="31"/>
+      <c r="BK31" s="31"/>
+      <c r="BL31" s="31"/>
+      <c r="BM31" s="31"/>
+      <c r="BN31" s="31"/>
       <c r="BO31" s="7"/>
       <c r="BP31" s="7"/>
       <c r="BQ31" s="7"/>
@@ -11020,9 +11041,9 @@
       <c r="BU31" s="7"/>
       <c r="BV31" s="7"/>
       <c r="BW31" s="7"/>
-      <c r="BX31" s="29"/>
-      <c r="BY31" s="29"/>
-      <c r="BZ31" s="29"/>
+      <c r="BX31" s="32"/>
+      <c r="BY31" s="32"/>
+      <c r="BZ31" s="32"/>
       <c r="CA31" s="6" t="s">
         <v>172</v>
       </c>
@@ -11131,7 +11152,7 @@
       <c r="AP33" s="4"/>
       <c r="AQ33" s="5"/>
       <c r="AS33" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="AT33" s="5"/>
       <c r="AU33" s="4"/>
@@ -11327,16 +11348,16 @@
       </c>
       <c r="AE35" s="13"/>
       <c r="AF35" s="13"/>
-      <c r="AG35" s="29" t="s">
+      <c r="AG35" s="30" t="s">
         <v>145</v>
       </c>
-      <c r="AH35" s="29"/>
-      <c r="AI35" s="29"/>
-      <c r="AJ35" s="29" t="s">
+      <c r="AH35" s="30"/>
+      <c r="AI35" s="30"/>
+      <c r="AJ35" s="30" t="s">
         <v>146</v>
       </c>
-      <c r="AK35" s="29"/>
-      <c r="AL35" s="29"/>
+      <c r="AK35" s="30"/>
+      <c r="AL35" s="30"/>
       <c r="AM35" s="6"/>
       <c r="AN35" s="6"/>
       <c r="AO35" s="6"/>
@@ -11454,11 +11475,11 @@
       </c>
       <c r="AF36" s="13"/>
       <c r="AG36" s="13"/>
-      <c r="AH36" s="29" t="s">
-        <v>186</v>
-      </c>
-      <c r="AI36" s="29"/>
-      <c r="AJ36" s="29"/>
+      <c r="AH36" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="AI36" s="30"/>
+      <c r="AJ36" s="30"/>
       <c r="AK36" s="13" t="s">
         <v>153</v>
       </c>
@@ -11468,11 +11489,11 @@
       <c r="AO36" s="9"/>
       <c r="AP36" s="9"/>
       <c r="AQ36" s="9"/>
-      <c r="AS36" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="AT36" s="7"/>
-      <c r="AU36" s="7"/>
+      <c r="AS36" s="31" t="s">
+        <v>188</v>
+      </c>
+      <c r="AT36" s="31"/>
+      <c r="AU36" s="31"/>
       <c r="AV36" s="7"/>
       <c r="AW36" s="7"/>
       <c r="AX36" s="7"/>
@@ -11696,11 +11717,11 @@
       </c>
       <c r="AD38" s="7"/>
       <c r="AE38" s="7"/>
-      <c r="AF38" s="30" t="s">
-        <v>189</v>
-      </c>
-      <c r="AG38" s="30"/>
-      <c r="AH38" s="30"/>
+      <c r="AF38" s="29" t="s">
+        <v>186</v>
+      </c>
+      <c r="AG38" s="29"/>
+      <c r="AH38" s="29"/>
       <c r="AI38" s="11"/>
       <c r="AJ38" s="11"/>
       <c r="AK38" s="11"/>
@@ -11723,17 +11744,17 @@
       <c r="BC38" s="7"/>
       <c r="BD38" s="7"/>
       <c r="BE38" s="7"/>
-      <c r="BF38" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="BG38" s="7"/>
-      <c r="BH38" s="7"/>
-      <c r="BI38" s="7"/>
-      <c r="BJ38" s="7"/>
-      <c r="BK38" s="7"/>
-      <c r="BL38" s="7"/>
-      <c r="BM38" s="7"/>
-      <c r="BN38" s="7"/>
+      <c r="BF38" s="31" t="s">
+        <v>188</v>
+      </c>
+      <c r="BG38" s="31"/>
+      <c r="BH38" s="31"/>
+      <c r="BI38" s="31"/>
+      <c r="BJ38" s="31"/>
+      <c r="BK38" s="31"/>
+      <c r="BL38" s="31"/>
+      <c r="BM38" s="31"/>
+      <c r="BN38" s="31"/>
       <c r="BO38" s="7"/>
       <c r="BP38" s="7"/>
       <c r="BQ38" s="7"/>
@@ -11743,11 +11764,11 @@
       <c r="BU38" s="7"/>
       <c r="BV38" s="7"/>
       <c r="BW38" s="7"/>
-      <c r="BX38" s="29" t="s">
-        <v>186</v>
-      </c>
-      <c r="BY38" s="29"/>
-      <c r="BZ38" s="29"/>
+      <c r="BX38" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="BY38" s="32"/>
+      <c r="BZ38" s="32"/>
       <c r="CA38" s="11"/>
       <c r="CB38" s="11"/>
       <c r="CC38" s="11"/>
@@ -11790,9 +11811,9 @@
       <c r="AC39" s="7"/>
       <c r="AD39" s="7"/>
       <c r="AE39" s="7"/>
-      <c r="AF39" s="30"/>
-      <c r="AG39" s="30"/>
-      <c r="AH39" s="30"/>
+      <c r="AF39" s="29"/>
+      <c r="AG39" s="29"/>
+      <c r="AH39" s="29"/>
       <c r="AI39" s="6"/>
       <c r="AJ39" s="6"/>
       <c r="AK39" s="6"/>
@@ -11815,15 +11836,15 @@
       <c r="BC39" s="7"/>
       <c r="BD39" s="7"/>
       <c r="BE39" s="7"/>
-      <c r="BF39" s="7"/>
-      <c r="BG39" s="7"/>
-      <c r="BH39" s="7"/>
-      <c r="BI39" s="7"/>
-      <c r="BJ39" s="7"/>
-      <c r="BK39" s="7"/>
-      <c r="BL39" s="7"/>
-      <c r="BM39" s="7"/>
-      <c r="BN39" s="7"/>
+      <c r="BF39" s="31"/>
+      <c r="BG39" s="31"/>
+      <c r="BH39" s="31"/>
+      <c r="BI39" s="31"/>
+      <c r="BJ39" s="31"/>
+      <c r="BK39" s="31"/>
+      <c r="BL39" s="31"/>
+      <c r="BM39" s="31"/>
+      <c r="BN39" s="31"/>
       <c r="BO39" s="7"/>
       <c r="BP39" s="7"/>
       <c r="BQ39" s="7"/>
@@ -11833,9 +11854,9 @@
       <c r="BU39" s="7"/>
       <c r="BV39" s="7"/>
       <c r="BW39" s="7"/>
-      <c r="BX39" s="29"/>
-      <c r="BY39" s="29"/>
-      <c r="BZ39" s="29"/>
+      <c r="BX39" s="32"/>
+      <c r="BY39" s="32"/>
+      <c r="BZ39" s="32"/>
       <c r="CA39" s="6"/>
       <c r="CB39" s="6"/>
       <c r="CC39" s="6"/>
@@ -11890,7 +11911,7 @@
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B41" s="15"/>
       <c r="C41" s="15"/>
@@ -11935,7 +11956,7 @@
       <c r="AP41" s="4"/>
       <c r="AQ41" s="5"/>
       <c r="AS41" s="15" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="AT41" s="15"/>
       <c r="AU41" s="4"/>
@@ -12049,14 +12070,14 @@
       <c r="F43" s="6"/>
       <c r="G43" s="6"/>
       <c r="H43" s="6"/>
-      <c r="I43" s="29" t="s">
-        <v>186</v>
-      </c>
-      <c r="J43" s="29"/>
-      <c r="K43" s="29"/>
-      <c r="L43" s="6"/>
-      <c r="M43" s="6"/>
-      <c r="N43" s="6"/>
+      <c r="I43" s="6"/>
+      <c r="J43" s="6"/>
+      <c r="K43" s="6"/>
+      <c r="L43" s="29" t="s">
+        <v>193</v>
+      </c>
+      <c r="M43" s="29"/>
+      <c r="N43" s="29"/>
       <c r="O43" s="6"/>
       <c r="P43" s="6"/>
       <c r="Q43" s="6"/>
@@ -12085,16 +12106,16 @@
       </c>
       <c r="AE43" s="7"/>
       <c r="AF43" s="7"/>
-      <c r="AG43" s="29" t="s">
+      <c r="AG43" s="30" t="s">
         <v>145</v>
       </c>
-      <c r="AH43" s="29"/>
-      <c r="AI43" s="29"/>
-      <c r="AJ43" s="29" t="s">
+      <c r="AH43" s="30"/>
+      <c r="AI43" s="30"/>
+      <c r="AJ43" s="30" t="s">
         <v>146</v>
       </c>
-      <c r="AK43" s="29"/>
-      <c r="AL43" s="29"/>
+      <c r="AK43" s="30"/>
+      <c r="AL43" s="30"/>
       <c r="AM43" s="6"/>
       <c r="AN43" s="6"/>
       <c r="AO43" s="6"/>
@@ -12108,14 +12129,14 @@
       <c r="AX43" s="6"/>
       <c r="AY43" s="6"/>
       <c r="AZ43" s="6"/>
-      <c r="BA43" s="29" t="s">
-        <v>192</v>
-      </c>
-      <c r="BB43" s="29"/>
-      <c r="BC43" s="29"/>
-      <c r="BD43" s="6"/>
-      <c r="BE43" s="6"/>
-      <c r="BF43" s="6"/>
+      <c r="BA43" s="6"/>
+      <c r="BB43" s="6"/>
+      <c r="BC43" s="6"/>
+      <c r="BD43" s="32" t="s">
+        <v>193</v>
+      </c>
+      <c r="BE43" s="32"/>
+      <c r="BF43" s="32"/>
       <c r="BG43" s="6"/>
       <c r="BH43" s="6"/>
       <c r="BI43" s="6"/>
@@ -12164,9 +12185,11 @@
       <c r="G44" s="6"/>
       <c r="H44" s="6"/>
       <c r="I44" s="6"/>
-      <c r="J44" s="6"/>
-      <c r="K44" s="6"/>
-      <c r="L44" s="6"/>
+      <c r="J44" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="K44" s="32"/>
+      <c r="L44" s="32"/>
       <c r="M44" s="20"/>
       <c r="N44" s="20"/>
       <c r="O44" s="20"/>
@@ -12200,11 +12223,11 @@
       </c>
       <c r="AF44" s="13"/>
       <c r="AG44" s="13"/>
-      <c r="AH44" s="29" t="s">
-        <v>186</v>
-      </c>
-      <c r="AI44" s="29"/>
-      <c r="AJ44" s="29"/>
+      <c r="AH44" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="AI44" s="30"/>
+      <c r="AJ44" s="30"/>
       <c r="AK44" s="6"/>
       <c r="AL44" s="6"/>
       <c r="AM44" s="6"/>
@@ -12223,9 +12246,11 @@
       <c r="AY44" s="6"/>
       <c r="AZ44" s="6"/>
       <c r="BA44" s="6"/>
-      <c r="BB44" s="6"/>
-      <c r="BC44" s="6"/>
-      <c r="BD44" s="6"/>
+      <c r="BB44" s="32" t="s">
+        <v>194</v>
+      </c>
+      <c r="BC44" s="32"/>
+      <c r="BD44" s="32"/>
       <c r="BE44" s="8"/>
       <c r="BF44" s="8"/>
       <c r="BG44" s="8"/>
@@ -12259,11 +12284,11 @@
       </c>
       <c r="BX44" s="13"/>
       <c r="BY44" s="13"/>
-      <c r="BZ44" s="29" t="s">
-        <v>192</v>
-      </c>
-      <c r="CA44" s="29"/>
-      <c r="CB44" s="29"/>
+      <c r="BZ44" s="30" t="s">
+        <v>195</v>
+      </c>
+      <c r="CA44" s="30"/>
+      <c r="CB44" s="30"/>
       <c r="CC44" s="6"/>
       <c r="CD44" s="6"/>
       <c r="CE44" s="6"/>
@@ -12341,16 +12366,16 @@
       </c>
       <c r="AX45" s="13"/>
       <c r="AY45" s="13"/>
-      <c r="AZ45" s="31" t="s">
-        <v>193</v>
-      </c>
-      <c r="BA45" s="31"/>
-      <c r="BB45" s="31"/>
-      <c r="BC45" s="31" t="s">
-        <v>194</v>
-      </c>
-      <c r="BD45" s="31"/>
-      <c r="BE45" s="31"/>
+      <c r="AZ45" s="33" t="s">
+        <v>196</v>
+      </c>
+      <c r="BA45" s="33"/>
+      <c r="BB45" s="33"/>
+      <c r="BC45" s="33" t="s">
+        <v>197</v>
+      </c>
+      <c r="BD45" s="33"/>
+      <c r="BE45" s="33"/>
       <c r="BF45" s="13" t="s">
         <v>157</v>
       </c>
@@ -12366,16 +12391,16 @@
       </c>
       <c r="BM45" s="10"/>
       <c r="BN45" s="10"/>
-      <c r="BO45" s="32" t="s">
+      <c r="BO45" s="34" t="s">
         <v>166</v>
       </c>
-      <c r="BP45" s="32"/>
-      <c r="BQ45" s="32"/>
-      <c r="BR45" s="32" t="s">
+      <c r="BP45" s="34"/>
+      <c r="BQ45" s="34"/>
+      <c r="BR45" s="34" t="s">
         <v>144</v>
       </c>
-      <c r="BS45" s="32"/>
-      <c r="BT45" s="32"/>
+      <c r="BS45" s="34"/>
+      <c r="BT45" s="34"/>
       <c r="BU45" s="6"/>
       <c r="BV45" s="6"/>
       <c r="BW45" s="6"/>
@@ -12392,7 +12417,7 @@
       <c r="CH45" s="6"/>
       <c r="CI45" s="6"/>
     </row>
-    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="7"/>
       <c r="B46" s="7"/>
       <c r="C46" s="7"/>
@@ -12424,11 +12449,11 @@
       <c r="AC46" s="7"/>
       <c r="AD46" s="7"/>
       <c r="AE46" s="7"/>
-      <c r="AF46" s="29" t="s">
-        <v>186</v>
-      </c>
-      <c r="AG46" s="29"/>
-      <c r="AH46" s="29"/>
+      <c r="AF46" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="AG46" s="32"/>
+      <c r="AH46" s="32"/>
       <c r="AI46" s="11"/>
       <c r="AJ46" s="11"/>
       <c r="AK46" s="11"/>
@@ -12475,11 +12500,11 @@
       <c r="BU46" s="7"/>
       <c r="BV46" s="7"/>
       <c r="BW46" s="7"/>
-      <c r="BX46" s="29" t="s">
-        <v>192</v>
-      </c>
-      <c r="BY46" s="29"/>
-      <c r="BZ46" s="29"/>
+      <c r="BX46" s="32" t="s">
+        <v>194</v>
+      </c>
+      <c r="BY46" s="32"/>
+      <c r="BZ46" s="32"/>
       <c r="CA46" s="11"/>
       <c r="CB46" s="11"/>
       <c r="CC46" s="11"/>
@@ -12522,9 +12547,9 @@
       <c r="AC47" s="7"/>
       <c r="AD47" s="7"/>
       <c r="AE47" s="7"/>
-      <c r="AF47" s="29"/>
-      <c r="AG47" s="29"/>
-      <c r="AH47" s="29"/>
+      <c r="AF47" s="32"/>
+      <c r="AG47" s="32"/>
+      <c r="AH47" s="32"/>
       <c r="AI47" s="6"/>
       <c r="AJ47" s="6"/>
       <c r="AK47" s="6"/>
@@ -12565,9 +12590,9 @@
       <c r="BU47" s="7"/>
       <c r="BV47" s="7"/>
       <c r="BW47" s="7"/>
-      <c r="BX47" s="29"/>
-      <c r="BY47" s="29"/>
-      <c r="BZ47" s="29"/>
+      <c r="BX47" s="32"/>
+      <c r="BY47" s="32"/>
+      <c r="BZ47" s="32"/>
       <c r="CA47" s="6"/>
       <c r="CB47" s="6"/>
       <c r="CC47" s="6"/>
@@ -14970,7 +14995,7 @@
       <c r="BP10" s="13"/>
       <c r="BQ10" s="13"/>
       <c r="BR10" s="13" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="BS10" s="13"/>
       <c r="BT10" s="13"/>
@@ -15064,7 +15089,7 @@
       <c r="AK11" s="6"/>
       <c r="AL11" s="6"/>
       <c r="AM11" s="6" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="AN11" s="6"/>
       <c r="AO11" s="6"/>
@@ -15733,7 +15758,7 @@
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>109</v>
@@ -15939,7 +15964,7 @@
       <c r="AK19" s="13"/>
       <c r="AL19" s="13"/>
       <c r="AM19" s="6" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="AN19" s="6"/>
       <c r="AO19" s="6"/>
@@ -15994,7 +16019,7 @@
       <c r="CC19" s="7"/>
       <c r="CD19" s="7"/>
       <c r="CE19" s="6" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="CF19" s="6"/>
       <c r="CG19" s="6"/>
@@ -16775,7 +16800,7 @@
       <c r="AK27" s="13"/>
       <c r="AL27" s="13"/>
       <c r="AM27" s="6" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="AN27" s="6"/>
       <c r="AO27" s="6"/>
@@ -16828,7 +16853,7 @@
       <c r="CC27" s="7"/>
       <c r="CD27" s="7"/>
       <c r="CE27" s="6" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="CF27" s="6"/>
       <c r="CG27" s="6"/>
@@ -17600,7 +17625,7 @@
       <c r="AK35" s="13"/>
       <c r="AL35" s="13"/>
       <c r="AM35" s="6" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="AN35" s="6"/>
       <c r="AO35" s="6"/>
@@ -17657,7 +17682,7 @@
       <c r="CC35" s="7"/>
       <c r="CD35" s="7"/>
       <c r="CE35" s="6" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="CF35" s="6"/>
       <c r="CG35" s="6"/>
@@ -19211,7 +19236,7 @@
       <c r="AP1" s="4"/>
       <c r="AQ1" s="5"/>
       <c r="AT1" s="3" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="AU1" s="4"/>
       <c r="AV1" s="4"/>
@@ -19494,7 +19519,7 @@
         <v>161</v>
       </c>
       <c r="AT4" s="7" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="AU4" s="7"/>
       <c r="AV4" s="7"/>
@@ -19502,7 +19527,7 @@
       <c r="AX4" s="8"/>
       <c r="AY4" s="6"/>
       <c r="AZ4" s="6" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="BA4" s="8" t="s">
         <v>56</v>
@@ -19591,8 +19616,8 @@
       <c r="AO5" s="6"/>
       <c r="AP5" s="6"/>
       <c r="AQ5" s="6"/>
-      <c r="AR5" s="33" t="s">
-        <v>201</v>
+      <c r="AR5" s="35" t="s">
+        <v>204</v>
       </c>
       <c r="AT5" s="7"/>
       <c r="AU5" s="7"/>
@@ -19601,7 +19626,7 @@
       <c r="AX5" s="7"/>
       <c r="AY5" s="7"/>
       <c r="AZ5" s="6" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="BA5" s="7" t="s">
         <v>172</v>
@@ -19661,10 +19686,10 @@
       <c r="V6" s="7"/>
       <c r="W6" s="7"/>
       <c r="X6" s="7" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="Y6" s="7" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="Z6" s="7"/>
       <c r="AA6" s="7"/>
@@ -19707,7 +19732,7 @@
       <c r="AW6" s="7"/>
       <c r="AX6" s="7"/>
       <c r="AY6" s="7" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="AZ6" s="7"/>
       <c r="BA6" s="7"/>
@@ -19716,7 +19741,7 @@
       <c r="BD6" s="6"/>
       <c r="BE6" s="11"/>
       <c r="BF6" s="6" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="BG6" s="11"/>
       <c r="BH6" s="11"/>
@@ -19781,7 +19806,7 @@
         <v>172</v>
       </c>
       <c r="BF7" s="6" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="BG7" s="6" t="s">
         <v>173</v>
@@ -19835,7 +19860,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -20398,8 +20423,8 @@
       <c r="AO13" s="6"/>
       <c r="AP13" s="6"/>
       <c r="AQ13" s="6"/>
-      <c r="AR13" s="33" t="s">
-        <v>201</v>
+      <c r="AR13" s="35" t="s">
+        <v>204</v>
       </c>
       <c r="AT13" s="7"/>
       <c r="AU13" s="7"/>
@@ -20512,10 +20537,10 @@
       </c>
       <c r="W14" s="7"/>
       <c r="X14" s="7" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="Y14" s="7" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="Z14" s="7"/>
       <c r="AA14" s="7"/>
@@ -20794,7 +20819,7 @@
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>109</v>
@@ -21265,8 +21290,8 @@
       <c r="AO21" s="6"/>
       <c r="AP21" s="6"/>
       <c r="AQ21" s="6"/>
-      <c r="AR21" s="33" t="s">
-        <v>201</v>
+      <c r="AR21" s="35" t="s">
+        <v>204</v>
       </c>
       <c r="AT21" s="7"/>
       <c r="AU21" s="7"/>
@@ -21375,10 +21400,10 @@
       </c>
       <c r="W22" s="7"/>
       <c r="X22" s="7" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="Y22" s="7" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="Z22" s="7"/>
       <c r="AA22" s="7"/>
@@ -22091,8 +22116,8 @@
       <c r="AO29" s="6"/>
       <c r="AP29" s="6"/>
       <c r="AQ29" s="6"/>
-      <c r="AR29" s="33" t="s">
-        <v>201</v>
+      <c r="AR29" s="35" t="s">
+        <v>204</v>
       </c>
       <c r="AT29" s="7"/>
       <c r="AU29" s="7"/>
@@ -22189,10 +22214,10 @@
       </c>
       <c r="W30" s="7"/>
       <c r="X30" s="7" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="Y30" s="7" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="Z30" s="7"/>
       <c r="AA30" s="7"/>
@@ -22259,7 +22284,7 @@
       </c>
       <c r="BP30" s="7"/>
       <c r="BQ30" s="7" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="BR30" s="7"/>
       <c r="BS30" s="7"/>
@@ -22764,7 +22789,7 @@
       <c r="AR36" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="AT36" s="34" t="s">
+      <c r="AT36" s="36" t="s">
         <v>34</v>
       </c>
       <c r="AU36" s="13" t="s">
@@ -22870,8 +22895,8 @@
       <c r="AO37" s="6"/>
       <c r="AP37" s="6"/>
       <c r="AQ37" s="6"/>
-      <c r="AR37" s="33" t="s">
-        <v>201</v>
+      <c r="AR37" s="35" t="s">
+        <v>204</v>
       </c>
       <c r="AT37" s="7" t="s">
         <v>35</v>
@@ -22954,10 +22979,10 @@
       </c>
       <c r="W38" s="7"/>
       <c r="X38" s="7" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="Y38" s="7" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="Z38" s="7"/>
       <c r="AA38" s="7"/>
@@ -22992,17 +23017,17 @@
       <c r="AW38" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="AX38" s="34" t="s">
+      <c r="AX38" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="AY38" s="34" t="s">
+      <c r="AY38" s="36" t="s">
         <v>52</v>
       </c>
-      <c r="AZ38" s="34"/>
-      <c r="BA38" s="34" t="s">
+      <c r="AZ38" s="36"/>
+      <c r="BA38" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="BB38" s="34" t="s">
+      <c r="BB38" s="36" t="s">
         <v>107</v>
       </c>
       <c r="BC38" s="11"/>
@@ -23065,9 +23090,9 @@
       <c r="AW39" s="7"/>
       <c r="AX39" s="7"/>
       <c r="AY39" s="7"/>
-      <c r="AZ39" s="34"/>
-      <c r="BA39" s="34"/>
-      <c r="BB39" s="34"/>
+      <c r="AZ39" s="36"/>
+      <c r="BA39" s="36"/>
+      <c r="BB39" s="36"/>
       <c r="BC39" s="11"/>
       <c r="BD39" s="6"/>
       <c r="BE39" s="6"/>
@@ -24312,8 +24337,8 @@
       </c>
       <c r="N5" s="6"/>
       <c r="O5" s="6"/>
-      <c r="P5" s="33" t="s">
-        <v>201</v>
+      <c r="P5" s="35" t="s">
+        <v>204</v>
       </c>
       <c r="R5" s="7"/>
       <c r="S5" s="7"/>
@@ -24444,7 +24469,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -24599,7 +24624,7 @@
       <c r="Z11" s="13"/>
       <c r="AA11" s="13"/>
       <c r="AB11" s="13"/>
-      <c r="AC11" s="35"/>
+      <c r="AC11" s="37"/>
       <c r="AD11" s="21"/>
       <c r="AE11" s="6"/>
       <c r="AF11" s="6"/>
@@ -24707,8 +24732,8 @@
       </c>
       <c r="N13" s="6"/>
       <c r="O13" s="6"/>
-      <c r="P13" s="33" t="s">
-        <v>201</v>
+      <c r="P13" s="35" t="s">
+        <v>204</v>
       </c>
       <c r="R13" s="7"/>
       <c r="S13" s="13"/>
@@ -24916,8 +24941,8 @@
       <c r="M19" s="13"/>
       <c r="N19" s="6"/>
       <c r="O19" s="6"/>
-      <c r="P19" s="36" t="s">
-        <v>207</v>
+      <c r="P19" s="38" t="s">
+        <v>210</v>
       </c>
       <c r="R19" s="7"/>
       <c r="S19" s="7"/>
@@ -24936,7 +24961,7 @@
       <c r="AF19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="34"/>
+      <c r="A20" s="36"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
@@ -25019,11 +25044,11 @@
       <c r="S22" s="7"/>
       <c r="T22" s="7"/>
       <c r="U22" s="7"/>
-      <c r="V22" s="34"/>
+      <c r="V22" s="36"/>
       <c r="W22" s="7"/>
       <c r="X22" s="7"/>
-      <c r="Y22" s="37"/>
-      <c r="Z22" s="37"/>
+      <c r="Y22" s="39"/>
+      <c r="Z22" s="39"/>
       <c r="AA22" s="11"/>
       <c r="AB22" s="6"/>
       <c r="AC22" s="11"/>
@@ -25051,11 +25076,11 @@
       <c r="S23" s="7"/>
       <c r="T23" s="7"/>
       <c r="U23" s="7"/>
-      <c r="V23" s="34"/>
-      <c r="W23" s="34"/>
+      <c r="V23" s="36"/>
+      <c r="W23" s="36"/>
       <c r="X23" s="7"/>
-      <c r="Y23" s="37"/>
-      <c r="Z23" s="37"/>
+      <c r="Y23" s="39"/>
+      <c r="Z23" s="39"/>
       <c r="AA23" s="11"/>
       <c r="AB23" s="6"/>
       <c r="AC23" s="6"/>
@@ -25192,7 +25217,7 @@
       <c r="M28" s="13"/>
       <c r="N28" s="6"/>
       <c r="O28" s="6"/>
-      <c r="R28" s="34"/>
+      <c r="R28" s="36"/>
       <c r="S28" s="7"/>
       <c r="T28" s="7"/>
       <c r="U28" s="7"/>
@@ -25246,8 +25271,8 @@
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
       <c r="E30" s="7"/>
-      <c r="F30" s="34"/>
-      <c r="G30" s="34"/>
+      <c r="F30" s="36"/>
+      <c r="G30" s="36"/>
       <c r="H30" s="7"/>
       <c r="I30" s="7"/>
       <c r="J30" s="11"/>
@@ -25260,9 +25285,9 @@
       <c r="S30" s="7"/>
       <c r="T30" s="7"/>
       <c r="U30" s="7"/>
-      <c r="V30" s="34"/>
-      <c r="W30" s="34"/>
-      <c r="X30" s="34"/>
+      <c r="V30" s="36"/>
+      <c r="W30" s="36"/>
+      <c r="X30" s="36"/>
       <c r="Y30" s="6"/>
       <c r="Z30" s="7"/>
       <c r="AA30" s="11"/>
@@ -25279,7 +25304,7 @@
       <c r="D31" s="7"/>
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
-      <c r="G31" s="34"/>
+      <c r="G31" s="36"/>
       <c r="H31" s="7"/>
       <c r="I31" s="7"/>
       <c r="J31" s="11"/>
@@ -25294,7 +25319,7 @@
       <c r="U31" s="7"/>
       <c r="V31" s="7"/>
       <c r="W31" s="7"/>
-      <c r="X31" s="34"/>
+      <c r="X31" s="36"/>
       <c r="Y31" s="6"/>
       <c r="Z31" s="7"/>
       <c r="AA31" s="11"/>
@@ -25357,7 +25382,7 @@
       <c r="A34" s="7"/>
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
-      <c r="D34" s="32"/>
+      <c r="D34" s="34"/>
       <c r="E34" s="6"/>
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
@@ -25433,7 +25458,7 @@
       <c r="M36" s="13"/>
       <c r="N36" s="6"/>
       <c r="O36" s="6"/>
-      <c r="R36" s="34"/>
+      <c r="R36" s="36"/>
       <c r="S36" s="13"/>
       <c r="T36" s="13"/>
       <c r="U36" s="13"/>
@@ -25472,7 +25497,7 @@
       <c r="V37" s="13"/>
       <c r="W37" s="13"/>
       <c r="X37" s="18"/>
-      <c r="Y37" s="38"/>
+      <c r="Y37" s="40"/>
       <c r="Z37" s="6"/>
       <c r="AA37" s="6"/>
       <c r="AB37" s="6"/>
@@ -25487,8 +25512,8 @@
       <c r="C38" s="7"/>
       <c r="D38" s="7"/>
       <c r="E38" s="7"/>
-      <c r="F38" s="34"/>
-      <c r="G38" s="34"/>
+      <c r="F38" s="36"/>
+      <c r="G38" s="36"/>
       <c r="H38" s="7"/>
       <c r="I38" s="7"/>
       <c r="J38" s="11"/>
@@ -25501,11 +25526,11 @@
       <c r="S38" s="7"/>
       <c r="T38" s="7"/>
       <c r="U38" s="7"/>
-      <c r="V38" s="34"/>
-      <c r="W38" s="34"/>
-      <c r="X38" s="34"/>
-      <c r="Y38" s="34"/>
-      <c r="Z38" s="34"/>
+      <c r="V38" s="36"/>
+      <c r="W38" s="36"/>
+      <c r="X38" s="36"/>
+      <c r="Y38" s="36"/>
+      <c r="Z38" s="36"/>
       <c r="AA38" s="11"/>
       <c r="AB38" s="6"/>
       <c r="AC38" s="11"/>
@@ -25520,7 +25545,7 @@
       <c r="D39" s="7"/>
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
-      <c r="G39" s="34"/>
+      <c r="G39" s="36"/>
       <c r="H39" s="7"/>
       <c r="I39" s="7"/>
       <c r="J39" s="11"/>
@@ -25535,9 +25560,9 @@
       <c r="U39" s="7"/>
       <c r="V39" s="7"/>
       <c r="W39" s="7"/>
-      <c r="X39" s="34"/>
-      <c r="Y39" s="34"/>
-      <c r="Z39" s="34"/>
+      <c r="X39" s="36"/>
+      <c r="Y39" s="36"/>
+      <c r="Z39" s="36"/>
       <c r="AA39" s="11"/>
       <c r="AB39" s="6"/>
       <c r="AC39" s="6"/>
@@ -25658,7 +25683,7 @@
       <c r="AF43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="34"/>
+      <c r="A44" s="36"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
@@ -25673,7 +25698,7 @@
       <c r="M44" s="6"/>
       <c r="N44" s="6"/>
       <c r="O44" s="6"/>
-      <c r="R44" s="34"/>
+      <c r="R44" s="36"/>
       <c r="S44" s="13"/>
       <c r="T44" s="13"/>
       <c r="U44" s="13"/>
@@ -25727,8 +25752,8 @@
       <c r="C46" s="7"/>
       <c r="D46" s="7"/>
       <c r="E46" s="7"/>
-      <c r="F46" s="34"/>
-      <c r="G46" s="34"/>
+      <c r="F46" s="36"/>
+      <c r="G46" s="36"/>
       <c r="H46" s="6"/>
       <c r="I46" s="7"/>
       <c r="J46" s="11"/>
@@ -25741,11 +25766,11 @@
       <c r="S46" s="7"/>
       <c r="T46" s="7"/>
       <c r="U46" s="7"/>
-      <c r="V46" s="34"/>
-      <c r="W46" s="34"/>
-      <c r="X46" s="34"/>
-      <c r="Y46" s="34"/>
-      <c r="Z46" s="34"/>
+      <c r="V46" s="36"/>
+      <c r="W46" s="36"/>
+      <c r="X46" s="36"/>
+      <c r="Y46" s="36"/>
+      <c r="Z46" s="36"/>
       <c r="AA46" s="11"/>
       <c r="AB46" s="6"/>
       <c r="AC46" s="11"/>
@@ -25760,7 +25785,7 @@
       <c r="D47" s="7"/>
       <c r="E47" s="7"/>
       <c r="F47" s="7"/>
-      <c r="G47" s="34"/>
+      <c r="G47" s="36"/>
       <c r="H47" s="6"/>
       <c r="I47" s="7"/>
       <c r="J47" s="11"/>
@@ -25775,9 +25800,9 @@
       <c r="U47" s="7"/>
       <c r="V47" s="7"/>
       <c r="W47" s="7"/>
-      <c r="X47" s="34"/>
-      <c r="Y47" s="34"/>
-      <c r="Z47" s="34"/>
+      <c r="X47" s="36"/>
+      <c r="Y47" s="36"/>
+      <c r="Z47" s="36"/>
       <c r="AA47" s="11"/>
       <c r="AB47" s="6"/>
       <c r="AC47" s="6"/>
@@ -25905,7 +25930,7 @@
       <c r="S52" s="7"/>
       <c r="T52" s="7"/>
       <c r="U52" s="7"/>
-      <c r="V52" s="39"/>
+      <c r="V52" s="41"/>
       <c r="W52" s="6"/>
       <c r="X52" s="13"/>
       <c r="Y52" s="14"/>
@@ -25954,11 +25979,11 @@
       <c r="B54" s="7"/>
       <c r="C54" s="7"/>
       <c r="D54" s="7"/>
-      <c r="E54" s="34"/>
+      <c r="E54" s="36"/>
       <c r="F54" s="7"/>
       <c r="G54" s="7"/>
-      <c r="H54" s="37"/>
-      <c r="I54" s="37"/>
+      <c r="H54" s="39"/>
+      <c r="I54" s="39"/>
       <c r="J54" s="11"/>
       <c r="K54" s="6"/>
       <c r="L54" s="11"/>
@@ -25986,11 +26011,11 @@
       <c r="B55" s="7"/>
       <c r="C55" s="7"/>
       <c r="D55" s="7"/>
-      <c r="E55" s="34"/>
-      <c r="F55" s="34"/>
+      <c r="E55" s="36"/>
+      <c r="F55" s="36"/>
       <c r="G55" s="7"/>
-      <c r="H55" s="37"/>
-      <c r="I55" s="37"/>
+      <c r="H55" s="39"/>
+      <c r="I55" s="39"/>
       <c r="J55" s="11"/>
       <c r="K55" s="6"/>
       <c r="L55" s="6"/>

</xml_diff>

<commit_message>
[Update] Layout images are updated.
</commit_message>
<xml_diff>
--- a/img/keymap.xlsx
+++ b/img/keymap.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2358" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2361" uniqueCount="210">
   <si>
     <t xml:space="preserve">標準</t>
   </si>
@@ -592,7 +592,7 @@
 Mode</t>
   </si>
   <si>
-    <t xml:space="preserve">Stdard
+    <t xml:space="preserve">Standard
 Mode</t>
   </si>
   <si>
@@ -614,9 +614,6 @@
   <si>
     <t xml:space="preserve">Cursor
 Mode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CurMode</t>
   </si>
   <si>
     <r>
@@ -7658,7 +7655,9 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="2" style="1" width="2.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="2" style="1" width="2.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="1" width="2.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="35" style="1" width="2.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="4.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="1" width="6.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="48" min="46" style="1" width="2.04"/>
@@ -10535,26 +10534,26 @@
       </c>
       <c r="Y27" s="6"/>
       <c r="Z27" s="6"/>
-      <c r="AA27" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="AB27" s="6"/>
-      <c r="AC27" s="6"/>
-      <c r="AD27" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="AE27" s="7"/>
-      <c r="AF27" s="7"/>
-      <c r="AG27" s="13" t="s">
+      <c r="AA27" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="AH27" s="13"/>
-      <c r="AI27" s="13"/>
-      <c r="AJ27" s="13" t="s">
+      <c r="AB27" s="13"/>
+      <c r="AC27" s="13"/>
+      <c r="AD27" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="AK27" s="13"/>
-      <c r="AL27" s="13"/>
+      <c r="AE27" s="13"/>
+      <c r="AF27" s="13"/>
+      <c r="AG27" s="30" t="s">
+        <v>145</v>
+      </c>
+      <c r="AH27" s="30"/>
+      <c r="AI27" s="30"/>
+      <c r="AJ27" s="30" t="s">
+        <v>146</v>
+      </c>
+      <c r="AK27" s="30"/>
+      <c r="AL27" s="30"/>
       <c r="AM27" s="6"/>
       <c r="AN27" s="6"/>
       <c r="AO27" s="6"/>
@@ -10940,20 +10939,22 @@
       <c r="BL30" s="31"/>
       <c r="BM30" s="31"/>
       <c r="BN30" s="31"/>
-      <c r="BO30" s="7"/>
-      <c r="BP30" s="7"/>
-      <c r="BQ30" s="7"/>
-      <c r="BR30" s="7"/>
-      <c r="BS30" s="7"/>
-      <c r="BT30" s="7"/>
+      <c r="BO30" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="BP30" s="32"/>
+      <c r="BQ30" s="32"/>
+      <c r="BR30" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="BS30" s="32"/>
+      <c r="BT30" s="32"/>
       <c r="BU30" s="7"/>
       <c r="BV30" s="7"/>
       <c r="BW30" s="7"/>
-      <c r="BX30" s="32" t="s">
-        <v>187</v>
-      </c>
-      <c r="BY30" s="32"/>
-      <c r="BZ30" s="32"/>
+      <c r="BX30" s="7"/>
+      <c r="BY30" s="7"/>
+      <c r="BZ30" s="7"/>
       <c r="CA30" s="11"/>
       <c r="CB30" s="11"/>
       <c r="CC30" s="11"/>
@@ -11032,18 +11033,18 @@
       <c r="BL31" s="31"/>
       <c r="BM31" s="31"/>
       <c r="BN31" s="31"/>
-      <c r="BO31" s="7"/>
-      <c r="BP31" s="7"/>
-      <c r="BQ31" s="7"/>
-      <c r="BR31" s="7"/>
-      <c r="BS31" s="7"/>
-      <c r="BT31" s="7"/>
+      <c r="BO31" s="32"/>
+      <c r="BP31" s="32"/>
+      <c r="BQ31" s="32"/>
+      <c r="BR31" s="32"/>
+      <c r="BS31" s="32"/>
+      <c r="BT31" s="32"/>
       <c r="BU31" s="7"/>
       <c r="BV31" s="7"/>
       <c r="BW31" s="7"/>
-      <c r="BX31" s="32"/>
-      <c r="BY31" s="32"/>
-      <c r="BZ31" s="32"/>
+      <c r="BX31" s="7"/>
+      <c r="BY31" s="7"/>
+      <c r="BZ31" s="7"/>
       <c r="CA31" s="6" t="s">
         <v>172</v>
       </c>
@@ -11435,11 +11436,11 @@
       </c>
       <c r="H36" s="13"/>
       <c r="I36" s="13"/>
-      <c r="J36" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="K36" s="13"/>
-      <c r="L36" s="13"/>
+      <c r="J36" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="K36" s="29"/>
+      <c r="L36" s="29"/>
       <c r="M36" s="20" t="s">
         <v>7</v>
       </c>
@@ -11717,11 +11718,11 @@
       </c>
       <c r="AD38" s="7"/>
       <c r="AE38" s="7"/>
-      <c r="AF38" s="29" t="s">
-        <v>186</v>
-      </c>
-      <c r="AG38" s="29"/>
-      <c r="AH38" s="29"/>
+      <c r="AF38" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="AG38" s="7"/>
+      <c r="AH38" s="7"/>
       <c r="AI38" s="11"/>
       <c r="AJ38" s="11"/>
       <c r="AK38" s="11"/>
@@ -11755,20 +11756,22 @@
       <c r="BL38" s="31"/>
       <c r="BM38" s="31"/>
       <c r="BN38" s="31"/>
-      <c r="BO38" s="7"/>
-      <c r="BP38" s="7"/>
-      <c r="BQ38" s="7"/>
-      <c r="BR38" s="7"/>
-      <c r="BS38" s="7"/>
-      <c r="BT38" s="7"/>
+      <c r="BO38" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="BP38" s="32"/>
+      <c r="BQ38" s="32"/>
+      <c r="BR38" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="BS38" s="32"/>
+      <c r="BT38" s="32"/>
       <c r="BU38" s="7"/>
       <c r="BV38" s="7"/>
       <c r="BW38" s="7"/>
-      <c r="BX38" s="32" t="s">
-        <v>187</v>
-      </c>
-      <c r="BY38" s="32"/>
-      <c r="BZ38" s="32"/>
+      <c r="BX38" s="7"/>
+      <c r="BY38" s="7"/>
+      <c r="BZ38" s="7"/>
       <c r="CA38" s="11"/>
       <c r="CB38" s="11"/>
       <c r="CC38" s="11"/>
@@ -11811,9 +11814,9 @@
       <c r="AC39" s="7"/>
       <c r="AD39" s="7"/>
       <c r="AE39" s="7"/>
-      <c r="AF39" s="29"/>
-      <c r="AG39" s="29"/>
-      <c r="AH39" s="29"/>
+      <c r="AF39" s="7"/>
+      <c r="AG39" s="7"/>
+      <c r="AH39" s="7"/>
       <c r="AI39" s="6"/>
       <c r="AJ39" s="6"/>
       <c r="AK39" s="6"/>
@@ -11845,18 +11848,18 @@
       <c r="BL39" s="31"/>
       <c r="BM39" s="31"/>
       <c r="BN39" s="31"/>
-      <c r="BO39" s="7"/>
-      <c r="BP39" s="7"/>
-      <c r="BQ39" s="7"/>
-      <c r="BR39" s="7"/>
-      <c r="BS39" s="7"/>
-      <c r="BT39" s="7"/>
+      <c r="BO39" s="32"/>
+      <c r="BP39" s="32"/>
+      <c r="BQ39" s="32"/>
+      <c r="BR39" s="32"/>
+      <c r="BS39" s="32"/>
+      <c r="BT39" s="32"/>
       <c r="BU39" s="7"/>
       <c r="BV39" s="7"/>
       <c r="BW39" s="7"/>
-      <c r="BX39" s="32"/>
-      <c r="BY39" s="32"/>
-      <c r="BZ39" s="32"/>
+      <c r="BX39" s="7"/>
+      <c r="BY39" s="7"/>
+      <c r="BZ39" s="7"/>
       <c r="CA39" s="6"/>
       <c r="CB39" s="6"/>
       <c r="CC39" s="6"/>
@@ -12174,11 +12177,11 @@
       <c r="CI43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B44" s="7"/>
-      <c r="C44" s="7"/>
+      <c r="A44" s="31" t="s">
+        <v>188</v>
+      </c>
+      <c r="B44" s="31"/>
+      <c r="C44" s="31"/>
       <c r="D44" s="6"/>
       <c r="E44" s="6"/>
       <c r="F44" s="6"/>
@@ -12223,11 +12226,11 @@
       </c>
       <c r="AF44" s="13"/>
       <c r="AG44" s="13"/>
-      <c r="AH44" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="AI44" s="30"/>
-      <c r="AJ44" s="30"/>
+      <c r="AH44" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="AI44" s="32"/>
+      <c r="AJ44" s="32"/>
       <c r="AK44" s="6"/>
       <c r="AL44" s="6"/>
       <c r="AM44" s="6"/>
@@ -12235,11 +12238,11 @@
       <c r="AO44" s="9"/>
       <c r="AP44" s="9"/>
       <c r="AQ44" s="9"/>
-      <c r="AS44" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="AT44" s="7"/>
-      <c r="AU44" s="7"/>
+      <c r="AS44" s="31" t="s">
+        <v>188</v>
+      </c>
+      <c r="AT44" s="31"/>
+      <c r="AU44" s="31"/>
       <c r="AV44" s="6"/>
       <c r="AW44" s="6"/>
       <c r="AX44" s="6"/>
@@ -12284,11 +12287,11 @@
       </c>
       <c r="BX44" s="13"/>
       <c r="BY44" s="13"/>
-      <c r="BZ44" s="30" t="s">
-        <v>195</v>
-      </c>
-      <c r="CA44" s="30"/>
-      <c r="CB44" s="30"/>
+      <c r="BZ44" s="32" t="s">
+        <v>194</v>
+      </c>
+      <c r="CA44" s="32"/>
+      <c r="CB44" s="32"/>
       <c r="CC44" s="6"/>
       <c r="CD44" s="6"/>
       <c r="CE44" s="6"/>
@@ -12367,12 +12370,12 @@
       <c r="AX45" s="13"/>
       <c r="AY45" s="13"/>
       <c r="AZ45" s="33" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="BA45" s="33"/>
       <c r="BB45" s="33"/>
       <c r="BC45" s="33" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="BD45" s="33"/>
       <c r="BE45" s="33"/>
@@ -12431,29 +12434,33 @@
       <c r="K46" s="7"/>
       <c r="L46" s="7"/>
       <c r="M46" s="7"/>
-      <c r="N46" s="7"/>
-      <c r="O46" s="7"/>
-      <c r="P46" s="7"/>
-      <c r="Q46" s="7"/>
-      <c r="R46" s="7"/>
-      <c r="S46" s="7"/>
-      <c r="T46" s="7"/>
-      <c r="U46" s="7"/>
-      <c r="V46" s="7"/>
-      <c r="W46" s="7"/>
-      <c r="X46" s="7"/>
-      <c r="Y46" s="7"/>
-      <c r="Z46" s="7"/>
-      <c r="AA46" s="7"/>
-      <c r="AB46" s="7"/>
+      <c r="N46" s="31" t="s">
+        <v>188</v>
+      </c>
+      <c r="O46" s="31"/>
+      <c r="P46" s="31"/>
+      <c r="Q46" s="31"/>
+      <c r="R46" s="31"/>
+      <c r="S46" s="31"/>
+      <c r="T46" s="31"/>
+      <c r="U46" s="31"/>
+      <c r="V46" s="31"/>
+      <c r="W46" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="X46" s="32"/>
+      <c r="Y46" s="32"/>
+      <c r="Z46" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA46" s="32"/>
+      <c r="AB46" s="32"/>
       <c r="AC46" s="7"/>
       <c r="AD46" s="7"/>
       <c r="AE46" s="7"/>
-      <c r="AF46" s="32" t="s">
-        <v>187</v>
-      </c>
-      <c r="AG46" s="32"/>
-      <c r="AH46" s="32"/>
+      <c r="AF46" s="7"/>
+      <c r="AG46" s="7"/>
+      <c r="AH46" s="7"/>
       <c r="AI46" s="11"/>
       <c r="AJ46" s="11"/>
       <c r="AK46" s="11"/>
@@ -12476,35 +12483,33 @@
       <c r="BC46" s="7"/>
       <c r="BD46" s="7"/>
       <c r="BE46" s="7"/>
-      <c r="BF46" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="BG46" s="7"/>
-      <c r="BH46" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="BI46" s="7"/>
-      <c r="BJ46" s="7"/>
-      <c r="BK46" s="7"/>
-      <c r="BL46" s="7"/>
-      <c r="BM46" s="7"/>
-      <c r="BN46" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="BO46" s="7"/>
-      <c r="BP46" s="7"/>
-      <c r="BQ46" s="7"/>
-      <c r="BR46" s="7"/>
-      <c r="BS46" s="7"/>
-      <c r="BT46" s="7"/>
+      <c r="BF46" s="31" t="s">
+        <v>188</v>
+      </c>
+      <c r="BG46" s="31"/>
+      <c r="BH46" s="31"/>
+      <c r="BI46" s="31"/>
+      <c r="BJ46" s="31"/>
+      <c r="BK46" s="31"/>
+      <c r="BL46" s="31"/>
+      <c r="BM46" s="31"/>
+      <c r="BN46" s="31"/>
+      <c r="BO46" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="BP46" s="32"/>
+      <c r="BQ46" s="32"/>
+      <c r="BR46" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="BS46" s="32"/>
+      <c r="BT46" s="32"/>
       <c r="BU46" s="7"/>
       <c r="BV46" s="7"/>
       <c r="BW46" s="7"/>
-      <c r="BX46" s="32" t="s">
-        <v>194</v>
-      </c>
-      <c r="BY46" s="32"/>
-      <c r="BZ46" s="32"/>
+      <c r="BX46" s="7"/>
+      <c r="BY46" s="7"/>
+      <c r="BZ46" s="7"/>
       <c r="CA46" s="11"/>
       <c r="CB46" s="11"/>
       <c r="CC46" s="11"/>
@@ -12529,27 +12534,27 @@
       <c r="K47" s="7"/>
       <c r="L47" s="7"/>
       <c r="M47" s="7"/>
-      <c r="N47" s="7"/>
-      <c r="O47" s="7"/>
-      <c r="P47" s="7"/>
-      <c r="Q47" s="7"/>
-      <c r="R47" s="7"/>
-      <c r="S47" s="7"/>
-      <c r="T47" s="7"/>
-      <c r="U47" s="7"/>
-      <c r="V47" s="7"/>
-      <c r="W47" s="7"/>
-      <c r="X47" s="7"/>
-      <c r="Y47" s="7"/>
-      <c r="Z47" s="7"/>
-      <c r="AA47" s="7"/>
-      <c r="AB47" s="7"/>
+      <c r="N47" s="31"/>
+      <c r="O47" s="31"/>
+      <c r="P47" s="31"/>
+      <c r="Q47" s="31"/>
+      <c r="R47" s="31"/>
+      <c r="S47" s="31"/>
+      <c r="T47" s="31"/>
+      <c r="U47" s="31"/>
+      <c r="V47" s="31"/>
+      <c r="W47" s="32"/>
+      <c r="X47" s="32"/>
+      <c r="Y47" s="32"/>
+      <c r="Z47" s="32"/>
+      <c r="AA47" s="32"/>
+      <c r="AB47" s="32"/>
       <c r="AC47" s="7"/>
       <c r="AD47" s="7"/>
       <c r="AE47" s="7"/>
-      <c r="AF47" s="32"/>
-      <c r="AG47" s="32"/>
-      <c r="AH47" s="32"/>
+      <c r="AF47" s="7"/>
+      <c r="AG47" s="7"/>
+      <c r="AH47" s="7"/>
       <c r="AI47" s="6"/>
       <c r="AJ47" s="6"/>
       <c r="AK47" s="6"/>
@@ -12572,27 +12577,27 @@
       <c r="BC47" s="7"/>
       <c r="BD47" s="7"/>
       <c r="BE47" s="7"/>
-      <c r="BF47" s="7"/>
-      <c r="BG47" s="7"/>
-      <c r="BH47" s="7"/>
-      <c r="BI47" s="7"/>
-      <c r="BJ47" s="7"/>
-      <c r="BK47" s="7"/>
-      <c r="BL47" s="7"/>
-      <c r="BM47" s="7"/>
-      <c r="BN47" s="7"/>
-      <c r="BO47" s="7"/>
-      <c r="BP47" s="7"/>
-      <c r="BQ47" s="7"/>
-      <c r="BR47" s="7"/>
-      <c r="BS47" s="7"/>
-      <c r="BT47" s="7"/>
+      <c r="BF47" s="31"/>
+      <c r="BG47" s="31"/>
+      <c r="BH47" s="31"/>
+      <c r="BI47" s="31"/>
+      <c r="BJ47" s="31"/>
+      <c r="BK47" s="31"/>
+      <c r="BL47" s="31"/>
+      <c r="BM47" s="31"/>
+      <c r="BN47" s="31"/>
+      <c r="BO47" s="32"/>
+      <c r="BP47" s="32"/>
+      <c r="BQ47" s="32"/>
+      <c r="BR47" s="32"/>
+      <c r="BS47" s="32"/>
+      <c r="BT47" s="32"/>
       <c r="BU47" s="7"/>
       <c r="BV47" s="7"/>
       <c r="BW47" s="7"/>
-      <c r="BX47" s="32"/>
-      <c r="BY47" s="32"/>
-      <c r="BZ47" s="32"/>
+      <c r="BX47" s="7"/>
+      <c r="BY47" s="7"/>
+      <c r="BZ47" s="7"/>
       <c r="CA47" s="6"/>
       <c r="CB47" s="6"/>
       <c r="CC47" s="6"/>
@@ -14995,7 +15000,7 @@
       <c r="BP10" s="13"/>
       <c r="BQ10" s="13"/>
       <c r="BR10" s="13" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="BS10" s="13"/>
       <c r="BT10" s="13"/>
@@ -15089,7 +15094,7 @@
       <c r="AK11" s="6"/>
       <c r="AL11" s="6"/>
       <c r="AM11" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AN11" s="6"/>
       <c r="AO11" s="6"/>
@@ -15758,7 +15763,7 @@
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>109</v>
@@ -15964,7 +15969,7 @@
       <c r="AK19" s="13"/>
       <c r="AL19" s="13"/>
       <c r="AM19" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AN19" s="6"/>
       <c r="AO19" s="6"/>
@@ -16019,7 +16024,7 @@
       <c r="CC19" s="7"/>
       <c r="CD19" s="7"/>
       <c r="CE19" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="CF19" s="6"/>
       <c r="CG19" s="6"/>
@@ -16800,7 +16805,7 @@
       <c r="AK27" s="13"/>
       <c r="AL27" s="13"/>
       <c r="AM27" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AN27" s="6"/>
       <c r="AO27" s="6"/>
@@ -16853,7 +16858,7 @@
       <c r="CC27" s="7"/>
       <c r="CD27" s="7"/>
       <c r="CE27" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="CF27" s="6"/>
       <c r="CG27" s="6"/>
@@ -17625,7 +17630,7 @@
       <c r="AK35" s="13"/>
       <c r="AL35" s="13"/>
       <c r="AM35" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AN35" s="6"/>
       <c r="AO35" s="6"/>
@@ -17682,7 +17687,7 @@
       <c r="CC35" s="7"/>
       <c r="CD35" s="7"/>
       <c r="CE35" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="CF35" s="6"/>
       <c r="CG35" s="6"/>
@@ -19236,7 +19241,7 @@
       <c r="AP1" s="4"/>
       <c r="AQ1" s="5"/>
       <c r="AT1" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AU1" s="4"/>
       <c r="AV1" s="4"/>
@@ -19519,7 +19524,7 @@
         <v>161</v>
       </c>
       <c r="AT4" s="7" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AU4" s="7"/>
       <c r="AV4" s="7"/>
@@ -19527,7 +19532,7 @@
       <c r="AX4" s="8"/>
       <c r="AY4" s="6"/>
       <c r="AZ4" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="BA4" s="8" t="s">
         <v>56</v>
@@ -19617,7 +19622,7 @@
       <c r="AP5" s="6"/>
       <c r="AQ5" s="6"/>
       <c r="AR5" s="35" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AT5" s="7"/>
       <c r="AU5" s="7"/>
@@ -19626,7 +19631,7 @@
       <c r="AX5" s="7"/>
       <c r="AY5" s="7"/>
       <c r="AZ5" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BA5" s="7" t="s">
         <v>172</v>
@@ -19686,10 +19691,10 @@
       <c r="V6" s="7"/>
       <c r="W6" s="7"/>
       <c r="X6" s="7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="Y6" s="7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="Z6" s="7"/>
       <c r="AA6" s="7"/>
@@ -19732,7 +19737,7 @@
       <c r="AW6" s="7"/>
       <c r="AX6" s="7"/>
       <c r="AY6" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AZ6" s="7"/>
       <c r="BA6" s="7"/>
@@ -19741,7 +19746,7 @@
       <c r="BD6" s="6"/>
       <c r="BE6" s="11"/>
       <c r="BF6" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="BG6" s="11"/>
       <c r="BH6" s="11"/>
@@ -19806,7 +19811,7 @@
         <v>172</v>
       </c>
       <c r="BF7" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="BG7" s="6" t="s">
         <v>173</v>
@@ -19860,7 +19865,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -20424,7 +20429,7 @@
       <c r="AP13" s="6"/>
       <c r="AQ13" s="6"/>
       <c r="AR13" s="35" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AT13" s="7"/>
       <c r="AU13" s="7"/>
@@ -20537,10 +20542,10 @@
       </c>
       <c r="W14" s="7"/>
       <c r="X14" s="7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="Y14" s="7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="Z14" s="7"/>
       <c r="AA14" s="7"/>
@@ -20819,7 +20824,7 @@
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>109</v>
@@ -21291,7 +21296,7 @@
       <c r="AP21" s="6"/>
       <c r="AQ21" s="6"/>
       <c r="AR21" s="35" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AT21" s="7"/>
       <c r="AU21" s="7"/>
@@ -21400,10 +21405,10 @@
       </c>
       <c r="W22" s="7"/>
       <c r="X22" s="7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="Y22" s="7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="Z22" s="7"/>
       <c r="AA22" s="7"/>
@@ -22117,7 +22122,7 @@
       <c r="AP29" s="6"/>
       <c r="AQ29" s="6"/>
       <c r="AR29" s="35" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AT29" s="7"/>
       <c r="AU29" s="7"/>
@@ -22214,10 +22219,10 @@
       </c>
       <c r="W30" s="7"/>
       <c r="X30" s="7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="Y30" s="7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="Z30" s="7"/>
       <c r="AA30" s="7"/>
@@ -22284,7 +22289,7 @@
       </c>
       <c r="BP30" s="7"/>
       <c r="BQ30" s="7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="BR30" s="7"/>
       <c r="BS30" s="7"/>
@@ -22896,7 +22901,7 @@
       <c r="AP37" s="6"/>
       <c r="AQ37" s="6"/>
       <c r="AR37" s="35" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AT37" s="7" t="s">
         <v>35</v>
@@ -22979,10 +22984,10 @@
       </c>
       <c r="W38" s="7"/>
       <c r="X38" s="7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="Y38" s="7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="Z38" s="7"/>
       <c r="AA38" s="7"/>
@@ -24338,7 +24343,7 @@
       <c r="N5" s="6"/>
       <c r="O5" s="6"/>
       <c r="P5" s="35" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="R5" s="7"/>
       <c r="S5" s="7"/>
@@ -24469,7 +24474,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -24733,7 +24738,7 @@
       <c r="N13" s="6"/>
       <c r="O13" s="6"/>
       <c r="P13" s="35" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="R13" s="7"/>
       <c r="S13" s="13"/>
@@ -24942,7 +24947,7 @@
       <c r="N19" s="6"/>
       <c r="O19" s="6"/>
       <c r="P19" s="38" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="R19" s="7"/>
       <c r="S19" s="7"/>

</xml_diff>

<commit_message>
[Update] Layout images are changed.
</commit_message>
<xml_diff>
--- a/img/keymap.xlsx
+++ b/img/keymap.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2340" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2340" uniqueCount="213">
   <si>
     <t xml:space="preserve">標準</t>
   </si>
@@ -587,18 +587,14 @@
     <t xml:space="preserve">sShift</t>
   </si>
   <si>
-    <t xml:space="preserve">SelCur
-Togle</t>
+    <t xml:space="preserve">Select
+Mode</t>
   </si>
   <si>
     <t xml:space="preserve">F14修飾</t>
   </si>
   <si>
     <t xml:space="preserve">SC+p</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Select
-Mode</t>
   </si>
   <si>
     <t xml:space="preserve">C+Space</t>
@@ -963,7 +959,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="42">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1078,10 +1074,6 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -9674,11 +9666,11 @@
       </c>
       <c r="M19" s="13"/>
       <c r="N19" s="13"/>
-      <c r="O19" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="P19" s="30"/>
-      <c r="Q19" s="30"/>
+      <c r="O19" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="P19" s="29"/>
+      <c r="Q19" s="29"/>
       <c r="R19" s="13" t="s">
         <v>138</v>
       </c>
@@ -9704,16 +9696,16 @@
       </c>
       <c r="AE19" s="13"/>
       <c r="AF19" s="13"/>
-      <c r="AG19" s="31" t="s">
+      <c r="AG19" s="30" t="s">
         <v>145</v>
       </c>
-      <c r="AH19" s="31"/>
-      <c r="AI19" s="31"/>
-      <c r="AJ19" s="31" t="s">
+      <c r="AH19" s="30"/>
+      <c r="AI19" s="30"/>
+      <c r="AJ19" s="30" t="s">
         <v>146</v>
       </c>
-      <c r="AK19" s="31"/>
-      <c r="AL19" s="31"/>
+      <c r="AK19" s="30"/>
+      <c r="AL19" s="30"/>
       <c r="AM19" s="6"/>
       <c r="AN19" s="6"/>
       <c r="AO19" s="6"/>
@@ -9807,11 +9799,11 @@
       </c>
       <c r="N20" s="20"/>
       <c r="O20" s="20"/>
-      <c r="P20" s="31" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q20" s="31"/>
-      <c r="R20" s="31"/>
+      <c r="P20" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q20" s="30"/>
+      <c r="R20" s="30"/>
       <c r="S20" s="6" t="s">
         <v>151</v>
       </c>
@@ -9865,11 +9857,11 @@
       </c>
       <c r="BC20" s="13"/>
       <c r="BD20" s="13"/>
-      <c r="BE20" s="32" t="s">
-        <v>192</v>
-      </c>
-      <c r="BF20" s="32"/>
-      <c r="BG20" s="32"/>
+      <c r="BE20" s="31" t="s">
+        <v>191</v>
+      </c>
+      <c r="BF20" s="31"/>
+      <c r="BG20" s="31"/>
       <c r="BH20" s="7"/>
       <c r="BI20" s="7"/>
       <c r="BJ20" s="7"/>
@@ -10493,11 +10485,11 @@
       </c>
       <c r="M27" s="13"/>
       <c r="N27" s="13"/>
-      <c r="O27" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="P27" s="30"/>
-      <c r="Q27" s="30"/>
+      <c r="O27" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="P27" s="29"/>
+      <c r="Q27" s="29"/>
       <c r="R27" s="13" t="s">
         <v>138</v>
       </c>
@@ -10523,16 +10515,16 @@
       </c>
       <c r="AE27" s="13"/>
       <c r="AF27" s="13"/>
-      <c r="AG27" s="31" t="s">
+      <c r="AG27" s="30" t="s">
         <v>145</v>
       </c>
-      <c r="AH27" s="31"/>
-      <c r="AI27" s="31"/>
-      <c r="AJ27" s="31" t="s">
+      <c r="AH27" s="30"/>
+      <c r="AI27" s="30"/>
+      <c r="AJ27" s="30" t="s">
         <v>146</v>
       </c>
-      <c r="AK27" s="31"/>
-      <c r="AL27" s="31"/>
+      <c r="AK27" s="30"/>
+      <c r="AL27" s="30"/>
       <c r="AM27" s="6"/>
       <c r="AN27" s="6"/>
       <c r="AO27" s="6"/>
@@ -10616,11 +10608,11 @@
       </c>
       <c r="N28" s="20"/>
       <c r="O28" s="20"/>
-      <c r="P28" s="31" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q28" s="31"/>
-      <c r="R28" s="31"/>
+      <c r="P28" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q28" s="30"/>
+      <c r="R28" s="30"/>
       <c r="S28" s="6" t="s">
         <v>151</v>
       </c>
@@ -10660,11 +10652,11 @@
       <c r="AO28" s="9"/>
       <c r="AP28" s="9"/>
       <c r="AQ28" s="9"/>
-      <c r="AS28" s="33" t="s">
-        <v>193</v>
-      </c>
-      <c r="AT28" s="33"/>
-      <c r="AU28" s="33"/>
+      <c r="AS28" s="32" t="s">
+        <v>192</v>
+      </c>
+      <c r="AT28" s="32"/>
+      <c r="AU28" s="32"/>
       <c r="AV28" s="7"/>
       <c r="AW28" s="7"/>
       <c r="AX28" s="7"/>
@@ -10907,27 +10899,27 @@
       <c r="BC30" s="7"/>
       <c r="BD30" s="7"/>
       <c r="BE30" s="7"/>
-      <c r="BF30" s="33" t="s">
-        <v>193</v>
-      </c>
-      <c r="BG30" s="33"/>
-      <c r="BH30" s="33"/>
-      <c r="BI30" s="33"/>
-      <c r="BJ30" s="33"/>
-      <c r="BK30" s="33"/>
-      <c r="BL30" s="33"/>
-      <c r="BM30" s="33"/>
-      <c r="BN30" s="33"/>
-      <c r="BO30" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="BP30" s="30"/>
-      <c r="BQ30" s="30"/>
-      <c r="BR30" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="BS30" s="30"/>
-      <c r="BT30" s="30"/>
+      <c r="BF30" s="32" t="s">
+        <v>192</v>
+      </c>
+      <c r="BG30" s="32"/>
+      <c r="BH30" s="32"/>
+      <c r="BI30" s="32"/>
+      <c r="BJ30" s="32"/>
+      <c r="BK30" s="32"/>
+      <c r="BL30" s="32"/>
+      <c r="BM30" s="32"/>
+      <c r="BN30" s="32"/>
+      <c r="BO30" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="BP30" s="29"/>
+      <c r="BQ30" s="29"/>
+      <c r="BR30" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="BS30" s="29"/>
+      <c r="BT30" s="29"/>
       <c r="BU30" s="7"/>
       <c r="BV30" s="7"/>
       <c r="BW30" s="7"/>
@@ -11003,21 +10995,21 @@
       <c r="BC31" s="7"/>
       <c r="BD31" s="7"/>
       <c r="BE31" s="7"/>
-      <c r="BF31" s="33"/>
-      <c r="BG31" s="33"/>
-      <c r="BH31" s="33"/>
-      <c r="BI31" s="33"/>
-      <c r="BJ31" s="33"/>
-      <c r="BK31" s="33"/>
-      <c r="BL31" s="33"/>
-      <c r="BM31" s="33"/>
-      <c r="BN31" s="33"/>
-      <c r="BO31" s="30"/>
-      <c r="BP31" s="30"/>
-      <c r="BQ31" s="30"/>
-      <c r="BR31" s="30"/>
-      <c r="BS31" s="30"/>
-      <c r="BT31" s="30"/>
+      <c r="BF31" s="32"/>
+      <c r="BG31" s="32"/>
+      <c r="BH31" s="32"/>
+      <c r="BI31" s="32"/>
+      <c r="BJ31" s="32"/>
+      <c r="BK31" s="32"/>
+      <c r="BL31" s="32"/>
+      <c r="BM31" s="32"/>
+      <c r="BN31" s="32"/>
+      <c r="BO31" s="29"/>
+      <c r="BP31" s="29"/>
+      <c r="BQ31" s="29"/>
+      <c r="BR31" s="29"/>
+      <c r="BS31" s="29"/>
+      <c r="BT31" s="29"/>
       <c r="BU31" s="7"/>
       <c r="BV31" s="7"/>
       <c r="BW31" s="7"/>
@@ -11134,7 +11126,7 @@
       <c r="AP33" s="4"/>
       <c r="AQ33" s="5"/>
       <c r="AS33" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT33" s="5"/>
       <c r="AU33" s="4"/>
@@ -11300,11 +11292,11 @@
       </c>
       <c r="M35" s="13"/>
       <c r="N35" s="13"/>
-      <c r="O35" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="P35" s="30"/>
-      <c r="Q35" s="30"/>
+      <c r="O35" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="P35" s="29"/>
+      <c r="Q35" s="29"/>
       <c r="R35" s="13" t="s">
         <v>138</v>
       </c>
@@ -11330,16 +11322,16 @@
       </c>
       <c r="AE35" s="13"/>
       <c r="AF35" s="13"/>
-      <c r="AG35" s="31" t="s">
+      <c r="AG35" s="30" t="s">
         <v>145</v>
       </c>
-      <c r="AH35" s="31"/>
-      <c r="AI35" s="31"/>
-      <c r="AJ35" s="31" t="s">
+      <c r="AH35" s="30"/>
+      <c r="AI35" s="30"/>
+      <c r="AJ35" s="30" t="s">
         <v>146</v>
       </c>
-      <c r="AK35" s="31"/>
-      <c r="AL35" s="31"/>
+      <c r="AK35" s="30"/>
+      <c r="AL35" s="30"/>
       <c r="AM35" s="6"/>
       <c r="AN35" s="6"/>
       <c r="AO35" s="6"/>
@@ -11427,11 +11419,11 @@
       </c>
       <c r="N36" s="20"/>
       <c r="O36" s="20"/>
-      <c r="P36" s="31" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q36" s="31"/>
-      <c r="R36" s="31"/>
+      <c r="P36" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q36" s="30"/>
+      <c r="R36" s="30"/>
       <c r="S36" s="6" t="s">
         <v>151</v>
       </c>
@@ -11471,11 +11463,11 @@
       <c r="AO36" s="9"/>
       <c r="AP36" s="9"/>
       <c r="AQ36" s="9"/>
-      <c r="AS36" s="33" t="s">
-        <v>193</v>
-      </c>
-      <c r="AT36" s="33"/>
-      <c r="AU36" s="33"/>
+      <c r="AS36" s="32" t="s">
+        <v>192</v>
+      </c>
+      <c r="AT36" s="32"/>
+      <c r="AU36" s="32"/>
       <c r="AV36" s="7"/>
       <c r="AW36" s="7"/>
       <c r="AX36" s="7"/>
@@ -11672,7 +11664,7 @@
       <c r="L38" s="7"/>
       <c r="M38" s="7"/>
       <c r="N38" s="7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="O38" s="7"/>
       <c r="P38" s="7" t="s">
@@ -11728,27 +11720,27 @@
       <c r="BC38" s="7"/>
       <c r="BD38" s="7"/>
       <c r="BE38" s="7"/>
-      <c r="BF38" s="33" t="s">
-        <v>193</v>
-      </c>
-      <c r="BG38" s="33"/>
-      <c r="BH38" s="33"/>
-      <c r="BI38" s="33"/>
-      <c r="BJ38" s="33"/>
-      <c r="BK38" s="33"/>
-      <c r="BL38" s="33"/>
-      <c r="BM38" s="33"/>
-      <c r="BN38" s="33"/>
-      <c r="BO38" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="BP38" s="30"/>
-      <c r="BQ38" s="30"/>
-      <c r="BR38" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="BS38" s="30"/>
-      <c r="BT38" s="30"/>
+      <c r="BF38" s="32" t="s">
+        <v>192</v>
+      </c>
+      <c r="BG38" s="32"/>
+      <c r="BH38" s="32"/>
+      <c r="BI38" s="32"/>
+      <c r="BJ38" s="32"/>
+      <c r="BK38" s="32"/>
+      <c r="BL38" s="32"/>
+      <c r="BM38" s="32"/>
+      <c r="BN38" s="32"/>
+      <c r="BO38" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="BP38" s="29"/>
+      <c r="BQ38" s="29"/>
+      <c r="BR38" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="BS38" s="29"/>
+      <c r="BT38" s="29"/>
       <c r="BU38" s="7"/>
       <c r="BV38" s="7"/>
       <c r="BW38" s="7"/>
@@ -11822,21 +11814,21 @@
       <c r="BC39" s="7"/>
       <c r="BD39" s="7"/>
       <c r="BE39" s="7"/>
-      <c r="BF39" s="33"/>
-      <c r="BG39" s="33"/>
-      <c r="BH39" s="33"/>
-      <c r="BI39" s="33"/>
-      <c r="BJ39" s="33"/>
-      <c r="BK39" s="33"/>
-      <c r="BL39" s="33"/>
-      <c r="BM39" s="33"/>
-      <c r="BN39" s="33"/>
-      <c r="BO39" s="30"/>
-      <c r="BP39" s="30"/>
-      <c r="BQ39" s="30"/>
-      <c r="BR39" s="30"/>
-      <c r="BS39" s="30"/>
-      <c r="BT39" s="30"/>
+      <c r="BF39" s="32"/>
+      <c r="BG39" s="32"/>
+      <c r="BH39" s="32"/>
+      <c r="BI39" s="32"/>
+      <c r="BJ39" s="32"/>
+      <c r="BK39" s="32"/>
+      <c r="BL39" s="32"/>
+      <c r="BM39" s="32"/>
+      <c r="BN39" s="32"/>
+      <c r="BO39" s="29"/>
+      <c r="BP39" s="29"/>
+      <c r="BQ39" s="29"/>
+      <c r="BR39" s="29"/>
+      <c r="BS39" s="29"/>
+      <c r="BT39" s="29"/>
       <c r="BU39" s="7"/>
       <c r="BV39" s="7"/>
       <c r="BW39" s="7"/>
@@ -11897,7 +11889,7 @@
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B41" s="15"/>
       <c r="C41" s="15"/>
@@ -11942,7 +11934,7 @@
       <c r="AP41" s="4"/>
       <c r="AQ41" s="5"/>
       <c r="AS41" s="15" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AT41" s="15"/>
       <c r="AU41" s="4"/>
@@ -12064,11 +12056,11 @@
       </c>
       <c r="M43" s="13"/>
       <c r="N43" s="13"/>
-      <c r="O43" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="P43" s="30"/>
-      <c r="Q43" s="30"/>
+      <c r="O43" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="P43" s="29"/>
+      <c r="Q43" s="29"/>
       <c r="R43" s="13" t="s">
         <v>138</v>
       </c>
@@ -12094,16 +12086,16 @@
       </c>
       <c r="AE43" s="7"/>
       <c r="AF43" s="7"/>
-      <c r="AG43" s="31" t="s">
+      <c r="AG43" s="30" t="s">
         <v>145</v>
       </c>
-      <c r="AH43" s="31"/>
-      <c r="AI43" s="31"/>
-      <c r="AJ43" s="31" t="s">
+      <c r="AH43" s="30"/>
+      <c r="AI43" s="30"/>
+      <c r="AJ43" s="30" t="s">
         <v>146</v>
       </c>
-      <c r="AK43" s="31"/>
-      <c r="AL43" s="31"/>
+      <c r="AK43" s="30"/>
+      <c r="AL43" s="30"/>
       <c r="AM43" s="6"/>
       <c r="AN43" s="6"/>
       <c r="AO43" s="6"/>
@@ -12125,11 +12117,11 @@
       </c>
       <c r="BE43" s="13"/>
       <c r="BF43" s="13"/>
-      <c r="BG43" s="30" t="s">
-        <v>198</v>
-      </c>
-      <c r="BH43" s="30"/>
-      <c r="BI43" s="30"/>
+      <c r="BG43" s="29" t="s">
+        <v>197</v>
+      </c>
+      <c r="BH43" s="29"/>
+      <c r="BI43" s="29"/>
       <c r="BJ43" s="13" t="s">
         <v>138</v>
       </c>
@@ -12164,11 +12156,11 @@
       <c r="CI43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="33" t="s">
-        <v>193</v>
-      </c>
-      <c r="B44" s="33"/>
-      <c r="C44" s="33"/>
+      <c r="A44" s="32" t="s">
+        <v>192</v>
+      </c>
+      <c r="B44" s="32"/>
+      <c r="C44" s="32"/>
       <c r="D44" s="6"/>
       <c r="E44" s="6"/>
       <c r="F44" s="6"/>
@@ -12219,11 +12211,11 @@
       <c r="AO44" s="9"/>
       <c r="AP44" s="9"/>
       <c r="AQ44" s="9"/>
-      <c r="AS44" s="33" t="s">
-        <v>193</v>
-      </c>
-      <c r="AT44" s="33"/>
-      <c r="AU44" s="33"/>
+      <c r="AS44" s="32" t="s">
+        <v>192</v>
+      </c>
+      <c r="AT44" s="32"/>
+      <c r="AU44" s="32"/>
       <c r="AV44" s="6"/>
       <c r="AW44" s="6"/>
       <c r="AX44" s="6"/>
@@ -12342,16 +12334,16 @@
       </c>
       <c r="AX45" s="13"/>
       <c r="AY45" s="13"/>
-      <c r="AZ45" s="34" t="s">
+      <c r="AZ45" s="33" t="s">
+        <v>198</v>
+      </c>
+      <c r="BA45" s="33"/>
+      <c r="BB45" s="33"/>
+      <c r="BC45" s="33" t="s">
         <v>199</v>
       </c>
-      <c r="BA45" s="34"/>
-      <c r="BB45" s="34"/>
-      <c r="BC45" s="34" t="s">
-        <v>200</v>
-      </c>
-      <c r="BD45" s="34"/>
-      <c r="BE45" s="34"/>
+      <c r="BD45" s="33"/>
+      <c r="BE45" s="33"/>
       <c r="BF45" s="13" t="s">
         <v>157</v>
       </c>
@@ -12367,16 +12359,16 @@
       </c>
       <c r="BM45" s="10"/>
       <c r="BN45" s="10"/>
-      <c r="BO45" s="35" t="s">
+      <c r="BO45" s="34" t="s">
         <v>166</v>
       </c>
-      <c r="BP45" s="35"/>
-      <c r="BQ45" s="35"/>
-      <c r="BR45" s="35" t="s">
+      <c r="BP45" s="34"/>
+      <c r="BQ45" s="34"/>
+      <c r="BR45" s="34" t="s">
         <v>144</v>
       </c>
-      <c r="BS45" s="35"/>
-      <c r="BT45" s="35"/>
+      <c r="BS45" s="34"/>
+      <c r="BT45" s="34"/>
       <c r="BU45" s="6"/>
       <c r="BV45" s="6"/>
       <c r="BW45" s="6"/>
@@ -12407,27 +12399,27 @@
       <c r="K46" s="7"/>
       <c r="L46" s="7"/>
       <c r="M46" s="7"/>
-      <c r="N46" s="33" t="s">
-        <v>193</v>
-      </c>
-      <c r="O46" s="33"/>
-      <c r="P46" s="33"/>
-      <c r="Q46" s="33"/>
-      <c r="R46" s="33"/>
-      <c r="S46" s="33"/>
-      <c r="T46" s="33"/>
-      <c r="U46" s="33"/>
-      <c r="V46" s="33"/>
-      <c r="W46" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="X46" s="30"/>
-      <c r="Y46" s="30"/>
-      <c r="Z46" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="AA46" s="30"/>
-      <c r="AB46" s="30"/>
+      <c r="N46" s="32" t="s">
+        <v>192</v>
+      </c>
+      <c r="O46" s="32"/>
+      <c r="P46" s="32"/>
+      <c r="Q46" s="32"/>
+      <c r="R46" s="32"/>
+      <c r="S46" s="32"/>
+      <c r="T46" s="32"/>
+      <c r="U46" s="32"/>
+      <c r="V46" s="32"/>
+      <c r="W46" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="X46" s="29"/>
+      <c r="Y46" s="29"/>
+      <c r="Z46" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA46" s="29"/>
+      <c r="AB46" s="29"/>
       <c r="AC46" s="7"/>
       <c r="AD46" s="7"/>
       <c r="AE46" s="7"/>
@@ -12456,27 +12448,27 @@
       <c r="BC46" s="7"/>
       <c r="BD46" s="7"/>
       <c r="BE46" s="7"/>
-      <c r="BF46" s="33" t="s">
-        <v>193</v>
-      </c>
-      <c r="BG46" s="33"/>
-      <c r="BH46" s="33"/>
-      <c r="BI46" s="33"/>
-      <c r="BJ46" s="33"/>
-      <c r="BK46" s="33"/>
-      <c r="BL46" s="33"/>
-      <c r="BM46" s="33"/>
-      <c r="BN46" s="33"/>
-      <c r="BO46" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="BP46" s="30"/>
-      <c r="BQ46" s="30"/>
-      <c r="BR46" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="BS46" s="30"/>
-      <c r="BT46" s="30"/>
+      <c r="BF46" s="32" t="s">
+        <v>192</v>
+      </c>
+      <c r="BG46" s="32"/>
+      <c r="BH46" s="32"/>
+      <c r="BI46" s="32"/>
+      <c r="BJ46" s="32"/>
+      <c r="BK46" s="32"/>
+      <c r="BL46" s="32"/>
+      <c r="BM46" s="32"/>
+      <c r="BN46" s="32"/>
+      <c r="BO46" s="29" t="s">
+        <v>197</v>
+      </c>
+      <c r="BP46" s="29"/>
+      <c r="BQ46" s="29"/>
+      <c r="BR46" s="29" t="s">
+        <v>197</v>
+      </c>
+      <c r="BS46" s="29"/>
+      <c r="BT46" s="29"/>
       <c r="BU46" s="7"/>
       <c r="BV46" s="7"/>
       <c r="BW46" s="7"/>
@@ -12507,21 +12499,21 @@
       <c r="K47" s="7"/>
       <c r="L47" s="7"/>
       <c r="M47" s="7"/>
-      <c r="N47" s="33"/>
-      <c r="O47" s="33"/>
-      <c r="P47" s="33"/>
-      <c r="Q47" s="33"/>
-      <c r="R47" s="33"/>
-      <c r="S47" s="33"/>
-      <c r="T47" s="33"/>
-      <c r="U47" s="33"/>
-      <c r="V47" s="33"/>
-      <c r="W47" s="30"/>
-      <c r="X47" s="30"/>
-      <c r="Y47" s="30"/>
-      <c r="Z47" s="30"/>
-      <c r="AA47" s="30"/>
-      <c r="AB47" s="30"/>
+      <c r="N47" s="32"/>
+      <c r="O47" s="32"/>
+      <c r="P47" s="32"/>
+      <c r="Q47" s="32"/>
+      <c r="R47" s="32"/>
+      <c r="S47" s="32"/>
+      <c r="T47" s="32"/>
+      <c r="U47" s="32"/>
+      <c r="V47" s="32"/>
+      <c r="W47" s="29"/>
+      <c r="X47" s="29"/>
+      <c r="Y47" s="29"/>
+      <c r="Z47" s="29"/>
+      <c r="AA47" s="29"/>
+      <c r="AB47" s="29"/>
       <c r="AC47" s="7"/>
       <c r="AD47" s="7"/>
       <c r="AE47" s="7"/>
@@ -12550,21 +12542,21 @@
       <c r="BC47" s="7"/>
       <c r="BD47" s="7"/>
       <c r="BE47" s="7"/>
-      <c r="BF47" s="33"/>
-      <c r="BG47" s="33"/>
-      <c r="BH47" s="33"/>
-      <c r="BI47" s="33"/>
-      <c r="BJ47" s="33"/>
-      <c r="BK47" s="33"/>
-      <c r="BL47" s="33"/>
-      <c r="BM47" s="33"/>
-      <c r="BN47" s="33"/>
-      <c r="BO47" s="30"/>
-      <c r="BP47" s="30"/>
-      <c r="BQ47" s="30"/>
-      <c r="BR47" s="30"/>
-      <c r="BS47" s="30"/>
-      <c r="BT47" s="30"/>
+      <c r="BF47" s="32"/>
+      <c r="BG47" s="32"/>
+      <c r="BH47" s="32"/>
+      <c r="BI47" s="32"/>
+      <c r="BJ47" s="32"/>
+      <c r="BK47" s="32"/>
+      <c r="BL47" s="32"/>
+      <c r="BM47" s="32"/>
+      <c r="BN47" s="32"/>
+      <c r="BO47" s="29"/>
+      <c r="BP47" s="29"/>
+      <c r="BQ47" s="29"/>
+      <c r="BR47" s="29"/>
+      <c r="BS47" s="29"/>
+      <c r="BT47" s="29"/>
       <c r="BU47" s="7"/>
       <c r="BV47" s="7"/>
       <c r="BW47" s="7"/>
@@ -14973,7 +14965,7 @@
       <c r="BP10" s="13"/>
       <c r="BQ10" s="13"/>
       <c r="BR10" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="BS10" s="13"/>
       <c r="BT10" s="13"/>
@@ -15067,7 +15059,7 @@
       <c r="AK11" s="6"/>
       <c r="AL11" s="6"/>
       <c r="AM11" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AN11" s="6"/>
       <c r="AO11" s="6"/>
@@ -15736,7 +15728,7 @@
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>109</v>
@@ -15942,7 +15934,7 @@
       <c r="AK19" s="13"/>
       <c r="AL19" s="13"/>
       <c r="AM19" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AN19" s="6"/>
       <c r="AO19" s="6"/>
@@ -15997,7 +15989,7 @@
       <c r="CC19" s="7"/>
       <c r="CD19" s="7"/>
       <c r="CE19" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="CF19" s="6"/>
       <c r="CG19" s="6"/>
@@ -16778,7 +16770,7 @@
       <c r="AK27" s="13"/>
       <c r="AL27" s="13"/>
       <c r="AM27" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AN27" s="6"/>
       <c r="AO27" s="6"/>
@@ -16831,7 +16823,7 @@
       <c r="CC27" s="7"/>
       <c r="CD27" s="7"/>
       <c r="CE27" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="CF27" s="6"/>
       <c r="CG27" s="6"/>
@@ -17603,7 +17595,7 @@
       <c r="AK35" s="13"/>
       <c r="AL35" s="13"/>
       <c r="AM35" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AN35" s="6"/>
       <c r="AO35" s="6"/>
@@ -17660,7 +17652,7 @@
       <c r="CC35" s="7"/>
       <c r="CD35" s="7"/>
       <c r="CE35" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="CF35" s="6"/>
       <c r="CG35" s="6"/>
@@ -19214,7 +19206,7 @@
       <c r="AP1" s="4"/>
       <c r="AQ1" s="5"/>
       <c r="AT1" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AU1" s="4"/>
       <c r="AV1" s="4"/>
@@ -19497,7 +19489,7 @@
         <v>161</v>
       </c>
       <c r="AT4" s="7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AU4" s="7"/>
       <c r="AV4" s="7"/>
@@ -19505,7 +19497,7 @@
       <c r="AX4" s="8"/>
       <c r="AY4" s="6"/>
       <c r="AZ4" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="BA4" s="8" t="s">
         <v>56</v>
@@ -19594,8 +19586,8 @@
       <c r="AO5" s="6"/>
       <c r="AP5" s="6"/>
       <c r="AQ5" s="6"/>
-      <c r="AR5" s="36" t="s">
-        <v>207</v>
+      <c r="AR5" s="35" t="s">
+        <v>206</v>
       </c>
       <c r="AT5" s="7"/>
       <c r="AU5" s="7"/>
@@ -19604,7 +19596,7 @@
       <c r="AX5" s="7"/>
       <c r="AY5" s="7"/>
       <c r="AZ5" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="BA5" s="7" t="s">
         <v>172</v>
@@ -19664,10 +19656,10 @@
       <c r="V6" s="7"/>
       <c r="W6" s="7"/>
       <c r="X6" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Y6" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Z6" s="7"/>
       <c r="AA6" s="7"/>
@@ -19710,7 +19702,7 @@
       <c r="AW6" s="7"/>
       <c r="AX6" s="7"/>
       <c r="AY6" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="AZ6" s="7"/>
       <c r="BA6" s="7"/>
@@ -19719,7 +19711,7 @@
       <c r="BD6" s="6"/>
       <c r="BE6" s="11"/>
       <c r="BF6" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="BG6" s="11"/>
       <c r="BH6" s="11"/>
@@ -19784,7 +19776,7 @@
         <v>172</v>
       </c>
       <c r="BF7" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="BG7" s="6" t="s">
         <v>173</v>
@@ -19838,7 +19830,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -20401,8 +20393,8 @@
       <c r="AO13" s="6"/>
       <c r="AP13" s="6"/>
       <c r="AQ13" s="6"/>
-      <c r="AR13" s="36" t="s">
-        <v>207</v>
+      <c r="AR13" s="35" t="s">
+        <v>206</v>
       </c>
       <c r="AT13" s="7"/>
       <c r="AU13" s="7"/>
@@ -20515,10 +20507,10 @@
       </c>
       <c r="W14" s="7"/>
       <c r="X14" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Y14" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Z14" s="7"/>
       <c r="AA14" s="7"/>
@@ -20797,7 +20789,7 @@
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>109</v>
@@ -21268,8 +21260,8 @@
       <c r="AO21" s="6"/>
       <c r="AP21" s="6"/>
       <c r="AQ21" s="6"/>
-      <c r="AR21" s="36" t="s">
-        <v>207</v>
+      <c r="AR21" s="35" t="s">
+        <v>206</v>
       </c>
       <c r="AT21" s="7"/>
       <c r="AU21" s="7"/>
@@ -21378,10 +21370,10 @@
       </c>
       <c r="W22" s="7"/>
       <c r="X22" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Y22" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Z22" s="7"/>
       <c r="AA22" s="7"/>
@@ -22094,8 +22086,8 @@
       <c r="AO29" s="6"/>
       <c r="AP29" s="6"/>
       <c r="AQ29" s="6"/>
-      <c r="AR29" s="36" t="s">
-        <v>207</v>
+      <c r="AR29" s="35" t="s">
+        <v>206</v>
       </c>
       <c r="AT29" s="7"/>
       <c r="AU29" s="7"/>
@@ -22192,10 +22184,10 @@
       </c>
       <c r="W30" s="7"/>
       <c r="X30" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Y30" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Z30" s="7"/>
       <c r="AA30" s="7"/>
@@ -22262,7 +22254,7 @@
       </c>
       <c r="BP30" s="7"/>
       <c r="BQ30" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="BR30" s="7"/>
       <c r="BS30" s="7"/>
@@ -22767,7 +22759,7 @@
       <c r="AR36" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="AT36" s="37" t="s">
+      <c r="AT36" s="36" t="s">
         <v>34</v>
       </c>
       <c r="AU36" s="13" t="s">
@@ -22873,8 +22865,8 @@
       <c r="AO37" s="6"/>
       <c r="AP37" s="6"/>
       <c r="AQ37" s="6"/>
-      <c r="AR37" s="36" t="s">
-        <v>207</v>
+      <c r="AR37" s="35" t="s">
+        <v>206</v>
       </c>
       <c r="AT37" s="7" t="s">
         <v>35</v>
@@ -22957,10 +22949,10 @@
       </c>
       <c r="W38" s="7"/>
       <c r="X38" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Y38" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Z38" s="7"/>
       <c r="AA38" s="7"/>
@@ -22995,17 +22987,17 @@
       <c r="AW38" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="AX38" s="37" t="s">
+      <c r="AX38" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="AY38" s="37" t="s">
+      <c r="AY38" s="36" t="s">
         <v>52</v>
       </c>
-      <c r="AZ38" s="37"/>
-      <c r="BA38" s="37" t="s">
+      <c r="AZ38" s="36"/>
+      <c r="BA38" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="BB38" s="37" t="s">
+      <c r="BB38" s="36" t="s">
         <v>107</v>
       </c>
       <c r="BC38" s="11"/>
@@ -23068,9 +23060,9 @@
       <c r="AW39" s="7"/>
       <c r="AX39" s="7"/>
       <c r="AY39" s="7"/>
-      <c r="AZ39" s="37"/>
-      <c r="BA39" s="37"/>
-      <c r="BB39" s="37"/>
+      <c r="AZ39" s="36"/>
+      <c r="BA39" s="36"/>
+      <c r="BB39" s="36"/>
       <c r="BC39" s="11"/>
       <c r="BD39" s="6"/>
       <c r="BE39" s="6"/>
@@ -24315,8 +24307,8 @@
       </c>
       <c r="N5" s="6"/>
       <c r="O5" s="6"/>
-      <c r="P5" s="36" t="s">
-        <v>207</v>
+      <c r="P5" s="35" t="s">
+        <v>206</v>
       </c>
       <c r="R5" s="7"/>
       <c r="S5" s="7"/>
@@ -24447,7 +24439,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -24602,7 +24594,7 @@
       <c r="Z11" s="13"/>
       <c r="AA11" s="13"/>
       <c r="AB11" s="13"/>
-      <c r="AC11" s="38"/>
+      <c r="AC11" s="37"/>
       <c r="AD11" s="21"/>
       <c r="AE11" s="6"/>
       <c r="AF11" s="6"/>
@@ -24710,8 +24702,8 @@
       </c>
       <c r="N13" s="6"/>
       <c r="O13" s="6"/>
-      <c r="P13" s="36" t="s">
-        <v>207</v>
+      <c r="P13" s="35" t="s">
+        <v>206</v>
       </c>
       <c r="R13" s="7"/>
       <c r="S13" s="13"/>
@@ -24919,8 +24911,8 @@
       <c r="M19" s="13"/>
       <c r="N19" s="6"/>
       <c r="O19" s="6"/>
-      <c r="P19" s="39" t="s">
-        <v>213</v>
+      <c r="P19" s="38" t="s">
+        <v>212</v>
       </c>
       <c r="R19" s="7"/>
       <c r="S19" s="7"/>
@@ -24939,7 +24931,7 @@
       <c r="AF19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="37"/>
+      <c r="A20" s="36"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
@@ -25022,11 +25014,11 @@
       <c r="S22" s="7"/>
       <c r="T22" s="7"/>
       <c r="U22" s="7"/>
-      <c r="V22" s="37"/>
+      <c r="V22" s="36"/>
       <c r="W22" s="7"/>
       <c r="X22" s="7"/>
-      <c r="Y22" s="40"/>
-      <c r="Z22" s="40"/>
+      <c r="Y22" s="39"/>
+      <c r="Z22" s="39"/>
       <c r="AA22" s="11"/>
       <c r="AB22" s="6"/>
       <c r="AC22" s="11"/>
@@ -25054,11 +25046,11 @@
       <c r="S23" s="7"/>
       <c r="T23" s="7"/>
       <c r="U23" s="7"/>
-      <c r="V23" s="37"/>
-      <c r="W23" s="37"/>
+      <c r="V23" s="36"/>
+      <c r="W23" s="36"/>
       <c r="X23" s="7"/>
-      <c r="Y23" s="40"/>
-      <c r="Z23" s="40"/>
+      <c r="Y23" s="39"/>
+      <c r="Z23" s="39"/>
       <c r="AA23" s="11"/>
       <c r="AB23" s="6"/>
       <c r="AC23" s="6"/>
@@ -25195,7 +25187,7 @@
       <c r="M28" s="13"/>
       <c r="N28" s="6"/>
       <c r="O28" s="6"/>
-      <c r="R28" s="37"/>
+      <c r="R28" s="36"/>
       <c r="S28" s="7"/>
       <c r="T28" s="7"/>
       <c r="U28" s="7"/>
@@ -25249,8 +25241,8 @@
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
       <c r="E30" s="7"/>
-      <c r="F30" s="37"/>
-      <c r="G30" s="37"/>
+      <c r="F30" s="36"/>
+      <c r="G30" s="36"/>
       <c r="H30" s="7"/>
       <c r="I30" s="7"/>
       <c r="J30" s="11"/>
@@ -25263,9 +25255,9 @@
       <c r="S30" s="7"/>
       <c r="T30" s="7"/>
       <c r="U30" s="7"/>
-      <c r="V30" s="37"/>
-      <c r="W30" s="37"/>
-      <c r="X30" s="37"/>
+      <c r="V30" s="36"/>
+      <c r="W30" s="36"/>
+      <c r="X30" s="36"/>
       <c r="Y30" s="6"/>
       <c r="Z30" s="7"/>
       <c r="AA30" s="11"/>
@@ -25282,7 +25274,7 @@
       <c r="D31" s="7"/>
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
-      <c r="G31" s="37"/>
+      <c r="G31" s="36"/>
       <c r="H31" s="7"/>
       <c r="I31" s="7"/>
       <c r="J31" s="11"/>
@@ -25297,7 +25289,7 @@
       <c r="U31" s="7"/>
       <c r="V31" s="7"/>
       <c r="W31" s="7"/>
-      <c r="X31" s="37"/>
+      <c r="X31" s="36"/>
       <c r="Y31" s="6"/>
       <c r="Z31" s="7"/>
       <c r="AA31" s="11"/>
@@ -25360,7 +25352,7 @@
       <c r="A34" s="7"/>
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
-      <c r="D34" s="35"/>
+      <c r="D34" s="34"/>
       <c r="E34" s="6"/>
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
@@ -25436,7 +25428,7 @@
       <c r="M36" s="13"/>
       <c r="N36" s="6"/>
       <c r="O36" s="6"/>
-      <c r="R36" s="37"/>
+      <c r="R36" s="36"/>
       <c r="S36" s="13"/>
       <c r="T36" s="13"/>
       <c r="U36" s="13"/>
@@ -25475,7 +25467,7 @@
       <c r="V37" s="13"/>
       <c r="W37" s="13"/>
       <c r="X37" s="18"/>
-      <c r="Y37" s="41"/>
+      <c r="Y37" s="40"/>
       <c r="Z37" s="6"/>
       <c r="AA37" s="6"/>
       <c r="AB37" s="6"/>
@@ -25490,8 +25482,8 @@
       <c r="C38" s="7"/>
       <c r="D38" s="7"/>
       <c r="E38" s="7"/>
-      <c r="F38" s="37"/>
-      <c r="G38" s="37"/>
+      <c r="F38" s="36"/>
+      <c r="G38" s="36"/>
       <c r="H38" s="7"/>
       <c r="I38" s="7"/>
       <c r="J38" s="11"/>
@@ -25504,11 +25496,11 @@
       <c r="S38" s="7"/>
       <c r="T38" s="7"/>
       <c r="U38" s="7"/>
-      <c r="V38" s="37"/>
-      <c r="W38" s="37"/>
-      <c r="X38" s="37"/>
-      <c r="Y38" s="37"/>
-      <c r="Z38" s="37"/>
+      <c r="V38" s="36"/>
+      <c r="W38" s="36"/>
+      <c r="X38" s="36"/>
+      <c r="Y38" s="36"/>
+      <c r="Z38" s="36"/>
       <c r="AA38" s="11"/>
       <c r="AB38" s="6"/>
       <c r="AC38" s="11"/>
@@ -25523,7 +25515,7 @@
       <c r="D39" s="7"/>
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
-      <c r="G39" s="37"/>
+      <c r="G39" s="36"/>
       <c r="H39" s="7"/>
       <c r="I39" s="7"/>
       <c r="J39" s="11"/>
@@ -25538,9 +25530,9 @@
       <c r="U39" s="7"/>
       <c r="V39" s="7"/>
       <c r="W39" s="7"/>
-      <c r="X39" s="37"/>
-      <c r="Y39" s="37"/>
-      <c r="Z39" s="37"/>
+      <c r="X39" s="36"/>
+      <c r="Y39" s="36"/>
+      <c r="Z39" s="36"/>
       <c r="AA39" s="11"/>
       <c r="AB39" s="6"/>
       <c r="AC39" s="6"/>
@@ -25661,7 +25653,7 @@
       <c r="AF43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="37"/>
+      <c r="A44" s="36"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
@@ -25676,7 +25668,7 @@
       <c r="M44" s="6"/>
       <c r="N44" s="6"/>
       <c r="O44" s="6"/>
-      <c r="R44" s="37"/>
+      <c r="R44" s="36"/>
       <c r="S44" s="13"/>
       <c r="T44" s="13"/>
       <c r="U44" s="13"/>
@@ -25730,8 +25722,8 @@
       <c r="C46" s="7"/>
       <c r="D46" s="7"/>
       <c r="E46" s="7"/>
-      <c r="F46" s="37"/>
-      <c r="G46" s="37"/>
+      <c r="F46" s="36"/>
+      <c r="G46" s="36"/>
       <c r="H46" s="6"/>
       <c r="I46" s="7"/>
       <c r="J46" s="11"/>
@@ -25744,11 +25736,11 @@
       <c r="S46" s="7"/>
       <c r="T46" s="7"/>
       <c r="U46" s="7"/>
-      <c r="V46" s="37"/>
-      <c r="W46" s="37"/>
-      <c r="X46" s="37"/>
-      <c r="Y46" s="37"/>
-      <c r="Z46" s="37"/>
+      <c r="V46" s="36"/>
+      <c r="W46" s="36"/>
+      <c r="X46" s="36"/>
+      <c r="Y46" s="36"/>
+      <c r="Z46" s="36"/>
       <c r="AA46" s="11"/>
       <c r="AB46" s="6"/>
       <c r="AC46" s="11"/>
@@ -25763,7 +25755,7 @@
       <c r="D47" s="7"/>
       <c r="E47" s="7"/>
       <c r="F47" s="7"/>
-      <c r="G47" s="37"/>
+      <c r="G47" s="36"/>
       <c r="H47" s="6"/>
       <c r="I47" s="7"/>
       <c r="J47" s="11"/>
@@ -25778,9 +25770,9 @@
       <c r="U47" s="7"/>
       <c r="V47" s="7"/>
       <c r="W47" s="7"/>
-      <c r="X47" s="37"/>
-      <c r="Y47" s="37"/>
-      <c r="Z47" s="37"/>
+      <c r="X47" s="36"/>
+      <c r="Y47" s="36"/>
+      <c r="Z47" s="36"/>
       <c r="AA47" s="11"/>
       <c r="AB47" s="6"/>
       <c r="AC47" s="6"/>
@@ -25908,7 +25900,7 @@
       <c r="S52" s="7"/>
       <c r="T52" s="7"/>
       <c r="U52" s="7"/>
-      <c r="V52" s="42"/>
+      <c r="V52" s="41"/>
       <c r="W52" s="6"/>
       <c r="X52" s="13"/>
       <c r="Y52" s="14"/>
@@ -25957,11 +25949,11 @@
       <c r="B54" s="7"/>
       <c r="C54" s="7"/>
       <c r="D54" s="7"/>
-      <c r="E54" s="37"/>
+      <c r="E54" s="36"/>
       <c r="F54" s="7"/>
       <c r="G54" s="7"/>
-      <c r="H54" s="40"/>
-      <c r="I54" s="40"/>
+      <c r="H54" s="39"/>
+      <c r="I54" s="39"/>
       <c r="J54" s="11"/>
       <c r="K54" s="6"/>
       <c r="L54" s="11"/>
@@ -25989,11 +25981,11 @@
       <c r="B55" s="7"/>
       <c r="C55" s="7"/>
       <c r="D55" s="7"/>
-      <c r="E55" s="37"/>
-      <c r="F55" s="37"/>
+      <c r="E55" s="36"/>
+      <c r="F55" s="36"/>
       <c r="G55" s="7"/>
-      <c r="H55" s="40"/>
-      <c r="I55" s="40"/>
+      <c r="H55" s="39"/>
+      <c r="I55" s="39"/>
       <c r="J55" s="11"/>
       <c r="K55" s="6"/>
       <c r="L55" s="6"/>

</xml_diff>

<commit_message>
[Update] Key layout images are updated.
</commit_message>
<xml_diff>
--- a/img/keymap.xlsx
+++ b/img/keymap.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2340" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2329" uniqueCount="211">
   <si>
     <t xml:space="preserve">標準</t>
   </si>
@@ -603,14 +603,7 @@
     <t xml:space="preserve">S+Tab</t>
   </si>
   <si>
-    <t xml:space="preserve">Standard
-Mode</t>
-  </si>
-  <si>
     <t xml:space="preserve">10Key Mode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Backspace</t>
   </si>
   <si>
     <t xml:space="preserve">Cursor Mode</t>
@@ -959,7 +952,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1085,10 +1078,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9774,9 +9763,7 @@
       <c r="CI19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
-        <v>34</v>
-      </c>
+      <c r="A20" s="7"/>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
       <c r="D20" s="13" t="s">
@@ -10050,7 +10037,9 @@
       </c>
       <c r="I22" s="7"/>
       <c r="J22" s="7"/>
-      <c r="K22" s="7"/>
+      <c r="K22" s="7" t="s">
+        <v>2</v>
+      </c>
       <c r="L22" s="7"/>
       <c r="M22" s="7"/>
       <c r="N22" s="7" t="s">
@@ -10583,9 +10572,7 @@
       <c r="CI27" s="7"/>
     </row>
     <row r="28" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
-        <v>34</v>
-      </c>
+      <c r="A28" s="7"/>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
       <c r="D28" s="13" t="s">
@@ -10652,11 +10639,9 @@
       <c r="AO28" s="9"/>
       <c r="AP28" s="9"/>
       <c r="AQ28" s="9"/>
-      <c r="AS28" s="32" t="s">
-        <v>192</v>
-      </c>
-      <c r="AT28" s="32"/>
-      <c r="AU28" s="32"/>
+      <c r="AS28" s="7"/>
+      <c r="AT28" s="7"/>
+      <c r="AU28" s="7"/>
       <c r="AV28" s="7"/>
       <c r="AW28" s="7"/>
       <c r="AX28" s="7"/>
@@ -10839,12 +10824,12 @@
       </c>
       <c r="I30" s="7"/>
       <c r="J30" s="7"/>
-      <c r="K30" s="7"/>
+      <c r="K30" s="7" t="s">
+        <v>2</v>
+      </c>
       <c r="L30" s="7"/>
       <c r="M30" s="7"/>
-      <c r="N30" s="7" t="s">
-        <v>52</v>
-      </c>
+      <c r="N30" s="7"/>
       <c r="O30" s="7"/>
       <c r="P30" s="7" t="s">
         <v>52</v>
@@ -10899,17 +10884,15 @@
       <c r="BC30" s="7"/>
       <c r="BD30" s="7"/>
       <c r="BE30" s="7"/>
-      <c r="BF30" s="32" t="s">
-        <v>192</v>
-      </c>
-      <c r="BG30" s="32"/>
-      <c r="BH30" s="32"/>
-      <c r="BI30" s="32"/>
-      <c r="BJ30" s="32"/>
-      <c r="BK30" s="32"/>
-      <c r="BL30" s="32"/>
-      <c r="BM30" s="32"/>
-      <c r="BN30" s="32"/>
+      <c r="BF30" s="7"/>
+      <c r="BG30" s="7"/>
+      <c r="BH30" s="7"/>
+      <c r="BI30" s="7"/>
+      <c r="BJ30" s="7"/>
+      <c r="BK30" s="7"/>
+      <c r="BL30" s="7"/>
+      <c r="BM30" s="7"/>
+      <c r="BN30" s="7"/>
       <c r="BO30" s="29" t="s">
         <v>187</v>
       </c>
@@ -10995,15 +10978,15 @@
       <c r="BC31" s="7"/>
       <c r="BD31" s="7"/>
       <c r="BE31" s="7"/>
-      <c r="BF31" s="32"/>
-      <c r="BG31" s="32"/>
-      <c r="BH31" s="32"/>
-      <c r="BI31" s="32"/>
-      <c r="BJ31" s="32"/>
-      <c r="BK31" s="32"/>
-      <c r="BL31" s="32"/>
-      <c r="BM31" s="32"/>
-      <c r="BN31" s="32"/>
+      <c r="BF31" s="7"/>
+      <c r="BG31" s="7"/>
+      <c r="BH31" s="7"/>
+      <c r="BI31" s="7"/>
+      <c r="BJ31" s="7"/>
+      <c r="BK31" s="7"/>
+      <c r="BL31" s="7"/>
+      <c r="BM31" s="7"/>
+      <c r="BN31" s="7"/>
       <c r="BO31" s="29"/>
       <c r="BP31" s="29"/>
       <c r="BQ31" s="29"/>
@@ -11080,9 +11063,7 @@
       <c r="AT32" s="12"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
-        <v>34</v>
-      </c>
+      <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
       <c r="D33" s="15"/>
@@ -11126,7 +11107,7 @@
       <c r="AP33" s="4"/>
       <c r="AQ33" s="5"/>
       <c r="AS33" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AT33" s="5"/>
       <c r="AU33" s="4"/>
@@ -11394,9 +11375,7 @@
       <c r="CI35" s="7"/>
     </row>
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7" t="s">
-        <v>34</v>
-      </c>
+      <c r="A36" s="7"/>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="13" t="s">
@@ -11463,11 +11442,9 @@
       <c r="AO36" s="9"/>
       <c r="AP36" s="9"/>
       <c r="AQ36" s="9"/>
-      <c r="AS36" s="32" t="s">
-        <v>192</v>
-      </c>
-      <c r="AT36" s="32"/>
-      <c r="AU36" s="32"/>
+      <c r="AS36" s="7"/>
+      <c r="AT36" s="7"/>
+      <c r="AU36" s="7"/>
       <c r="AV36" s="7"/>
       <c r="AW36" s="7"/>
       <c r="AX36" s="7"/>
@@ -11660,12 +11637,12 @@
       </c>
       <c r="I38" s="7"/>
       <c r="J38" s="7"/>
-      <c r="K38" s="7"/>
+      <c r="K38" s="7" t="s">
+        <v>2</v>
+      </c>
       <c r="L38" s="7"/>
       <c r="M38" s="7"/>
-      <c r="N38" s="7" t="s">
-        <v>194</v>
-      </c>
+      <c r="N38" s="7"/>
       <c r="O38" s="7"/>
       <c r="P38" s="7" t="s">
         <v>52</v>
@@ -11720,17 +11697,15 @@
       <c r="BC38" s="7"/>
       <c r="BD38" s="7"/>
       <c r="BE38" s="7"/>
-      <c r="BF38" s="32" t="s">
-        <v>192</v>
-      </c>
-      <c r="BG38" s="32"/>
-      <c r="BH38" s="32"/>
-      <c r="BI38" s="32"/>
-      <c r="BJ38" s="32"/>
-      <c r="BK38" s="32"/>
-      <c r="BL38" s="32"/>
-      <c r="BM38" s="32"/>
-      <c r="BN38" s="32"/>
+      <c r="BF38" s="7"/>
+      <c r="BG38" s="7"/>
+      <c r="BH38" s="7"/>
+      <c r="BI38" s="7"/>
+      <c r="BJ38" s="7"/>
+      <c r="BK38" s="7"/>
+      <c r="BL38" s="7"/>
+      <c r="BM38" s="7"/>
+      <c r="BN38" s="7"/>
       <c r="BO38" s="29" t="s">
         <v>187</v>
       </c>
@@ -11814,15 +11789,15 @@
       <c r="BC39" s="7"/>
       <c r="BD39" s="7"/>
       <c r="BE39" s="7"/>
-      <c r="BF39" s="32"/>
-      <c r="BG39" s="32"/>
-      <c r="BH39" s="32"/>
-      <c r="BI39" s="32"/>
-      <c r="BJ39" s="32"/>
-      <c r="BK39" s="32"/>
-      <c r="BL39" s="32"/>
-      <c r="BM39" s="32"/>
-      <c r="BN39" s="32"/>
+      <c r="BF39" s="7"/>
+      <c r="BG39" s="7"/>
+      <c r="BH39" s="7"/>
+      <c r="BI39" s="7"/>
+      <c r="BJ39" s="7"/>
+      <c r="BK39" s="7"/>
+      <c r="BL39" s="7"/>
+      <c r="BM39" s="7"/>
+      <c r="BN39" s="7"/>
       <c r="BO39" s="29"/>
       <c r="BP39" s="29"/>
       <c r="BQ39" s="29"/>
@@ -11846,50 +11821,53 @@
       <c r="CI39" s="24"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D40" s="26"/>
-      <c r="E40" s="26"/>
-      <c r="F40" s="26"/>
-      <c r="G40" s="27"/>
-      <c r="H40" s="27"/>
-      <c r="I40" s="27"/>
-      <c r="J40" s="27"/>
-      <c r="K40" s="27"/>
-      <c r="L40" s="27"/>
-      <c r="M40" s="27"/>
-      <c r="N40" s="27"/>
-      <c r="O40" s="27"/>
-      <c r="P40" s="27"/>
-      <c r="Q40" s="27"/>
-      <c r="R40" s="27"/>
-      <c r="S40" s="27"/>
-      <c r="T40" s="27"/>
-      <c r="U40" s="27"/>
-      <c r="V40" s="27"/>
-      <c r="W40" s="27"/>
-      <c r="X40" s="27"/>
-      <c r="Y40" s="27"/>
-      <c r="Z40" s="27"/>
-      <c r="AA40" s="27"/>
-      <c r="AB40" s="27"/>
-      <c r="AC40" s="27"/>
-      <c r="AD40" s="27"/>
-      <c r="AE40" s="27"/>
-      <c r="AF40" s="27"/>
-      <c r="AG40" s="27"/>
-      <c r="AH40" s="27"/>
-      <c r="AI40" s="27"/>
-      <c r="AJ40" s="27"/>
-      <c r="AK40" s="27"/>
-      <c r="AL40" s="27"/>
-      <c r="AM40" s="27"/>
-      <c r="AN40" s="27"/>
-      <c r="AO40" s="27"/>
-      <c r="AP40" s="27"/>
-      <c r="AQ40" s="28"/>
+      <c r="A40" s="12"/>
+      <c r="B40" s="12"/>
+      <c r="C40" s="12"/>
+      <c r="D40" s="12"/>
+      <c r="E40" s="12"/>
+      <c r="F40" s="12"/>
+      <c r="G40" s="12"/>
+      <c r="H40" s="12"/>
+      <c r="I40" s="12"/>
+      <c r="J40" s="12"/>
+      <c r="K40" s="12"/>
+      <c r="L40" s="12"/>
+      <c r="M40" s="12"/>
+      <c r="N40" s="12"/>
+      <c r="O40" s="12"/>
+      <c r="P40" s="12"/>
+      <c r="Q40" s="12"/>
+      <c r="R40" s="12"/>
+      <c r="S40" s="12"/>
+      <c r="T40" s="12"/>
+      <c r="U40" s="12"/>
+      <c r="V40" s="12"/>
+      <c r="W40" s="12"/>
+      <c r="X40" s="12"/>
+      <c r="Y40" s="12"/>
+      <c r="Z40" s="12"/>
+      <c r="AA40" s="12"/>
+      <c r="AB40" s="12"/>
+      <c r="AC40" s="12"/>
+      <c r="AD40" s="12"/>
+      <c r="AE40" s="12"/>
+      <c r="AF40" s="12"/>
+      <c r="AG40" s="12"/>
+      <c r="AH40" s="12"/>
+      <c r="AI40" s="12"/>
+      <c r="AJ40" s="12"/>
+      <c r="AK40" s="12"/>
+      <c r="AL40" s="12"/>
+      <c r="AM40" s="12"/>
+      <c r="AN40" s="12"/>
+      <c r="AO40" s="12"/>
+      <c r="AP40" s="12"/>
+      <c r="AQ40" s="12"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B41" s="15"/>
       <c r="C41" s="15"/>
@@ -11934,7 +11912,7 @@
       <c r="AP41" s="4"/>
       <c r="AQ41" s="5"/>
       <c r="AS41" s="15" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="AT41" s="15"/>
       <c r="AU41" s="4"/>
@@ -12118,7 +12096,7 @@
       <c r="BE43" s="13"/>
       <c r="BF43" s="13"/>
       <c r="BG43" s="29" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="BH43" s="29"/>
       <c r="BI43" s="29"/>
@@ -12156,11 +12134,9 @@
       <c r="CI43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="32" t="s">
-        <v>192</v>
-      </c>
-      <c r="B44" s="32"/>
-      <c r="C44" s="32"/>
+      <c r="A44" s="7"/>
+      <c r="B44" s="7"/>
+      <c r="C44" s="7"/>
       <c r="D44" s="6"/>
       <c r="E44" s="6"/>
       <c r="F44" s="6"/>
@@ -12211,11 +12187,9 @@
       <c r="AO44" s="9"/>
       <c r="AP44" s="9"/>
       <c r="AQ44" s="9"/>
-      <c r="AS44" s="32" t="s">
-        <v>192</v>
-      </c>
-      <c r="AT44" s="32"/>
-      <c r="AU44" s="32"/>
+      <c r="AS44" s="7"/>
+      <c r="AT44" s="7"/>
+      <c r="AU44" s="7"/>
       <c r="AV44" s="6"/>
       <c r="AW44" s="6"/>
       <c r="AX44" s="6"/>
@@ -12334,16 +12308,16 @@
       </c>
       <c r="AX45" s="13"/>
       <c r="AY45" s="13"/>
-      <c r="AZ45" s="33" t="s">
-        <v>198</v>
-      </c>
-      <c r="BA45" s="33"/>
-      <c r="BB45" s="33"/>
-      <c r="BC45" s="33" t="s">
-        <v>199</v>
-      </c>
-      <c r="BD45" s="33"/>
-      <c r="BE45" s="33"/>
+      <c r="AZ45" s="32" t="s">
+        <v>196</v>
+      </c>
+      <c r="BA45" s="32"/>
+      <c r="BB45" s="32"/>
+      <c r="BC45" s="32" t="s">
+        <v>197</v>
+      </c>
+      <c r="BD45" s="32"/>
+      <c r="BE45" s="32"/>
       <c r="BF45" s="13" t="s">
         <v>157</v>
       </c>
@@ -12359,16 +12333,16 @@
       </c>
       <c r="BM45" s="10"/>
       <c r="BN45" s="10"/>
-      <c r="BO45" s="34" t="s">
+      <c r="BO45" s="33" t="s">
         <v>166</v>
       </c>
-      <c r="BP45" s="34"/>
-      <c r="BQ45" s="34"/>
-      <c r="BR45" s="34" t="s">
+      <c r="BP45" s="33"/>
+      <c r="BQ45" s="33"/>
+      <c r="BR45" s="33" t="s">
         <v>144</v>
       </c>
-      <c r="BS45" s="34"/>
-      <c r="BT45" s="34"/>
+      <c r="BS45" s="33"/>
+      <c r="BT45" s="33"/>
       <c r="BU45" s="6"/>
       <c r="BV45" s="6"/>
       <c r="BW45" s="6"/>
@@ -12399,17 +12373,15 @@
       <c r="K46" s="7"/>
       <c r="L46" s="7"/>
       <c r="M46" s="7"/>
-      <c r="N46" s="32" t="s">
-        <v>192</v>
-      </c>
-      <c r="O46" s="32"/>
-      <c r="P46" s="32"/>
-      <c r="Q46" s="32"/>
-      <c r="R46" s="32"/>
-      <c r="S46" s="32"/>
-      <c r="T46" s="32"/>
-      <c r="U46" s="32"/>
-      <c r="V46" s="32"/>
+      <c r="N46" s="7"/>
+      <c r="O46" s="7"/>
+      <c r="P46" s="7"/>
+      <c r="Q46" s="7"/>
+      <c r="R46" s="7"/>
+      <c r="S46" s="7"/>
+      <c r="T46" s="7"/>
+      <c r="U46" s="7"/>
+      <c r="V46" s="7"/>
       <c r="W46" s="29" t="s">
         <v>187</v>
       </c>
@@ -12448,24 +12420,22 @@
       <c r="BC46" s="7"/>
       <c r="BD46" s="7"/>
       <c r="BE46" s="7"/>
-      <c r="BF46" s="32" t="s">
-        <v>192</v>
-      </c>
-      <c r="BG46" s="32"/>
-      <c r="BH46" s="32"/>
-      <c r="BI46" s="32"/>
-      <c r="BJ46" s="32"/>
-      <c r="BK46" s="32"/>
-      <c r="BL46" s="32"/>
-      <c r="BM46" s="32"/>
-      <c r="BN46" s="32"/>
+      <c r="BF46" s="7"/>
+      <c r="BG46" s="7"/>
+      <c r="BH46" s="7"/>
+      <c r="BI46" s="7"/>
+      <c r="BJ46" s="7"/>
+      <c r="BK46" s="7"/>
+      <c r="BL46" s="7"/>
+      <c r="BM46" s="7"/>
+      <c r="BN46" s="7"/>
       <c r="BO46" s="29" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="BP46" s="29"/>
       <c r="BQ46" s="29"/>
       <c r="BR46" s="29" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="BS46" s="29"/>
       <c r="BT46" s="29"/>
@@ -12499,15 +12469,15 @@
       <c r="K47" s="7"/>
       <c r="L47" s="7"/>
       <c r="M47" s="7"/>
-      <c r="N47" s="32"/>
-      <c r="O47" s="32"/>
-      <c r="P47" s="32"/>
-      <c r="Q47" s="32"/>
-      <c r="R47" s="32"/>
-      <c r="S47" s="32"/>
-      <c r="T47" s="32"/>
-      <c r="U47" s="32"/>
-      <c r="V47" s="32"/>
+      <c r="N47" s="7"/>
+      <c r="O47" s="7"/>
+      <c r="P47" s="7"/>
+      <c r="Q47" s="7"/>
+      <c r="R47" s="7"/>
+      <c r="S47" s="7"/>
+      <c r="T47" s="7"/>
+      <c r="U47" s="7"/>
+      <c r="V47" s="7"/>
       <c r="W47" s="29"/>
       <c r="X47" s="29"/>
       <c r="Y47" s="29"/>
@@ -12542,15 +12512,15 @@
       <c r="BC47" s="7"/>
       <c r="BD47" s="7"/>
       <c r="BE47" s="7"/>
-      <c r="BF47" s="32"/>
-      <c r="BG47" s="32"/>
-      <c r="BH47" s="32"/>
-      <c r="BI47" s="32"/>
-      <c r="BJ47" s="32"/>
-      <c r="BK47" s="32"/>
-      <c r="BL47" s="32"/>
-      <c r="BM47" s="32"/>
-      <c r="BN47" s="32"/>
+      <c r="BF47" s="7"/>
+      <c r="BG47" s="7"/>
+      <c r="BH47" s="7"/>
+      <c r="BI47" s="7"/>
+      <c r="BJ47" s="7"/>
+      <c r="BK47" s="7"/>
+      <c r="BL47" s="7"/>
+      <c r="BM47" s="7"/>
+      <c r="BN47" s="7"/>
       <c r="BO47" s="29"/>
       <c r="BP47" s="29"/>
       <c r="BQ47" s="29"/>
@@ -12574,49 +12544,45 @@
       <c r="CI47" s="6"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="26"/>
-      <c r="B48" s="26"/>
-      <c r="C48" s="26"/>
-      <c r="D48" s="26"/>
-      <c r="E48" s="26"/>
-      <c r="F48" s="26"/>
-      <c r="G48" s="27"/>
-      <c r="H48" s="27"/>
-      <c r="I48" s="27"/>
-      <c r="J48" s="27"/>
-      <c r="K48" s="27"/>
-      <c r="L48" s="27"/>
-      <c r="M48" s="27"/>
-      <c r="N48" s="27"/>
-      <c r="O48" s="27"/>
-      <c r="P48" s="27"/>
-      <c r="Q48" s="27"/>
-      <c r="R48" s="27"/>
-      <c r="S48" s="27"/>
-      <c r="T48" s="27"/>
-      <c r="U48" s="27"/>
-      <c r="V48" s="27"/>
-      <c r="W48" s="27"/>
-      <c r="X48" s="27"/>
-      <c r="Y48" s="27"/>
-      <c r="Z48" s="27"/>
-      <c r="AA48" s="27"/>
-      <c r="AB48" s="27"/>
-      <c r="AC48" s="27"/>
-      <c r="AD48" s="27"/>
-      <c r="AE48" s="27"/>
-      <c r="AF48" s="27"/>
-      <c r="AG48" s="27"/>
-      <c r="AH48" s="27"/>
-      <c r="AI48" s="27"/>
-      <c r="AJ48" s="27"/>
-      <c r="AK48" s="27"/>
-      <c r="AL48" s="27"/>
-      <c r="AM48" s="27"/>
-      <c r="AN48" s="27"/>
-      <c r="AO48" s="27"/>
-      <c r="AP48" s="27"/>
-      <c r="AQ48" s="28"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="2"/>
+      <c r="G48" s="2"/>
+      <c r="H48" s="2"/>
+      <c r="I48" s="2"/>
+      <c r="J48" s="2"/>
+      <c r="K48" s="2"/>
+      <c r="L48" s="2"/>
+      <c r="M48" s="2"/>
+      <c r="N48" s="2"/>
+      <c r="O48" s="2"/>
+      <c r="P48" s="2"/>
+      <c r="Q48" s="2"/>
+      <c r="R48" s="2"/>
+      <c r="S48" s="2"/>
+      <c r="T48" s="2"/>
+      <c r="U48" s="2"/>
+      <c r="V48" s="2"/>
+      <c r="W48" s="2"/>
+      <c r="X48" s="2"/>
+      <c r="Y48" s="2"/>
+      <c r="Z48" s="2"/>
+      <c r="AA48" s="2"/>
+      <c r="AB48" s="2"/>
+      <c r="AC48" s="2"/>
+      <c r="AD48" s="2"/>
+      <c r="AE48" s="2"/>
+      <c r="AF48" s="2"/>
+      <c r="AG48" s="2"/>
+      <c r="AH48" s="2"/>
+      <c r="AI48" s="2"/>
+      <c r="AJ48" s="2"/>
+      <c r="AK48" s="2"/>
+      <c r="AL48" s="2"/>
+      <c r="AM48" s="2"/>
+      <c r="AN48" s="2"/>
+      <c r="AO48" s="2"/>
+      <c r="AP48" s="2"/>
+      <c r="AQ48" s="2"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3"/>
@@ -14965,7 +14931,7 @@
       <c r="BP10" s="13"/>
       <c r="BQ10" s="13"/>
       <c r="BR10" s="13" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="BS10" s="13"/>
       <c r="BT10" s="13"/>
@@ -15059,7 +15025,7 @@
       <c r="AK11" s="6"/>
       <c r="AL11" s="6"/>
       <c r="AM11" s="6" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="AN11" s="6"/>
       <c r="AO11" s="6"/>
@@ -15728,7 +15694,7 @@
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>109</v>
@@ -15934,7 +15900,7 @@
       <c r="AK19" s="13"/>
       <c r="AL19" s="13"/>
       <c r="AM19" s="6" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="AN19" s="6"/>
       <c r="AO19" s="6"/>
@@ -15989,7 +15955,7 @@
       <c r="CC19" s="7"/>
       <c r="CD19" s="7"/>
       <c r="CE19" s="6" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="CF19" s="6"/>
       <c r="CG19" s="6"/>
@@ -16770,7 +16736,7 @@
       <c r="AK27" s="13"/>
       <c r="AL27" s="13"/>
       <c r="AM27" s="6" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="AN27" s="6"/>
       <c r="AO27" s="6"/>
@@ -16823,7 +16789,7 @@
       <c r="CC27" s="7"/>
       <c r="CD27" s="7"/>
       <c r="CE27" s="6" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="CF27" s="6"/>
       <c r="CG27" s="6"/>
@@ -17595,7 +17561,7 @@
       <c r="AK35" s="13"/>
       <c r="AL35" s="13"/>
       <c r="AM35" s="6" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="AN35" s="6"/>
       <c r="AO35" s="6"/>
@@ -17652,7 +17618,7 @@
       <c r="CC35" s="7"/>
       <c r="CD35" s="7"/>
       <c r="CE35" s="6" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="CF35" s="6"/>
       <c r="CG35" s="6"/>
@@ -19206,7 +19172,7 @@
       <c r="AP1" s="4"/>
       <c r="AQ1" s="5"/>
       <c r="AT1" s="3" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="AU1" s="4"/>
       <c r="AV1" s="4"/>
@@ -19489,7 +19455,7 @@
         <v>161</v>
       </c>
       <c r="AT4" s="7" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="AU4" s="7"/>
       <c r="AV4" s="7"/>
@@ -19497,7 +19463,7 @@
       <c r="AX4" s="8"/>
       <c r="AY4" s="6"/>
       <c r="AZ4" s="6" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="BA4" s="8" t="s">
         <v>56</v>
@@ -19586,8 +19552,8 @@
       <c r="AO5" s="6"/>
       <c r="AP5" s="6"/>
       <c r="AQ5" s="6"/>
-      <c r="AR5" s="35" t="s">
-        <v>206</v>
+      <c r="AR5" s="34" t="s">
+        <v>204</v>
       </c>
       <c r="AT5" s="7"/>
       <c r="AU5" s="7"/>
@@ -19596,7 +19562,7 @@
       <c r="AX5" s="7"/>
       <c r="AY5" s="7"/>
       <c r="AZ5" s="6" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="BA5" s="7" t="s">
         <v>172</v>
@@ -19656,10 +19622,10 @@
       <c r="V6" s="7"/>
       <c r="W6" s="7"/>
       <c r="X6" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="Y6" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="Z6" s="7"/>
       <c r="AA6" s="7"/>
@@ -19702,7 +19668,7 @@
       <c r="AW6" s="7"/>
       <c r="AX6" s="7"/>
       <c r="AY6" s="7" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="AZ6" s="7"/>
       <c r="BA6" s="7"/>
@@ -19711,7 +19677,7 @@
       <c r="BD6" s="6"/>
       <c r="BE6" s="11"/>
       <c r="BF6" s="6" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="BG6" s="11"/>
       <c r="BH6" s="11"/>
@@ -19776,7 +19742,7 @@
         <v>172</v>
       </c>
       <c r="BF7" s="6" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="BG7" s="6" t="s">
         <v>173</v>
@@ -19830,7 +19796,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -20393,8 +20359,8 @@
       <c r="AO13" s="6"/>
       <c r="AP13" s="6"/>
       <c r="AQ13" s="6"/>
-      <c r="AR13" s="35" t="s">
-        <v>206</v>
+      <c r="AR13" s="34" t="s">
+        <v>204</v>
       </c>
       <c r="AT13" s="7"/>
       <c r="AU13" s="7"/>
@@ -20507,10 +20473,10 @@
       </c>
       <c r="W14" s="7"/>
       <c r="X14" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="Y14" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="Z14" s="7"/>
       <c r="AA14" s="7"/>
@@ -20789,7 +20755,7 @@
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>109</v>
@@ -21260,8 +21226,8 @@
       <c r="AO21" s="6"/>
       <c r="AP21" s="6"/>
       <c r="AQ21" s="6"/>
-      <c r="AR21" s="35" t="s">
-        <v>206</v>
+      <c r="AR21" s="34" t="s">
+        <v>204</v>
       </c>
       <c r="AT21" s="7"/>
       <c r="AU21" s="7"/>
@@ -21370,10 +21336,10 @@
       </c>
       <c r="W22" s="7"/>
       <c r="X22" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="Y22" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="Z22" s="7"/>
       <c r="AA22" s="7"/>
@@ -22086,8 +22052,8 @@
       <c r="AO29" s="6"/>
       <c r="AP29" s="6"/>
       <c r="AQ29" s="6"/>
-      <c r="AR29" s="35" t="s">
-        <v>206</v>
+      <c r="AR29" s="34" t="s">
+        <v>204</v>
       </c>
       <c r="AT29" s="7"/>
       <c r="AU29" s="7"/>
@@ -22184,10 +22150,10 @@
       </c>
       <c r="W30" s="7"/>
       <c r="X30" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="Y30" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="Z30" s="7"/>
       <c r="AA30" s="7"/>
@@ -22254,7 +22220,7 @@
       </c>
       <c r="BP30" s="7"/>
       <c r="BQ30" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="BR30" s="7"/>
       <c r="BS30" s="7"/>
@@ -22759,7 +22725,7 @@
       <c r="AR36" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="AT36" s="36" t="s">
+      <c r="AT36" s="35" t="s">
         <v>34</v>
       </c>
       <c r="AU36" s="13" t="s">
@@ -22865,8 +22831,8 @@
       <c r="AO37" s="6"/>
       <c r="AP37" s="6"/>
       <c r="AQ37" s="6"/>
-      <c r="AR37" s="35" t="s">
-        <v>206</v>
+      <c r="AR37" s="34" t="s">
+        <v>204</v>
       </c>
       <c r="AT37" s="7" t="s">
         <v>35</v>
@@ -22949,10 +22915,10 @@
       </c>
       <c r="W38" s="7"/>
       <c r="X38" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="Y38" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="Z38" s="7"/>
       <c r="AA38" s="7"/>
@@ -22987,17 +22953,17 @@
       <c r="AW38" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="AX38" s="36" t="s">
+      <c r="AX38" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="AY38" s="36" t="s">
+      <c r="AY38" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="AZ38" s="36"/>
-      <c r="BA38" s="36" t="s">
+      <c r="AZ38" s="35"/>
+      <c r="BA38" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="BB38" s="36" t="s">
+      <c r="BB38" s="35" t="s">
         <v>107</v>
       </c>
       <c r="BC38" s="11"/>
@@ -23060,9 +23026,9 @@
       <c r="AW39" s="7"/>
       <c r="AX39" s="7"/>
       <c r="AY39" s="7"/>
-      <c r="AZ39" s="36"/>
-      <c r="BA39" s="36"/>
-      <c r="BB39" s="36"/>
+      <c r="AZ39" s="35"/>
+      <c r="BA39" s="35"/>
+      <c r="BB39" s="35"/>
       <c r="BC39" s="11"/>
       <c r="BD39" s="6"/>
       <c r="BE39" s="6"/>
@@ -24307,8 +24273,8 @@
       </c>
       <c r="N5" s="6"/>
       <c r="O5" s="6"/>
-      <c r="P5" s="35" t="s">
-        <v>206</v>
+      <c r="P5" s="34" t="s">
+        <v>204</v>
       </c>
       <c r="R5" s="7"/>
       <c r="S5" s="7"/>
@@ -24439,7 +24405,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -24594,7 +24560,7 @@
       <c r="Z11" s="13"/>
       <c r="AA11" s="13"/>
       <c r="AB11" s="13"/>
-      <c r="AC11" s="37"/>
+      <c r="AC11" s="36"/>
       <c r="AD11" s="21"/>
       <c r="AE11" s="6"/>
       <c r="AF11" s="6"/>
@@ -24702,8 +24668,8 @@
       </c>
       <c r="N13" s="6"/>
       <c r="O13" s="6"/>
-      <c r="P13" s="35" t="s">
-        <v>206</v>
+      <c r="P13" s="34" t="s">
+        <v>204</v>
       </c>
       <c r="R13" s="7"/>
       <c r="S13" s="13"/>
@@ -24911,8 +24877,8 @@
       <c r="M19" s="13"/>
       <c r="N19" s="6"/>
       <c r="O19" s="6"/>
-      <c r="P19" s="38" t="s">
-        <v>212</v>
+      <c r="P19" s="37" t="s">
+        <v>210</v>
       </c>
       <c r="R19" s="7"/>
       <c r="S19" s="7"/>
@@ -24931,7 +24897,7 @@
       <c r="AF19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="36"/>
+      <c r="A20" s="35"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
@@ -25014,11 +24980,11 @@
       <c r="S22" s="7"/>
       <c r="T22" s="7"/>
       <c r="U22" s="7"/>
-      <c r="V22" s="36"/>
+      <c r="V22" s="35"/>
       <c r="W22" s="7"/>
       <c r="X22" s="7"/>
-      <c r="Y22" s="39"/>
-      <c r="Z22" s="39"/>
+      <c r="Y22" s="38"/>
+      <c r="Z22" s="38"/>
       <c r="AA22" s="11"/>
       <c r="AB22" s="6"/>
       <c r="AC22" s="11"/>
@@ -25046,11 +25012,11 @@
       <c r="S23" s="7"/>
       <c r="T23" s="7"/>
       <c r="U23" s="7"/>
-      <c r="V23" s="36"/>
-      <c r="W23" s="36"/>
+      <c r="V23" s="35"/>
+      <c r="W23" s="35"/>
       <c r="X23" s="7"/>
-      <c r="Y23" s="39"/>
-      <c r="Z23" s="39"/>
+      <c r="Y23" s="38"/>
+      <c r="Z23" s="38"/>
       <c r="AA23" s="11"/>
       <c r="AB23" s="6"/>
       <c r="AC23" s="6"/>
@@ -25187,7 +25153,7 @@
       <c r="M28" s="13"/>
       <c r="N28" s="6"/>
       <c r="O28" s="6"/>
-      <c r="R28" s="36"/>
+      <c r="R28" s="35"/>
       <c r="S28" s="7"/>
       <c r="T28" s="7"/>
       <c r="U28" s="7"/>
@@ -25241,8 +25207,8 @@
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
       <c r="E30" s="7"/>
-      <c r="F30" s="36"/>
-      <c r="G30" s="36"/>
+      <c r="F30" s="35"/>
+      <c r="G30" s="35"/>
       <c r="H30" s="7"/>
       <c r="I30" s="7"/>
       <c r="J30" s="11"/>
@@ -25255,9 +25221,9 @@
       <c r="S30" s="7"/>
       <c r="T30" s="7"/>
       <c r="U30" s="7"/>
-      <c r="V30" s="36"/>
-      <c r="W30" s="36"/>
-      <c r="X30" s="36"/>
+      <c r="V30" s="35"/>
+      <c r="W30" s="35"/>
+      <c r="X30" s="35"/>
       <c r="Y30" s="6"/>
       <c r="Z30" s="7"/>
       <c r="AA30" s="11"/>
@@ -25274,7 +25240,7 @@
       <c r="D31" s="7"/>
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
-      <c r="G31" s="36"/>
+      <c r="G31" s="35"/>
       <c r="H31" s="7"/>
       <c r="I31" s="7"/>
       <c r="J31" s="11"/>
@@ -25289,7 +25255,7 @@
       <c r="U31" s="7"/>
       <c r="V31" s="7"/>
       <c r="W31" s="7"/>
-      <c r="X31" s="36"/>
+      <c r="X31" s="35"/>
       <c r="Y31" s="6"/>
       <c r="Z31" s="7"/>
       <c r="AA31" s="11"/>
@@ -25352,7 +25318,7 @@
       <c r="A34" s="7"/>
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
-      <c r="D34" s="34"/>
+      <c r="D34" s="33"/>
       <c r="E34" s="6"/>
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
@@ -25428,7 +25394,7 @@
       <c r="M36" s="13"/>
       <c r="N36" s="6"/>
       <c r="O36" s="6"/>
-      <c r="R36" s="36"/>
+      <c r="R36" s="35"/>
       <c r="S36" s="13"/>
       <c r="T36" s="13"/>
       <c r="U36" s="13"/>
@@ -25467,7 +25433,7 @@
       <c r="V37" s="13"/>
       <c r="W37" s="13"/>
       <c r="X37" s="18"/>
-      <c r="Y37" s="40"/>
+      <c r="Y37" s="39"/>
       <c r="Z37" s="6"/>
       <c r="AA37" s="6"/>
       <c r="AB37" s="6"/>
@@ -25482,8 +25448,8 @@
       <c r="C38" s="7"/>
       <c r="D38" s="7"/>
       <c r="E38" s="7"/>
-      <c r="F38" s="36"/>
-      <c r="G38" s="36"/>
+      <c r="F38" s="35"/>
+      <c r="G38" s="35"/>
       <c r="H38" s="7"/>
       <c r="I38" s="7"/>
       <c r="J38" s="11"/>
@@ -25496,11 +25462,11 @@
       <c r="S38" s="7"/>
       <c r="T38" s="7"/>
       <c r="U38" s="7"/>
-      <c r="V38" s="36"/>
-      <c r="W38" s="36"/>
-      <c r="X38" s="36"/>
-      <c r="Y38" s="36"/>
-      <c r="Z38" s="36"/>
+      <c r="V38" s="35"/>
+      <c r="W38" s="35"/>
+      <c r="X38" s="35"/>
+      <c r="Y38" s="35"/>
+      <c r="Z38" s="35"/>
       <c r="AA38" s="11"/>
       <c r="AB38" s="6"/>
       <c r="AC38" s="11"/>
@@ -25515,7 +25481,7 @@
       <c r="D39" s="7"/>
       <c r="E39" s="7"/>
       <c r="F39" s="7"/>
-      <c r="G39" s="36"/>
+      <c r="G39" s="35"/>
       <c r="H39" s="7"/>
       <c r="I39" s="7"/>
       <c r="J39" s="11"/>
@@ -25530,9 +25496,9 @@
       <c r="U39" s="7"/>
       <c r="V39" s="7"/>
       <c r="W39" s="7"/>
-      <c r="X39" s="36"/>
-      <c r="Y39" s="36"/>
-      <c r="Z39" s="36"/>
+      <c r="X39" s="35"/>
+      <c r="Y39" s="35"/>
+      <c r="Z39" s="35"/>
       <c r="AA39" s="11"/>
       <c r="AB39" s="6"/>
       <c r="AC39" s="6"/>
@@ -25653,7 +25619,7 @@
       <c r="AF43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="36"/>
+      <c r="A44" s="35"/>
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
       <c r="D44" s="7"/>
@@ -25668,7 +25634,7 @@
       <c r="M44" s="6"/>
       <c r="N44" s="6"/>
       <c r="O44" s="6"/>
-      <c r="R44" s="36"/>
+      <c r="R44" s="35"/>
       <c r="S44" s="13"/>
       <c r="T44" s="13"/>
       <c r="U44" s="13"/>
@@ -25722,8 +25688,8 @@
       <c r="C46" s="7"/>
       <c r="D46" s="7"/>
       <c r="E46" s="7"/>
-      <c r="F46" s="36"/>
-      <c r="G46" s="36"/>
+      <c r="F46" s="35"/>
+      <c r="G46" s="35"/>
       <c r="H46" s="6"/>
       <c r="I46" s="7"/>
       <c r="J46" s="11"/>
@@ -25736,11 +25702,11 @@
       <c r="S46" s="7"/>
       <c r="T46" s="7"/>
       <c r="U46" s="7"/>
-      <c r="V46" s="36"/>
-      <c r="W46" s="36"/>
-      <c r="X46" s="36"/>
-      <c r="Y46" s="36"/>
-      <c r="Z46" s="36"/>
+      <c r="V46" s="35"/>
+      <c r="W46" s="35"/>
+      <c r="X46" s="35"/>
+      <c r="Y46" s="35"/>
+      <c r="Z46" s="35"/>
       <c r="AA46" s="11"/>
       <c r="AB46" s="6"/>
       <c r="AC46" s="11"/>
@@ -25755,7 +25721,7 @@
       <c r="D47" s="7"/>
       <c r="E47" s="7"/>
       <c r="F47" s="7"/>
-      <c r="G47" s="36"/>
+      <c r="G47" s="35"/>
       <c r="H47" s="6"/>
       <c r="I47" s="7"/>
       <c r="J47" s="11"/>
@@ -25770,9 +25736,9 @@
       <c r="U47" s="7"/>
       <c r="V47" s="7"/>
       <c r="W47" s="7"/>
-      <c r="X47" s="36"/>
-      <c r="Y47" s="36"/>
-      <c r="Z47" s="36"/>
+      <c r="X47" s="35"/>
+      <c r="Y47" s="35"/>
+      <c r="Z47" s="35"/>
       <c r="AA47" s="11"/>
       <c r="AB47" s="6"/>
       <c r="AC47" s="6"/>
@@ -25900,7 +25866,7 @@
       <c r="S52" s="7"/>
       <c r="T52" s="7"/>
       <c r="U52" s="7"/>
-      <c r="V52" s="41"/>
+      <c r="V52" s="40"/>
       <c r="W52" s="6"/>
       <c r="X52" s="13"/>
       <c r="Y52" s="14"/>
@@ -25949,11 +25915,11 @@
       <c r="B54" s="7"/>
       <c r="C54" s="7"/>
       <c r="D54" s="7"/>
-      <c r="E54" s="36"/>
+      <c r="E54" s="35"/>
       <c r="F54" s="7"/>
       <c r="G54" s="7"/>
-      <c r="H54" s="39"/>
-      <c r="I54" s="39"/>
+      <c r="H54" s="38"/>
+      <c r="I54" s="38"/>
       <c r="J54" s="11"/>
       <c r="K54" s="6"/>
       <c r="L54" s="11"/>
@@ -25981,11 +25947,11 @@
       <c r="B55" s="7"/>
       <c r="C55" s="7"/>
       <c r="D55" s="7"/>
-      <c r="E55" s="36"/>
-      <c r="F55" s="36"/>
+      <c r="E55" s="35"/>
+      <c r="F55" s="35"/>
       <c r="G55" s="7"/>
-      <c r="H55" s="39"/>
-      <c r="I55" s="39"/>
+      <c r="H55" s="38"/>
+      <c r="I55" s="38"/>
       <c r="J55" s="11"/>
       <c r="K55" s="6"/>
       <c r="L55" s="6"/>

</xml_diff>

<commit_message>
feat: add keymap documentation and m6 asset with updated script references
</commit_message>
<xml_diff>
--- a/img/keymap.xlsx
+++ b/img/keymap.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="7"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="roman_table" sheetId="1" state="visible" r:id="rId3"/>
@@ -4746,11 +4746,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="32898233"/>
-        <c:axId val="25760029"/>
+        <c:axId val="81620111"/>
+        <c:axId val="26171528"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="32898233"/>
+        <c:axId val="81620111"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4817,13 +4817,13 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25760029"/>
+        <c:crossAx val="26171528"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="1"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="25760029"/>
+        <c:axId val="26171528"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="30"/>
@@ -4900,7 +4900,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="32898233"/>
+        <c:crossAx val="81620111"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -4938,9 +4938,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>57240</xdr:colOff>
+      <xdr:colOff>56880</xdr:colOff>
       <xdr:row>28</xdr:row>
-      <xdr:rowOff>50760</xdr:rowOff>
+      <xdr:rowOff>50400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -4949,7 +4949,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="1662120" y="478080"/>
-        <a:ext cx="7336080" cy="4124520"/>
+        <a:ext cx="7335720" cy="4124160"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -21630,7 +21630,7 @@
       <c r="CW44" s="47"/>
       <c r="CX44" s="47"/>
       <c r="CY44" s="47" t="s">
-        <v>463</v>
+        <v>495</v>
       </c>
       <c r="CZ44" s="47"/>
       <c r="DA44" s="47"/>
@@ -21782,23 +21782,21 @@
       <c r="CL45" s="40"/>
       <c r="CM45" s="40"/>
       <c r="CN45" s="47" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="CO45" s="47"/>
       <c r="CP45" s="47"/>
       <c r="CQ45" s="47" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="CR45" s="47"/>
       <c r="CS45" s="47"/>
       <c r="CT45" s="47" t="s">
-        <v>497</v>
+        <v>463</v>
       </c>
       <c r="CU45" s="47"/>
       <c r="CV45" s="47"/>
-      <c r="CW45" s="77" t="s">
-        <v>463</v>
-      </c>
+      <c r="CW45" s="77"/>
       <c r="CX45" s="77"/>
       <c r="CY45" s="77"/>
       <c r="CZ45" s="47" t="s">
@@ -21951,9 +21949,11 @@
       <c r="CL46" s="42"/>
       <c r="CM46" s="42"/>
       <c r="CN46" s="42"/>
-      <c r="CO46" s="34"/>
-      <c r="CP46" s="34"/>
-      <c r="CQ46" s="34"/>
+      <c r="CO46" s="47" t="s">
+        <v>501</v>
+      </c>
+      <c r="CP46" s="47"/>
+      <c r="CQ46" s="47"/>
       <c r="CR46" s="47" t="s">
         <v>467</v>
       </c>
@@ -48609,15 +48609,15 @@
       <c r="K15" s="62"/>
       <c r="L15" s="62"/>
       <c r="M15" s="62"/>
-      <c r="N15" s="0"/>
-      <c r="O15" s="0"/>
-      <c r="P15" s="0"/>
-      <c r="Q15" s="0"/>
-      <c r="R15" s="0"/>
-      <c r="S15" s="0"/>
-      <c r="T15" s="0"/>
-      <c r="U15" s="0"/>
-      <c r="V15" s="0"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+      <c r="P15" s="1"/>
+      <c r="Q15" s="1"/>
+      <c r="R15" s="1"/>
+      <c r="S15" s="1"/>
+      <c r="T15" s="1"/>
+      <c r="U15" s="1"/>
+      <c r="V15" s="1"/>
       <c r="W15" s="62"/>
       <c r="X15" s="62"/>
       <c r="Y15" s="62"/>
@@ -48794,15 +48794,15 @@
       <c r="K16" s="62"/>
       <c r="L16" s="62"/>
       <c r="M16" s="62"/>
-      <c r="N16" s="0"/>
-      <c r="O16" s="0"/>
-      <c r="P16" s="0"/>
-      <c r="Q16" s="0"/>
-      <c r="R16" s="0"/>
-      <c r="S16" s="0"/>
-      <c r="T16" s="0"/>
-      <c r="U16" s="0"/>
-      <c r="V16" s="0"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="1"/>
+      <c r="R16" s="1"/>
+      <c r="S16" s="1"/>
+      <c r="T16" s="1"/>
+      <c r="U16" s="1"/>
+      <c r="V16" s="1"/>
       <c r="W16" s="62"/>
       <c r="X16" s="62"/>
       <c r="Y16" s="62"/>

</xml_diff>